<commit_message>
Add results and executed notebooks from the model 1.5.0 run
Full pipeline (45/45) on the merged base. All movement vs model 1.4.0 is
the NTD entity, as intended: averted NTD DALYs x0.72 (nigeria, india) and
x0.77 (ethiopia 45ppm) under the power-law elasticity; anemia, LBWSG, and
maternal-disorders averted DALYs are identical to the DALY, confirming the
variance-space SD correction is inert under the fixed-shift effect model.

External validity: the Ethiopia 45ppm NTD-affected-pregnancy reduction is
now 58.4% (was 76.4%), just below the Tessema-trial-anchored expectation
of ~61-63% at the scenario's realized dose with coverage mixing -- the old
setting overshot the trial by ~14pp, the new one undershoots by ~3pp.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JpDueU6WT9Sj1m2BsoASHM
</commit_message>
<xml_diff>
--- a/5000_analyze_results/results_spreadsheet.xlsx
+++ b/5000_analyze_results/results_spreadsheet.xlsx
@@ -920,7 +920,7 @@
         <v>362.8529849538489</v>
       </c>
       <c r="G5" s="3">
-        <v>22.21240835871268</v>
+        <v>15.87131876495009</v>
       </c>
       <c r="H5" s="4">
         <f>IF(F5=0,0,G5/F5)</f>
@@ -960,7 +960,7 @@
         <v>4684.597214204819</v>
       </c>
       <c r="T5" s="3">
-        <v>286.7723034750288</v>
+        <v>204.9059502197524</v>
       </c>
       <c r="U5" s="4">
         <f>IF(S5=0,0,T5/S5)</f>
@@ -1017,7 +1017,7 @@
         <v>320.5427437766894</v>
       </c>
       <c r="G6" s="3">
-        <v>15.97156975435937</v>
+        <v>11.4178093054627</v>
       </c>
       <c r="H6" s="4">
         <f>IF(F6=0,0,G6/F6)</f>
@@ -1057,7 +1057,7 @@
         <v>4138.352740079671</v>
       </c>
       <c r="T6" s="3">
-        <v>206.200236129423</v>
+        <v>147.4091157648745</v>
       </c>
       <c r="U6" s="4">
         <f>IF(S6=0,0,T6/S6)</f>
@@ -1114,7 +1114,7 @@
         <v>287.7720482472399</v>
       </c>
       <c r="G7" s="3">
-        <v>13.40039457662957</v>
+        <v>9.581140009551017</v>
       </c>
       <c r="H7" s="4">
         <f>IF(F7=0,0,G7/F7)</f>
@@ -1154,7 +1154,7 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T7" s="3">
-        <v>173.0051941309189</v>
+        <v>123.6968790634523</v>
       </c>
       <c r="U7" s="4">
         <f>IF(S7=0,0,T7/S7)</f>
@@ -1211,7 +1211,7 @@
         <v>271.3548595424364</v>
       </c>
       <c r="G8" s="3">
-        <v>11.70526956314346</v>
+        <v>8.370468320719199</v>
       </c>
       <c r="H8" s="4">
         <f>IF(F8=0,0,G8/F8)</f>
@@ -1251,7 +1251,7 @@
         <v>3503.314763237015</v>
       </c>
       <c r="T8" s="3">
-        <v>151.1203585495996</v>
+        <v>108.0665564369497</v>
       </c>
       <c r="U8" s="4">
         <f>IF(S8=0,0,T8/S8)</f>
@@ -1308,7 +1308,7 @@
         <v>231.1015430943892</v>
       </c>
       <c r="G9" s="3">
-        <v>4.177694050613908</v>
+        <v>2.991144416980329</v>
       </c>
       <c r="H9" s="4">
         <f>IF(F9=0,0,G9/F9)</f>
@@ -1348,7 +1348,7 @@
         <v>2983.6261237209</v>
       </c>
       <c r="T9" s="3">
-        <v>53.93593196923712</v>
+        <v>38.61703605622006</v>
       </c>
       <c r="U9" s="4">
         <f>IF(S9=0,0,T9/S9)</f>
@@ -1528,7 +1528,7 @@
         <v>362.8529849538489</v>
       </c>
       <c r="G14" s="3">
-        <v>208.4237176868842</v>
+        <v>151.0014963206652</v>
       </c>
       <c r="H14" s="4">
         <f>IF(F14=0,0,G14/F14)</f>
@@ -1568,7 +1568,7 @@
         <v>4684.597214204819</v>
       </c>
       <c r="T14" s="3">
-        <v>2690.845074278154</v>
+        <v>1949.498056615184</v>
       </c>
       <c r="U14" s="4">
         <f>IF(S14=0,0,T14/S14)</f>
@@ -1625,7 +1625,7 @@
         <v>320.5427437766894</v>
       </c>
       <c r="G15" s="3">
-        <v>168.1301289690394</v>
+        <v>121.1169850777707</v>
       </c>
       <c r="H15" s="4">
         <f>IF(F15=0,0,G15/F15)</f>
@@ -1665,7 +1665,7 @@
         <v>4138.352740079671</v>
       </c>
       <c r="T15" s="3">
-        <v>2170.636501426152</v>
+        <v>1563.675412399809</v>
       </c>
       <c r="U15" s="4">
         <f>IF(S15=0,0,T15/S15)</f>
@@ -1722,7 +1722,7 @@
         <v>287.7720482472399</v>
       </c>
       <c r="G16" s="3">
-        <v>152.6827367323572</v>
+        <v>110.0570853730647</v>
       </c>
       <c r="H16" s="4">
         <f>IF(F16=0,0,G16/F16)</f>
@@ -1762,7 +1762,7 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T16" s="3">
-        <v>1971.203635666774</v>
+        <v>1420.887072508819</v>
       </c>
       <c r="U16" s="4">
         <f>IF(S16=0,0,T16/S16)</f>
@@ -1819,7 +1819,7 @@
         <v>271.3548595424364</v>
       </c>
       <c r="G17" s="3">
-        <v>142.3193796941794</v>
+        <v>102.5231161409741</v>
       </c>
       <c r="H17" s="4">
         <f>IF(F17=0,0,G17/F17)</f>
@@ -1859,7 +1859,7 @@
         <v>3503.314763237015</v>
       </c>
       <c r="T17" s="3">
-        <v>1837.407978681804</v>
+        <v>1323.620100098366</v>
       </c>
       <c r="U17" s="4">
         <f>IF(S17=0,0,T17/S17)</f>
@@ -1916,7 +1916,7 @@
         <v>231.1015430943892</v>
       </c>
       <c r="G18" s="3">
-        <v>93.97803135922382</v>
+        <v>67.11521448847459</v>
       </c>
       <c r="H18" s="4">
         <f>IF(F18=0,0,G18/F18)</f>
@@ -1956,7 +1956,7 @@
         <v>2983.6261237209</v>
       </c>
       <c r="T18" s="3">
-        <v>1213.299165660351</v>
+        <v>866.487971329369</v>
       </c>
       <c r="U18" s="4">
         <f>IF(S18=0,0,T18/S18)</f>
@@ -2136,7 +2136,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G23" s="3">
-        <v>213.4118382061803</v>
+        <v>153.5338348629944</v>
       </c>
       <c r="H23" s="4">
         <f>IF(F23=0,0,G23/F23)</f>
@@ -2146,7 +2146,7 @@
         <v>1024.476057384201</v>
       </c>
       <c r="J23" s="3">
-        <v>88.45305872836965</v>
+        <v>88.45306222013221</v>
       </c>
       <c r="K23" s="4">
         <f>IF(I23=0,0,J23/I23)</f>
@@ -2176,7 +2176,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T23" s="3">
-        <v>6584.73744802172</v>
+        <v>4737.225453182307</v>
       </c>
       <c r="U23" s="4">
         <f>IF(S23=0,0,T23/S23)</f>
@@ -2186,7 +2186,7 @@
         <v>25177467.03377928</v>
       </c>
       <c r="W23" s="3">
-        <v>1717880.25111318</v>
+        <v>1717881.090067629</v>
       </c>
       <c r="X23" s="4">
         <f>IF(V23=0,0,W23/V23)</f>
@@ -2233,7 +2233,7 @@
         <v>422.0532339939541</v>
       </c>
       <c r="G24" s="3">
-        <v>208.3471500632799</v>
+        <v>149.5731184765907</v>
       </c>
       <c r="H24" s="4">
         <f>IF(F24=0,0,G24/F24)</f>
@@ -2243,7 +2243,7 @@
         <v>968.8874507802924</v>
       </c>
       <c r="J24" s="3">
-        <v>89.17516949223425</v>
+        <v>89.17520191574422</v>
       </c>
       <c r="K24" s="4">
         <f>IF(I24=0,0,J24/I24)</f>
@@ -2273,7 +2273,7 @@
         <v>13022.28479122008</v>
       </c>
       <c r="T24" s="3">
-        <v>6428.468508316091</v>
+        <v>4615.01912325346</v>
       </c>
       <c r="U24" s="4">
         <f>IF(S24=0,0,T24/S24)</f>
@@ -2283,7 +2283,7 @@
         <v>24716781.60947407</v>
       </c>
       <c r="W24" s="3">
-        <v>1817087.458511882</v>
+        <v>1817089.165172193</v>
       </c>
       <c r="X24" s="4">
         <f>IF(V24=0,0,W24/V24)</f>
@@ -2330,7 +2330,7 @@
         <v>382.0743136549376</v>
       </c>
       <c r="G25" s="3">
-        <v>157.1453841591108</v>
+        <v>112.1956276633881</v>
       </c>
       <c r="H25" s="4">
         <f>IF(F25=0,0,G25/F25)</f>
@@ -2340,7 +2340,7 @@
         <v>792.6568327877751</v>
       </c>
       <c r="J25" s="3">
-        <v>82.16157690995256</v>
+        <v>82.16165372872993</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
@@ -2370,7 +2370,7 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T25" s="3">
-        <v>4848.658371315645</v>
+        <v>3461.751499772323</v>
       </c>
       <c r="U25" s="4">
         <f>IF(S25=0,0,T25/S25)</f>
@@ -2380,7 +2380,7 @@
         <v>22756394.15398703</v>
       </c>
       <c r="W25" s="3">
-        <v>1928602.185540609</v>
+        <v>1928604.090877723</v>
       </c>
       <c r="X25" s="4">
         <f>IF(V25=0,0,W25/V25)</f>
@@ -2427,7 +2427,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G26" s="3">
-        <v>121.0430906924064</v>
+        <v>86.23155739396391</v>
       </c>
       <c r="H26" s="4">
         <f>IF(F26=0,0,G26/F26)</f>
@@ -2437,7 +2437,7 @@
         <v>714.5868735320346</v>
       </c>
       <c r="J26" s="3">
-        <v>76.42899579097144</v>
+        <v>76.42915899969695</v>
       </c>
       <c r="K26" s="4">
         <f>IF(I26=0,0,J26/I26)</f>
@@ -2467,7 +2467,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T26" s="3">
-        <v>3734.736455137735</v>
+        <v>2660.640430943183</v>
       </c>
       <c r="U26" s="4">
         <f>IF(S26=0,0,T26/S26)</f>
@@ -2477,7 +2477,7 @@
         <v>21413420.36871202</v>
       </c>
       <c r="W26" s="3">
-        <v>1904396.2780747</v>
+        <v>1904396.797904398</v>
       </c>
       <c r="X26" s="4">
         <f>IF(V26=0,0,W26/V26)</f>
@@ -2524,7 +2524,7 @@
         <v>297.4602934996698</v>
       </c>
       <c r="G27" s="3">
-        <v>99.54060524581827</v>
+        <v>70.86872059774323</v>
       </c>
       <c r="H27" s="4">
         <f>IF(F27=0,0,G27/F27)</f>
@@ -2564,7 +2564,7 @@
         <v>9178.019131321482</v>
       </c>
       <c r="T27" s="3">
-        <v>3071.285812775053</v>
+        <v>2186.626207504518</v>
       </c>
       <c r="U27" s="4">
         <f>IF(S27=0,0,T27/S27)</f>
@@ -2744,7 +2744,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G32" s="3">
-        <v>44.60952190125041</v>
+        <v>31.81246083158365</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
@@ -2754,7 +2754,7 @@
         <v>1024.476057384201</v>
       </c>
       <c r="J32" s="3">
-        <v>32.68367144466716</v>
+        <v>32.68368291760166</v>
       </c>
       <c r="K32" s="4">
         <f>IF(I32=0,0,J32/I32)</f>
@@ -2784,7 +2784,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T32" s="3">
-        <v>1376.409068355992</v>
+        <v>981.560835201064</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
@@ -2794,7 +2794,7 @@
         <v>25177467.03377928</v>
       </c>
       <c r="W32" s="3">
-        <v>626040.2107638977</v>
+        <v>626042.9301561825</v>
       </c>
       <c r="X32" s="4">
         <f>IF(V32=0,0,W32/V32)</f>
@@ -2841,7 +2841,7 @@
         <v>422.0532339939541</v>
       </c>
       <c r="G33" s="3">
-        <v>82.11660802380734</v>
+        <v>58.43364202621579</v>
       </c>
       <c r="H33" s="4">
         <f>IF(F33=0,0,G33/F33)</f>
@@ -2851,7 +2851,7 @@
         <v>968.8874507802924</v>
       </c>
       <c r="J33" s="3">
-        <v>42.90435799123114</v>
+        <v>42.90436372769834</v>
       </c>
       <c r="K33" s="4">
         <f>IF(I33=0,0,J33/I33)</f>
@@ -2881,7 +2881,7 @@
         <v>13022.28479122008</v>
       </c>
       <c r="T33" s="3">
-        <v>2533.675303600032</v>
+        <v>1802.94680046093</v>
       </c>
       <c r="U33" s="4">
         <f>IF(S33=0,0,T33/S33)</f>
@@ -2891,7 +2891,7 @@
         <v>24716781.60947407</v>
       </c>
       <c r="W33" s="3">
-        <v>861730.5522282757</v>
+        <v>861731.9117797464</v>
       </c>
       <c r="X33" s="4">
         <f>IF(V33=0,0,W33/V33)</f>
@@ -2938,7 +2938,7 @@
         <v>382.0743136549376</v>
       </c>
       <c r="G34" s="3">
-        <v>98.872168911535</v>
+        <v>70.32625266599533</v>
       </c>
       <c r="H34" s="4">
         <f>IF(F34=0,0,G34/F34)</f>
@@ -2948,7 +2948,7 @@
         <v>792.6568327877751</v>
       </c>
       <c r="J34" s="3">
-        <v>47.95443374507281</v>
+        <v>47.95450258267846</v>
       </c>
       <c r="K34" s="4">
         <f>IF(I34=0,0,J34/I34)</f>
@@ -2978,7 +2978,7 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T34" s="3">
-        <v>3050.661475348556</v>
+        <v>2169.888575072522</v>
       </c>
       <c r="U34" s="4">
         <f>IF(S34=0,0,T34/S34)</f>
@@ -3035,7 +3035,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G35" s="3">
-        <v>111.0000684404046</v>
+        <v>79.01499632789695</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
@@ -3075,7 +3075,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T35" s="3">
-        <v>3424.862995118233</v>
+        <v>2437.97630744804</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
@@ -3132,7 +3132,7 @@
         <v>297.4602934996698</v>
       </c>
       <c r="G36" s="3">
-        <v>106.0000459180257</v>
+        <v>75.51235895096086</v>
       </c>
       <c r="H36" s="4">
         <f>IF(F36=0,0,G36/F36)</f>
@@ -3172,7 +3172,7 @@
         <v>9178.019131321482</v>
       </c>
       <c r="T36" s="3">
-        <v>3270.58928743266</v>
+        <v>2329.903823294328</v>
       </c>
       <c r="U36" s="4">
         <f>IF(S36=0,0,T36/S36)</f>
@@ -3345,14 +3345,14 @@
         <v>0</v>
       </c>
       <c r="E41" s="3">
-        <f>M41+P41</f>
+        <f>P41+M41</f>
         <v>0</v>
       </c>
       <c r="F41" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G41" s="3">
-        <v>81.86999988549339</v>
+        <v>58.98240259960004</v>
       </c>
       <c r="H41" s="4">
         <f>IF(F41=0,0,G41/F41)</f>
@@ -3392,7 +3392,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T41" s="3">
-        <v>1158.665071812607</v>
+        <v>834.748379618052</v>
       </c>
       <c r="U41" s="4">
         <f>IF(S41=0,0,T41/S41)</f>
@@ -3442,14 +3442,14 @@
         <v>0</v>
       </c>
       <c r="E42" s="3">
-        <f>M42+P42</f>
+        <f>P42+M42</f>
         <v>0</v>
       </c>
       <c r="F42" s="3">
         <v>147.7607036391234</v>
       </c>
       <c r="G42" s="3">
-        <v>82.20269740785589</v>
+        <v>59.41247823140031</v>
       </c>
       <c r="H42" s="4">
         <f>IF(F42=0,0,G42/F42)</f>
@@ -3489,7 +3489,7 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T42" s="3">
-        <v>1163.373573085103</v>
+        <v>840.835024463559</v>
       </c>
       <c r="U42" s="4">
         <f>IF(S42=0,0,T42/S42)</f>
@@ -3539,14 +3539,14 @@
         <v>0</v>
       </c>
       <c r="E43" s="3">
-        <f>M43+P43</f>
+        <f>P43+M43</f>
         <v>0</v>
       </c>
       <c r="F43" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G43" s="3">
-        <v>81.3780121199603</v>
+        <v>59.19812501773825</v>
       </c>
       <c r="H43" s="4">
         <f>IF(F43=0,0,G43/F43)</f>
@@ -3586,7 +3586,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T43" s="3">
-        <v>1151.702215571254</v>
+        <v>837.8013908731305</v>
       </c>
       <c r="U43" s="4">
         <f>IF(S43=0,0,T43/S43)</f>
@@ -3636,14 +3636,14 @@
         <v>0</v>
       </c>
       <c r="E44" s="3">
-        <f>M44+P44</f>
+        <f>P44+M44</f>
         <v>0</v>
       </c>
       <c r="F44" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G44" s="3">
-        <v>39.16266033894262</v>
+        <v>27.88815467106953</v>
       </c>
       <c r="H44" s="4">
         <f>IF(F44=0,0,G44/F44)</f>
@@ -3683,7 +3683,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T44" s="3">
-        <v>554.2495018622074</v>
+        <v>394.6870743846359</v>
       </c>
       <c r="U44" s="4">
         <f>IF(S44=0,0,T44/S44)</f>
@@ -3733,14 +3733,14 @@
         <v>0</v>
       </c>
       <c r="E45" s="3">
-        <f>M45+P45</f>
+        <f>P45+M45</f>
         <v>0</v>
       </c>
       <c r="F45" s="3">
         <v>93.49564395607489</v>
       </c>
       <c r="G45" s="3">
-        <v>22.85792253853465</v>
+        <v>16.262542548974</v>
       </c>
       <c r="H45" s="4">
         <f>IF(F45=0,0,G45/F45)</f>
@@ -3780,7 +3780,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T45" s="3">
-        <v>323.4967203693753</v>
+        <v>230.1556132492594</v>
       </c>
       <c r="U45" s="4">
         <f>IF(S45=0,0,T45/S45)</f>
@@ -3953,14 +3953,14 @@
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>M50+P50</f>
+        <f>P50+M50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G50" s="3">
-        <v>133.9952818442369</v>
+        <v>105.1172530897168</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
@@ -4000,7 +4000,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T50" s="3">
-        <v>1896.36806006779</v>
+        <v>1487.671793945145</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
@@ -4050,14 +4050,14 @@
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>M51+P51</f>
+        <f>P51+M51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
         <v>147.7607036391234</v>
       </c>
       <c r="G51" s="3">
-        <v>129.7820746858701</v>
+        <v>102.7420072452102</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
@@ -4097,7 +4097,7 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T51" s="3">
-        <v>1836.740650985853</v>
+        <v>1454.056130077464</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
@@ -4147,14 +4147,14 @@
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>M52+P52</f>
+        <f>P52+M52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G52" s="3">
-        <v>121.2448620347747</v>
+        <v>97.48822698814803</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
@@ -4194,7 +4194,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T52" s="3">
-        <v>1715.917759532378</v>
+        <v>1379.702011507161</v>
       </c>
       <c r="U52" s="4">
         <f>IF(S52=0,0,T52/S52)</f>
@@ -4244,14 +4244,14 @@
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>M53+P53</f>
+        <f>P53+M53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G53" s="3">
-        <v>83.96254109871973</v>
+        <v>62.28901992946243</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
@@ -4291,7 +4291,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T53" s="3">
-        <v>1188.279758736814</v>
+        <v>881.5452772767835</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
@@ -4341,14 +4341,14 @@
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>M54+P54</f>
+        <f>P54+M54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
         <v>93.49564395607489</v>
       </c>
       <c r="G54" s="3">
-        <v>56.21002423112071</v>
+        <v>40.86638015373273</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
@@ -4388,7 +4388,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T54" s="3">
-        <v>795.512298197524</v>
+        <v>578.3613944274123</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>
@@ -4561,14 +4561,14 @@
         <v>0</v>
       </c>
       <c r="E59" s="3">
-        <f>M59+P59</f>
+        <f>P59+M59</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G59" s="3">
-        <v>127.8303805653116</v>
+        <v>98.37588727255856</v>
       </c>
       <c r="H59" s="4">
         <f>IF(F59=0,0,G59/F59)</f>
@@ -4608,7 +4608,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T59" s="3">
-        <v>1809.119302365895</v>
+        <v>1392.264622581062</v>
       </c>
       <c r="U59" s="4">
         <f>IF(S59=0,0,T59/S59)</f>
@@ -4658,14 +4658,14 @@
         <v>0</v>
       </c>
       <c r="E60" s="3">
-        <f>M60+P60</f>
+        <f>P60+M60</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
         <v>147.7607036391234</v>
       </c>
       <c r="G60" s="3">
-        <v>124.3897710242896</v>
+        <v>96.54985248064214</v>
       </c>
       <c r="H60" s="4">
         <f>IF(F60=0,0,G60/F60)</f>
@@ -4705,7 +4705,7 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T60" s="3">
-        <v>1760.426080104955</v>
+        <v>1366.42166745382</v>
       </c>
       <c r="U60" s="4">
         <f>IF(S60=0,0,T60/S60)</f>
@@ -4755,14 +4755,14 @@
         <v>0</v>
       </c>
       <c r="E61" s="3">
-        <f>M61+P61</f>
+        <f>P61+M61</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G61" s="3">
-        <v>117.0373671682523</v>
+        <v>92.2087189913087</v>
       </c>
       <c r="H61" s="4">
         <f>IF(F61=0,0,G61/F61)</f>
@@ -4802,7 +4802,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T61" s="3">
-        <v>1656.371193653684</v>
+        <v>1304.983781131581</v>
       </c>
       <c r="U61" s="4">
         <f>IF(S61=0,0,T61/S61)</f>
@@ -4852,14 +4852,14 @@
         <v>0</v>
       </c>
       <c r="E62" s="3">
-        <f>M62+P62</f>
+        <f>P62+M62</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G62" s="3">
-        <v>76.88625128893909</v>
+        <v>56.33344127694023</v>
       </c>
       <c r="H62" s="4">
         <f>IF(F62=0,0,G62/F62)</f>
@@ -4899,7 +4899,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T62" s="3">
-        <v>1088.132575982645</v>
+        <v>797.2589577853753</v>
       </c>
       <c r="U62" s="4">
         <f>IF(S62=0,0,T62/S62)</f>
@@ -4949,14 +4949,14 @@
         <v>0</v>
       </c>
       <c r="E63" s="3">
-        <f>M63+P63</f>
+        <f>P63+M63</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
         <v>93.49564395607489</v>
       </c>
       <c r="G63" s="3">
-        <v>50.20618165273297</v>
+        <v>36.20808203369917</v>
       </c>
       <c r="H63" s="4">
         <f>IF(F63=0,0,G63/F63)</f>
@@ -4996,7 +4996,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T63" s="3">
-        <v>710.5429235551791</v>
+        <v>512.4348360626602</v>
       </c>
       <c r="U63" s="4">
         <f>IF(S63=0,0,T63/S63)</f>

</xml_diff>

<commit_message>
changes from snakemake run
</commit_message>
<xml_diff>
--- a/5000_analyze_results/results_spreadsheet.xlsx
+++ b/5000_analyze_results/results_spreadsheet.xlsx
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="43">
   <si>
     <t>DALYs Averted by Fortification (1000s)</t>
   </si>
@@ -303,6 +303,12 @@
   </si>
   <si>
     <t>Ethiopia -- Salt-- DFS-IoFA preliminary standard 45 ppm</t>
+  </si>
+  <si>
+    <t>Nigeria -- Salt-- 25% NRV per average intake</t>
+  </si>
+  <si>
+    <t>Nigeria -- Salt-- 100% NRV per average intake</t>
   </si>
 </sst>
 </file>
@@ -683,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD63"/>
+  <dimension ref="A1:AD81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -3341,11 +3347,11 @@
         <v>0</v>
       </c>
       <c r="D41" s="3">
-        <f>J41+G41</f>
+        <f>G41+J41</f>
         <v>0</v>
       </c>
       <c r="E41" s="3">
-        <f>P41+M41</f>
+        <f>M41+P41</f>
         <v>0</v>
       </c>
       <c r="F41" s="3">
@@ -3438,11 +3444,11 @@
         <v>0</v>
       </c>
       <c r="D42" s="3">
-        <f>J42+G42</f>
+        <f>G42+J42</f>
         <v>0</v>
       </c>
       <c r="E42" s="3">
-        <f>P42+M42</f>
+        <f>M42+P42</f>
         <v>0</v>
       </c>
       <c r="F42" s="3">
@@ -3535,11 +3541,11 @@
         <v>0</v>
       </c>
       <c r="D43" s="3">
-        <f>J43+G43</f>
+        <f>G43+J43</f>
         <v>0</v>
       </c>
       <c r="E43" s="3">
-        <f>P43+M43</f>
+        <f>M43+P43</f>
         <v>0</v>
       </c>
       <c r="F43" s="3">
@@ -3632,11 +3638,11 @@
         <v>0</v>
       </c>
       <c r="D44" s="3">
-        <f>J44+G44</f>
+        <f>G44+J44</f>
         <v>0</v>
       </c>
       <c r="E44" s="3">
-        <f>P44+M44</f>
+        <f>M44+P44</f>
         <v>0</v>
       </c>
       <c r="F44" s="3">
@@ -3729,11 +3735,11 @@
         <v>0</v>
       </c>
       <c r="D45" s="3">
-        <f>J45+G45</f>
+        <f>G45+J45</f>
         <v>0</v>
       </c>
       <c r="E45" s="3">
-        <f>P45+M45</f>
+        <f>M45+P45</f>
         <v>0</v>
       </c>
       <c r="F45" s="3">
@@ -3949,11 +3955,11 @@
         <v>0</v>
       </c>
       <c r="D50" s="3">
-        <f>J50+G50</f>
+        <f>G50+J50</f>
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>P50+M50</f>
+        <f>M50+P50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
@@ -4046,11 +4052,11 @@
         <v>0</v>
       </c>
       <c r="D51" s="3">
-        <f>J51+G51</f>
+        <f>G51+J51</f>
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>P51+M51</f>
+        <f>M51+P51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
@@ -4143,11 +4149,11 @@
         <v>0</v>
       </c>
       <c r="D52" s="3">
-        <f>J52+G52</f>
+        <f>G52+J52</f>
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>P52+M52</f>
+        <f>M52+P52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
@@ -4240,11 +4246,11 @@
         <v>0</v>
       </c>
       <c r="D53" s="3">
-        <f>J53+G53</f>
+        <f>G53+J53</f>
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>P53+M53</f>
+        <f>M53+P53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
@@ -4337,11 +4343,11 @@
         <v>0</v>
       </c>
       <c r="D54" s="3">
-        <f>J54+G54</f>
+        <f>G54+J54</f>
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>P54+M54</f>
+        <f>M54+P54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
@@ -4557,11 +4563,11 @@
         <v>0</v>
       </c>
       <c r="D59" s="3">
-        <f>J59+G59</f>
+        <f>G59+J59</f>
         <v>0</v>
       </c>
       <c r="E59" s="3">
-        <f>P59+M59</f>
+        <f>M59+P59</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
@@ -4654,11 +4660,11 @@
         <v>0</v>
       </c>
       <c r="D60" s="3">
-        <f>J60+G60</f>
+        <f>G60+J60</f>
         <v>0</v>
       </c>
       <c r="E60" s="3">
-        <f>P60+M60</f>
+        <f>M60+P60</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
@@ -4751,11 +4757,11 @@
         <v>0</v>
       </c>
       <c r="D61" s="3">
-        <f>J61+G61</f>
+        <f>G61+J61</f>
         <v>0</v>
       </c>
       <c r="E61" s="3">
-        <f>P61+M61</f>
+        <f>M61+P61</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
@@ -4848,11 +4854,11 @@
         <v>0</v>
       </c>
       <c r="D62" s="3">
-        <f>J62+G62</f>
+        <f>G62+J62</f>
         <v>0</v>
       </c>
       <c r="E62" s="3">
-        <f>P62+M62</f>
+        <f>M62+P62</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
@@ -4945,11 +4951,11 @@
         <v>0</v>
       </c>
       <c r="D63" s="3">
-        <f>J63+G63</f>
+        <f>G63+J63</f>
         <v>0</v>
       </c>
       <c r="E63" s="3">
-        <f>P63+M63</f>
+        <f>M63+P63</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
@@ -5030,6 +5036,1222 @@
       </c>
       <c r="AD63" s="4">
         <f>IF(AB63=0,0,AC63/AB63)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:30">
+      <c r="A65" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="66" spans="1:30">
+      <c r="B66" t="s">
+        <v>28</v>
+      </c>
+      <c r="C66" s="3">
+        <f>C68+C69+C70+C71+C72</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="3">
+        <f>D68+D69+D70+D71+D72</f>
+        <v>0</v>
+      </c>
+      <c r="E66" s="3">
+        <f>E68+E69+E70+E71+E72</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="3">
+        <f>F68+F69+F70+F71+F72</f>
+        <v>0</v>
+      </c>
+      <c r="G66" s="3">
+        <f>G68+G69+G70+G71+G72</f>
+        <v>0</v>
+      </c>
+      <c r="H66" s="4">
+        <f>IF(F66=0,0,G66/F66)</f>
+        <v>0</v>
+      </c>
+      <c r="I66" s="3">
+        <f>I68+I69+I70+I71+I72</f>
+        <v>0</v>
+      </c>
+      <c r="J66" s="3">
+        <f>J68+J69+J70+J71+J72</f>
+        <v>0</v>
+      </c>
+      <c r="K66" s="4">
+        <f>IF(I66=0,0,J66/I66)</f>
+        <v>0</v>
+      </c>
+      <c r="L66" s="3">
+        <f>L68+L69+L70+L71+L72</f>
+        <v>0</v>
+      </c>
+      <c r="M66" s="3">
+        <f>M68+M69+M70+M71+M72</f>
+        <v>0</v>
+      </c>
+      <c r="N66" s="4">
+        <f>IF(L66=0,0,M66/L66)</f>
+        <v>0</v>
+      </c>
+      <c r="O66" s="3">
+        <f>O68+O69+O70+O71+O72</f>
+        <v>0</v>
+      </c>
+      <c r="P66" s="3">
+        <f>P68+P69+P70+P71+P72</f>
+        <v>0</v>
+      </c>
+      <c r="Q66" s="4">
+        <f>IF(O66=0,0,P66/O66)</f>
+        <v>0</v>
+      </c>
+      <c r="S66" s="3">
+        <f>S68+S69+S70+S71+S72</f>
+        <v>0</v>
+      </c>
+      <c r="T66" s="3">
+        <f>T68+T69+T70+T71+T72</f>
+        <v>0</v>
+      </c>
+      <c r="U66" s="4">
+        <f>IF(S66=0,0,T66/S66)</f>
+        <v>0</v>
+      </c>
+      <c r="V66" s="3">
+        <f>V68+V69+V70+V71+V72</f>
+        <v>0</v>
+      </c>
+      <c r="W66" s="3">
+        <f>W68+W69+W70+W71+W72</f>
+        <v>0</v>
+      </c>
+      <c r="X66" s="4">
+        <f>IF(V66=0,0,W66/V66)</f>
+        <v>0</v>
+      </c>
+      <c r="Y66" s="3">
+        <f>Y68+Y69+Y70+Y71+Y72</f>
+        <v>0</v>
+      </c>
+      <c r="Z66" s="3">
+        <f>Z68+Z69+Z70+Z71+Z72</f>
+        <v>0</v>
+      </c>
+      <c r="AA66" s="4">
+        <f>IF(Y66=0,0,Z66/Y66)</f>
+        <v>0</v>
+      </c>
+      <c r="AB66" s="3">
+        <f>AB68+AB69+AB70+AB71+AB72</f>
+        <v>0</v>
+      </c>
+      <c r="AC66" s="3">
+        <f>AC68+AC69+AC70+AC71+AC72</f>
+        <v>0</v>
+      </c>
+      <c r="AD66" s="4">
+        <f>IF(AB66=0,0,AC66/AB66)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:30">
+      <c r="A67" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="68" spans="1:30">
+      <c r="B68" t="s">
+        <v>30</v>
+      </c>
+      <c r="C68" s="3">
+        <f>J68+M68+G68+P68</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="3">
+        <f>G68</f>
+        <v>0</v>
+      </c>
+      <c r="E68" s="3">
+        <f>J68+M68+P68</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="3">
+        <v>412.7408750394843</v>
+      </c>
+      <c r="G68" s="3">
+        <v>146.8879599840255</v>
+      </c>
+      <c r="H68" s="4">
+        <f>IF(F68=0,0,G68/F68)</f>
+        <v>0</v>
+      </c>
+      <c r="I68" s="3">
+        <v>0</v>
+      </c>
+      <c r="J68" s="3">
+        <v>0</v>
+      </c>
+      <c r="K68" s="4">
+        <f>IF(I68=0,0,J68/I68)</f>
+        <v>0</v>
+      </c>
+      <c r="L68" s="3">
+        <v>0</v>
+      </c>
+      <c r="M68" s="3">
+        <v>0</v>
+      </c>
+      <c r="N68" s="4">
+        <f>IF(L68=0,0,M68/L68)</f>
+        <v>0</v>
+      </c>
+      <c r="O68" s="3">
+        <v>0</v>
+      </c>
+      <c r="P68" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="4">
+        <f>IF(O68=0,0,P68/O68)</f>
+        <v>0</v>
+      </c>
+      <c r="S68" s="3">
+        <v>12734.95565684622</v>
+      </c>
+      <c r="T68" s="3">
+        <v>4532.169625172734</v>
+      </c>
+      <c r="U68" s="4">
+        <f>IF(S68=0,0,T68/S68)</f>
+        <v>0</v>
+      </c>
+      <c r="V68" s="3">
+        <v>0</v>
+      </c>
+      <c r="W68" s="3">
+        <v>0</v>
+      </c>
+      <c r="X68" s="4">
+        <f>IF(V68=0,0,W68/V68)</f>
+        <v>0</v>
+      </c>
+      <c r="Y68" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z68" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="4">
+        <f>IF(Y68=0,0,Z68/Y68)</f>
+        <v>0</v>
+      </c>
+      <c r="AB68" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC68" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD68" s="4">
+        <f>IF(AB68=0,0,AC68/AB68)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:30">
+      <c r="B69" t="s">
+        <v>31</v>
+      </c>
+      <c r="C69" s="3">
+        <f>J69+M69+G69+P69</f>
+        <v>0</v>
+      </c>
+      <c r="D69" s="3">
+        <f>G69</f>
+        <v>0</v>
+      </c>
+      <c r="E69" s="3">
+        <f>J69+M69+P69</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="3">
+        <v>422.0532339939541</v>
+      </c>
+      <c r="G69" s="3">
+        <v>141.7344183926904</v>
+      </c>
+      <c r="H69" s="4">
+        <f>IF(F69=0,0,G69/F69)</f>
+        <v>0</v>
+      </c>
+      <c r="I69" s="3">
+        <v>0</v>
+      </c>
+      <c r="J69" s="3">
+        <v>0</v>
+      </c>
+      <c r="K69" s="4">
+        <f>IF(I69=0,0,J69/I69)</f>
+        <v>0</v>
+      </c>
+      <c r="L69" s="3">
+        <v>0</v>
+      </c>
+      <c r="M69" s="3">
+        <v>0</v>
+      </c>
+      <c r="N69" s="4">
+        <f>IF(L69=0,0,M69/L69)</f>
+        <v>0</v>
+      </c>
+      <c r="O69" s="3">
+        <v>0</v>
+      </c>
+      <c r="P69" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="4">
+        <f>IF(O69=0,0,P69/O69)</f>
+        <v>0</v>
+      </c>
+      <c r="S69" s="3">
+        <v>13022.28479122008</v>
+      </c>
+      <c r="T69" s="3">
+        <v>4373.159147630166</v>
+      </c>
+      <c r="U69" s="4">
+        <f>IF(S69=0,0,T69/S69)</f>
+        <v>0</v>
+      </c>
+      <c r="V69" s="3">
+        <v>0</v>
+      </c>
+      <c r="W69" s="3">
+        <v>0</v>
+      </c>
+      <c r="X69" s="4">
+        <f>IF(V69=0,0,W69/V69)</f>
+        <v>0</v>
+      </c>
+      <c r="Y69" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="4">
+        <f>IF(Y69=0,0,Z69/Y69)</f>
+        <v>0</v>
+      </c>
+      <c r="AB69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD69" s="4">
+        <f>IF(AB69=0,0,AC69/AB69)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:30">
+      <c r="B70" t="s">
+        <v>32</v>
+      </c>
+      <c r="C70" s="3">
+        <f>J70+M70+G70+P70</f>
+        <v>0</v>
+      </c>
+      <c r="D70" s="3">
+        <f>G70</f>
+        <v>0</v>
+      </c>
+      <c r="E70" s="3">
+        <f>J70+M70+P70</f>
+        <v>0</v>
+      </c>
+      <c r="F70" s="3">
+        <v>382.0743136549376</v>
+      </c>
+      <c r="G70" s="3">
+        <v>124.6559480289836</v>
+      </c>
+      <c r="H70" s="4">
+        <f>IF(F70=0,0,G70/F70)</f>
+        <v>0</v>
+      </c>
+      <c r="I70" s="3">
+        <v>0</v>
+      </c>
+      <c r="J70" s="3">
+        <v>0</v>
+      </c>
+      <c r="K70" s="4">
+        <f>IF(I70=0,0,J70/I70)</f>
+        <v>0</v>
+      </c>
+      <c r="L70" s="3">
+        <v>0</v>
+      </c>
+      <c r="M70" s="3">
+        <v>0</v>
+      </c>
+      <c r="N70" s="4">
+        <f>IF(L70=0,0,M70/L70)</f>
+        <v>0</v>
+      </c>
+      <c r="O70" s="3">
+        <v>0</v>
+      </c>
+      <c r="P70" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="4">
+        <f>IF(O70=0,0,P70/O70)</f>
+        <v>0</v>
+      </c>
+      <c r="S70" s="3">
+        <v>11788.75109364953</v>
+      </c>
+      <c r="T70" s="3">
+        <v>3846.209732339612</v>
+      </c>
+      <c r="U70" s="4">
+        <f>IF(S70=0,0,T70/S70)</f>
+        <v>0</v>
+      </c>
+      <c r="V70" s="3">
+        <v>0</v>
+      </c>
+      <c r="W70" s="3">
+        <v>0</v>
+      </c>
+      <c r="X70" s="4">
+        <f>IF(V70=0,0,W70/V70)</f>
+        <v>0</v>
+      </c>
+      <c r="Y70" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z70" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="4">
+        <f>IF(Y70=0,0,Z70/Y70)</f>
+        <v>0</v>
+      </c>
+      <c r="AB70" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC70" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD70" s="4">
+        <f>IF(AB70=0,0,AC70/AB70)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:30">
+      <c r="B71" t="s">
+        <v>33</v>
+      </c>
+      <c r="C71" s="3">
+        <f>J71+M71+G71+P71</f>
+        <v>0</v>
+      </c>
+      <c r="D71" s="3">
+        <f>G71</f>
+        <v>0</v>
+      </c>
+      <c r="E71" s="3">
+        <f>J71+M71+P71</f>
+        <v>0</v>
+      </c>
+      <c r="F71" s="3">
+        <v>338.6701578384149</v>
+      </c>
+      <c r="G71" s="3">
+        <v>106.5823973125179</v>
+      </c>
+      <c r="H71" s="4">
+        <f>IF(F71=0,0,G71/F71)</f>
+        <v>0</v>
+      </c>
+      <c r="I71" s="3">
+        <v>0</v>
+      </c>
+      <c r="J71" s="3">
+        <v>0</v>
+      </c>
+      <c r="K71" s="4">
+        <f>IF(I71=0,0,J71/I71)</f>
+        <v>0</v>
+      </c>
+      <c r="L71" s="3">
+        <v>0</v>
+      </c>
+      <c r="M71" s="3">
+        <v>0</v>
+      </c>
+      <c r="N71" s="4">
+        <f>IF(L71=0,0,M71/L71)</f>
+        <v>0</v>
+      </c>
+      <c r="O71" s="3">
+        <v>0</v>
+      </c>
+      <c r="P71" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="4">
+        <f>IF(O71=0,0,P71/O71)</f>
+        <v>0</v>
+      </c>
+      <c r="S71" s="3">
+        <v>10449.53311676904</v>
+      </c>
+      <c r="T71" s="3">
+        <v>3288.557508256084</v>
+      </c>
+      <c r="U71" s="4">
+        <f>IF(S71=0,0,T71/S71)</f>
+        <v>0</v>
+      </c>
+      <c r="V71" s="3">
+        <v>0</v>
+      </c>
+      <c r="W71" s="3">
+        <v>0</v>
+      </c>
+      <c r="X71" s="4">
+        <f>IF(V71=0,0,W71/V71)</f>
+        <v>0</v>
+      </c>
+      <c r="Y71" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z71" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA71" s="4">
+        <f>IF(Y71=0,0,Z71/Y71)</f>
+        <v>0</v>
+      </c>
+      <c r="AB71" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC71" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD71" s="4">
+        <f>IF(AB71=0,0,AC71/AB71)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:30">
+      <c r="B72" t="s">
+        <v>34</v>
+      </c>
+      <c r="C72" s="3">
+        <f>J72+M72+G72+P72</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="3">
+        <f>G72</f>
+        <v>0</v>
+      </c>
+      <c r="E72" s="3">
+        <f>J72+M72+P72</f>
+        <v>0</v>
+      </c>
+      <c r="F72" s="3">
+        <v>297.4602934996698</v>
+      </c>
+      <c r="G72" s="3">
+        <v>93.75383596516214</v>
+      </c>
+      <c r="H72" s="4">
+        <f>IF(F72=0,0,G72/F72)</f>
+        <v>0</v>
+      </c>
+      <c r="I72" s="3">
+        <v>0</v>
+      </c>
+      <c r="J72" s="3">
+        <v>0</v>
+      </c>
+      <c r="K72" s="4">
+        <f>IF(I72=0,0,J72/I72)</f>
+        <v>0</v>
+      </c>
+      <c r="L72" s="3">
+        <v>0</v>
+      </c>
+      <c r="M72" s="3">
+        <v>0</v>
+      </c>
+      <c r="N72" s="4">
+        <f>IF(L72=0,0,M72/L72)</f>
+        <v>0</v>
+      </c>
+      <c r="O72" s="3">
+        <v>0</v>
+      </c>
+      <c r="P72" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="4">
+        <f>IF(O72=0,0,P72/O72)</f>
+        <v>0</v>
+      </c>
+      <c r="S72" s="3">
+        <v>9178.019131321482</v>
+      </c>
+      <c r="T72" s="3">
+        <v>2892.73734655274</v>
+      </c>
+      <c r="U72" s="4">
+        <f>IF(S72=0,0,T72/S72)</f>
+        <v>0</v>
+      </c>
+      <c r="V72" s="3">
+        <v>0</v>
+      </c>
+      <c r="W72" s="3">
+        <v>0</v>
+      </c>
+      <c r="X72" s="4">
+        <f>IF(V72=0,0,W72/V72)</f>
+        <v>0</v>
+      </c>
+      <c r="Y72" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="4">
+        <f>IF(Y72=0,0,Z72/Y72)</f>
+        <v>0</v>
+      </c>
+      <c r="AB72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD72" s="4">
+        <f>IF(AB72=0,0,AC72/AB72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:30">
+      <c r="A74" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="75" spans="1:30">
+      <c r="B75" t="s">
+        <v>28</v>
+      </c>
+      <c r="C75" s="3">
+        <f>C77+C78+C79+C80+C81</f>
+        <v>0</v>
+      </c>
+      <c r="D75" s="3">
+        <f>D77+D78+D79+D80+D81</f>
+        <v>0</v>
+      </c>
+      <c r="E75" s="3">
+        <f>E77+E78+E79+E80+E81</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="3">
+        <f>F77+F78+F79+F80+F81</f>
+        <v>0</v>
+      </c>
+      <c r="G75" s="3">
+        <f>G77+G78+G79+G80+G81</f>
+        <v>0</v>
+      </c>
+      <c r="H75" s="4">
+        <f>IF(F75=0,0,G75/F75)</f>
+        <v>0</v>
+      </c>
+      <c r="I75" s="3">
+        <f>I77+I78+I79+I80+I81</f>
+        <v>0</v>
+      </c>
+      <c r="J75" s="3">
+        <f>J77+J78+J79+J80+J81</f>
+        <v>0</v>
+      </c>
+      <c r="K75" s="4">
+        <f>IF(I75=0,0,J75/I75)</f>
+        <v>0</v>
+      </c>
+      <c r="L75" s="3">
+        <f>L77+L78+L79+L80+L81</f>
+        <v>0</v>
+      </c>
+      <c r="M75" s="3">
+        <f>M77+M78+M79+M80+M81</f>
+        <v>0</v>
+      </c>
+      <c r="N75" s="4">
+        <f>IF(L75=0,0,M75/L75)</f>
+        <v>0</v>
+      </c>
+      <c r="O75" s="3">
+        <f>O77+O78+O79+O80+O81</f>
+        <v>0</v>
+      </c>
+      <c r="P75" s="3">
+        <f>P77+P78+P79+P80+P81</f>
+        <v>0</v>
+      </c>
+      <c r="Q75" s="4">
+        <f>IF(O75=0,0,P75/O75)</f>
+        <v>0</v>
+      </c>
+      <c r="S75" s="3">
+        <f>S77+S78+S79+S80+S81</f>
+        <v>0</v>
+      </c>
+      <c r="T75" s="3">
+        <f>T77+T78+T79+T80+T81</f>
+        <v>0</v>
+      </c>
+      <c r="U75" s="4">
+        <f>IF(S75=0,0,T75/S75)</f>
+        <v>0</v>
+      </c>
+      <c r="V75" s="3">
+        <f>V77+V78+V79+V80+V81</f>
+        <v>0</v>
+      </c>
+      <c r="W75" s="3">
+        <f>W77+W78+W79+W80+W81</f>
+        <v>0</v>
+      </c>
+      <c r="X75" s="4">
+        <f>IF(V75=0,0,W75/V75)</f>
+        <v>0</v>
+      </c>
+      <c r="Y75" s="3">
+        <f>Y77+Y78+Y79+Y80+Y81</f>
+        <v>0</v>
+      </c>
+      <c r="Z75" s="3">
+        <f>Z77+Z78+Z79+Z80+Z81</f>
+        <v>0</v>
+      </c>
+      <c r="AA75" s="4">
+        <f>IF(Y75=0,0,Z75/Y75)</f>
+        <v>0</v>
+      </c>
+      <c r="AB75" s="3">
+        <f>AB77+AB78+AB79+AB80+AB81</f>
+        <v>0</v>
+      </c>
+      <c r="AC75" s="3">
+        <f>AC77+AC78+AC79+AC80+AC81</f>
+        <v>0</v>
+      </c>
+      <c r="AD75" s="4">
+        <f>IF(AB75=0,0,AC75/AB75)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:30">
+      <c r="A76" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="77" spans="1:30">
+      <c r="B77" t="s">
+        <v>30</v>
+      </c>
+      <c r="C77" s="3">
+        <f>J77+M77+G77+P77</f>
+        <v>0</v>
+      </c>
+      <c r="D77" s="3">
+        <f>G77</f>
+        <v>0</v>
+      </c>
+      <c r="E77" s="3">
+        <f>J77+M77+P77</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="3">
+        <v>412.7408750394843</v>
+      </c>
+      <c r="G77" s="3">
+        <v>270.6215288307627</v>
+      </c>
+      <c r="H77" s="4">
+        <f>IF(F77=0,0,G77/F77)</f>
+        <v>0</v>
+      </c>
+      <c r="I77" s="3">
+        <v>0</v>
+      </c>
+      <c r="J77" s="3">
+        <v>0</v>
+      </c>
+      <c r="K77" s="4">
+        <f>IF(I77=0,0,J77/I77)</f>
+        <v>0</v>
+      </c>
+      <c r="L77" s="3">
+        <v>0</v>
+      </c>
+      <c r="M77" s="3">
+        <v>0</v>
+      </c>
+      <c r="N77" s="4">
+        <f>IF(L77=0,0,M77/L77)</f>
+        <v>0</v>
+      </c>
+      <c r="O77" s="3">
+        <v>0</v>
+      </c>
+      <c r="P77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="4">
+        <f>IF(O77=0,0,P77/O77)</f>
+        <v>0</v>
+      </c>
+      <c r="S77" s="3">
+        <v>12734.95565684622</v>
+      </c>
+      <c r="T77" s="3">
+        <v>8349.919714440697</v>
+      </c>
+      <c r="U77" s="4">
+        <f>IF(S77=0,0,T77/S77)</f>
+        <v>0</v>
+      </c>
+      <c r="V77" s="3">
+        <v>0</v>
+      </c>
+      <c r="W77" s="3">
+        <v>0</v>
+      </c>
+      <c r="X77" s="4">
+        <f>IF(V77=0,0,W77/V77)</f>
+        <v>0</v>
+      </c>
+      <c r="Y77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="4">
+        <f>IF(Y77=0,0,Z77/Y77)</f>
+        <v>0</v>
+      </c>
+      <c r="AB77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD77" s="4">
+        <f>IF(AB77=0,0,AC77/AB77)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:30">
+      <c r="B78" t="s">
+        <v>31</v>
+      </c>
+      <c r="C78" s="3">
+        <f>J78+M78+G78+P78</f>
+        <v>0</v>
+      </c>
+      <c r="D78" s="3">
+        <f>G78</f>
+        <v>0</v>
+      </c>
+      <c r="E78" s="3">
+        <f>J78+M78+P78</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="3">
+        <v>422.0532339939541</v>
+      </c>
+      <c r="G78" s="3">
+        <v>268.8415075664349</v>
+      </c>
+      <c r="H78" s="4">
+        <f>IF(F78=0,0,G78/F78)</f>
+        <v>0</v>
+      </c>
+      <c r="I78" s="3">
+        <v>0</v>
+      </c>
+      <c r="J78" s="3">
+        <v>0</v>
+      </c>
+      <c r="K78" s="4">
+        <f>IF(I78=0,0,J78/I78)</f>
+        <v>0</v>
+      </c>
+      <c r="L78" s="3">
+        <v>0</v>
+      </c>
+      <c r="M78" s="3">
+        <v>0</v>
+      </c>
+      <c r="N78" s="4">
+        <f>IF(L78=0,0,M78/L78)</f>
+        <v>0</v>
+      </c>
+      <c r="O78" s="3">
+        <v>0</v>
+      </c>
+      <c r="P78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="4">
+        <f>IF(O78=0,0,P78/O78)</f>
+        <v>0</v>
+      </c>
+      <c r="S78" s="3">
+        <v>13022.28479122008</v>
+      </c>
+      <c r="T78" s="3">
+        <v>8294.99786579343</v>
+      </c>
+      <c r="U78" s="4">
+        <f>IF(S78=0,0,T78/S78)</f>
+        <v>0</v>
+      </c>
+      <c r="V78" s="3">
+        <v>0</v>
+      </c>
+      <c r="W78" s="3">
+        <v>0</v>
+      </c>
+      <c r="X78" s="4">
+        <f>IF(V78=0,0,W78/V78)</f>
+        <v>0</v>
+      </c>
+      <c r="Y78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="4">
+        <f>IF(Y78=0,0,Z78/Y78)</f>
+        <v>0</v>
+      </c>
+      <c r="AB78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD78" s="4">
+        <f>IF(AB78=0,0,AC78/AB78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:30">
+      <c r="B79" t="s">
+        <v>32</v>
+      </c>
+      <c r="C79" s="3">
+        <f>J79+M79+G79+P79</f>
+        <v>0</v>
+      </c>
+      <c r="D79" s="3">
+        <f>G79</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="3">
+        <f>J79+M79+P79</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="3">
+        <v>382.0743136549376</v>
+      </c>
+      <c r="G79" s="3">
+        <v>239.83782878063</v>
+      </c>
+      <c r="H79" s="4">
+        <f>IF(F79=0,0,G79/F79)</f>
+        <v>0</v>
+      </c>
+      <c r="I79" s="3">
+        <v>0</v>
+      </c>
+      <c r="J79" s="3">
+        <v>0</v>
+      </c>
+      <c r="K79" s="4">
+        <f>IF(I79=0,0,J79/I79)</f>
+        <v>0</v>
+      </c>
+      <c r="L79" s="3">
+        <v>0</v>
+      </c>
+      <c r="M79" s="3">
+        <v>0</v>
+      </c>
+      <c r="N79" s="4">
+        <f>IF(L79=0,0,M79/L79)</f>
+        <v>0</v>
+      </c>
+      <c r="O79" s="3">
+        <v>0</v>
+      </c>
+      <c r="P79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="4">
+        <f>IF(O79=0,0,P79/O79)</f>
+        <v>0</v>
+      </c>
+      <c r="S79" s="3">
+        <v>11788.75109364953</v>
+      </c>
+      <c r="T79" s="3">
+        <v>7400.100884273723</v>
+      </c>
+      <c r="U79" s="4">
+        <f>IF(S79=0,0,T79/S79)</f>
+        <v>0</v>
+      </c>
+      <c r="V79" s="3">
+        <v>0</v>
+      </c>
+      <c r="W79" s="3">
+        <v>0</v>
+      </c>
+      <c r="X79" s="4">
+        <f>IF(V79=0,0,W79/V79)</f>
+        <v>0</v>
+      </c>
+      <c r="Y79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="4">
+        <f>IF(Y79=0,0,Z79/Y79)</f>
+        <v>0</v>
+      </c>
+      <c r="AB79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD79" s="4">
+        <f>IF(AB79=0,0,AC79/AB79)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:30">
+      <c r="B80" t="s">
+        <v>33</v>
+      </c>
+      <c r="C80" s="3">
+        <f>J80+M80+G80+P80</f>
+        <v>0</v>
+      </c>
+      <c r="D80" s="3">
+        <f>G80</f>
+        <v>0</v>
+      </c>
+      <c r="E80" s="3">
+        <f>J80+M80+P80</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="3">
+        <v>338.6701578384149</v>
+      </c>
+      <c r="G80" s="3">
+        <v>208.6917795068874</v>
+      </c>
+      <c r="H80" s="4">
+        <f>IF(F80=0,0,G80/F80)</f>
+        <v>0</v>
+      </c>
+      <c r="I80" s="3">
+        <v>0</v>
+      </c>
+      <c r="J80" s="3">
+        <v>0</v>
+      </c>
+      <c r="K80" s="4">
+        <f>IF(I80=0,0,J80/I80)</f>
+        <v>0</v>
+      </c>
+      <c r="L80" s="3">
+        <v>0</v>
+      </c>
+      <c r="M80" s="3">
+        <v>0</v>
+      </c>
+      <c r="N80" s="4">
+        <f>IF(L80=0,0,M80/L80)</f>
+        <v>0</v>
+      </c>
+      <c r="O80" s="3">
+        <v>0</v>
+      </c>
+      <c r="P80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="4">
+        <f>IF(O80=0,0,P80/O80)</f>
+        <v>0</v>
+      </c>
+      <c r="S80" s="3">
+        <v>10449.53311676904</v>
+      </c>
+      <c r="T80" s="3">
+        <v>6439.101912826773</v>
+      </c>
+      <c r="U80" s="4">
+        <f>IF(S80=0,0,T80/S80)</f>
+        <v>0</v>
+      </c>
+      <c r="V80" s="3">
+        <v>0</v>
+      </c>
+      <c r="W80" s="3">
+        <v>0</v>
+      </c>
+      <c r="X80" s="4">
+        <f>IF(V80=0,0,W80/V80)</f>
+        <v>0</v>
+      </c>
+      <c r="Y80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="4">
+        <f>IF(Y80=0,0,Z80/Y80)</f>
+        <v>0</v>
+      </c>
+      <c r="AB80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD80" s="4">
+        <f>IF(AB80=0,0,AC80/AB80)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="2:30">
+      <c r="B81" t="s">
+        <v>34</v>
+      </c>
+      <c r="C81" s="3">
+        <f>J81+M81+G81+P81</f>
+        <v>0</v>
+      </c>
+      <c r="D81" s="3">
+        <f>G81</f>
+        <v>0</v>
+      </c>
+      <c r="E81" s="3">
+        <f>J81+M81+P81</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="3">
+        <v>297.4602934996698</v>
+      </c>
+      <c r="G81" s="3">
+        <v>183.4401220978905</v>
+      </c>
+      <c r="H81" s="4">
+        <f>IF(F81=0,0,G81/F81)</f>
+        <v>0</v>
+      </c>
+      <c r="I81" s="3">
+        <v>0</v>
+      </c>
+      <c r="J81" s="3">
+        <v>0</v>
+      </c>
+      <c r="K81" s="4">
+        <f>IF(I81=0,0,J81/I81)</f>
+        <v>0</v>
+      </c>
+      <c r="L81" s="3">
+        <v>0</v>
+      </c>
+      <c r="M81" s="3">
+        <v>0</v>
+      </c>
+      <c r="N81" s="4">
+        <f>IF(L81=0,0,M81/L81)</f>
+        <v>0</v>
+      </c>
+      <c r="O81" s="3">
+        <v>0</v>
+      </c>
+      <c r="P81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q81" s="4">
+        <f>IF(O81=0,0,P81/O81)</f>
+        <v>0</v>
+      </c>
+      <c r="S81" s="3">
+        <v>9178.019131321482</v>
+      </c>
+      <c r="T81" s="3">
+        <v>5659.972059659975</v>
+      </c>
+      <c r="U81" s="4">
+        <f>IF(S81=0,0,T81/S81)</f>
+        <v>0</v>
+      </c>
+      <c r="V81" s="3">
+        <v>0</v>
+      </c>
+      <c r="W81" s="3">
+        <v>0</v>
+      </c>
+      <c r="X81" s="4">
+        <f>IF(V81=0,0,W81/V81)</f>
+        <v>0</v>
+      </c>
+      <c r="Y81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="4">
+        <f>IF(Y81=0,0,Z81/Y81)</f>
+        <v>0</v>
+      </c>
+      <c r="AB81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD81" s="4">
+        <f>IF(AB81=0,0,AC81/AB81)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add results and executed notebooks from the Nigeria wheat iron test run (MIC-7549)
</commit_message>
<xml_diff>
--- a/5000_analyze_results/results_spreadsheet.xlsx
+++ b/5000_analyze_results/results_spreadsheet.xlsx
@@ -19,58 +19,6 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="J39" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Based on correlation between serum folate and hemoglobin</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K39" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Based on correlation between serum folate and hemoglobin</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W39" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Based on correlation between serum folate and hemoglobin</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X39" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Based on correlation between serum folate and hemoglobin</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="J48" authorId="0">
       <text>
         <r>
@@ -175,12 +123,64 @@
         </r>
       </text>
     </comment>
+    <comment ref="J66" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Based on correlation between serum folate and hemoglobin</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K66" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Based on correlation between serum folate and hemoglobin</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W66" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Based on correlation between serum folate and hemoglobin</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X66" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Based on correlation between serum folate and hemoglobin</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="42">
   <si>
     <t>DALYs Averted by Fortification (1000s)</t>
   </si>
@@ -294,6 +294,9 @@
   </si>
   <si>
     <t>Nigeria -- Rice</t>
+  </si>
+  <si>
+    <t>Nigeria -- Wheat</t>
   </si>
   <si>
     <t>Ethiopia -- Salt-- 25% NRV per average intake</t>
@@ -683,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD63"/>
+  <dimension ref="A1:AD72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -930,7 +933,7 @@
         <v>4771.261231090824</v>
       </c>
       <c r="J5" s="3">
-        <v>288.4337566118361</v>
+        <v>288.4337566118371</v>
       </c>
       <c r="K5" s="4">
         <f>IF(I5=0,0,J5/I5)</f>
@@ -1027,7 +1030,7 @@
         <v>4315.21265961095</v>
       </c>
       <c r="J6" s="3">
-        <v>254.1003600447956</v>
+        <v>254.1003600447951</v>
       </c>
       <c r="K6" s="4">
         <f>IF(I6=0,0,J6/I6)</f>
@@ -1121,10 +1124,10 @@
         <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>4220.065012527612</v>
+        <v>4220.06501252761</v>
       </c>
       <c r="J7" s="3">
-        <v>227.9834892376838</v>
+        <v>227.9834892376829</v>
       </c>
       <c r="K7" s="4">
         <f>IF(I7=0,0,J7/I7)</f>
@@ -1221,7 +1224,7 @@
         <v>3866.462901477351</v>
       </c>
       <c r="J8" s="3">
-        <v>196.466800308214</v>
+        <v>196.4668003082145</v>
       </c>
       <c r="K8" s="4">
         <f>IF(I8=0,0,J8/I8)</f>
@@ -1315,10 +1318,10 @@
         <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>3364.297008165505</v>
+        <v>3364.297008165506</v>
       </c>
       <c r="J9" s="3">
-        <v>97.66824302014476</v>
+        <v>97.6682430201457</v>
       </c>
       <c r="K9" s="4">
         <f>IF(I9=0,0,J9/I9)</f>
@@ -1578,7 +1581,7 @@
         <v>131696392.1412486</v>
       </c>
       <c r="W14" s="3">
-        <v>10296243.37165028</v>
+        <v>10296243.37165025</v>
       </c>
       <c r="X14" s="4">
         <f>IF(V14=0,0,W14/V14)</f>
@@ -1635,7 +1638,7 @@
         <v>4315.21265961095</v>
       </c>
       <c r="J15" s="3">
-        <v>433.8825937981489</v>
+        <v>433.8825937981484</v>
       </c>
       <c r="K15" s="4">
         <f>IF(I15=0,0,J15/I15)</f>
@@ -1729,10 +1732,10 @@
         <v>0</v>
       </c>
       <c r="I16" s="3">
-        <v>4220.065012527612</v>
+        <v>4220.06501252761</v>
       </c>
       <c r="J16" s="3">
-        <v>424.9209438963709</v>
+        <v>424.92094389637</v>
       </c>
       <c r="K16" s="4">
         <f>IF(I16=0,0,J16/I16)</f>
@@ -1923,10 +1926,10 @@
         <v>0</v>
       </c>
       <c r="I18" s="3">
-        <v>3364.297008165505</v>
+        <v>3364.297008165506</v>
       </c>
       <c r="J18" s="3">
-        <v>311.568357023593</v>
+        <v>311.5683570235935</v>
       </c>
       <c r="K18" s="4">
         <f>IF(I18=0,0,J18/I18)</f>
@@ -2340,7 +2343,7 @@
         <v>792.6568327877751</v>
       </c>
       <c r="J25" s="3">
-        <v>82.16165372872993</v>
+        <v>82.16165372872982</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
@@ -3045,7 +3048,7 @@
         <v>714.5868735320346</v>
       </c>
       <c r="J35" s="3">
-        <v>51.68573642029148</v>
+        <v>51.68573642029136</v>
       </c>
       <c r="K35" s="4">
         <f>IF(I35=0,0,J35/I35)</f>
@@ -3085,7 +3088,7 @@
         <v>21413420.36871202</v>
       </c>
       <c r="W35" s="3">
-        <v>1269177.296716779</v>
+        <v>1269177.296716776</v>
       </c>
       <c r="X35" s="4">
         <f>IF(V35=0,0,W35/V35)</f>
@@ -3142,7 +3145,7 @@
         <v>607.1996095192959</v>
       </c>
       <c r="J36" s="3">
-        <v>49.91319984393485</v>
+        <v>49.91319984393473</v>
       </c>
       <c r="K36" s="4">
         <f>IF(I36=0,0,J36/I36)</f>
@@ -3246,11 +3249,11 @@
         <f>I41+I42+I43+I44+I45</f>
         <v>0</v>
       </c>
-      <c r="J39" s="6">
+      <c r="J39" s="3">
         <f>J41+J42+J43+J44+J45</f>
         <v>0</v>
       </c>
-      <c r="K39" s="7">
+      <c r="K39" s="4">
         <f>IF(I39=0,0,J39/I39)</f>
         <v>0</v>
       </c>
@@ -3294,11 +3297,11 @@
         <f>V41+V42+V43+V44+V45</f>
         <v>0</v>
       </c>
-      <c r="W39" s="6">
+      <c r="W39" s="3">
         <f>W41+W42+W43+W44+W45</f>
         <v>0</v>
       </c>
-      <c r="X39" s="7">
+      <c r="X39" s="4">
         <f>IF(V39=0,0,W39/V39)</f>
         <v>0</v>
       </c>
@@ -3341,88 +3344,88 @@
         <v>0</v>
       </c>
       <c r="D41" s="3">
-        <f>J41+G41</f>
+        <f>G41</f>
         <v>0</v>
       </c>
       <c r="E41" s="3">
-        <f>P41+M41</f>
+        <f>J41+M41+P41</f>
         <v>0</v>
       </c>
       <c r="F41" s="3">
-        <v>155.3366697637048</v>
+        <v>0</v>
       </c>
       <c r="G41" s="3">
-        <v>58.98240259960004</v>
+        <v>0</v>
       </c>
       <c r="H41" s="4">
         <f>IF(F41=0,0,G41/F41)</f>
         <v>0</v>
       </c>
       <c r="I41" s="3">
-        <v>382.3073643284127</v>
-      </c>
-      <c r="J41" s="6">
-        <v>8.688572781210882</v>
-      </c>
-      <c r="K41" s="7">
+        <v>1024.476057384201</v>
+      </c>
+      <c r="J41" s="3">
+        <v>32.68368291760166</v>
+      </c>
+      <c r="K41" s="4">
         <f>IF(I41=0,0,J41/I41)</f>
         <v>0</v>
       </c>
       <c r="L41" s="3">
-        <v>0</v>
+        <v>15352.83741703859</v>
       </c>
       <c r="M41" s="3">
-        <v>0</v>
+        <v>3.522455788802355</v>
       </c>
       <c r="N41" s="4">
         <f>IF(L41=0,0,M41/L41)</f>
         <v>0</v>
       </c>
       <c r="O41" s="3">
-        <v>0</v>
+        <v>503.5634310516943</v>
       </c>
       <c r="P41" s="3">
-        <v>0</v>
+        <v>3.068380574589828</v>
       </c>
       <c r="Q41" s="4">
         <f>IF(O41=0,0,P41/O41)</f>
         <v>0</v>
       </c>
       <c r="S41" s="3">
-        <v>2198.402026122217</v>
+        <v>0</v>
       </c>
       <c r="T41" s="3">
-        <v>834.748379618052</v>
+        <v>0</v>
       </c>
       <c r="U41" s="4">
         <f>IF(S41=0,0,T41/S41)</f>
         <v>0</v>
       </c>
       <c r="V41" s="3">
-        <v>9070418.669545408</v>
-      </c>
-      <c r="W41" s="6">
-        <v>206244.2943557166</v>
-      </c>
-      <c r="X41" s="7">
+        <v>25177467.03377928</v>
+      </c>
+      <c r="W41" s="3">
+        <v>626042.9301561825</v>
+      </c>
+      <c r="X41" s="4">
         <f>IF(V41=0,0,W41/V41)</f>
         <v>0</v>
       </c>
       <c r="Y41" s="3">
-        <v>0</v>
+        <v>2561085.175981381</v>
       </c>
       <c r="Z41" s="3">
-        <v>0</v>
+        <v>21648.69212072948</v>
       </c>
       <c r="AA41" s="4">
         <f>IF(Y41=0,0,Z41/Y41)</f>
         <v>0</v>
       </c>
       <c r="AB41" s="3">
-        <v>0</v>
+        <v>172903.801774421</v>
       </c>
       <c r="AC41" s="3">
-        <v>0</v>
+        <v>39.10155138786649</v>
       </c>
       <c r="AD41" s="4">
         <f>IF(AB41=0,0,AC41/AB41)</f>
@@ -3438,88 +3441,88 @@
         <v>0</v>
       </c>
       <c r="D42" s="3">
-        <f>J42+G42</f>
+        <f>G42</f>
         <v>0</v>
       </c>
       <c r="E42" s="3">
-        <f>P42+M42</f>
+        <f>J42+M42+P42</f>
         <v>0</v>
       </c>
       <c r="F42" s="3">
-        <v>147.7607036391234</v>
+        <v>0</v>
       </c>
       <c r="G42" s="3">
-        <v>59.41247823140031</v>
+        <v>0</v>
       </c>
       <c r="H42" s="4">
         <f>IF(F42=0,0,G42/F42)</f>
         <v>0</v>
       </c>
       <c r="I42" s="3">
-        <v>245.090682899663</v>
-      </c>
-      <c r="J42" s="6">
-        <v>7.531359140255663</v>
-      </c>
-      <c r="K42" s="7">
+        <v>968.8874507802924</v>
+      </c>
+      <c r="J42" s="3">
+        <v>42.90436372769834</v>
+      </c>
+      <c r="K42" s="4">
         <f>IF(I42=0,0,J42/I42)</f>
         <v>0</v>
       </c>
       <c r="L42" s="3">
-        <v>0</v>
+        <v>15897.14811387405</v>
       </c>
       <c r="M42" s="3">
-        <v>0</v>
+        <v>4.837213344274089</v>
       </c>
       <c r="N42" s="4">
         <f>IF(L42=0,0,M42/L42)</f>
         <v>0</v>
       </c>
       <c r="O42" s="3">
-        <v>0</v>
+        <v>427.6878840211459</v>
       </c>
       <c r="P42" s="3">
-        <v>0</v>
+        <v>5.825020013755769</v>
       </c>
       <c r="Q42" s="4">
         <f>IF(O42=0,0,P42/O42)</f>
         <v>0</v>
       </c>
       <c r="S42" s="3">
-        <v>2091.183174942721</v>
+        <v>0</v>
       </c>
       <c r="T42" s="3">
-        <v>840.835024463559</v>
+        <v>0</v>
       </c>
       <c r="U42" s="4">
         <f>IF(S42=0,0,T42/S42)</f>
         <v>0</v>
       </c>
       <c r="V42" s="3">
-        <v>7100767.677214347</v>
-      </c>
-      <c r="W42" s="6">
-        <v>238006.6357756918</v>
-      </c>
-      <c r="X42" s="7">
+        <v>24716781.60947407</v>
+      </c>
+      <c r="W42" s="3">
+        <v>861731.9117797464</v>
+      </c>
+      <c r="X42" s="4">
         <f>IF(V42=0,0,W42/V42)</f>
         <v>0</v>
       </c>
       <c r="Y42" s="3">
-        <v>0</v>
+        <v>2216806.226901517</v>
       </c>
       <c r="Z42" s="3">
-        <v>0</v>
+        <v>30569.74919843301</v>
       </c>
       <c r="AA42" s="4">
         <f>IF(Y42=0,0,Z42/Y42)</f>
         <v>0</v>
       </c>
       <c r="AB42" s="3">
-        <v>0</v>
+        <v>179047.6330362356</v>
       </c>
       <c r="AC42" s="3">
-        <v>0</v>
+        <v>53.76463315828005</v>
       </c>
       <c r="AD42" s="4">
         <f>IF(AB42=0,0,AC42/AB42)</f>
@@ -3535,88 +3538,88 @@
         <v>0</v>
       </c>
       <c r="D43" s="3">
-        <f>J43+G43</f>
+        <f>G43</f>
         <v>0</v>
       </c>
       <c r="E43" s="3">
-        <f>P43+M43</f>
+        <f>J43+M43+P43</f>
         <v>0</v>
       </c>
       <c r="F43" s="3">
-        <v>134.4880808162132</v>
+        <v>0</v>
       </c>
       <c r="G43" s="3">
-        <v>59.19812501773825</v>
+        <v>0</v>
       </c>
       <c r="H43" s="4">
         <f>IF(F43=0,0,G43/F43)</f>
         <v>0</v>
       </c>
       <c r="I43" s="3">
-        <v>200.4130880433794</v>
-      </c>
-      <c r="J43" s="6">
-        <v>8.333503383573669</v>
-      </c>
-      <c r="K43" s="7">
+        <v>792.6568327877751</v>
+      </c>
+      <c r="J43" s="3">
+        <v>47.95450258267846</v>
+      </c>
+      <c r="K43" s="4">
         <f>IF(I43=0,0,J43/I43)</f>
         <v>0</v>
       </c>
       <c r="L43" s="3">
-        <v>0</v>
+        <v>14099.36149543928</v>
       </c>
       <c r="M43" s="3">
-        <v>0</v>
+        <v>7.771691316105425</v>
       </c>
       <c r="N43" s="4">
         <f>IF(L43=0,0,M43/L43)</f>
         <v>0</v>
       </c>
       <c r="O43" s="3">
-        <v>0</v>
+        <v>410.8336896551561</v>
       </c>
       <c r="P43" s="3">
-        <v>0</v>
+        <v>6.801244757992798</v>
       </c>
       <c r="Q43" s="4">
         <f>IF(O43=0,0,P43/O43)</f>
         <v>0</v>
       </c>
       <c r="S43" s="3">
-        <v>1903.342396907326</v>
+        <v>0</v>
       </c>
       <c r="T43" s="3">
-        <v>837.8013908731305</v>
+        <v>0</v>
       </c>
       <c r="U43" s="4">
         <f>IF(S43=0,0,T43/S43)</f>
         <v>0</v>
       </c>
       <c r="V43" s="3">
-        <v>6292834.208210533</v>
-      </c>
-      <c r="W43" s="6">
-        <v>279483.1369019002</v>
-      </c>
-      <c r="X43" s="7">
+        <v>22756394.15398703</v>
+      </c>
+      <c r="W43" s="3">
+        <v>1108078.306488663</v>
+      </c>
+      <c r="X43" s="4">
         <f>IF(V43=0,0,W43/V43)</f>
         <v>0</v>
       </c>
       <c r="Y43" s="3">
-        <v>0</v>
+        <v>2114085.557833027</v>
       </c>
       <c r="Z43" s="3">
-        <v>0</v>
+        <v>36469.94504468259</v>
       </c>
       <c r="AA43" s="4">
         <f>IF(Y43=0,0,Z43/Y43)</f>
         <v>0</v>
       </c>
       <c r="AB43" s="3">
-        <v>0</v>
+        <v>158763.7032537926</v>
       </c>
       <c r="AC43" s="3">
-        <v>0</v>
+        <v>86.34925931482576</v>
       </c>
       <c r="AD43" s="4">
         <f>IF(AB43=0,0,AC43/AB43)</f>
@@ -3632,88 +3635,88 @@
         <v>0</v>
       </c>
       <c r="D44" s="3">
-        <f>J44+G44</f>
+        <f>G44</f>
         <v>0</v>
       </c>
       <c r="E44" s="3">
-        <f>P44+M44</f>
+        <f>J44+M44+P44</f>
         <v>0</v>
       </c>
       <c r="F44" s="3">
-        <v>118.5139506930648</v>
+        <v>0</v>
       </c>
       <c r="G44" s="3">
-        <v>27.88815467106953</v>
+        <v>0</v>
       </c>
       <c r="H44" s="4">
         <f>IF(F44=0,0,G44/F44)</f>
         <v>0</v>
       </c>
       <c r="I44" s="3">
-        <v>193.9015574705648</v>
-      </c>
-      <c r="J44" s="6">
-        <v>3.251090114021907</v>
-      </c>
-      <c r="K44" s="7">
+        <v>714.5868735320346</v>
+      </c>
+      <c r="J44" s="3">
+        <v>51.68573642029136</v>
+      </c>
+      <c r="K44" s="4">
         <f>IF(I44=0,0,J44/I44)</f>
         <v>0</v>
       </c>
       <c r="L44" s="3">
-        <v>0</v>
+        <v>12459.036398116</v>
       </c>
       <c r="M44" s="3">
-        <v>0</v>
+        <v>5.284773733304814</v>
       </c>
       <c r="N44" s="4">
         <f>IF(L44=0,0,M44/L44)</f>
         <v>0</v>
       </c>
       <c r="O44" s="3">
-        <v>0</v>
+        <v>388.5202631627004</v>
       </c>
       <c r="P44" s="3">
-        <v>0</v>
+        <v>6.425640266744071</v>
       </c>
       <c r="Q44" s="4">
         <f>IF(O44=0,0,P44/O44)</f>
         <v>0</v>
       </c>
       <c r="S44" s="3">
-        <v>1677.268540156761</v>
+        <v>0</v>
       </c>
       <c r="T44" s="3">
-        <v>394.6870743846359</v>
+        <v>0</v>
       </c>
       <c r="U44" s="4">
         <f>IF(S44=0,0,T44/S44)</f>
         <v>0</v>
       </c>
       <c r="V44" s="3">
-        <v>6053045.584847068</v>
-      </c>
-      <c r="W44" s="6">
-        <v>115470.6967978468</v>
-      </c>
-      <c r="X44" s="7">
+        <v>21413420.36871202</v>
+      </c>
+      <c r="W44" s="3">
+        <v>1269177.296716776</v>
+      </c>
+      <c r="X44" s="4">
         <f>IF(V44=0,0,W44/V44)</f>
         <v>0</v>
       </c>
       <c r="Y44" s="3">
-        <v>0</v>
+        <v>1925897.452986733</v>
       </c>
       <c r="Z44" s="3">
-        <v>0</v>
+        <v>35243.3810336343</v>
       </c>
       <c r="AA44" s="4">
         <f>IF(Y44=0,0,Z44/Y44)</f>
         <v>0</v>
       </c>
       <c r="AB44" s="3">
-        <v>0</v>
+        <v>140314.2879239626</v>
       </c>
       <c r="AC44" s="3">
-        <v>0</v>
+        <v>58.65232708177064</v>
       </c>
       <c r="AD44" s="4">
         <f>IF(AB44=0,0,AC44/AB44)</f>
@@ -3729,88 +3732,88 @@
         <v>0</v>
       </c>
       <c r="D45" s="3">
-        <f>J45+G45</f>
+        <f>G45</f>
         <v>0</v>
       </c>
       <c r="E45" s="3">
-        <f>P45+M45</f>
+        <f>J45+M45+P45</f>
         <v>0</v>
       </c>
       <c r="F45" s="3">
-        <v>93.49564395607489</v>
+        <v>0</v>
       </c>
       <c r="G45" s="3">
-        <v>16.262542548974</v>
+        <v>0</v>
       </c>
       <c r="H45" s="4">
         <f>IF(F45=0,0,G45/F45)</f>
         <v>0</v>
       </c>
       <c r="I45" s="3">
-        <v>136.6145524202559</v>
-      </c>
-      <c r="J45" s="6">
-        <v>2.460393484535132</v>
-      </c>
-      <c r="K45" s="7">
+        <v>607.1996095192959</v>
+      </c>
+      <c r="J45" s="3">
+        <v>49.91319984393473</v>
+      </c>
+      <c r="K45" s="4">
         <f>IF(I45=0,0,J45/I45)</f>
         <v>0</v>
       </c>
       <c r="L45" s="3">
-        <v>0</v>
+        <v>9475.405513778041</v>
       </c>
       <c r="M45" s="3">
-        <v>0</v>
+        <v>8.366401425374672</v>
       </c>
       <c r="N45" s="4">
         <f>IF(L45=0,0,M45/L45)</f>
         <v>0</v>
       </c>
       <c r="O45" s="3">
-        <v>0</v>
+        <v>285.742923347472</v>
       </c>
       <c r="P45" s="3">
-        <v>0</v>
+        <v>6.236481271973287</v>
       </c>
       <c r="Q45" s="4">
         <f>IF(O45=0,0,P45/O45)</f>
         <v>0</v>
       </c>
       <c r="S45" s="3">
-        <v>1323.196985098892</v>
+        <v>0</v>
       </c>
       <c r="T45" s="3">
-        <v>230.1556132492594</v>
+        <v>0</v>
       </c>
       <c r="U45" s="4">
         <f>IF(S45=0,0,T45/S45)</f>
         <v>0</v>
       </c>
       <c r="V45" s="3">
-        <v>4890905.466101354</v>
-      </c>
-      <c r="W45" s="6">
-        <v>96394.34072632995</v>
-      </c>
-      <c r="X45" s="7">
+        <v>19850211.7121278</v>
+      </c>
+      <c r="W45" s="3">
+        <v>1356137.905176748</v>
+      </c>
+      <c r="X45" s="4">
         <f>IF(V45=0,0,W45/V45)</f>
         <v>0</v>
       </c>
       <c r="Y45" s="3">
-        <v>0</v>
+        <v>1405792.016991551</v>
       </c>
       <c r="Z45" s="3">
-        <v>0</v>
+        <v>30795.86643654411</v>
       </c>
       <c r="AA45" s="4">
         <f>IF(Y45=0,0,Z45/Y45)</f>
         <v>0</v>
       </c>
       <c r="AB45" s="3">
-        <v>0</v>
+        <v>106730.9429757299</v>
       </c>
       <c r="AC45" s="3">
-        <v>0</v>
+        <v>92.86618454611744</v>
       </c>
       <c r="AD45" s="4">
         <f>IF(AB45=0,0,AC45/AB45)</f>
@@ -3953,24 +3956,24 @@
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>P50+M50</f>
+        <f>M50+P50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G50" s="3">
-        <v>105.1172530897168</v>
+        <v>58.98240259960004</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
         <v>0</v>
       </c>
       <c r="I50" s="3">
-        <v>382.3073643284127</v>
+        <v>382.3073643284126</v>
       </c>
       <c r="J50" s="6">
-        <v>30.38027252396196</v>
+        <v>8.688572781210823</v>
       </c>
       <c r="K50" s="7">
         <f>IF(I50=0,0,J50/I50)</f>
@@ -4000,7 +4003,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T50" s="3">
-        <v>1487.671793945145</v>
+        <v>834.748379618052</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
@@ -4010,7 +4013,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W50" s="6">
-        <v>763318.428798628</v>
+        <v>206244.2943557147</v>
       </c>
       <c r="X50" s="7">
         <f>IF(V50=0,0,W50/V50)</f>
@@ -4050,14 +4053,14 @@
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>P51+M51</f>
+        <f>M51+P51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
         <v>147.7607036391234</v>
       </c>
       <c r="G51" s="3">
-        <v>102.7420072452102</v>
+        <v>59.41247823140031</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
@@ -4067,7 +4070,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J51" s="6">
-        <v>25.02248949374902</v>
+        <v>7.531359140255693</v>
       </c>
       <c r="K51" s="7">
         <f>IF(I51=0,0,J51/I51)</f>
@@ -4097,17 +4100,17 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T51" s="3">
-        <v>1454.056130077464</v>
+        <v>840.835024463559</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
         <v>0</v>
       </c>
       <c r="V51" s="3">
-        <v>7100767.677214347</v>
+        <v>7100767.677214348</v>
       </c>
       <c r="W51" s="6">
-        <v>836476.8330573235</v>
+        <v>238006.6357756928</v>
       </c>
       <c r="X51" s="7">
         <f>IF(V51=0,0,W51/V51)</f>
@@ -4147,14 +4150,14 @@
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>P52+M52</f>
+        <f>M52+P52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G52" s="3">
-        <v>97.48822698814803</v>
+        <v>59.19812501773825</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
@@ -4164,7 +4167,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J52" s="6">
-        <v>26.68454090976095</v>
+        <v>8.333503383573669</v>
       </c>
       <c r="K52" s="7">
         <f>IF(I52=0,0,J52/I52)</f>
@@ -4194,7 +4197,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T52" s="3">
-        <v>1379.702011507161</v>
+        <v>837.8013908731305</v>
       </c>
       <c r="U52" s="4">
         <f>IF(S52=0,0,T52/S52)</f>
@@ -4204,7 +4207,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W52" s="6">
-        <v>949876.6631412003</v>
+        <v>279483.1369019002</v>
       </c>
       <c r="X52" s="7">
         <f>IF(V52=0,0,W52/V52)</f>
@@ -4244,14 +4247,14 @@
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>P53+M53</f>
+        <f>M53+P53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G53" s="3">
-        <v>62.28901992946243</v>
+        <v>27.88815467106953</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
@@ -4261,7 +4264,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J53" s="6">
-        <v>11.86059618587699</v>
+        <v>3.251090114021907</v>
       </c>
       <c r="K53" s="7">
         <f>IF(I53=0,0,J53/I53)</f>
@@ -4291,7 +4294,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T53" s="3">
-        <v>881.5452772767835</v>
+        <v>394.6870743846359</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
@@ -4301,7 +4304,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W53" s="6">
-        <v>432629.1184659526</v>
+        <v>115470.6967978468</v>
       </c>
       <c r="X53" s="7">
         <f>IF(V53=0,0,W53/V53)</f>
@@ -4341,14 +4344,14 @@
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>P54+M54</f>
+        <f>M54+P54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
         <v>93.49564395607489</v>
       </c>
       <c r="G54" s="3">
-        <v>40.86638015373273</v>
+        <v>16.262542548974</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
@@ -4358,7 +4361,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J54" s="6">
-        <v>9.160355738468628</v>
+        <v>2.460393484535132</v>
       </c>
       <c r="K54" s="7">
         <f>IF(I54=0,0,J54/I54)</f>
@@ -4388,7 +4391,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T54" s="3">
-        <v>578.3613944274123</v>
+        <v>230.1556132492594</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>
@@ -4398,7 +4401,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W54" s="6">
-        <v>365344.9764395468</v>
+        <v>96394.34072632995</v>
       </c>
       <c r="X54" s="7">
         <f>IF(V54=0,0,W54/V54)</f>
@@ -4561,24 +4564,24 @@
         <v>0</v>
       </c>
       <c r="E59" s="3">
-        <f>P59+M59</f>
+        <f>M59+P59</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G59" s="3">
-        <v>98.37588727255856</v>
+        <v>105.1172530897168</v>
       </c>
       <c r="H59" s="4">
         <f>IF(F59=0,0,G59/F59)</f>
         <v>0</v>
       </c>
       <c r="I59" s="3">
-        <v>382.3073643284127</v>
+        <v>382.3073643284126</v>
       </c>
       <c r="J59" s="6">
-        <v>25.16365196989442</v>
+        <v>30.38027252396196</v>
       </c>
       <c r="K59" s="7">
         <f>IF(I59=0,0,J59/I59)</f>
@@ -4608,7 +4611,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T59" s="3">
-        <v>1392.264622581062</v>
+        <v>1487.671793945145</v>
       </c>
       <c r="U59" s="4">
         <f>IF(S59=0,0,T59/S59)</f>
@@ -4618,7 +4621,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W59" s="6">
-        <v>623324.3944149893</v>
+        <v>763318.428798628</v>
       </c>
       <c r="X59" s="7">
         <f>IF(V59=0,0,W59/V59)</f>
@@ -4658,14 +4661,14 @@
         <v>0</v>
       </c>
       <c r="E60" s="3">
-        <f>P60+M60</f>
+        <f>M60+P60</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
         <v>147.7607036391234</v>
       </c>
       <c r="G60" s="3">
-        <v>96.54985248064214</v>
+        <v>102.7420072452102</v>
       </c>
       <c r="H60" s="4">
         <f>IF(F60=0,0,G60/F60)</f>
@@ -4675,7 +4678,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J60" s="6">
-        <v>21.00591395392729</v>
+        <v>25.02248949374902</v>
       </c>
       <c r="K60" s="7">
         <f>IF(I60=0,0,J60/I60)</f>
@@ -4705,17 +4708,17 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T60" s="3">
-        <v>1366.42166745382</v>
+        <v>1454.056130077464</v>
       </c>
       <c r="U60" s="4">
         <f>IF(S60=0,0,T60/S60)</f>
         <v>0</v>
       </c>
       <c r="V60" s="3">
-        <v>7100767.677214347</v>
+        <v>7100767.677214348</v>
       </c>
       <c r="W60" s="6">
-        <v>692794.20388046</v>
+        <v>836476.8330573244</v>
       </c>
       <c r="X60" s="7">
         <f>IF(V60=0,0,W60/V60)</f>
@@ -4755,14 +4758,14 @@
         <v>0</v>
       </c>
       <c r="E61" s="3">
-        <f>P61+M61</f>
+        <f>M61+P61</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G61" s="3">
-        <v>92.2087189913087</v>
+        <v>97.48822698814803</v>
       </c>
       <c r="H61" s="4">
         <f>IF(F61=0,0,G61/F61)</f>
@@ -4772,7 +4775,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J61" s="6">
-        <v>22.61656617855845</v>
+        <v>26.68454090976095</v>
       </c>
       <c r="K61" s="7">
         <f>IF(I61=0,0,J61/I61)</f>
@@ -4802,7 +4805,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T61" s="3">
-        <v>1304.983781131581</v>
+        <v>1379.702011507161</v>
       </c>
       <c r="U61" s="4">
         <f>IF(S61=0,0,T61/S61)</f>
@@ -4812,7 +4815,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W61" s="6">
-        <v>794041.0575617198</v>
+        <v>949876.6631412003</v>
       </c>
       <c r="X61" s="7">
         <f>IF(V61=0,0,W61/V61)</f>
@@ -4852,14 +4855,14 @@
         <v>0</v>
       </c>
       <c r="E62" s="3">
-        <f>P62+M62</f>
+        <f>M62+P62</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G62" s="3">
-        <v>56.33344127694023</v>
+        <v>62.28901992946243</v>
       </c>
       <c r="H62" s="4">
         <f>IF(F62=0,0,G62/F62)</f>
@@ -4869,7 +4872,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J62" s="6">
-        <v>9.710502579285967</v>
+        <v>11.86059618587699</v>
       </c>
       <c r="K62" s="7">
         <f>IF(I62=0,0,J62/I62)</f>
@@ -4899,7 +4902,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T62" s="3">
-        <v>797.2589577853753</v>
+        <v>881.5452772767835</v>
       </c>
       <c r="U62" s="4">
         <f>IF(S62=0,0,T62/S62)</f>
@@ -4909,7 +4912,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W62" s="6">
-        <v>351805.066879469</v>
+        <v>432629.1184659526</v>
       </c>
       <c r="X62" s="7">
         <f>IF(V62=0,0,W62/V62)</f>
@@ -4949,14 +4952,14 @@
         <v>0</v>
       </c>
       <c r="E63" s="3">
-        <f>P63+M63</f>
+        <f>M63+P63</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
         <v>93.49564395607489</v>
       </c>
       <c r="G63" s="3">
-        <v>36.20808203369917</v>
+        <v>40.86638015373273</v>
       </c>
       <c r="H63" s="4">
         <f>IF(F63=0,0,G63/F63)</f>
@@ -4966,7 +4969,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J63" s="6">
-        <v>7.458779051449644</v>
+        <v>9.160355738468613</v>
       </c>
       <c r="K63" s="7">
         <f>IF(I63=0,0,J63/I63)</f>
@@ -4996,7 +4999,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T63" s="3">
-        <v>512.4348360626602</v>
+        <v>578.3613944274123</v>
       </c>
       <c r="U63" s="4">
         <f>IF(S63=0,0,T63/S63)</f>
@@ -5006,7 +5009,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W63" s="6">
-        <v>296120.1093025655</v>
+        <v>365344.9764395468</v>
       </c>
       <c r="X63" s="7">
         <f>IF(V63=0,0,W63/V63)</f>
@@ -5030,6 +5033,614 @@
       </c>
       <c r="AD63" s="4">
         <f>IF(AB63=0,0,AC63/AB63)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:30">
+      <c r="A65" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="66" spans="1:30">
+      <c r="B66" t="s">
+        <v>28</v>
+      </c>
+      <c r="C66" s="3">
+        <f>C68+C69+C70+C71+C72</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="3">
+        <f>D68+D69+D70+D71+D72</f>
+        <v>0</v>
+      </c>
+      <c r="E66" s="3">
+        <f>E68+E69+E70+E71+E72</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="3">
+        <f>F68+F69+F70+F71+F72</f>
+        <v>0</v>
+      </c>
+      <c r="G66" s="3">
+        <f>G68+G69+G70+G71+G72</f>
+        <v>0</v>
+      </c>
+      <c r="H66" s="4">
+        <f>IF(F66=0,0,G66/F66)</f>
+        <v>0</v>
+      </c>
+      <c r="I66" s="3">
+        <f>I68+I69+I70+I71+I72</f>
+        <v>0</v>
+      </c>
+      <c r="J66" s="6">
+        <f>J68+J69+J70+J71+J72</f>
+        <v>0</v>
+      </c>
+      <c r="K66" s="7">
+        <f>IF(I66=0,0,J66/I66)</f>
+        <v>0</v>
+      </c>
+      <c r="L66" s="3">
+        <f>L68+L69+L70+L71+L72</f>
+        <v>0</v>
+      </c>
+      <c r="M66" s="3">
+        <f>M68+M69+M70+M71+M72</f>
+        <v>0</v>
+      </c>
+      <c r="N66" s="4">
+        <f>IF(L66=0,0,M66/L66)</f>
+        <v>0</v>
+      </c>
+      <c r="O66" s="3">
+        <f>O68+O69+O70+O71+O72</f>
+        <v>0</v>
+      </c>
+      <c r="P66" s="3">
+        <f>P68+P69+P70+P71+P72</f>
+        <v>0</v>
+      </c>
+      <c r="Q66" s="4">
+        <f>IF(O66=0,0,P66/O66)</f>
+        <v>0</v>
+      </c>
+      <c r="S66" s="3">
+        <f>S68+S69+S70+S71+S72</f>
+        <v>0</v>
+      </c>
+      <c r="T66" s="3">
+        <f>T68+T69+T70+T71+T72</f>
+        <v>0</v>
+      </c>
+      <c r="U66" s="4">
+        <f>IF(S66=0,0,T66/S66)</f>
+        <v>0</v>
+      </c>
+      <c r="V66" s="3">
+        <f>V68+V69+V70+V71+V72</f>
+        <v>0</v>
+      </c>
+      <c r="W66" s="6">
+        <f>W68+W69+W70+W71+W72</f>
+        <v>0</v>
+      </c>
+      <c r="X66" s="7">
+        <f>IF(V66=0,0,W66/V66)</f>
+        <v>0</v>
+      </c>
+      <c r="Y66" s="3">
+        <f>Y68+Y69+Y70+Y71+Y72</f>
+        <v>0</v>
+      </c>
+      <c r="Z66" s="3">
+        <f>Z68+Z69+Z70+Z71+Z72</f>
+        <v>0</v>
+      </c>
+      <c r="AA66" s="4">
+        <f>IF(Y66=0,0,Z66/Y66)</f>
+        <v>0</v>
+      </c>
+      <c r="AB66" s="3">
+        <f>AB68+AB69+AB70+AB71+AB72</f>
+        <v>0</v>
+      </c>
+      <c r="AC66" s="3">
+        <f>AC68+AC69+AC70+AC71+AC72</f>
+        <v>0</v>
+      </c>
+      <c r="AD66" s="4">
+        <f>IF(AB66=0,0,AC66/AB66)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:30">
+      <c r="A67" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="68" spans="1:30">
+      <c r="B68" t="s">
+        <v>30</v>
+      </c>
+      <c r="C68" s="3">
+        <f>J68+M68+G68+P68</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="3">
+        <f>J68+G68</f>
+        <v>0</v>
+      </c>
+      <c r="E68" s="3">
+        <f>M68+P68</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="3">
+        <v>155.3366697637048</v>
+      </c>
+      <c r="G68" s="3">
+        <v>98.37588727255856</v>
+      </c>
+      <c r="H68" s="4">
+        <f>IF(F68=0,0,G68/F68)</f>
+        <v>0</v>
+      </c>
+      <c r="I68" s="3">
+        <v>382.3073643284126</v>
+      </c>
+      <c r="J68" s="6">
+        <v>25.16365196989442</v>
+      </c>
+      <c r="K68" s="7">
+        <f>IF(I68=0,0,J68/I68)</f>
+        <v>0</v>
+      </c>
+      <c r="L68" s="3">
+        <v>0</v>
+      </c>
+      <c r="M68" s="3">
+        <v>0</v>
+      </c>
+      <c r="N68" s="4">
+        <f>IF(L68=0,0,M68/L68)</f>
+        <v>0</v>
+      </c>
+      <c r="O68" s="3">
+        <v>0</v>
+      </c>
+      <c r="P68" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="4">
+        <f>IF(O68=0,0,P68/O68)</f>
+        <v>0</v>
+      </c>
+      <c r="S68" s="3">
+        <v>2198.402026122217</v>
+      </c>
+      <c r="T68" s="3">
+        <v>1392.264622581062</v>
+      </c>
+      <c r="U68" s="4">
+        <f>IF(S68=0,0,T68/S68)</f>
+        <v>0</v>
+      </c>
+      <c r="V68" s="3">
+        <v>9070418.669545408</v>
+      </c>
+      <c r="W68" s="6">
+        <v>623324.3944149893</v>
+      </c>
+      <c r="X68" s="7">
+        <f>IF(V68=0,0,W68/V68)</f>
+        <v>0</v>
+      </c>
+      <c r="Y68" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z68" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="4">
+        <f>IF(Y68=0,0,Z68/Y68)</f>
+        <v>0</v>
+      </c>
+      <c r="AB68" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC68" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD68" s="4">
+        <f>IF(AB68=0,0,AC68/AB68)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:30">
+      <c r="B69" t="s">
+        <v>31</v>
+      </c>
+      <c r="C69" s="3">
+        <f>J69+M69+G69+P69</f>
+        <v>0</v>
+      </c>
+      <c r="D69" s="3">
+        <f>J69+G69</f>
+        <v>0</v>
+      </c>
+      <c r="E69" s="3">
+        <f>M69+P69</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="3">
+        <v>147.7607036391234</v>
+      </c>
+      <c r="G69" s="3">
+        <v>96.54985248064214</v>
+      </c>
+      <c r="H69" s="4">
+        <f>IF(F69=0,0,G69/F69)</f>
+        <v>0</v>
+      </c>
+      <c r="I69" s="3">
+        <v>245.090682899663</v>
+      </c>
+      <c r="J69" s="6">
+        <v>21.00591395392729</v>
+      </c>
+      <c r="K69" s="7">
+        <f>IF(I69=0,0,J69/I69)</f>
+        <v>0</v>
+      </c>
+      <c r="L69" s="3">
+        <v>0</v>
+      </c>
+      <c r="M69" s="3">
+        <v>0</v>
+      </c>
+      <c r="N69" s="4">
+        <f>IF(L69=0,0,M69/L69)</f>
+        <v>0</v>
+      </c>
+      <c r="O69" s="3">
+        <v>0</v>
+      </c>
+      <c r="P69" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="4">
+        <f>IF(O69=0,0,P69/O69)</f>
+        <v>0</v>
+      </c>
+      <c r="S69" s="3">
+        <v>2091.183174942721</v>
+      </c>
+      <c r="T69" s="3">
+        <v>1366.42166745382</v>
+      </c>
+      <c r="U69" s="4">
+        <f>IF(S69=0,0,T69/S69)</f>
+        <v>0</v>
+      </c>
+      <c r="V69" s="3">
+        <v>7100767.677214348</v>
+      </c>
+      <c r="W69" s="6">
+        <v>692794.2038804609</v>
+      </c>
+      <c r="X69" s="7">
+        <f>IF(V69=0,0,W69/V69)</f>
+        <v>0</v>
+      </c>
+      <c r="Y69" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="4">
+        <f>IF(Y69=0,0,Z69/Y69)</f>
+        <v>0</v>
+      </c>
+      <c r="AB69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD69" s="4">
+        <f>IF(AB69=0,0,AC69/AB69)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:30">
+      <c r="B70" t="s">
+        <v>32</v>
+      </c>
+      <c r="C70" s="3">
+        <f>J70+M70+G70+P70</f>
+        <v>0</v>
+      </c>
+      <c r="D70" s="3">
+        <f>J70+G70</f>
+        <v>0</v>
+      </c>
+      <c r="E70" s="3">
+        <f>M70+P70</f>
+        <v>0</v>
+      </c>
+      <c r="F70" s="3">
+        <v>134.4880808162132</v>
+      </c>
+      <c r="G70" s="3">
+        <v>92.2087189913087</v>
+      </c>
+      <c r="H70" s="4">
+        <f>IF(F70=0,0,G70/F70)</f>
+        <v>0</v>
+      </c>
+      <c r="I70" s="3">
+        <v>200.4130880433794</v>
+      </c>
+      <c r="J70" s="6">
+        <v>22.61656617855842</v>
+      </c>
+      <c r="K70" s="7">
+        <f>IF(I70=0,0,J70/I70)</f>
+        <v>0</v>
+      </c>
+      <c r="L70" s="3">
+        <v>0</v>
+      </c>
+      <c r="M70" s="3">
+        <v>0</v>
+      </c>
+      <c r="N70" s="4">
+        <f>IF(L70=0,0,M70/L70)</f>
+        <v>0</v>
+      </c>
+      <c r="O70" s="3">
+        <v>0</v>
+      </c>
+      <c r="P70" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="4">
+        <f>IF(O70=0,0,P70/O70)</f>
+        <v>0</v>
+      </c>
+      <c r="S70" s="3">
+        <v>1903.342396907326</v>
+      </c>
+      <c r="T70" s="3">
+        <v>1304.983781131581</v>
+      </c>
+      <c r="U70" s="4">
+        <f>IF(S70=0,0,T70/S70)</f>
+        <v>0</v>
+      </c>
+      <c r="V70" s="3">
+        <v>6292834.208210533</v>
+      </c>
+      <c r="W70" s="6">
+        <v>794041.0575617198</v>
+      </c>
+      <c r="X70" s="7">
+        <f>IF(V70=0,0,W70/V70)</f>
+        <v>0</v>
+      </c>
+      <c r="Y70" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z70" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="4">
+        <f>IF(Y70=0,0,Z70/Y70)</f>
+        <v>0</v>
+      </c>
+      <c r="AB70" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC70" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD70" s="4">
+        <f>IF(AB70=0,0,AC70/AB70)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:30">
+      <c r="B71" t="s">
+        <v>33</v>
+      </c>
+      <c r="C71" s="3">
+        <f>J71+M71+G71+P71</f>
+        <v>0</v>
+      </c>
+      <c r="D71" s="3">
+        <f>J71+G71</f>
+        <v>0</v>
+      </c>
+      <c r="E71" s="3">
+        <f>M71+P71</f>
+        <v>0</v>
+      </c>
+      <c r="F71" s="3">
+        <v>118.5139506930648</v>
+      </c>
+      <c r="G71" s="3">
+        <v>56.33344127694023</v>
+      </c>
+      <c r="H71" s="4">
+        <f>IF(F71=0,0,G71/F71)</f>
+        <v>0</v>
+      </c>
+      <c r="I71" s="3">
+        <v>193.9015574705648</v>
+      </c>
+      <c r="J71" s="6">
+        <v>9.710502579285997</v>
+      </c>
+      <c r="K71" s="7">
+        <f>IF(I71=0,0,J71/I71)</f>
+        <v>0</v>
+      </c>
+      <c r="L71" s="3">
+        <v>0</v>
+      </c>
+      <c r="M71" s="3">
+        <v>0</v>
+      </c>
+      <c r="N71" s="4">
+        <f>IF(L71=0,0,M71/L71)</f>
+        <v>0</v>
+      </c>
+      <c r="O71" s="3">
+        <v>0</v>
+      </c>
+      <c r="P71" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="4">
+        <f>IF(O71=0,0,P71/O71)</f>
+        <v>0</v>
+      </c>
+      <c r="S71" s="3">
+        <v>1677.268540156761</v>
+      </c>
+      <c r="T71" s="3">
+        <v>797.2589577853753</v>
+      </c>
+      <c r="U71" s="4">
+        <f>IF(S71=0,0,T71/S71)</f>
+        <v>0</v>
+      </c>
+      <c r="V71" s="3">
+        <v>6053045.584847068</v>
+      </c>
+      <c r="W71" s="6">
+        <v>351805.066879469</v>
+      </c>
+      <c r="X71" s="7">
+        <f>IF(V71=0,0,W71/V71)</f>
+        <v>0</v>
+      </c>
+      <c r="Y71" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z71" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA71" s="4">
+        <f>IF(Y71=0,0,Z71/Y71)</f>
+        <v>0</v>
+      </c>
+      <c r="AB71" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC71" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD71" s="4">
+        <f>IF(AB71=0,0,AC71/AB71)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:30">
+      <c r="B72" t="s">
+        <v>34</v>
+      </c>
+      <c r="C72" s="3">
+        <f>J72+M72+G72+P72</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="3">
+        <f>J72+G72</f>
+        <v>0</v>
+      </c>
+      <c r="E72" s="3">
+        <f>M72+P72</f>
+        <v>0</v>
+      </c>
+      <c r="F72" s="3">
+        <v>93.49564395607489</v>
+      </c>
+      <c r="G72" s="3">
+        <v>36.20808203369917</v>
+      </c>
+      <c r="H72" s="4">
+        <f>IF(F72=0,0,G72/F72)</f>
+        <v>0</v>
+      </c>
+      <c r="I72" s="3">
+        <v>136.6145524202559</v>
+      </c>
+      <c r="J72" s="6">
+        <v>7.45877905144963</v>
+      </c>
+      <c r="K72" s="7">
+        <f>IF(I72=0,0,J72/I72)</f>
+        <v>0</v>
+      </c>
+      <c r="L72" s="3">
+        <v>0</v>
+      </c>
+      <c r="M72" s="3">
+        <v>0</v>
+      </c>
+      <c r="N72" s="4">
+        <f>IF(L72=0,0,M72/L72)</f>
+        <v>0</v>
+      </c>
+      <c r="O72" s="3">
+        <v>0</v>
+      </c>
+      <c r="P72" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="4">
+        <f>IF(O72=0,0,P72/O72)</f>
+        <v>0</v>
+      </c>
+      <c r="S72" s="3">
+        <v>1323.196985098892</v>
+      </c>
+      <c r="T72" s="3">
+        <v>512.4348360626602</v>
+      </c>
+      <c r="U72" s="4">
+        <f>IF(S72=0,0,T72/S72)</f>
+        <v>0</v>
+      </c>
+      <c r="V72" s="3">
+        <v>4890905.466101354</v>
+      </c>
+      <c r="W72" s="6">
+        <v>296120.1093025655</v>
+      </c>
+      <c r="X72" s="7">
+        <f>IF(V72=0,0,W72/V72)</f>
+        <v>0</v>
+      </c>
+      <c r="Y72" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="4">
+        <f>IF(Y72=0,0,Z72/Y72)</f>
+        <v>0</v>
+      </c>
+      <c r="AB72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD72" s="4">
+        <f>IF(AB72=0,0,AC72/AB72)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add results and executed notebooks from the Nigeria salt folate test run (MIC-7572)
</commit_message>
<xml_diff>
--- a/5000_analyze_results/results_spreadsheet.xlsx
+++ b/5000_analyze_results/results_spreadsheet.xlsx
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="44">
   <si>
     <t>DALYs Averted by Fortification (1000s)</t>
   </si>
@@ -306,6 +306,12 @@
   </si>
   <si>
     <t>Ethiopia -- Salt-- DFS-IoFA preliminary standard 45 ppm</t>
+  </si>
+  <si>
+    <t>Nigeria -- Salt-- 25% NRV per average intake</t>
+  </si>
+  <si>
+    <t>Nigeria -- Salt-- 100% NRV per average intake</t>
   </si>
 </sst>
 </file>
@@ -686,7 +692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD72"/>
+  <dimension ref="A1:AD90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -1020,7 +1026,7 @@
         <v>320.5427437766894</v>
       </c>
       <c r="G6" s="3">
-        <v>11.4178093054627</v>
+        <v>11.41780930546322</v>
       </c>
       <c r="H6" s="4">
         <f>IF(F6=0,0,G6/F6)</f>
@@ -1060,7 +1066,7 @@
         <v>4138.352740079671</v>
       </c>
       <c r="T6" s="3">
-        <v>147.4091157648745</v>
+        <v>147.4091157648822</v>
       </c>
       <c r="U6" s="4">
         <f>IF(S6=0,0,T6/S6)</f>
@@ -1157,7 +1163,7 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T7" s="3">
-        <v>123.6968790634523</v>
+        <v>123.6968790634528</v>
       </c>
       <c r="U7" s="4">
         <f>IF(S7=0,0,T7/S7)</f>
@@ -1211,10 +1217,10 @@
         <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>271.3548595424364</v>
+        <v>271.3548595424359</v>
       </c>
       <c r="G8" s="3">
-        <v>8.370468320719199</v>
+        <v>8.370468320719258</v>
       </c>
       <c r="H8" s="4">
         <f>IF(F8=0,0,G8/F8)</f>
@@ -1251,10 +1257,10 @@
         <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>3503.314763237015</v>
+        <v>3503.314763237009</v>
       </c>
       <c r="T8" s="3">
-        <v>108.0665564369497</v>
+        <v>108.0665564369501</v>
       </c>
       <c r="U8" s="4">
         <f>IF(S8=0,0,T8/S8)</f>
@@ -1308,10 +1314,10 @@
         <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>231.1015430943892</v>
+        <v>231.1015430943887</v>
       </c>
       <c r="G9" s="3">
-        <v>2.991144416980329</v>
+        <v>2.991144416980678</v>
       </c>
       <c r="H9" s="4">
         <f>IF(F9=0,0,G9/F9)</f>
@@ -1348,10 +1354,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="3">
-        <v>2983.6261237209</v>
+        <v>2983.626123720895</v>
       </c>
       <c r="T9" s="3">
-        <v>38.61703605622006</v>
+        <v>38.61703605622597</v>
       </c>
       <c r="U9" s="4">
         <f>IF(S9=0,0,T9/S9)</f>
@@ -1531,7 +1537,7 @@
         <v>362.8529849538489</v>
       </c>
       <c r="G14" s="3">
-        <v>151.0014963206652</v>
+        <v>151.0014963206656</v>
       </c>
       <c r="H14" s="4">
         <f>IF(F14=0,0,G14/F14)</f>
@@ -1571,7 +1577,7 @@
         <v>4684.597214204819</v>
       </c>
       <c r="T14" s="3">
-        <v>1949.498056615184</v>
+        <v>1949.498056615189</v>
       </c>
       <c r="U14" s="4">
         <f>IF(S14=0,0,T14/S14)</f>
@@ -1725,7 +1731,7 @@
         <v>287.7720482472399</v>
       </c>
       <c r="G16" s="3">
-        <v>110.0570853730647</v>
+        <v>110.057085373065</v>
       </c>
       <c r="H16" s="4">
         <f>IF(F16=0,0,G16/F16)</f>
@@ -1765,7 +1771,7 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T16" s="3">
-        <v>1420.887072508819</v>
+        <v>1420.887072508823</v>
       </c>
       <c r="U16" s="4">
         <f>IF(S16=0,0,T16/S16)</f>
@@ -1819,10 +1825,10 @@
         <v>0</v>
       </c>
       <c r="F17" s="3">
-        <v>271.3548595424364</v>
+        <v>271.3548595424359</v>
       </c>
       <c r="G17" s="3">
-        <v>102.5231161409741</v>
+        <v>102.523116140974</v>
       </c>
       <c r="H17" s="4">
         <f>IF(F17=0,0,G17/F17)</f>
@@ -1859,10 +1865,10 @@
         <v>0</v>
       </c>
       <c r="S17" s="3">
-        <v>3503.314763237015</v>
+        <v>3503.314763237009</v>
       </c>
       <c r="T17" s="3">
-        <v>1323.620100098366</v>
+        <v>1323.620100098364</v>
       </c>
       <c r="U17" s="4">
         <f>IF(S17=0,0,T17/S17)</f>
@@ -1916,10 +1922,10 @@
         <v>0</v>
       </c>
       <c r="F18" s="3">
-        <v>231.1015430943892</v>
+        <v>231.1015430943887</v>
       </c>
       <c r="G18" s="3">
-        <v>67.11521448847459</v>
+        <v>67.11521448847442</v>
       </c>
       <c r="H18" s="4">
         <f>IF(F18=0,0,G18/F18)</f>
@@ -1956,10 +1962,10 @@
         <v>0</v>
       </c>
       <c r="S18" s="3">
-        <v>2983.6261237209</v>
+        <v>2983.626123720895</v>
       </c>
       <c r="T18" s="3">
-        <v>866.487971329369</v>
+        <v>866.4879713293681</v>
       </c>
       <c r="U18" s="4">
         <f>IF(S18=0,0,T18/S18)</f>
@@ -2139,7 +2145,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G23" s="3">
-        <v>153.5338348629944</v>
+        <v>153.5338348629948</v>
       </c>
       <c r="H23" s="4">
         <f>IF(F23=0,0,G23/F23)</f>
@@ -2179,7 +2185,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T23" s="3">
-        <v>4737.225453182307</v>
+        <v>4737.225453182322</v>
       </c>
       <c r="U23" s="4">
         <f>IF(S23=0,0,T23/S23)</f>
@@ -2236,7 +2242,7 @@
         <v>422.0532339939541</v>
       </c>
       <c r="G24" s="3">
-        <v>149.5731184765907</v>
+        <v>149.5731184765912</v>
       </c>
       <c r="H24" s="4">
         <f>IF(F24=0,0,G24/F24)</f>
@@ -2276,7 +2282,7 @@
         <v>13022.28479122008</v>
       </c>
       <c r="T24" s="3">
-        <v>4615.01912325346</v>
+        <v>4615.019123253476</v>
       </c>
       <c r="U24" s="4">
         <f>IF(S24=0,0,T24/S24)</f>
@@ -2373,7 +2379,7 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T25" s="3">
-        <v>3461.751499772323</v>
+        <v>3461.751499772321</v>
       </c>
       <c r="U25" s="4">
         <f>IF(S25=0,0,T25/S25)</f>
@@ -2430,7 +2436,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G26" s="3">
-        <v>86.23155739396391</v>
+        <v>86.23155739396429</v>
       </c>
       <c r="H26" s="4">
         <f>IF(F26=0,0,G26/F26)</f>
@@ -2470,7 +2476,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T26" s="3">
-        <v>2660.640430943183</v>
+        <v>2660.640430943196</v>
       </c>
       <c r="U26" s="4">
         <f>IF(S26=0,0,T26/S26)</f>
@@ -2747,7 +2753,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G32" s="3">
-        <v>31.81246083158365</v>
+        <v>31.81246083158429</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
@@ -2787,7 +2793,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T32" s="3">
-        <v>981.560835201064</v>
+        <v>981.560835201084</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
@@ -3038,7 +3044,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G35" s="3">
-        <v>79.01499632789695</v>
+        <v>79.01499632789736</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
@@ -3078,7 +3084,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T35" s="3">
-        <v>2437.97630744804</v>
+        <v>2437.976307448053</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
@@ -3956,14 +3962,14 @@
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>M50+P50</f>
+        <f>P50+M50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G50" s="3">
-        <v>58.98240259960004</v>
+        <v>58.98240259960006</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
@@ -4003,7 +4009,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T50" s="3">
-        <v>834.748379618052</v>
+        <v>834.7483796180522</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
@@ -4053,14 +4059,14 @@
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>M51+P51</f>
+        <f>P51+M51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
-        <v>147.7607036391234</v>
+        <v>147.7607036391231</v>
       </c>
       <c r="G51" s="3">
-        <v>59.41247823140031</v>
+        <v>59.41247823140037</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
@@ -4097,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="S51" s="3">
-        <v>2091.183174942721</v>
+        <v>2091.183174942718</v>
       </c>
       <c r="T51" s="3">
-        <v>840.835024463559</v>
+        <v>840.8350244635603</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
@@ -4150,14 +4156,14 @@
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>M52+P52</f>
+        <f>P52+M52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G52" s="3">
-        <v>59.19812501773825</v>
+        <v>59.19812501773821</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
@@ -4247,14 +4253,14 @@
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>M53+P53</f>
+        <f>P53+M53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G53" s="3">
-        <v>27.88815467106953</v>
+        <v>27.88815467106969</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
@@ -4294,7 +4300,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T53" s="3">
-        <v>394.6870743846359</v>
+        <v>394.6870743846378</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
@@ -4344,14 +4350,14 @@
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>M54+P54</f>
+        <f>P54+M54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
-        <v>93.49564395607489</v>
+        <v>93.49564395607474</v>
       </c>
       <c r="G54" s="3">
-        <v>16.262542548974</v>
+        <v>16.26254254897413</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
@@ -4388,10 +4394,10 @@
         <v>0</v>
       </c>
       <c r="S54" s="3">
-        <v>1323.196985098892</v>
+        <v>1323.19698509889</v>
       </c>
       <c r="T54" s="3">
-        <v>230.1556132492594</v>
+        <v>230.1556132492615</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>
@@ -4564,7 +4570,7 @@
         <v>0</v>
       </c>
       <c r="E59" s="3">
-        <f>M59+P59</f>
+        <f>P59+M59</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
@@ -4661,14 +4667,14 @@
         <v>0</v>
       </c>
       <c r="E60" s="3">
-        <f>M60+P60</f>
+        <f>P60+M60</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
-        <v>147.7607036391234</v>
+        <v>147.7607036391231</v>
       </c>
       <c r="G60" s="3">
-        <v>102.7420072452102</v>
+        <v>102.74200724521</v>
       </c>
       <c r="H60" s="4">
         <f>IF(F60=0,0,G60/F60)</f>
@@ -4705,10 +4711,10 @@
         <v>0</v>
       </c>
       <c r="S60" s="3">
-        <v>2091.183174942721</v>
+        <v>2091.183174942718</v>
       </c>
       <c r="T60" s="3">
-        <v>1454.056130077464</v>
+        <v>1454.056130077462</v>
       </c>
       <c r="U60" s="4">
         <f>IF(S60=0,0,T60/S60)</f>
@@ -4758,14 +4764,14 @@
         <v>0</v>
       </c>
       <c r="E61" s="3">
-        <f>M61+P61</f>
+        <f>P61+M61</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G61" s="3">
-        <v>97.48822698814803</v>
+        <v>97.488226988148</v>
       </c>
       <c r="H61" s="4">
         <f>IF(F61=0,0,G61/F61)</f>
@@ -4855,14 +4861,14 @@
         <v>0</v>
       </c>
       <c r="E62" s="3">
-        <f>M62+P62</f>
+        <f>P62+M62</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G62" s="3">
-        <v>62.28901992946243</v>
+        <v>62.28901992946252</v>
       </c>
       <c r="H62" s="4">
         <f>IF(F62=0,0,G62/F62)</f>
@@ -4902,7 +4908,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T62" s="3">
-        <v>881.5452772767835</v>
+        <v>881.545277276785</v>
       </c>
       <c r="U62" s="4">
         <f>IF(S62=0,0,T62/S62)</f>
@@ -4952,14 +4958,14 @@
         <v>0</v>
       </c>
       <c r="E63" s="3">
-        <f>M63+P63</f>
+        <f>P63+M63</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
-        <v>93.49564395607489</v>
+        <v>93.49564395607474</v>
       </c>
       <c r="G63" s="3">
-        <v>40.86638015373273</v>
+        <v>40.86638015373266</v>
       </c>
       <c r="H63" s="4">
         <f>IF(F63=0,0,G63/F63)</f>
@@ -4996,10 +5002,10 @@
         <v>0</v>
       </c>
       <c r="S63" s="3">
-        <v>1323.196985098892</v>
+        <v>1323.19698509889</v>
       </c>
       <c r="T63" s="3">
-        <v>578.3613944274123</v>
+        <v>578.3613944274117</v>
       </c>
       <c r="U63" s="4">
         <f>IF(S63=0,0,T63/S63)</f>
@@ -5172,14 +5178,14 @@
         <v>0</v>
       </c>
       <c r="E68" s="3">
-        <f>M68+P68</f>
+        <f>P68+M68</f>
         <v>0</v>
       </c>
       <c r="F68" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G68" s="3">
-        <v>98.37588727255856</v>
+        <v>98.37588727255864</v>
       </c>
       <c r="H68" s="4">
         <f>IF(F68=0,0,G68/F68)</f>
@@ -5219,7 +5225,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T68" s="3">
-        <v>1392.264622581062</v>
+        <v>1392.264622581063</v>
       </c>
       <c r="U68" s="4">
         <f>IF(S68=0,0,T68/S68)</f>
@@ -5269,14 +5275,14 @@
         <v>0</v>
       </c>
       <c r="E69" s="3">
-        <f>M69+P69</f>
+        <f>P69+M69</f>
         <v>0</v>
       </c>
       <c r="F69" s="3">
-        <v>147.7607036391234</v>
+        <v>147.7607036391231</v>
       </c>
       <c r="G69" s="3">
-        <v>96.54985248064214</v>
+        <v>96.54985248064197</v>
       </c>
       <c r="H69" s="4">
         <f>IF(F69=0,0,G69/F69)</f>
@@ -5313,10 +5319,10 @@
         <v>0</v>
       </c>
       <c r="S69" s="3">
-        <v>2091.183174942721</v>
+        <v>2091.183174942718</v>
       </c>
       <c r="T69" s="3">
-        <v>1366.42166745382</v>
+        <v>1366.421667453817</v>
       </c>
       <c r="U69" s="4">
         <f>IF(S69=0,0,T69/S69)</f>
@@ -5366,14 +5372,14 @@
         <v>0</v>
       </c>
       <c r="E70" s="3">
-        <f>M70+P70</f>
+        <f>P70+M70</f>
         <v>0</v>
       </c>
       <c r="F70" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G70" s="3">
-        <v>92.2087189913087</v>
+        <v>92.20871899130873</v>
       </c>
       <c r="H70" s="4">
         <f>IF(F70=0,0,G70/F70)</f>
@@ -5463,7 +5469,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="3">
-        <f>M71+P71</f>
+        <f>P71+M71</f>
         <v>0</v>
       </c>
       <c r="F71" s="3">
@@ -5560,14 +5566,14 @@
         <v>0</v>
       </c>
       <c r="E72" s="3">
-        <f>M72+P72</f>
+        <f>P72+M72</f>
         <v>0</v>
       </c>
       <c r="F72" s="3">
-        <v>93.49564395607489</v>
+        <v>93.49564395607474</v>
       </c>
       <c r="G72" s="3">
-        <v>36.20808203369917</v>
+        <v>36.20808203369902</v>
       </c>
       <c r="H72" s="4">
         <f>IF(F72=0,0,G72/F72)</f>
@@ -5604,10 +5610,10 @@
         <v>0</v>
       </c>
       <c r="S72" s="3">
-        <v>1323.196985098892</v>
+        <v>1323.19698509889</v>
       </c>
       <c r="T72" s="3">
-        <v>512.4348360626602</v>
+        <v>512.4348360626584</v>
       </c>
       <c r="U72" s="4">
         <f>IF(S72=0,0,T72/S72)</f>
@@ -5641,6 +5647,1222 @@
       </c>
       <c r="AD72" s="4">
         <f>IF(AB72=0,0,AC72/AB72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:30">
+      <c r="A74" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="75" spans="1:30">
+      <c r="B75" t="s">
+        <v>28</v>
+      </c>
+      <c r="C75" s="3">
+        <f>C77+C78+C79+C80+C81</f>
+        <v>0</v>
+      </c>
+      <c r="D75" s="3">
+        <f>D77+D78+D79+D80+D81</f>
+        <v>0</v>
+      </c>
+      <c r="E75" s="3">
+        <f>E77+E78+E79+E80+E81</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="3">
+        <f>F77+F78+F79+F80+F81</f>
+        <v>0</v>
+      </c>
+      <c r="G75" s="3">
+        <f>G77+G78+G79+G80+G81</f>
+        <v>0</v>
+      </c>
+      <c r="H75" s="4">
+        <f>IF(F75=0,0,G75/F75)</f>
+        <v>0</v>
+      </c>
+      <c r="I75" s="3">
+        <f>I77+I78+I79+I80+I81</f>
+        <v>0</v>
+      </c>
+      <c r="J75" s="3">
+        <f>J77+J78+J79+J80+J81</f>
+        <v>0</v>
+      </c>
+      <c r="K75" s="4">
+        <f>IF(I75=0,0,J75/I75)</f>
+        <v>0</v>
+      </c>
+      <c r="L75" s="3">
+        <f>L77+L78+L79+L80+L81</f>
+        <v>0</v>
+      </c>
+      <c r="M75" s="3">
+        <f>M77+M78+M79+M80+M81</f>
+        <v>0</v>
+      </c>
+      <c r="N75" s="4">
+        <f>IF(L75=0,0,M75/L75)</f>
+        <v>0</v>
+      </c>
+      <c r="O75" s="3">
+        <f>O77+O78+O79+O80+O81</f>
+        <v>0</v>
+      </c>
+      <c r="P75" s="3">
+        <f>P77+P78+P79+P80+P81</f>
+        <v>0</v>
+      </c>
+      <c r="Q75" s="4">
+        <f>IF(O75=0,0,P75/O75)</f>
+        <v>0</v>
+      </c>
+      <c r="S75" s="3">
+        <f>S77+S78+S79+S80+S81</f>
+        <v>0</v>
+      </c>
+      <c r="T75" s="3">
+        <f>T77+T78+T79+T80+T81</f>
+        <v>0</v>
+      </c>
+      <c r="U75" s="4">
+        <f>IF(S75=0,0,T75/S75)</f>
+        <v>0</v>
+      </c>
+      <c r="V75" s="3">
+        <f>V77+V78+V79+V80+V81</f>
+        <v>0</v>
+      </c>
+      <c r="W75" s="3">
+        <f>W77+W78+W79+W80+W81</f>
+        <v>0</v>
+      </c>
+      <c r="X75" s="4">
+        <f>IF(V75=0,0,W75/V75)</f>
+        <v>0</v>
+      </c>
+      <c r="Y75" s="3">
+        <f>Y77+Y78+Y79+Y80+Y81</f>
+        <v>0</v>
+      </c>
+      <c r="Z75" s="3">
+        <f>Z77+Z78+Z79+Z80+Z81</f>
+        <v>0</v>
+      </c>
+      <c r="AA75" s="4">
+        <f>IF(Y75=0,0,Z75/Y75)</f>
+        <v>0</v>
+      </c>
+      <c r="AB75" s="3">
+        <f>AB77+AB78+AB79+AB80+AB81</f>
+        <v>0</v>
+      </c>
+      <c r="AC75" s="3">
+        <f>AC77+AC78+AC79+AC80+AC81</f>
+        <v>0</v>
+      </c>
+      <c r="AD75" s="4">
+        <f>IF(AB75=0,0,AC75/AB75)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:30">
+      <c r="A76" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="77" spans="1:30">
+      <c r="B77" t="s">
+        <v>30</v>
+      </c>
+      <c r="C77" s="3">
+        <f>J77+M77+G77+P77</f>
+        <v>0</v>
+      </c>
+      <c r="D77" s="3">
+        <f>G77</f>
+        <v>0</v>
+      </c>
+      <c r="E77" s="3">
+        <f>J77+M77+P77</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="3">
+        <v>412.7408750394843</v>
+      </c>
+      <c r="G77" s="3">
+        <v>146.8879599840255</v>
+      </c>
+      <c r="H77" s="4">
+        <f>IF(F77=0,0,G77/F77)</f>
+        <v>0</v>
+      </c>
+      <c r="I77" s="3">
+        <v>0</v>
+      </c>
+      <c r="J77" s="3">
+        <v>0</v>
+      </c>
+      <c r="K77" s="4">
+        <f>IF(I77=0,0,J77/I77)</f>
+        <v>0</v>
+      </c>
+      <c r="L77" s="3">
+        <v>0</v>
+      </c>
+      <c r="M77" s="3">
+        <v>0</v>
+      </c>
+      <c r="N77" s="4">
+        <f>IF(L77=0,0,M77/L77)</f>
+        <v>0</v>
+      </c>
+      <c r="O77" s="3">
+        <v>0</v>
+      </c>
+      <c r="P77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="4">
+        <f>IF(O77=0,0,P77/O77)</f>
+        <v>0</v>
+      </c>
+      <c r="S77" s="3">
+        <v>12734.95565684622</v>
+      </c>
+      <c r="T77" s="3">
+        <v>4532.169625172735</v>
+      </c>
+      <c r="U77" s="4">
+        <f>IF(S77=0,0,T77/S77)</f>
+        <v>0</v>
+      </c>
+      <c r="V77" s="3">
+        <v>0</v>
+      </c>
+      <c r="W77" s="3">
+        <v>0</v>
+      </c>
+      <c r="X77" s="4">
+        <f>IF(V77=0,0,W77/V77)</f>
+        <v>0</v>
+      </c>
+      <c r="Y77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="4">
+        <f>IF(Y77=0,0,Z77/Y77)</f>
+        <v>0</v>
+      </c>
+      <c r="AB77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD77" s="4">
+        <f>IF(AB77=0,0,AC77/AB77)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:30">
+      <c r="B78" t="s">
+        <v>31</v>
+      </c>
+      <c r="C78" s="3">
+        <f>J78+M78+G78+P78</f>
+        <v>0</v>
+      </c>
+      <c r="D78" s="3">
+        <f>G78</f>
+        <v>0</v>
+      </c>
+      <c r="E78" s="3">
+        <f>J78+M78+P78</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="3">
+        <v>422.0532339939541</v>
+      </c>
+      <c r="G78" s="3">
+        <v>141.7344183926904</v>
+      </c>
+      <c r="H78" s="4">
+        <f>IF(F78=0,0,G78/F78)</f>
+        <v>0</v>
+      </c>
+      <c r="I78" s="3">
+        <v>0</v>
+      </c>
+      <c r="J78" s="3">
+        <v>0</v>
+      </c>
+      <c r="K78" s="4">
+        <f>IF(I78=0,0,J78/I78)</f>
+        <v>0</v>
+      </c>
+      <c r="L78" s="3">
+        <v>0</v>
+      </c>
+      <c r="M78" s="3">
+        <v>0</v>
+      </c>
+      <c r="N78" s="4">
+        <f>IF(L78=0,0,M78/L78)</f>
+        <v>0</v>
+      </c>
+      <c r="O78" s="3">
+        <v>0</v>
+      </c>
+      <c r="P78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="4">
+        <f>IF(O78=0,0,P78/O78)</f>
+        <v>0</v>
+      </c>
+      <c r="S78" s="3">
+        <v>13022.28479122008</v>
+      </c>
+      <c r="T78" s="3">
+        <v>4373.159147630166</v>
+      </c>
+      <c r="U78" s="4">
+        <f>IF(S78=0,0,T78/S78)</f>
+        <v>0</v>
+      </c>
+      <c r="V78" s="3">
+        <v>0</v>
+      </c>
+      <c r="W78" s="3">
+        <v>0</v>
+      </c>
+      <c r="X78" s="4">
+        <f>IF(V78=0,0,W78/V78)</f>
+        <v>0</v>
+      </c>
+      <c r="Y78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="4">
+        <f>IF(Y78=0,0,Z78/Y78)</f>
+        <v>0</v>
+      </c>
+      <c r="AB78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD78" s="4">
+        <f>IF(AB78=0,0,AC78/AB78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:30">
+      <c r="B79" t="s">
+        <v>32</v>
+      </c>
+      <c r="C79" s="3">
+        <f>J79+M79+G79+P79</f>
+        <v>0</v>
+      </c>
+      <c r="D79" s="3">
+        <f>G79</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="3">
+        <f>J79+M79+P79</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="3">
+        <v>382.0743136549376</v>
+      </c>
+      <c r="G79" s="3">
+        <v>124.6559480289836</v>
+      </c>
+      <c r="H79" s="4">
+        <f>IF(F79=0,0,G79/F79)</f>
+        <v>0</v>
+      </c>
+      <c r="I79" s="3">
+        <v>0</v>
+      </c>
+      <c r="J79" s="3">
+        <v>0</v>
+      </c>
+      <c r="K79" s="4">
+        <f>IF(I79=0,0,J79/I79)</f>
+        <v>0</v>
+      </c>
+      <c r="L79" s="3">
+        <v>0</v>
+      </c>
+      <c r="M79" s="3">
+        <v>0</v>
+      </c>
+      <c r="N79" s="4">
+        <f>IF(L79=0,0,M79/L79)</f>
+        <v>0</v>
+      </c>
+      <c r="O79" s="3">
+        <v>0</v>
+      </c>
+      <c r="P79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="4">
+        <f>IF(O79=0,0,P79/O79)</f>
+        <v>0</v>
+      </c>
+      <c r="S79" s="3">
+        <v>11788.75109364953</v>
+      </c>
+      <c r="T79" s="3">
+        <v>3846.209732339612</v>
+      </c>
+      <c r="U79" s="4">
+        <f>IF(S79=0,0,T79/S79)</f>
+        <v>0</v>
+      </c>
+      <c r="V79" s="3">
+        <v>0</v>
+      </c>
+      <c r="W79" s="3">
+        <v>0</v>
+      </c>
+      <c r="X79" s="4">
+        <f>IF(V79=0,0,W79/V79)</f>
+        <v>0</v>
+      </c>
+      <c r="Y79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="4">
+        <f>IF(Y79=0,0,Z79/Y79)</f>
+        <v>0</v>
+      </c>
+      <c r="AB79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD79" s="4">
+        <f>IF(AB79=0,0,AC79/AB79)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:30">
+      <c r="B80" t="s">
+        <v>33</v>
+      </c>
+      <c r="C80" s="3">
+        <f>J80+M80+G80+P80</f>
+        <v>0</v>
+      </c>
+      <c r="D80" s="3">
+        <f>G80</f>
+        <v>0</v>
+      </c>
+      <c r="E80" s="3">
+        <f>J80+M80+P80</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="3">
+        <v>338.6701578384149</v>
+      </c>
+      <c r="G80" s="3">
+        <v>106.5823973125179</v>
+      </c>
+      <c r="H80" s="4">
+        <f>IF(F80=0,0,G80/F80)</f>
+        <v>0</v>
+      </c>
+      <c r="I80" s="3">
+        <v>0</v>
+      </c>
+      <c r="J80" s="3">
+        <v>0</v>
+      </c>
+      <c r="K80" s="4">
+        <f>IF(I80=0,0,J80/I80)</f>
+        <v>0</v>
+      </c>
+      <c r="L80" s="3">
+        <v>0</v>
+      </c>
+      <c r="M80" s="3">
+        <v>0</v>
+      </c>
+      <c r="N80" s="4">
+        <f>IF(L80=0,0,M80/L80)</f>
+        <v>0</v>
+      </c>
+      <c r="O80" s="3">
+        <v>0</v>
+      </c>
+      <c r="P80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="4">
+        <f>IF(O80=0,0,P80/O80)</f>
+        <v>0</v>
+      </c>
+      <c r="S80" s="3">
+        <v>10449.53311676904</v>
+      </c>
+      <c r="T80" s="3">
+        <v>3288.557508256084</v>
+      </c>
+      <c r="U80" s="4">
+        <f>IF(S80=0,0,T80/S80)</f>
+        <v>0</v>
+      </c>
+      <c r="V80" s="3">
+        <v>0</v>
+      </c>
+      <c r="W80" s="3">
+        <v>0</v>
+      </c>
+      <c r="X80" s="4">
+        <f>IF(V80=0,0,W80/V80)</f>
+        <v>0</v>
+      </c>
+      <c r="Y80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="4">
+        <f>IF(Y80=0,0,Z80/Y80)</f>
+        <v>0</v>
+      </c>
+      <c r="AB80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD80" s="4">
+        <f>IF(AB80=0,0,AC80/AB80)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:30">
+      <c r="B81" t="s">
+        <v>34</v>
+      </c>
+      <c r="C81" s="3">
+        <f>J81+M81+G81+P81</f>
+        <v>0</v>
+      </c>
+      <c r="D81" s="3">
+        <f>G81</f>
+        <v>0</v>
+      </c>
+      <c r="E81" s="3">
+        <f>J81+M81+P81</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="3">
+        <v>297.4602934996698</v>
+      </c>
+      <c r="G81" s="3">
+        <v>93.75383596516214</v>
+      </c>
+      <c r="H81" s="4">
+        <f>IF(F81=0,0,G81/F81)</f>
+        <v>0</v>
+      </c>
+      <c r="I81" s="3">
+        <v>0</v>
+      </c>
+      <c r="J81" s="3">
+        <v>0</v>
+      </c>
+      <c r="K81" s="4">
+        <f>IF(I81=0,0,J81/I81)</f>
+        <v>0</v>
+      </c>
+      <c r="L81" s="3">
+        <v>0</v>
+      </c>
+      <c r="M81" s="3">
+        <v>0</v>
+      </c>
+      <c r="N81" s="4">
+        <f>IF(L81=0,0,M81/L81)</f>
+        <v>0</v>
+      </c>
+      <c r="O81" s="3">
+        <v>0</v>
+      </c>
+      <c r="P81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q81" s="4">
+        <f>IF(O81=0,0,P81/O81)</f>
+        <v>0</v>
+      </c>
+      <c r="S81" s="3">
+        <v>9178.019131321482</v>
+      </c>
+      <c r="T81" s="3">
+        <v>2892.73734655274</v>
+      </c>
+      <c r="U81" s="4">
+        <f>IF(S81=0,0,T81/S81)</f>
+        <v>0</v>
+      </c>
+      <c r="V81" s="3">
+        <v>0</v>
+      </c>
+      <c r="W81" s="3">
+        <v>0</v>
+      </c>
+      <c r="X81" s="4">
+        <f>IF(V81=0,0,W81/V81)</f>
+        <v>0</v>
+      </c>
+      <c r="Y81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="4">
+        <f>IF(Y81=0,0,Z81/Y81)</f>
+        <v>0</v>
+      </c>
+      <c r="AB81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD81" s="4">
+        <f>IF(AB81=0,0,AC81/AB81)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:30">
+      <c r="A83" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="84" spans="1:30">
+      <c r="B84" t="s">
+        <v>28</v>
+      </c>
+      <c r="C84" s="3">
+        <f>C86+C87+C88+C89+C90</f>
+        <v>0</v>
+      </c>
+      <c r="D84" s="3">
+        <f>D86+D87+D88+D89+D90</f>
+        <v>0</v>
+      </c>
+      <c r="E84" s="3">
+        <f>E86+E87+E88+E89+E90</f>
+        <v>0</v>
+      </c>
+      <c r="F84" s="3">
+        <f>F86+F87+F88+F89+F90</f>
+        <v>0</v>
+      </c>
+      <c r="G84" s="3">
+        <f>G86+G87+G88+G89+G90</f>
+        <v>0</v>
+      </c>
+      <c r="H84" s="4">
+        <f>IF(F84=0,0,G84/F84)</f>
+        <v>0</v>
+      </c>
+      <c r="I84" s="3">
+        <f>I86+I87+I88+I89+I90</f>
+        <v>0</v>
+      </c>
+      <c r="J84" s="3">
+        <f>J86+J87+J88+J89+J90</f>
+        <v>0</v>
+      </c>
+      <c r="K84" s="4">
+        <f>IF(I84=0,0,J84/I84)</f>
+        <v>0</v>
+      </c>
+      <c r="L84" s="3">
+        <f>L86+L87+L88+L89+L90</f>
+        <v>0</v>
+      </c>
+      <c r="M84" s="3">
+        <f>M86+M87+M88+M89+M90</f>
+        <v>0</v>
+      </c>
+      <c r="N84" s="4">
+        <f>IF(L84=0,0,M84/L84)</f>
+        <v>0</v>
+      </c>
+      <c r="O84" s="3">
+        <f>O86+O87+O88+O89+O90</f>
+        <v>0</v>
+      </c>
+      <c r="P84" s="3">
+        <f>P86+P87+P88+P89+P90</f>
+        <v>0</v>
+      </c>
+      <c r="Q84" s="4">
+        <f>IF(O84=0,0,P84/O84)</f>
+        <v>0</v>
+      </c>
+      <c r="S84" s="3">
+        <f>S86+S87+S88+S89+S90</f>
+        <v>0</v>
+      </c>
+      <c r="T84" s="3">
+        <f>T86+T87+T88+T89+T90</f>
+        <v>0</v>
+      </c>
+      <c r="U84" s="4">
+        <f>IF(S84=0,0,T84/S84)</f>
+        <v>0</v>
+      </c>
+      <c r="V84" s="3">
+        <f>V86+V87+V88+V89+V90</f>
+        <v>0</v>
+      </c>
+      <c r="W84" s="3">
+        <f>W86+W87+W88+W89+W90</f>
+        <v>0</v>
+      </c>
+      <c r="X84" s="4">
+        <f>IF(V84=0,0,W84/V84)</f>
+        <v>0</v>
+      </c>
+      <c r="Y84" s="3">
+        <f>Y86+Y87+Y88+Y89+Y90</f>
+        <v>0</v>
+      </c>
+      <c r="Z84" s="3">
+        <f>Z86+Z87+Z88+Z89+Z90</f>
+        <v>0</v>
+      </c>
+      <c r="AA84" s="4">
+        <f>IF(Y84=0,0,Z84/Y84)</f>
+        <v>0</v>
+      </c>
+      <c r="AB84" s="3">
+        <f>AB86+AB87+AB88+AB89+AB90</f>
+        <v>0</v>
+      </c>
+      <c r="AC84" s="3">
+        <f>AC86+AC87+AC88+AC89+AC90</f>
+        <v>0</v>
+      </c>
+      <c r="AD84" s="4">
+        <f>IF(AB84=0,0,AC84/AB84)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:30">
+      <c r="A85" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="86" spans="1:30">
+      <c r="B86" t="s">
+        <v>30</v>
+      </c>
+      <c r="C86" s="3">
+        <f>J86+M86+G86+P86</f>
+        <v>0</v>
+      </c>
+      <c r="D86" s="3">
+        <f>G86</f>
+        <v>0</v>
+      </c>
+      <c r="E86" s="3">
+        <f>J86+M86+P86</f>
+        <v>0</v>
+      </c>
+      <c r="F86" s="3">
+        <v>412.7408750394843</v>
+      </c>
+      <c r="G86" s="3">
+        <v>270.621528830763</v>
+      </c>
+      <c r="H86" s="4">
+        <f>IF(F86=0,0,G86/F86)</f>
+        <v>0</v>
+      </c>
+      <c r="I86" s="3">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3">
+        <v>0</v>
+      </c>
+      <c r="K86" s="4">
+        <f>IF(I86=0,0,J86/I86)</f>
+        <v>0</v>
+      </c>
+      <c r="L86" s="3">
+        <v>0</v>
+      </c>
+      <c r="M86" s="3">
+        <v>0</v>
+      </c>
+      <c r="N86" s="4">
+        <f>IF(L86=0,0,M86/L86)</f>
+        <v>0</v>
+      </c>
+      <c r="O86" s="3">
+        <v>0</v>
+      </c>
+      <c r="P86" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="4">
+        <f>IF(O86=0,0,P86/O86)</f>
+        <v>0</v>
+      </c>
+      <c r="S86" s="3">
+        <v>12734.95565684622</v>
+      </c>
+      <c r="T86" s="3">
+        <v>8349.919714440704</v>
+      </c>
+      <c r="U86" s="4">
+        <f>IF(S86=0,0,T86/S86)</f>
+        <v>0</v>
+      </c>
+      <c r="V86" s="3">
+        <v>0</v>
+      </c>
+      <c r="W86" s="3">
+        <v>0</v>
+      </c>
+      <c r="X86" s="4">
+        <f>IF(V86=0,0,W86/V86)</f>
+        <v>0</v>
+      </c>
+      <c r="Y86" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z86" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA86" s="4">
+        <f>IF(Y86=0,0,Z86/Y86)</f>
+        <v>0</v>
+      </c>
+      <c r="AB86" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC86" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD86" s="4">
+        <f>IF(AB86=0,0,AC86/AB86)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:30">
+      <c r="B87" t="s">
+        <v>31</v>
+      </c>
+      <c r="C87" s="3">
+        <f>J87+M87+G87+P87</f>
+        <v>0</v>
+      </c>
+      <c r="D87" s="3">
+        <f>G87</f>
+        <v>0</v>
+      </c>
+      <c r="E87" s="3">
+        <f>J87+M87+P87</f>
+        <v>0</v>
+      </c>
+      <c r="F87" s="3">
+        <v>422.0532339939541</v>
+      </c>
+      <c r="G87" s="3">
+        <v>268.8415075664349</v>
+      </c>
+      <c r="H87" s="4">
+        <f>IF(F87=0,0,G87/F87)</f>
+        <v>0</v>
+      </c>
+      <c r="I87" s="3">
+        <v>0</v>
+      </c>
+      <c r="J87" s="3">
+        <v>0</v>
+      </c>
+      <c r="K87" s="4">
+        <f>IF(I87=0,0,J87/I87)</f>
+        <v>0</v>
+      </c>
+      <c r="L87" s="3">
+        <v>0</v>
+      </c>
+      <c r="M87" s="3">
+        <v>0</v>
+      </c>
+      <c r="N87" s="4">
+        <f>IF(L87=0,0,M87/L87)</f>
+        <v>0</v>
+      </c>
+      <c r="O87" s="3">
+        <v>0</v>
+      </c>
+      <c r="P87" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q87" s="4">
+        <f>IF(O87=0,0,P87/O87)</f>
+        <v>0</v>
+      </c>
+      <c r="S87" s="3">
+        <v>13022.28479122008</v>
+      </c>
+      <c r="T87" s="3">
+        <v>8294.997865793428</v>
+      </c>
+      <c r="U87" s="4">
+        <f>IF(S87=0,0,T87/S87)</f>
+        <v>0</v>
+      </c>
+      <c r="V87" s="3">
+        <v>0</v>
+      </c>
+      <c r="W87" s="3">
+        <v>0</v>
+      </c>
+      <c r="X87" s="4">
+        <f>IF(V87=0,0,W87/V87)</f>
+        <v>0</v>
+      </c>
+      <c r="Y87" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA87" s="4">
+        <f>IF(Y87=0,0,Z87/Y87)</f>
+        <v>0</v>
+      </c>
+      <c r="AB87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD87" s="4">
+        <f>IF(AB87=0,0,AC87/AB87)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:30">
+      <c r="B88" t="s">
+        <v>32</v>
+      </c>
+      <c r="C88" s="3">
+        <f>J88+M88+G88+P88</f>
+        <v>0</v>
+      </c>
+      <c r="D88" s="3">
+        <f>G88</f>
+        <v>0</v>
+      </c>
+      <c r="E88" s="3">
+        <f>J88+M88+P88</f>
+        <v>0</v>
+      </c>
+      <c r="F88" s="3">
+        <v>382.0743136549376</v>
+      </c>
+      <c r="G88" s="3">
+        <v>239.83782878063</v>
+      </c>
+      <c r="H88" s="4">
+        <f>IF(F88=0,0,G88/F88)</f>
+        <v>0</v>
+      </c>
+      <c r="I88" s="3">
+        <v>0</v>
+      </c>
+      <c r="J88" s="3">
+        <v>0</v>
+      </c>
+      <c r="K88" s="4">
+        <f>IF(I88=0,0,J88/I88)</f>
+        <v>0</v>
+      </c>
+      <c r="L88" s="3">
+        <v>0</v>
+      </c>
+      <c r="M88" s="3">
+        <v>0</v>
+      </c>
+      <c r="N88" s="4">
+        <f>IF(L88=0,0,M88/L88)</f>
+        <v>0</v>
+      </c>
+      <c r="O88" s="3">
+        <v>0</v>
+      </c>
+      <c r="P88" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="4">
+        <f>IF(O88=0,0,P88/O88)</f>
+        <v>0</v>
+      </c>
+      <c r="S88" s="3">
+        <v>11788.75109364953</v>
+      </c>
+      <c r="T88" s="3">
+        <v>7400.100884273723</v>
+      </c>
+      <c r="U88" s="4">
+        <f>IF(S88=0,0,T88/S88)</f>
+        <v>0</v>
+      </c>
+      <c r="V88" s="3">
+        <v>0</v>
+      </c>
+      <c r="W88" s="3">
+        <v>0</v>
+      </c>
+      <c r="X88" s="4">
+        <f>IF(V88=0,0,W88/V88)</f>
+        <v>0</v>
+      </c>
+      <c r="Y88" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z88" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA88" s="4">
+        <f>IF(Y88=0,0,Z88/Y88)</f>
+        <v>0</v>
+      </c>
+      <c r="AB88" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC88" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD88" s="4">
+        <f>IF(AB88=0,0,AC88/AB88)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:30">
+      <c r="B89" t="s">
+        <v>33</v>
+      </c>
+      <c r="C89" s="3">
+        <f>J89+M89+G89+P89</f>
+        <v>0</v>
+      </c>
+      <c r="D89" s="3">
+        <f>G89</f>
+        <v>0</v>
+      </c>
+      <c r="E89" s="3">
+        <f>J89+M89+P89</f>
+        <v>0</v>
+      </c>
+      <c r="F89" s="3">
+        <v>338.6701578384149</v>
+      </c>
+      <c r="G89" s="3">
+        <v>208.6917795068874</v>
+      </c>
+      <c r="H89" s="4">
+        <f>IF(F89=0,0,G89/F89)</f>
+        <v>0</v>
+      </c>
+      <c r="I89" s="3">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3">
+        <v>0</v>
+      </c>
+      <c r="K89" s="4">
+        <f>IF(I89=0,0,J89/I89)</f>
+        <v>0</v>
+      </c>
+      <c r="L89" s="3">
+        <v>0</v>
+      </c>
+      <c r="M89" s="3">
+        <v>0</v>
+      </c>
+      <c r="N89" s="4">
+        <f>IF(L89=0,0,M89/L89)</f>
+        <v>0</v>
+      </c>
+      <c r="O89" s="3">
+        <v>0</v>
+      </c>
+      <c r="P89" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q89" s="4">
+        <f>IF(O89=0,0,P89/O89)</f>
+        <v>0</v>
+      </c>
+      <c r="S89" s="3">
+        <v>10449.53311676904</v>
+      </c>
+      <c r="T89" s="3">
+        <v>6439.101912826773</v>
+      </c>
+      <c r="U89" s="4">
+        <f>IF(S89=0,0,T89/S89)</f>
+        <v>0</v>
+      </c>
+      <c r="V89" s="3">
+        <v>0</v>
+      </c>
+      <c r="W89" s="3">
+        <v>0</v>
+      </c>
+      <c r="X89" s="4">
+        <f>IF(V89=0,0,W89/V89)</f>
+        <v>0</v>
+      </c>
+      <c r="Y89" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA89" s="4">
+        <f>IF(Y89=0,0,Z89/Y89)</f>
+        <v>0</v>
+      </c>
+      <c r="AB89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD89" s="4">
+        <f>IF(AB89=0,0,AC89/AB89)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:30">
+      <c r="B90" t="s">
+        <v>34</v>
+      </c>
+      <c r="C90" s="3">
+        <f>J90+M90+G90+P90</f>
+        <v>0</v>
+      </c>
+      <c r="D90" s="3">
+        <f>G90</f>
+        <v>0</v>
+      </c>
+      <c r="E90" s="3">
+        <f>J90+M90+P90</f>
+        <v>0</v>
+      </c>
+      <c r="F90" s="3">
+        <v>297.4602934996698</v>
+      </c>
+      <c r="G90" s="3">
+        <v>183.4401220978906</v>
+      </c>
+      <c r="H90" s="4">
+        <f>IF(F90=0,0,G90/F90)</f>
+        <v>0</v>
+      </c>
+      <c r="I90" s="3">
+        <v>0</v>
+      </c>
+      <c r="J90" s="3">
+        <v>0</v>
+      </c>
+      <c r="K90" s="4">
+        <f>IF(I90=0,0,J90/I90)</f>
+        <v>0</v>
+      </c>
+      <c r="L90" s="3">
+        <v>0</v>
+      </c>
+      <c r="M90" s="3">
+        <v>0</v>
+      </c>
+      <c r="N90" s="4">
+        <f>IF(L90=0,0,M90/L90)</f>
+        <v>0</v>
+      </c>
+      <c r="O90" s="3">
+        <v>0</v>
+      </c>
+      <c r="P90" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="4">
+        <f>IF(O90=0,0,P90/O90)</f>
+        <v>0</v>
+      </c>
+      <c r="S90" s="3">
+        <v>9178.019131321482</v>
+      </c>
+      <c r="T90" s="3">
+        <v>5659.972059659981</v>
+      </c>
+      <c r="U90" s="4">
+        <f>IF(S90=0,0,T90/S90)</f>
+        <v>0</v>
+      </c>
+      <c r="V90" s="3">
+        <v>0</v>
+      </c>
+      <c r="W90" s="3">
+        <v>0</v>
+      </c>
+      <c r="X90" s="4">
+        <f>IF(V90=0,0,W90/V90)</f>
+        <v>0</v>
+      </c>
+      <c r="Y90" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z90" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="4">
+        <f>IF(Y90=0,0,Z90/Y90)</f>
+        <v>0</v>
+      </c>
+      <c r="AB90" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC90" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD90" s="4">
+        <f>IF(AB90=0,0,AC90/AB90)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Albrja/mic 7572/nigeria salt folic acid (#47)
</commit_message>
<xml_diff>
--- a/5000_analyze_results/results_spreadsheet.xlsx
+++ b/5000_analyze_results/results_spreadsheet.xlsx
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="44">
   <si>
     <t>DALYs Averted by Fortification (1000s)</t>
   </si>
@@ -306,6 +306,12 @@
   </si>
   <si>
     <t>Ethiopia -- Salt-- DFS-IoFA preliminary standard 45 ppm</t>
+  </si>
+  <si>
+    <t>Nigeria -- Salt-- 25% NRV per average intake</t>
+  </si>
+  <si>
+    <t>Nigeria -- Salt-- 100% NRV per average intake</t>
   </si>
 </sst>
 </file>
@@ -686,7 +692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD72"/>
+  <dimension ref="A1:AD90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -1020,7 +1026,7 @@
         <v>320.5427437766894</v>
       </c>
       <c r="G6" s="3">
-        <v>11.4178093054627</v>
+        <v>11.41780930546322</v>
       </c>
       <c r="H6" s="4">
         <f>IF(F6=0,0,G6/F6)</f>
@@ -1060,7 +1066,7 @@
         <v>4138.352740079671</v>
       </c>
       <c r="T6" s="3">
-        <v>147.4091157648745</v>
+        <v>147.4091157648822</v>
       </c>
       <c r="U6" s="4">
         <f>IF(S6=0,0,T6/S6)</f>
@@ -1157,7 +1163,7 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T7" s="3">
-        <v>123.6968790634523</v>
+        <v>123.6968790634528</v>
       </c>
       <c r="U7" s="4">
         <f>IF(S7=0,0,T7/S7)</f>
@@ -1211,10 +1217,10 @@
         <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>271.3548595424364</v>
+        <v>271.3548595424359</v>
       </c>
       <c r="G8" s="3">
-        <v>8.370468320719199</v>
+        <v>8.370468320719258</v>
       </c>
       <c r="H8" s="4">
         <f>IF(F8=0,0,G8/F8)</f>
@@ -1251,10 +1257,10 @@
         <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>3503.314763237015</v>
+        <v>3503.314763237009</v>
       </c>
       <c r="T8" s="3">
-        <v>108.0665564369497</v>
+        <v>108.0665564369501</v>
       </c>
       <c r="U8" s="4">
         <f>IF(S8=0,0,T8/S8)</f>
@@ -1308,10 +1314,10 @@
         <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>231.1015430943892</v>
+        <v>231.1015430943887</v>
       </c>
       <c r="G9" s="3">
-        <v>2.991144416980329</v>
+        <v>2.991144416980678</v>
       </c>
       <c r="H9" s="4">
         <f>IF(F9=0,0,G9/F9)</f>
@@ -1348,10 +1354,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="3">
-        <v>2983.6261237209</v>
+        <v>2983.626123720895</v>
       </c>
       <c r="T9" s="3">
-        <v>38.61703605622006</v>
+        <v>38.61703605622597</v>
       </c>
       <c r="U9" s="4">
         <f>IF(S9=0,0,T9/S9)</f>
@@ -1531,7 +1537,7 @@
         <v>362.8529849538489</v>
       </c>
       <c r="G14" s="3">
-        <v>151.0014963206652</v>
+        <v>151.0014963206656</v>
       </c>
       <c r="H14" s="4">
         <f>IF(F14=0,0,G14/F14)</f>
@@ -1571,7 +1577,7 @@
         <v>4684.597214204819</v>
       </c>
       <c r="T14" s="3">
-        <v>1949.498056615184</v>
+        <v>1949.498056615189</v>
       </c>
       <c r="U14" s="4">
         <f>IF(S14=0,0,T14/S14)</f>
@@ -1725,7 +1731,7 @@
         <v>287.7720482472399</v>
       </c>
       <c r="G16" s="3">
-        <v>110.0570853730647</v>
+        <v>110.057085373065</v>
       </c>
       <c r="H16" s="4">
         <f>IF(F16=0,0,G16/F16)</f>
@@ -1765,7 +1771,7 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T16" s="3">
-        <v>1420.887072508819</v>
+        <v>1420.887072508823</v>
       </c>
       <c r="U16" s="4">
         <f>IF(S16=0,0,T16/S16)</f>
@@ -1819,10 +1825,10 @@
         <v>0</v>
       </c>
       <c r="F17" s="3">
-        <v>271.3548595424364</v>
+        <v>271.3548595424359</v>
       </c>
       <c r="G17" s="3">
-        <v>102.5231161409741</v>
+        <v>102.523116140974</v>
       </c>
       <c r="H17" s="4">
         <f>IF(F17=0,0,G17/F17)</f>
@@ -1859,10 +1865,10 @@
         <v>0</v>
       </c>
       <c r="S17" s="3">
-        <v>3503.314763237015</v>
+        <v>3503.314763237009</v>
       </c>
       <c r="T17" s="3">
-        <v>1323.620100098366</v>
+        <v>1323.620100098364</v>
       </c>
       <c r="U17" s="4">
         <f>IF(S17=0,0,T17/S17)</f>
@@ -1916,10 +1922,10 @@
         <v>0</v>
       </c>
       <c r="F18" s="3">
-        <v>231.1015430943892</v>
+        <v>231.1015430943887</v>
       </c>
       <c r="G18" s="3">
-        <v>67.11521448847459</v>
+        <v>67.11521448847442</v>
       </c>
       <c r="H18" s="4">
         <f>IF(F18=0,0,G18/F18)</f>
@@ -1956,10 +1962,10 @@
         <v>0</v>
       </c>
       <c r="S18" s="3">
-        <v>2983.6261237209</v>
+        <v>2983.626123720895</v>
       </c>
       <c r="T18" s="3">
-        <v>866.487971329369</v>
+        <v>866.4879713293681</v>
       </c>
       <c r="U18" s="4">
         <f>IF(S18=0,0,T18/S18)</f>
@@ -2139,7 +2145,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G23" s="3">
-        <v>153.5338348629944</v>
+        <v>153.5338348629948</v>
       </c>
       <c r="H23" s="4">
         <f>IF(F23=0,0,G23/F23)</f>
@@ -2179,7 +2185,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T23" s="3">
-        <v>4737.225453182307</v>
+        <v>4737.225453182322</v>
       </c>
       <c r="U23" s="4">
         <f>IF(S23=0,0,T23/S23)</f>
@@ -2236,7 +2242,7 @@
         <v>422.0532339939541</v>
       </c>
       <c r="G24" s="3">
-        <v>149.5731184765907</v>
+        <v>149.5731184765912</v>
       </c>
       <c r="H24" s="4">
         <f>IF(F24=0,0,G24/F24)</f>
@@ -2276,7 +2282,7 @@
         <v>13022.28479122008</v>
       </c>
       <c r="T24" s="3">
-        <v>4615.01912325346</v>
+        <v>4615.019123253476</v>
       </c>
       <c r="U24" s="4">
         <f>IF(S24=0,0,T24/S24)</f>
@@ -2373,7 +2379,7 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T25" s="3">
-        <v>3461.751499772323</v>
+        <v>3461.751499772321</v>
       </c>
       <c r="U25" s="4">
         <f>IF(S25=0,0,T25/S25)</f>
@@ -2430,7 +2436,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G26" s="3">
-        <v>86.23155739396391</v>
+        <v>86.23155739396429</v>
       </c>
       <c r="H26" s="4">
         <f>IF(F26=0,0,G26/F26)</f>
@@ -2470,7 +2476,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T26" s="3">
-        <v>2660.640430943183</v>
+        <v>2660.640430943196</v>
       </c>
       <c r="U26" s="4">
         <f>IF(S26=0,0,T26/S26)</f>
@@ -2747,7 +2753,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G32" s="3">
-        <v>31.81246083158365</v>
+        <v>31.81246083158429</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
@@ -2787,7 +2793,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T32" s="3">
-        <v>981.560835201064</v>
+        <v>981.560835201084</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
@@ -3038,7 +3044,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G35" s="3">
-        <v>79.01499632789695</v>
+        <v>79.01499632789736</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
@@ -3078,7 +3084,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T35" s="3">
-        <v>2437.97630744804</v>
+        <v>2437.976307448053</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
@@ -3956,14 +3962,14 @@
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>M50+P50</f>
+        <f>P50+M50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G50" s="3">
-        <v>58.98240259960004</v>
+        <v>58.98240259960006</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
@@ -4003,7 +4009,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T50" s="3">
-        <v>834.748379618052</v>
+        <v>834.7483796180522</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
@@ -4053,14 +4059,14 @@
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>M51+P51</f>
+        <f>P51+M51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
-        <v>147.7607036391234</v>
+        <v>147.7607036391231</v>
       </c>
       <c r="G51" s="3">
-        <v>59.41247823140031</v>
+        <v>59.41247823140037</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
@@ -4097,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="S51" s="3">
-        <v>2091.183174942721</v>
+        <v>2091.183174942718</v>
       </c>
       <c r="T51" s="3">
-        <v>840.835024463559</v>
+        <v>840.8350244635603</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
@@ -4150,14 +4156,14 @@
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>M52+P52</f>
+        <f>P52+M52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G52" s="3">
-        <v>59.19812501773825</v>
+        <v>59.19812501773821</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
@@ -4247,14 +4253,14 @@
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>M53+P53</f>
+        <f>P53+M53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G53" s="3">
-        <v>27.88815467106953</v>
+        <v>27.88815467106969</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
@@ -4294,7 +4300,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T53" s="3">
-        <v>394.6870743846359</v>
+        <v>394.6870743846378</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
@@ -4344,14 +4350,14 @@
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>M54+P54</f>
+        <f>P54+M54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
-        <v>93.49564395607489</v>
+        <v>93.49564395607474</v>
       </c>
       <c r="G54" s="3">
-        <v>16.262542548974</v>
+        <v>16.26254254897413</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
@@ -4388,10 +4394,10 @@
         <v>0</v>
       </c>
       <c r="S54" s="3">
-        <v>1323.196985098892</v>
+        <v>1323.19698509889</v>
       </c>
       <c r="T54" s="3">
-        <v>230.1556132492594</v>
+        <v>230.1556132492615</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>
@@ -4564,7 +4570,7 @@
         <v>0</v>
       </c>
       <c r="E59" s="3">
-        <f>M59+P59</f>
+        <f>P59+M59</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
@@ -4661,14 +4667,14 @@
         <v>0</v>
       </c>
       <c r="E60" s="3">
-        <f>M60+P60</f>
+        <f>P60+M60</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
-        <v>147.7607036391234</v>
+        <v>147.7607036391231</v>
       </c>
       <c r="G60" s="3">
-        <v>102.7420072452102</v>
+        <v>102.74200724521</v>
       </c>
       <c r="H60" s="4">
         <f>IF(F60=0,0,G60/F60)</f>
@@ -4705,10 +4711,10 @@
         <v>0</v>
       </c>
       <c r="S60" s="3">
-        <v>2091.183174942721</v>
+        <v>2091.183174942718</v>
       </c>
       <c r="T60" s="3">
-        <v>1454.056130077464</v>
+        <v>1454.056130077462</v>
       </c>
       <c r="U60" s="4">
         <f>IF(S60=0,0,T60/S60)</f>
@@ -4758,14 +4764,14 @@
         <v>0</v>
       </c>
       <c r="E61" s="3">
-        <f>M61+P61</f>
+        <f>P61+M61</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G61" s="3">
-        <v>97.48822698814803</v>
+        <v>97.488226988148</v>
       </c>
       <c r="H61" s="4">
         <f>IF(F61=0,0,G61/F61)</f>
@@ -4855,14 +4861,14 @@
         <v>0</v>
       </c>
       <c r="E62" s="3">
-        <f>M62+P62</f>
+        <f>P62+M62</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G62" s="3">
-        <v>62.28901992946243</v>
+        <v>62.28901992946252</v>
       </c>
       <c r="H62" s="4">
         <f>IF(F62=0,0,G62/F62)</f>
@@ -4902,7 +4908,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T62" s="3">
-        <v>881.5452772767835</v>
+        <v>881.545277276785</v>
       </c>
       <c r="U62" s="4">
         <f>IF(S62=0,0,T62/S62)</f>
@@ -4952,14 +4958,14 @@
         <v>0</v>
       </c>
       <c r="E63" s="3">
-        <f>M63+P63</f>
+        <f>P63+M63</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
-        <v>93.49564395607489</v>
+        <v>93.49564395607474</v>
       </c>
       <c r="G63" s="3">
-        <v>40.86638015373273</v>
+        <v>40.86638015373266</v>
       </c>
       <c r="H63" s="4">
         <f>IF(F63=0,0,G63/F63)</f>
@@ -4996,10 +5002,10 @@
         <v>0</v>
       </c>
       <c r="S63" s="3">
-        <v>1323.196985098892</v>
+        <v>1323.19698509889</v>
       </c>
       <c r="T63" s="3">
-        <v>578.3613944274123</v>
+        <v>578.3613944274117</v>
       </c>
       <c r="U63" s="4">
         <f>IF(S63=0,0,T63/S63)</f>
@@ -5172,14 +5178,14 @@
         <v>0</v>
       </c>
       <c r="E68" s="3">
-        <f>M68+P68</f>
+        <f>P68+M68</f>
         <v>0</v>
       </c>
       <c r="F68" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G68" s="3">
-        <v>98.37588727255856</v>
+        <v>98.37588727255864</v>
       </c>
       <c r="H68" s="4">
         <f>IF(F68=0,0,G68/F68)</f>
@@ -5219,7 +5225,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T68" s="3">
-        <v>1392.264622581062</v>
+        <v>1392.264622581063</v>
       </c>
       <c r="U68" s="4">
         <f>IF(S68=0,0,T68/S68)</f>
@@ -5269,14 +5275,14 @@
         <v>0</v>
       </c>
       <c r="E69" s="3">
-        <f>M69+P69</f>
+        <f>P69+M69</f>
         <v>0</v>
       </c>
       <c r="F69" s="3">
-        <v>147.7607036391234</v>
+        <v>147.7607036391231</v>
       </c>
       <c r="G69" s="3">
-        <v>96.54985248064214</v>
+        <v>96.54985248064197</v>
       </c>
       <c r="H69" s="4">
         <f>IF(F69=0,0,G69/F69)</f>
@@ -5313,10 +5319,10 @@
         <v>0</v>
       </c>
       <c r="S69" s="3">
-        <v>2091.183174942721</v>
+        <v>2091.183174942718</v>
       </c>
       <c r="T69" s="3">
-        <v>1366.42166745382</v>
+        <v>1366.421667453817</v>
       </c>
       <c r="U69" s="4">
         <f>IF(S69=0,0,T69/S69)</f>
@@ -5366,14 +5372,14 @@
         <v>0</v>
       </c>
       <c r="E70" s="3">
-        <f>M70+P70</f>
+        <f>P70+M70</f>
         <v>0</v>
       </c>
       <c r="F70" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G70" s="3">
-        <v>92.2087189913087</v>
+        <v>92.20871899130873</v>
       </c>
       <c r="H70" s="4">
         <f>IF(F70=0,0,G70/F70)</f>
@@ -5463,7 +5469,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="3">
-        <f>M71+P71</f>
+        <f>P71+M71</f>
         <v>0</v>
       </c>
       <c r="F71" s="3">
@@ -5560,14 +5566,14 @@
         <v>0</v>
       </c>
       <c r="E72" s="3">
-        <f>M72+P72</f>
+        <f>P72+M72</f>
         <v>0</v>
       </c>
       <c r="F72" s="3">
-        <v>93.49564395607489</v>
+        <v>93.49564395607474</v>
       </c>
       <c r="G72" s="3">
-        <v>36.20808203369917</v>
+        <v>36.20808203369902</v>
       </c>
       <c r="H72" s="4">
         <f>IF(F72=0,0,G72/F72)</f>
@@ -5604,10 +5610,10 @@
         <v>0</v>
       </c>
       <c r="S72" s="3">
-        <v>1323.196985098892</v>
+        <v>1323.19698509889</v>
       </c>
       <c r="T72" s="3">
-        <v>512.4348360626602</v>
+        <v>512.4348360626584</v>
       </c>
       <c r="U72" s="4">
         <f>IF(S72=0,0,T72/S72)</f>
@@ -5641,6 +5647,1222 @@
       </c>
       <c r="AD72" s="4">
         <f>IF(AB72=0,0,AC72/AB72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:30">
+      <c r="A74" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="75" spans="1:30">
+      <c r="B75" t="s">
+        <v>28</v>
+      </c>
+      <c r="C75" s="3">
+        <f>C77+C78+C79+C80+C81</f>
+        <v>0</v>
+      </c>
+      <c r="D75" s="3">
+        <f>D77+D78+D79+D80+D81</f>
+        <v>0</v>
+      </c>
+      <c r="E75" s="3">
+        <f>E77+E78+E79+E80+E81</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="3">
+        <f>F77+F78+F79+F80+F81</f>
+        <v>0</v>
+      </c>
+      <c r="G75" s="3">
+        <f>G77+G78+G79+G80+G81</f>
+        <v>0</v>
+      </c>
+      <c r="H75" s="4">
+        <f>IF(F75=0,0,G75/F75)</f>
+        <v>0</v>
+      </c>
+      <c r="I75" s="3">
+        <f>I77+I78+I79+I80+I81</f>
+        <v>0</v>
+      </c>
+      <c r="J75" s="3">
+        <f>J77+J78+J79+J80+J81</f>
+        <v>0</v>
+      </c>
+      <c r="K75" s="4">
+        <f>IF(I75=0,0,J75/I75)</f>
+        <v>0</v>
+      </c>
+      <c r="L75" s="3">
+        <f>L77+L78+L79+L80+L81</f>
+        <v>0</v>
+      </c>
+      <c r="M75" s="3">
+        <f>M77+M78+M79+M80+M81</f>
+        <v>0</v>
+      </c>
+      <c r="N75" s="4">
+        <f>IF(L75=0,0,M75/L75)</f>
+        <v>0</v>
+      </c>
+      <c r="O75" s="3">
+        <f>O77+O78+O79+O80+O81</f>
+        <v>0</v>
+      </c>
+      <c r="P75" s="3">
+        <f>P77+P78+P79+P80+P81</f>
+        <v>0</v>
+      </c>
+      <c r="Q75" s="4">
+        <f>IF(O75=0,0,P75/O75)</f>
+        <v>0</v>
+      </c>
+      <c r="S75" s="3">
+        <f>S77+S78+S79+S80+S81</f>
+        <v>0</v>
+      </c>
+      <c r="T75" s="3">
+        <f>T77+T78+T79+T80+T81</f>
+        <v>0</v>
+      </c>
+      <c r="U75" s="4">
+        <f>IF(S75=0,0,T75/S75)</f>
+        <v>0</v>
+      </c>
+      <c r="V75" s="3">
+        <f>V77+V78+V79+V80+V81</f>
+        <v>0</v>
+      </c>
+      <c r="W75" s="3">
+        <f>W77+W78+W79+W80+W81</f>
+        <v>0</v>
+      </c>
+      <c r="X75" s="4">
+        <f>IF(V75=0,0,W75/V75)</f>
+        <v>0</v>
+      </c>
+      <c r="Y75" s="3">
+        <f>Y77+Y78+Y79+Y80+Y81</f>
+        <v>0</v>
+      </c>
+      <c r="Z75" s="3">
+        <f>Z77+Z78+Z79+Z80+Z81</f>
+        <v>0</v>
+      </c>
+      <c r="AA75" s="4">
+        <f>IF(Y75=0,0,Z75/Y75)</f>
+        <v>0</v>
+      </c>
+      <c r="AB75" s="3">
+        <f>AB77+AB78+AB79+AB80+AB81</f>
+        <v>0</v>
+      </c>
+      <c r="AC75" s="3">
+        <f>AC77+AC78+AC79+AC80+AC81</f>
+        <v>0</v>
+      </c>
+      <c r="AD75" s="4">
+        <f>IF(AB75=0,0,AC75/AB75)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:30">
+      <c r="A76" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="77" spans="1:30">
+      <c r="B77" t="s">
+        <v>30</v>
+      </c>
+      <c r="C77" s="3">
+        <f>J77+M77+G77+P77</f>
+        <v>0</v>
+      </c>
+      <c r="D77" s="3">
+        <f>G77</f>
+        <v>0</v>
+      </c>
+      <c r="E77" s="3">
+        <f>J77+M77+P77</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="3">
+        <v>412.7408750394843</v>
+      </c>
+      <c r="G77" s="3">
+        <v>146.8879599840255</v>
+      </c>
+      <c r="H77" s="4">
+        <f>IF(F77=0,0,G77/F77)</f>
+        <v>0</v>
+      </c>
+      <c r="I77" s="3">
+        <v>0</v>
+      </c>
+      <c r="J77" s="3">
+        <v>0</v>
+      </c>
+      <c r="K77" s="4">
+        <f>IF(I77=0,0,J77/I77)</f>
+        <v>0</v>
+      </c>
+      <c r="L77" s="3">
+        <v>0</v>
+      </c>
+      <c r="M77" s="3">
+        <v>0</v>
+      </c>
+      <c r="N77" s="4">
+        <f>IF(L77=0,0,M77/L77)</f>
+        <v>0</v>
+      </c>
+      <c r="O77" s="3">
+        <v>0</v>
+      </c>
+      <c r="P77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="4">
+        <f>IF(O77=0,0,P77/O77)</f>
+        <v>0</v>
+      </c>
+      <c r="S77" s="3">
+        <v>12734.95565684622</v>
+      </c>
+      <c r="T77" s="3">
+        <v>4532.169625172735</v>
+      </c>
+      <c r="U77" s="4">
+        <f>IF(S77=0,0,T77/S77)</f>
+        <v>0</v>
+      </c>
+      <c r="V77" s="3">
+        <v>0</v>
+      </c>
+      <c r="W77" s="3">
+        <v>0</v>
+      </c>
+      <c r="X77" s="4">
+        <f>IF(V77=0,0,W77/V77)</f>
+        <v>0</v>
+      </c>
+      <c r="Y77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="4">
+        <f>IF(Y77=0,0,Z77/Y77)</f>
+        <v>0</v>
+      </c>
+      <c r="AB77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD77" s="4">
+        <f>IF(AB77=0,0,AC77/AB77)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:30">
+      <c r="B78" t="s">
+        <v>31</v>
+      </c>
+      <c r="C78" s="3">
+        <f>J78+M78+G78+P78</f>
+        <v>0</v>
+      </c>
+      <c r="D78" s="3">
+        <f>G78</f>
+        <v>0</v>
+      </c>
+      <c r="E78" s="3">
+        <f>J78+M78+P78</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="3">
+        <v>422.0532339939541</v>
+      </c>
+      <c r="G78" s="3">
+        <v>141.7344183926904</v>
+      </c>
+      <c r="H78" s="4">
+        <f>IF(F78=0,0,G78/F78)</f>
+        <v>0</v>
+      </c>
+      <c r="I78" s="3">
+        <v>0</v>
+      </c>
+      <c r="J78" s="3">
+        <v>0</v>
+      </c>
+      <c r="K78" s="4">
+        <f>IF(I78=0,0,J78/I78)</f>
+        <v>0</v>
+      </c>
+      <c r="L78" s="3">
+        <v>0</v>
+      </c>
+      <c r="M78" s="3">
+        <v>0</v>
+      </c>
+      <c r="N78" s="4">
+        <f>IF(L78=0,0,M78/L78)</f>
+        <v>0</v>
+      </c>
+      <c r="O78" s="3">
+        <v>0</v>
+      </c>
+      <c r="P78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="4">
+        <f>IF(O78=0,0,P78/O78)</f>
+        <v>0</v>
+      </c>
+      <c r="S78" s="3">
+        <v>13022.28479122008</v>
+      </c>
+      <c r="T78" s="3">
+        <v>4373.159147630166</v>
+      </c>
+      <c r="U78" s="4">
+        <f>IF(S78=0,0,T78/S78)</f>
+        <v>0</v>
+      </c>
+      <c r="V78" s="3">
+        <v>0</v>
+      </c>
+      <c r="W78" s="3">
+        <v>0</v>
+      </c>
+      <c r="X78" s="4">
+        <f>IF(V78=0,0,W78/V78)</f>
+        <v>0</v>
+      </c>
+      <c r="Y78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="4">
+        <f>IF(Y78=0,0,Z78/Y78)</f>
+        <v>0</v>
+      </c>
+      <c r="AB78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD78" s="4">
+        <f>IF(AB78=0,0,AC78/AB78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:30">
+      <c r="B79" t="s">
+        <v>32</v>
+      </c>
+      <c r="C79" s="3">
+        <f>J79+M79+G79+P79</f>
+        <v>0</v>
+      </c>
+      <c r="D79" s="3">
+        <f>G79</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="3">
+        <f>J79+M79+P79</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="3">
+        <v>382.0743136549376</v>
+      </c>
+      <c r="G79" s="3">
+        <v>124.6559480289836</v>
+      </c>
+      <c r="H79" s="4">
+        <f>IF(F79=0,0,G79/F79)</f>
+        <v>0</v>
+      </c>
+      <c r="I79" s="3">
+        <v>0</v>
+      </c>
+      <c r="J79" s="3">
+        <v>0</v>
+      </c>
+      <c r="K79" s="4">
+        <f>IF(I79=0,0,J79/I79)</f>
+        <v>0</v>
+      </c>
+      <c r="L79" s="3">
+        <v>0</v>
+      </c>
+      <c r="M79" s="3">
+        <v>0</v>
+      </c>
+      <c r="N79" s="4">
+        <f>IF(L79=0,0,M79/L79)</f>
+        <v>0</v>
+      </c>
+      <c r="O79" s="3">
+        <v>0</v>
+      </c>
+      <c r="P79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="4">
+        <f>IF(O79=0,0,P79/O79)</f>
+        <v>0</v>
+      </c>
+      <c r="S79" s="3">
+        <v>11788.75109364953</v>
+      </c>
+      <c r="T79" s="3">
+        <v>3846.209732339612</v>
+      </c>
+      <c r="U79" s="4">
+        <f>IF(S79=0,0,T79/S79)</f>
+        <v>0</v>
+      </c>
+      <c r="V79" s="3">
+        <v>0</v>
+      </c>
+      <c r="W79" s="3">
+        <v>0</v>
+      </c>
+      <c r="X79" s="4">
+        <f>IF(V79=0,0,W79/V79)</f>
+        <v>0</v>
+      </c>
+      <c r="Y79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="4">
+        <f>IF(Y79=0,0,Z79/Y79)</f>
+        <v>0</v>
+      </c>
+      <c r="AB79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD79" s="4">
+        <f>IF(AB79=0,0,AC79/AB79)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:30">
+      <c r="B80" t="s">
+        <v>33</v>
+      </c>
+      <c r="C80" s="3">
+        <f>J80+M80+G80+P80</f>
+        <v>0</v>
+      </c>
+      <c r="D80" s="3">
+        <f>G80</f>
+        <v>0</v>
+      </c>
+      <c r="E80" s="3">
+        <f>J80+M80+P80</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="3">
+        <v>338.6701578384149</v>
+      </c>
+      <c r="G80" s="3">
+        <v>106.5823973125179</v>
+      </c>
+      <c r="H80" s="4">
+        <f>IF(F80=0,0,G80/F80)</f>
+        <v>0</v>
+      </c>
+      <c r="I80" s="3">
+        <v>0</v>
+      </c>
+      <c r="J80" s="3">
+        <v>0</v>
+      </c>
+      <c r="K80" s="4">
+        <f>IF(I80=0,0,J80/I80)</f>
+        <v>0</v>
+      </c>
+      <c r="L80" s="3">
+        <v>0</v>
+      </c>
+      <c r="M80" s="3">
+        <v>0</v>
+      </c>
+      <c r="N80" s="4">
+        <f>IF(L80=0,0,M80/L80)</f>
+        <v>0</v>
+      </c>
+      <c r="O80" s="3">
+        <v>0</v>
+      </c>
+      <c r="P80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="4">
+        <f>IF(O80=0,0,P80/O80)</f>
+        <v>0</v>
+      </c>
+      <c r="S80" s="3">
+        <v>10449.53311676904</v>
+      </c>
+      <c r="T80" s="3">
+        <v>3288.557508256084</v>
+      </c>
+      <c r="U80" s="4">
+        <f>IF(S80=0,0,T80/S80)</f>
+        <v>0</v>
+      </c>
+      <c r="V80" s="3">
+        <v>0</v>
+      </c>
+      <c r="W80" s="3">
+        <v>0</v>
+      </c>
+      <c r="X80" s="4">
+        <f>IF(V80=0,0,W80/V80)</f>
+        <v>0</v>
+      </c>
+      <c r="Y80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="4">
+        <f>IF(Y80=0,0,Z80/Y80)</f>
+        <v>0</v>
+      </c>
+      <c r="AB80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD80" s="4">
+        <f>IF(AB80=0,0,AC80/AB80)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:30">
+      <c r="B81" t="s">
+        <v>34</v>
+      </c>
+      <c r="C81" s="3">
+        <f>J81+M81+G81+P81</f>
+        <v>0</v>
+      </c>
+      <c r="D81" s="3">
+        <f>G81</f>
+        <v>0</v>
+      </c>
+      <c r="E81" s="3">
+        <f>J81+M81+P81</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="3">
+        <v>297.4602934996698</v>
+      </c>
+      <c r="G81" s="3">
+        <v>93.75383596516214</v>
+      </c>
+      <c r="H81" s="4">
+        <f>IF(F81=0,0,G81/F81)</f>
+        <v>0</v>
+      </c>
+      <c r="I81" s="3">
+        <v>0</v>
+      </c>
+      <c r="J81" s="3">
+        <v>0</v>
+      </c>
+      <c r="K81" s="4">
+        <f>IF(I81=0,0,J81/I81)</f>
+        <v>0</v>
+      </c>
+      <c r="L81" s="3">
+        <v>0</v>
+      </c>
+      <c r="M81" s="3">
+        <v>0</v>
+      </c>
+      <c r="N81" s="4">
+        <f>IF(L81=0,0,M81/L81)</f>
+        <v>0</v>
+      </c>
+      <c r="O81" s="3">
+        <v>0</v>
+      </c>
+      <c r="P81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q81" s="4">
+        <f>IF(O81=0,0,P81/O81)</f>
+        <v>0</v>
+      </c>
+      <c r="S81" s="3">
+        <v>9178.019131321482</v>
+      </c>
+      <c r="T81" s="3">
+        <v>2892.73734655274</v>
+      </c>
+      <c r="U81" s="4">
+        <f>IF(S81=0,0,T81/S81)</f>
+        <v>0</v>
+      </c>
+      <c r="V81" s="3">
+        <v>0</v>
+      </c>
+      <c r="W81" s="3">
+        <v>0</v>
+      </c>
+      <c r="X81" s="4">
+        <f>IF(V81=0,0,W81/V81)</f>
+        <v>0</v>
+      </c>
+      <c r="Y81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="4">
+        <f>IF(Y81=0,0,Z81/Y81)</f>
+        <v>0</v>
+      </c>
+      <c r="AB81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD81" s="4">
+        <f>IF(AB81=0,0,AC81/AB81)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:30">
+      <c r="A83" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="84" spans="1:30">
+      <c r="B84" t="s">
+        <v>28</v>
+      </c>
+      <c r="C84" s="3">
+        <f>C86+C87+C88+C89+C90</f>
+        <v>0</v>
+      </c>
+      <c r="D84" s="3">
+        <f>D86+D87+D88+D89+D90</f>
+        <v>0</v>
+      </c>
+      <c r="E84" s="3">
+        <f>E86+E87+E88+E89+E90</f>
+        <v>0</v>
+      </c>
+      <c r="F84" s="3">
+        <f>F86+F87+F88+F89+F90</f>
+        <v>0</v>
+      </c>
+      <c r="G84" s="3">
+        <f>G86+G87+G88+G89+G90</f>
+        <v>0</v>
+      </c>
+      <c r="H84" s="4">
+        <f>IF(F84=0,0,G84/F84)</f>
+        <v>0</v>
+      </c>
+      <c r="I84" s="3">
+        <f>I86+I87+I88+I89+I90</f>
+        <v>0</v>
+      </c>
+      <c r="J84" s="3">
+        <f>J86+J87+J88+J89+J90</f>
+        <v>0</v>
+      </c>
+      <c r="K84" s="4">
+        <f>IF(I84=0,0,J84/I84)</f>
+        <v>0</v>
+      </c>
+      <c r="L84" s="3">
+        <f>L86+L87+L88+L89+L90</f>
+        <v>0</v>
+      </c>
+      <c r="M84" s="3">
+        <f>M86+M87+M88+M89+M90</f>
+        <v>0</v>
+      </c>
+      <c r="N84" s="4">
+        <f>IF(L84=0,0,M84/L84)</f>
+        <v>0</v>
+      </c>
+      <c r="O84" s="3">
+        <f>O86+O87+O88+O89+O90</f>
+        <v>0</v>
+      </c>
+      <c r="P84" s="3">
+        <f>P86+P87+P88+P89+P90</f>
+        <v>0</v>
+      </c>
+      <c r="Q84" s="4">
+        <f>IF(O84=0,0,P84/O84)</f>
+        <v>0</v>
+      </c>
+      <c r="S84" s="3">
+        <f>S86+S87+S88+S89+S90</f>
+        <v>0</v>
+      </c>
+      <c r="T84" s="3">
+        <f>T86+T87+T88+T89+T90</f>
+        <v>0</v>
+      </c>
+      <c r="U84" s="4">
+        <f>IF(S84=0,0,T84/S84)</f>
+        <v>0</v>
+      </c>
+      <c r="V84" s="3">
+        <f>V86+V87+V88+V89+V90</f>
+        <v>0</v>
+      </c>
+      <c r="W84" s="3">
+        <f>W86+W87+W88+W89+W90</f>
+        <v>0</v>
+      </c>
+      <c r="X84" s="4">
+        <f>IF(V84=0,0,W84/V84)</f>
+        <v>0</v>
+      </c>
+      <c r="Y84" s="3">
+        <f>Y86+Y87+Y88+Y89+Y90</f>
+        <v>0</v>
+      </c>
+      <c r="Z84" s="3">
+        <f>Z86+Z87+Z88+Z89+Z90</f>
+        <v>0</v>
+      </c>
+      <c r="AA84" s="4">
+        <f>IF(Y84=0,0,Z84/Y84)</f>
+        <v>0</v>
+      </c>
+      <c r="AB84" s="3">
+        <f>AB86+AB87+AB88+AB89+AB90</f>
+        <v>0</v>
+      </c>
+      <c r="AC84" s="3">
+        <f>AC86+AC87+AC88+AC89+AC90</f>
+        <v>0</v>
+      </c>
+      <c r="AD84" s="4">
+        <f>IF(AB84=0,0,AC84/AB84)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:30">
+      <c r="A85" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="86" spans="1:30">
+      <c r="B86" t="s">
+        <v>30</v>
+      </c>
+      <c r="C86" s="3">
+        <f>J86+M86+G86+P86</f>
+        <v>0</v>
+      </c>
+      <c r="D86" s="3">
+        <f>G86</f>
+        <v>0</v>
+      </c>
+      <c r="E86" s="3">
+        <f>J86+M86+P86</f>
+        <v>0</v>
+      </c>
+      <c r="F86" s="3">
+        <v>412.7408750394843</v>
+      </c>
+      <c r="G86" s="3">
+        <v>270.621528830763</v>
+      </c>
+      <c r="H86" s="4">
+        <f>IF(F86=0,0,G86/F86)</f>
+        <v>0</v>
+      </c>
+      <c r="I86" s="3">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3">
+        <v>0</v>
+      </c>
+      <c r="K86" s="4">
+        <f>IF(I86=0,0,J86/I86)</f>
+        <v>0</v>
+      </c>
+      <c r="L86" s="3">
+        <v>0</v>
+      </c>
+      <c r="M86" s="3">
+        <v>0</v>
+      </c>
+      <c r="N86" s="4">
+        <f>IF(L86=0,0,M86/L86)</f>
+        <v>0</v>
+      </c>
+      <c r="O86" s="3">
+        <v>0</v>
+      </c>
+      <c r="P86" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="4">
+        <f>IF(O86=0,0,P86/O86)</f>
+        <v>0</v>
+      </c>
+      <c r="S86" s="3">
+        <v>12734.95565684622</v>
+      </c>
+      <c r="T86" s="3">
+        <v>8349.919714440704</v>
+      </c>
+      <c r="U86" s="4">
+        <f>IF(S86=0,0,T86/S86)</f>
+        <v>0</v>
+      </c>
+      <c r="V86" s="3">
+        <v>0</v>
+      </c>
+      <c r="W86" s="3">
+        <v>0</v>
+      </c>
+      <c r="X86" s="4">
+        <f>IF(V86=0,0,W86/V86)</f>
+        <v>0</v>
+      </c>
+      <c r="Y86" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z86" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA86" s="4">
+        <f>IF(Y86=0,0,Z86/Y86)</f>
+        <v>0</v>
+      </c>
+      <c r="AB86" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC86" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD86" s="4">
+        <f>IF(AB86=0,0,AC86/AB86)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:30">
+      <c r="B87" t="s">
+        <v>31</v>
+      </c>
+      <c r="C87" s="3">
+        <f>J87+M87+G87+P87</f>
+        <v>0</v>
+      </c>
+      <c r="D87" s="3">
+        <f>G87</f>
+        <v>0</v>
+      </c>
+      <c r="E87" s="3">
+        <f>J87+M87+P87</f>
+        <v>0</v>
+      </c>
+      <c r="F87" s="3">
+        <v>422.0532339939541</v>
+      </c>
+      <c r="G87" s="3">
+        <v>268.8415075664349</v>
+      </c>
+      <c r="H87" s="4">
+        <f>IF(F87=0,0,G87/F87)</f>
+        <v>0</v>
+      </c>
+      <c r="I87" s="3">
+        <v>0</v>
+      </c>
+      <c r="J87" s="3">
+        <v>0</v>
+      </c>
+      <c r="K87" s="4">
+        <f>IF(I87=0,0,J87/I87)</f>
+        <v>0</v>
+      </c>
+      <c r="L87" s="3">
+        <v>0</v>
+      </c>
+      <c r="M87" s="3">
+        <v>0</v>
+      </c>
+      <c r="N87" s="4">
+        <f>IF(L87=0,0,M87/L87)</f>
+        <v>0</v>
+      </c>
+      <c r="O87" s="3">
+        <v>0</v>
+      </c>
+      <c r="P87" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q87" s="4">
+        <f>IF(O87=0,0,P87/O87)</f>
+        <v>0</v>
+      </c>
+      <c r="S87" s="3">
+        <v>13022.28479122008</v>
+      </c>
+      <c r="T87" s="3">
+        <v>8294.997865793428</v>
+      </c>
+      <c r="U87" s="4">
+        <f>IF(S87=0,0,T87/S87)</f>
+        <v>0</v>
+      </c>
+      <c r="V87" s="3">
+        <v>0</v>
+      </c>
+      <c r="W87" s="3">
+        <v>0</v>
+      </c>
+      <c r="X87" s="4">
+        <f>IF(V87=0,0,W87/V87)</f>
+        <v>0</v>
+      </c>
+      <c r="Y87" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA87" s="4">
+        <f>IF(Y87=0,0,Z87/Y87)</f>
+        <v>0</v>
+      </c>
+      <c r="AB87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD87" s="4">
+        <f>IF(AB87=0,0,AC87/AB87)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:30">
+      <c r="B88" t="s">
+        <v>32</v>
+      </c>
+      <c r="C88" s="3">
+        <f>J88+M88+G88+P88</f>
+        <v>0</v>
+      </c>
+      <c r="D88" s="3">
+        <f>G88</f>
+        <v>0</v>
+      </c>
+      <c r="E88" s="3">
+        <f>J88+M88+P88</f>
+        <v>0</v>
+      </c>
+      <c r="F88" s="3">
+        <v>382.0743136549376</v>
+      </c>
+      <c r="G88" s="3">
+        <v>239.83782878063</v>
+      </c>
+      <c r="H88" s="4">
+        <f>IF(F88=0,0,G88/F88)</f>
+        <v>0</v>
+      </c>
+      <c r="I88" s="3">
+        <v>0</v>
+      </c>
+      <c r="J88" s="3">
+        <v>0</v>
+      </c>
+      <c r="K88" s="4">
+        <f>IF(I88=0,0,J88/I88)</f>
+        <v>0</v>
+      </c>
+      <c r="L88" s="3">
+        <v>0</v>
+      </c>
+      <c r="M88" s="3">
+        <v>0</v>
+      </c>
+      <c r="N88" s="4">
+        <f>IF(L88=0,0,M88/L88)</f>
+        <v>0</v>
+      </c>
+      <c r="O88" s="3">
+        <v>0</v>
+      </c>
+      <c r="P88" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="4">
+        <f>IF(O88=0,0,P88/O88)</f>
+        <v>0</v>
+      </c>
+      <c r="S88" s="3">
+        <v>11788.75109364953</v>
+      </c>
+      <c r="T88" s="3">
+        <v>7400.100884273723</v>
+      </c>
+      <c r="U88" s="4">
+        <f>IF(S88=0,0,T88/S88)</f>
+        <v>0</v>
+      </c>
+      <c r="V88" s="3">
+        <v>0</v>
+      </c>
+      <c r="W88" s="3">
+        <v>0</v>
+      </c>
+      <c r="X88" s="4">
+        <f>IF(V88=0,0,W88/V88)</f>
+        <v>0</v>
+      </c>
+      <c r="Y88" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z88" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA88" s="4">
+        <f>IF(Y88=0,0,Z88/Y88)</f>
+        <v>0</v>
+      </c>
+      <c r="AB88" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC88" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD88" s="4">
+        <f>IF(AB88=0,0,AC88/AB88)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:30">
+      <c r="B89" t="s">
+        <v>33</v>
+      </c>
+      <c r="C89" s="3">
+        <f>J89+M89+G89+P89</f>
+        <v>0</v>
+      </c>
+      <c r="D89" s="3">
+        <f>G89</f>
+        <v>0</v>
+      </c>
+      <c r="E89" s="3">
+        <f>J89+M89+P89</f>
+        <v>0</v>
+      </c>
+      <c r="F89" s="3">
+        <v>338.6701578384149</v>
+      </c>
+      <c r="G89" s="3">
+        <v>208.6917795068874</v>
+      </c>
+      <c r="H89" s="4">
+        <f>IF(F89=0,0,G89/F89)</f>
+        <v>0</v>
+      </c>
+      <c r="I89" s="3">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3">
+        <v>0</v>
+      </c>
+      <c r="K89" s="4">
+        <f>IF(I89=0,0,J89/I89)</f>
+        <v>0</v>
+      </c>
+      <c r="L89" s="3">
+        <v>0</v>
+      </c>
+      <c r="M89" s="3">
+        <v>0</v>
+      </c>
+      <c r="N89" s="4">
+        <f>IF(L89=0,0,M89/L89)</f>
+        <v>0</v>
+      </c>
+      <c r="O89" s="3">
+        <v>0</v>
+      </c>
+      <c r="P89" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q89" s="4">
+        <f>IF(O89=0,0,P89/O89)</f>
+        <v>0</v>
+      </c>
+      <c r="S89" s="3">
+        <v>10449.53311676904</v>
+      </c>
+      <c r="T89" s="3">
+        <v>6439.101912826773</v>
+      </c>
+      <c r="U89" s="4">
+        <f>IF(S89=0,0,T89/S89)</f>
+        <v>0</v>
+      </c>
+      <c r="V89" s="3">
+        <v>0</v>
+      </c>
+      <c r="W89" s="3">
+        <v>0</v>
+      </c>
+      <c r="X89" s="4">
+        <f>IF(V89=0,0,W89/V89)</f>
+        <v>0</v>
+      </c>
+      <c r="Y89" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA89" s="4">
+        <f>IF(Y89=0,0,Z89/Y89)</f>
+        <v>0</v>
+      </c>
+      <c r="AB89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC89" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD89" s="4">
+        <f>IF(AB89=0,0,AC89/AB89)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:30">
+      <c r="B90" t="s">
+        <v>34</v>
+      </c>
+      <c r="C90" s="3">
+        <f>J90+M90+G90+P90</f>
+        <v>0</v>
+      </c>
+      <c r="D90" s="3">
+        <f>G90</f>
+        <v>0</v>
+      </c>
+      <c r="E90" s="3">
+        <f>J90+M90+P90</f>
+        <v>0</v>
+      </c>
+      <c r="F90" s="3">
+        <v>297.4602934996698</v>
+      </c>
+      <c r="G90" s="3">
+        <v>183.4401220978906</v>
+      </c>
+      <c r="H90" s="4">
+        <f>IF(F90=0,0,G90/F90)</f>
+        <v>0</v>
+      </c>
+      <c r="I90" s="3">
+        <v>0</v>
+      </c>
+      <c r="J90" s="3">
+        <v>0</v>
+      </c>
+      <c r="K90" s="4">
+        <f>IF(I90=0,0,J90/I90)</f>
+        <v>0</v>
+      </c>
+      <c r="L90" s="3">
+        <v>0</v>
+      </c>
+      <c r="M90" s="3">
+        <v>0</v>
+      </c>
+      <c r="N90" s="4">
+        <f>IF(L90=0,0,M90/L90)</f>
+        <v>0</v>
+      </c>
+      <c r="O90" s="3">
+        <v>0</v>
+      </c>
+      <c r="P90" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="4">
+        <f>IF(O90=0,0,P90/O90)</f>
+        <v>0</v>
+      </c>
+      <c r="S90" s="3">
+        <v>9178.019131321482</v>
+      </c>
+      <c r="T90" s="3">
+        <v>5659.972059659981</v>
+      </c>
+      <c r="U90" s="4">
+        <f>IF(S90=0,0,T90/S90)</f>
+        <v>0</v>
+      </c>
+      <c r="V90" s="3">
+        <v>0</v>
+      </c>
+      <c r="W90" s="3">
+        <v>0</v>
+      </c>
+      <c r="X90" s="4">
+        <f>IF(V90=0,0,W90/V90)</f>
+        <v>0</v>
+      </c>
+      <c r="Y90" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z90" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="4">
+        <f>IF(Y90=0,0,Z90/Y90)</f>
+        <v>0</v>
+      </c>
+      <c r="AB90" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC90" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD90" s="4">
+        <f>IF(AB90=0,0,AC90/AB90)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
run snakemake with updated data
</commit_message>
<xml_diff>
--- a/5000_analyze_results/results_spreadsheet.xlsx
+++ b/5000_analyze_results/results_spreadsheet.xlsx
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="42">
   <si>
     <t>DALYs Averted by Fortification (1000s)</t>
   </si>
@@ -306,12 +306,6 @@
   </si>
   <si>
     <t>Ethiopia -- Salt-- DFS-IoFA preliminary standard 45 ppm</t>
-  </si>
-  <si>
-    <t>Nigeria -- Salt-- 25% NRV per average intake</t>
-  </si>
-  <si>
-    <t>Nigeria -- Salt-- 100% NRV per average intake</t>
   </si>
 </sst>
 </file>
@@ -692,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD90"/>
+  <dimension ref="A1:AD72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -939,7 +933,7 @@
         <v>4771.261231090824</v>
       </c>
       <c r="J5" s="3">
-        <v>288.4337566118371</v>
+        <v>288.4337566118361</v>
       </c>
       <c r="K5" s="4">
         <f>IF(I5=0,0,J5/I5)</f>
@@ -1026,7 +1020,7 @@
         <v>320.5427437766894</v>
       </c>
       <c r="G6" s="3">
-        <v>11.41780930546322</v>
+        <v>11.4178093054627</v>
       </c>
       <c r="H6" s="4">
         <f>IF(F6=0,0,G6/F6)</f>
@@ -1036,7 +1030,7 @@
         <v>4315.21265961095</v>
       </c>
       <c r="J6" s="3">
-        <v>254.1003600447951</v>
+        <v>254.1003600447956</v>
       </c>
       <c r="K6" s="4">
         <f>IF(I6=0,0,J6/I6)</f>
@@ -1066,7 +1060,7 @@
         <v>4138.352740079671</v>
       </c>
       <c r="T6" s="3">
-        <v>147.4091157648822</v>
+        <v>147.4091157648745</v>
       </c>
       <c r="U6" s="4">
         <f>IF(S6=0,0,T6/S6)</f>
@@ -1130,10 +1124,10 @@
         <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>4220.06501252761</v>
+        <v>4220.065012527612</v>
       </c>
       <c r="J7" s="3">
-        <v>227.9834892376829</v>
+        <v>227.9834892376838</v>
       </c>
       <c r="K7" s="4">
         <f>IF(I7=0,0,J7/I7)</f>
@@ -1163,7 +1157,7 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T7" s="3">
-        <v>123.6968790634528</v>
+        <v>123.6968790634523</v>
       </c>
       <c r="U7" s="4">
         <f>IF(S7=0,0,T7/S7)</f>
@@ -1217,10 +1211,10 @@
         <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>271.3548595424359</v>
+        <v>271.3548595424364</v>
       </c>
       <c r="G8" s="3">
-        <v>8.370468320719258</v>
+        <v>8.370468320719199</v>
       </c>
       <c r="H8" s="4">
         <f>IF(F8=0,0,G8/F8)</f>
@@ -1230,7 +1224,7 @@
         <v>3866.462901477351</v>
       </c>
       <c r="J8" s="3">
-        <v>196.4668003082145</v>
+        <v>196.466800308214</v>
       </c>
       <c r="K8" s="4">
         <f>IF(I8=0,0,J8/I8)</f>
@@ -1257,10 +1251,10 @@
         <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>3503.314763237009</v>
+        <v>3503.314763237015</v>
       </c>
       <c r="T8" s="3">
-        <v>108.0665564369501</v>
+        <v>108.0665564369497</v>
       </c>
       <c r="U8" s="4">
         <f>IF(S8=0,0,T8/S8)</f>
@@ -1314,20 +1308,20 @@
         <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>231.1015430943887</v>
+        <v>231.1015430943892</v>
       </c>
       <c r="G9" s="3">
-        <v>2.991144416980678</v>
+        <v>2.991144416980329</v>
       </c>
       <c r="H9" s="4">
         <f>IF(F9=0,0,G9/F9)</f>
         <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>3364.297008165506</v>
+        <v>3364.297008165505</v>
       </c>
       <c r="J9" s="3">
-        <v>97.6682430201457</v>
+        <v>97.66824302014476</v>
       </c>
       <c r="K9" s="4">
         <f>IF(I9=0,0,J9/I9)</f>
@@ -1354,10 +1348,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="3">
-        <v>2983.626123720895</v>
+        <v>2983.6261237209</v>
       </c>
       <c r="T9" s="3">
-        <v>38.61703605622597</v>
+        <v>38.61703605622006</v>
       </c>
       <c r="U9" s="4">
         <f>IF(S9=0,0,T9/S9)</f>
@@ -1537,7 +1531,7 @@
         <v>362.8529849538489</v>
       </c>
       <c r="G14" s="3">
-        <v>151.0014963206656</v>
+        <v>151.0014963206652</v>
       </c>
       <c r="H14" s="4">
         <f>IF(F14=0,0,G14/F14)</f>
@@ -1577,7 +1571,7 @@
         <v>4684.597214204819</v>
       </c>
       <c r="T14" s="3">
-        <v>1949.498056615189</v>
+        <v>1949.498056615184</v>
       </c>
       <c r="U14" s="4">
         <f>IF(S14=0,0,T14/S14)</f>
@@ -1587,7 +1581,7 @@
         <v>131696392.1412486</v>
       </c>
       <c r="W14" s="3">
-        <v>10296243.37165025</v>
+        <v>10296243.37165028</v>
       </c>
       <c r="X14" s="4">
         <f>IF(V14=0,0,W14/V14)</f>
@@ -1644,7 +1638,7 @@
         <v>4315.21265961095</v>
       </c>
       <c r="J15" s="3">
-        <v>433.8825937981484</v>
+        <v>433.8825937981489</v>
       </c>
       <c r="K15" s="4">
         <f>IF(I15=0,0,J15/I15)</f>
@@ -1731,17 +1725,17 @@
         <v>287.7720482472399</v>
       </c>
       <c r="G16" s="3">
-        <v>110.057085373065</v>
+        <v>110.0570853730647</v>
       </c>
       <c r="H16" s="4">
         <f>IF(F16=0,0,G16/F16)</f>
         <v>0</v>
       </c>
       <c r="I16" s="3">
-        <v>4220.06501252761</v>
+        <v>4220.065012527612</v>
       </c>
       <c r="J16" s="3">
-        <v>424.92094389637</v>
+        <v>424.9209438963709</v>
       </c>
       <c r="K16" s="4">
         <f>IF(I16=0,0,J16/I16)</f>
@@ -1771,7 +1765,7 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T16" s="3">
-        <v>1420.887072508823</v>
+        <v>1420.887072508819</v>
       </c>
       <c r="U16" s="4">
         <f>IF(S16=0,0,T16/S16)</f>
@@ -1825,10 +1819,10 @@
         <v>0</v>
       </c>
       <c r="F17" s="3">
-        <v>271.3548595424359</v>
+        <v>271.3548595424364</v>
       </c>
       <c r="G17" s="3">
-        <v>102.523116140974</v>
+        <v>102.5231161409741</v>
       </c>
       <c r="H17" s="4">
         <f>IF(F17=0,0,G17/F17)</f>
@@ -1865,10 +1859,10 @@
         <v>0</v>
       </c>
       <c r="S17" s="3">
-        <v>3503.314763237009</v>
+        <v>3503.314763237015</v>
       </c>
       <c r="T17" s="3">
-        <v>1323.620100098364</v>
+        <v>1323.620100098366</v>
       </c>
       <c r="U17" s="4">
         <f>IF(S17=0,0,T17/S17)</f>
@@ -1922,20 +1916,20 @@
         <v>0</v>
       </c>
       <c r="F18" s="3">
-        <v>231.1015430943887</v>
+        <v>231.1015430943892</v>
       </c>
       <c r="G18" s="3">
-        <v>67.11521448847442</v>
+        <v>67.11521448847459</v>
       </c>
       <c r="H18" s="4">
         <f>IF(F18=0,0,G18/F18)</f>
         <v>0</v>
       </c>
       <c r="I18" s="3">
-        <v>3364.297008165506</v>
+        <v>3364.297008165505</v>
       </c>
       <c r="J18" s="3">
-        <v>311.5683570235935</v>
+        <v>311.568357023593</v>
       </c>
       <c r="K18" s="4">
         <f>IF(I18=0,0,J18/I18)</f>
@@ -1962,10 +1956,10 @@
         <v>0</v>
       </c>
       <c r="S18" s="3">
-        <v>2983.626123720895</v>
+        <v>2983.6261237209</v>
       </c>
       <c r="T18" s="3">
-        <v>866.4879713293681</v>
+        <v>866.487971329369</v>
       </c>
       <c r="U18" s="4">
         <f>IF(S18=0,0,T18/S18)</f>
@@ -2145,7 +2139,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G23" s="3">
-        <v>153.5338348629948</v>
+        <v>203.0197823281202</v>
       </c>
       <c r="H23" s="4">
         <f>IF(F23=0,0,G23/F23)</f>
@@ -2155,7 +2149,7 @@
         <v>1024.476057384201</v>
       </c>
       <c r="J23" s="3">
-        <v>88.45306222013221</v>
+        <v>151.6692552821839</v>
       </c>
       <c r="K23" s="4">
         <f>IF(I23=0,0,J23/I23)</f>
@@ -2165,7 +2159,7 @@
         <v>15352.83741703859</v>
       </c>
       <c r="M23" s="3">
-        <v>39.48982839281298</v>
+        <v>69.56725985433347</v>
       </c>
       <c r="N23" s="4">
         <f>IF(L23=0,0,M23/L23)</f>
@@ -2175,7 +2169,7 @@
         <v>503.5634310516943</v>
       </c>
       <c r="P23" s="3">
-        <v>12.79225539798773</v>
+        <v>21.01036396919185</v>
       </c>
       <c r="Q23" s="4">
         <f>IF(O23=0,0,P23/O23)</f>
@@ -2185,7 +2179,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T23" s="3">
-        <v>4737.225453182322</v>
+        <v>6264.094694192449</v>
       </c>
       <c r="U23" s="4">
         <f>IF(S23=0,0,T23/S23)</f>
@@ -2195,7 +2189,7 @@
         <v>25177467.03377928</v>
       </c>
       <c r="W23" s="3">
-        <v>1717881.090067629</v>
+        <v>2945174.443318196</v>
       </c>
       <c r="X23" s="4">
         <f>IF(V23=0,0,W23/V23)</f>
@@ -2205,7 +2199,7 @@
         <v>2561085.175981381</v>
       </c>
       <c r="Z23" s="3">
-        <v>67791.24937985884</v>
+        <v>116196.6057628184</v>
       </c>
       <c r="AA23" s="4">
         <f>IF(Y23=0,0,Z23/Y23)</f>
@@ -2215,7 +2209,7 @@
         <v>172903.801774421</v>
       </c>
       <c r="AC23" s="3">
-        <v>438.2632218054205</v>
+        <v>772.255639909883</v>
       </c>
       <c r="AD23" s="4">
         <f>IF(AB23=0,0,AC23/AB23)</f>
@@ -2242,7 +2236,7 @@
         <v>422.0532339939541</v>
       </c>
       <c r="G24" s="3">
-        <v>149.5731184765912</v>
+        <v>198.5663656707619</v>
       </c>
       <c r="H24" s="4">
         <f>IF(F24=0,0,G24/F24)</f>
@@ -2252,7 +2246,7 @@
         <v>968.8874507802924</v>
       </c>
       <c r="J24" s="3">
-        <v>89.17520191574422</v>
+        <v>150.8926468475667</v>
       </c>
       <c r="K24" s="4">
         <f>IF(I24=0,0,J24/I24)</f>
@@ -2262,7 +2256,7 @@
         <v>15897.14811387405</v>
       </c>
       <c r="M24" s="3">
-        <v>35.37980973197706</v>
+        <v>66.02582374739833</v>
       </c>
       <c r="N24" s="4">
         <f>IF(L24=0,0,M24/L24)</f>
@@ -2272,7 +2266,7 @@
         <v>427.6878840211459</v>
       </c>
       <c r="P24" s="3">
-        <v>13.53889125172485</v>
+        <v>21.73464126741991</v>
       </c>
       <c r="Q24" s="4">
         <f>IF(O24=0,0,P24/O24)</f>
@@ -2282,7 +2276,7 @@
         <v>13022.28479122008</v>
       </c>
       <c r="T24" s="3">
-        <v>4615.019123253476</v>
+        <v>6126.686293225393</v>
       </c>
       <c r="U24" s="4">
         <f>IF(S24=0,0,T24/S24)</f>
@@ -2292,7 +2286,7 @@
         <v>24716781.60947407</v>
       </c>
       <c r="W24" s="3">
-        <v>1817089.165172193</v>
+        <v>3073981.15008124</v>
       </c>
       <c r="X24" s="4">
         <f>IF(V24=0,0,W24/V24)</f>
@@ -2302,7 +2296,7 @@
         <v>2216806.226901517</v>
       </c>
       <c r="Z24" s="3">
-        <v>66880.27345653391</v>
+        <v>113084.6469390318</v>
       </c>
       <c r="AA24" s="4">
         <f>IF(Y24=0,0,Z24/Y24)</f>
@@ -2312,7 +2306,7 @@
         <v>179047.6330362356</v>
       </c>
       <c r="AC24" s="3">
-        <v>392.6447451862332</v>
+        <v>733.1540885220165</v>
       </c>
       <c r="AD24" s="4">
         <f>IF(AB24=0,0,AC24/AB24)</f>
@@ -2339,7 +2333,7 @@
         <v>382.0743136549376</v>
       </c>
       <c r="G25" s="3">
-        <v>112.1956276633881</v>
+        <v>154.1818427005811</v>
       </c>
       <c r="H25" s="4">
         <f>IF(F25=0,0,G25/F25)</f>
@@ -2349,7 +2343,7 @@
         <v>792.6568327877751</v>
       </c>
       <c r="J25" s="3">
-        <v>82.16165372872982</v>
+        <v>138.7460097809298</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
@@ -2359,7 +2353,7 @@
         <v>14099.36149543928</v>
       </c>
       <c r="M25" s="3">
-        <v>27.60176385746338</v>
+        <v>48.02046110171266</v>
       </c>
       <c r="N25" s="4">
         <f>IF(L25=0,0,M25/L25)</f>
@@ -2369,7 +2363,7 @@
         <v>410.8336896551561</v>
       </c>
       <c r="P25" s="3">
-        <v>11.78004676621949</v>
+        <v>20.00392896381795</v>
       </c>
       <c r="Q25" s="4">
         <f>IF(O25=0,0,P25/O25)</f>
@@ -2379,7 +2373,7 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T25" s="3">
-        <v>3461.751499772321</v>
+        <v>4757.219477462471</v>
       </c>
       <c r="U25" s="4">
         <f>IF(S25=0,0,T25/S25)</f>
@@ -2389,7 +2383,7 @@
         <v>22756394.15398703</v>
       </c>
       <c r="W25" s="3">
-        <v>1928604.090877723</v>
+        <v>3255095.686233584</v>
       </c>
       <c r="X25" s="4">
         <f>IF(V25=0,0,W25/V25)</f>
@@ -2399,7 +2393,7 @@
         <v>2114085.557833027</v>
       </c>
       <c r="Z25" s="3">
-        <v>62040.71386387013</v>
+        <v>104646.7324492342</v>
       </c>
       <c r="AA25" s="4">
         <f>IF(Y25=0,0,Z25/Y25)</f>
@@ -2409,7 +2403,7 @@
         <v>158763.7032537926</v>
       </c>
       <c r="AC25" s="3">
-        <v>306.2954858714365</v>
+        <v>532.758637659339</v>
       </c>
       <c r="AD25" s="4">
         <f>IF(AB25=0,0,AC25/AB25)</f>
@@ -2436,7 +2430,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G26" s="3">
-        <v>86.23155739396429</v>
+        <v>120.7918882652273</v>
       </c>
       <c r="H26" s="4">
         <f>IF(F26=0,0,G26/F26)</f>
@@ -2446,7 +2440,7 @@
         <v>714.5868735320346</v>
       </c>
       <c r="J26" s="3">
-        <v>76.42915899969695</v>
+        <v>127.9421658211542</v>
       </c>
       <c r="K26" s="4">
         <f>IF(I26=0,0,J26/I26)</f>
@@ -2456,7 +2450,7 @@
         <v>12459.036398116</v>
       </c>
       <c r="M26" s="3">
-        <v>20.53776044135541</v>
+        <v>33.00900104676187</v>
       </c>
       <c r="N26" s="4">
         <f>IF(L26=0,0,M26/L26)</f>
@@ -2466,7 +2460,7 @@
         <v>388.5202631627004</v>
       </c>
       <c r="P26" s="3">
-        <v>9.655606483098177</v>
+        <v>16.30620732857898</v>
       </c>
       <c r="Q26" s="4">
         <f>IF(O26=0,0,P26/O26)</f>
@@ -2476,7 +2470,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T26" s="3">
-        <v>2660.640430943196</v>
+        <v>3726.985704086702</v>
       </c>
       <c r="U26" s="4">
         <f>IF(S26=0,0,T26/S26)</f>
@@ -2486,7 +2480,7 @@
         <v>21413420.36871202</v>
       </c>
       <c r="W26" s="3">
-        <v>1904396.797904398</v>
+        <v>3188030.275738072</v>
       </c>
       <c r="X26" s="4">
         <f>IF(V26=0,0,W26/V26)</f>
@@ -2496,7 +2490,7 @@
         <v>1925897.452986733</v>
       </c>
       <c r="Z26" s="3">
-        <v>51998.83105193265</v>
+        <v>86993.32044937275</v>
       </c>
       <c r="AA26" s="4">
         <f>IF(Y26=0,0,Z26/Y26)</f>
@@ -2506,7 +2500,7 @@
         <v>140314.2879239626</v>
       </c>
       <c r="AC26" s="3">
-        <v>228.0923830957618</v>
+        <v>366.5770442610374</v>
       </c>
       <c r="AD26" s="4">
         <f>IF(AB26=0,0,AC26/AB26)</f>
@@ -2533,7 +2527,7 @@
         <v>297.4602934996698</v>
       </c>
       <c r="G27" s="3">
-        <v>70.86872059774323</v>
+        <v>100.604253937639</v>
       </c>
       <c r="H27" s="4">
         <f>IF(F27=0,0,G27/F27)</f>
@@ -2543,7 +2537,7 @@
         <v>607.1996095192959</v>
       </c>
       <c r="J27" s="3">
-        <v>68.60541800043255</v>
+        <v>115.4369858740715</v>
       </c>
       <c r="K27" s="4">
         <f>IF(I27=0,0,J27/I27)</f>
@@ -2553,7 +2547,7 @@
         <v>9475.405513778041</v>
       </c>
       <c r="M27" s="3">
-        <v>16.14096631298959</v>
+        <v>26.1176055910252</v>
       </c>
       <c r="N27" s="4">
         <f>IF(L27=0,0,M27/L27)</f>
@@ -2563,7 +2557,7 @@
         <v>285.742923347472</v>
       </c>
       <c r="P27" s="3">
-        <v>8.734874414667255</v>
+        <v>14.29403973296256</v>
       </c>
       <c r="Q27" s="4">
         <f>IF(O27=0,0,P27/O27)</f>
@@ -2573,7 +2567,7 @@
         <v>9178.019131321482</v>
       </c>
       <c r="T27" s="3">
-        <v>2186.626207504518</v>
+        <v>3104.104270417525</v>
       </c>
       <c r="U27" s="4">
         <f>IF(S27=0,0,T27/S27)</f>
@@ -2583,7 +2577,7 @@
         <v>19850211.7121278</v>
       </c>
       <c r="W27" s="3">
-        <v>1891366.608428925</v>
+        <v>3182528.287519272</v>
       </c>
       <c r="X27" s="4">
         <f>IF(V27=0,0,W27/V27)</f>
@@ -2593,7 +2587,7 @@
         <v>1405792.016991551</v>
       </c>
       <c r="Z27" s="3">
-        <v>42910.21947404603</v>
+        <v>72425.83938977448</v>
       </c>
       <c r="AA27" s="4">
         <f>IF(Y27=0,0,Z27/Y27)</f>
@@ -2603,7 +2597,7 @@
         <v>106730.9429757299</v>
       </c>
       <c r="AC27" s="3">
-        <v>179.2154438609432</v>
+        <v>290.0031727931782</v>
       </c>
       <c r="AD27" s="4">
         <f>IF(AB27=0,0,AC27/AB27)</f>
@@ -2753,7 +2747,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G32" s="3">
-        <v>31.81246083158429</v>
+        <v>35.73618465235695</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
@@ -2763,7 +2757,7 @@
         <v>1024.476057384201</v>
       </c>
       <c r="J32" s="3">
-        <v>32.68368291760166</v>
+        <v>37.27986362662178</v>
       </c>
       <c r="K32" s="4">
         <f>IF(I32=0,0,J32/I32)</f>
@@ -2773,7 +2767,7 @@
         <v>15352.83741703859</v>
       </c>
       <c r="M32" s="3">
-        <v>3.522455788802355</v>
+        <v>3.962234379850328</v>
       </c>
       <c r="N32" s="4">
         <f>IF(L32=0,0,M32/L32)</f>
@@ -2783,7 +2777,7 @@
         <v>503.5634310516943</v>
       </c>
       <c r="P32" s="3">
-        <v>3.068380574589828</v>
+        <v>3.925692564837344</v>
       </c>
       <c r="Q32" s="4">
         <f>IF(O32=0,0,P32/O32)</f>
@@ -2793,7 +2787,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T32" s="3">
-        <v>981.560835201084</v>
+        <v>1102.625774219956</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
@@ -2803,7 +2797,7 @@
         <v>25177467.03377928</v>
       </c>
       <c r="W32" s="3">
-        <v>626042.9301561825</v>
+        <v>714061.0112777613</v>
       </c>
       <c r="X32" s="4">
         <f>IF(V32=0,0,W32/V32)</f>
@@ -2813,7 +2807,7 @@
         <v>2561085.175981381</v>
       </c>
       <c r="Z32" s="3">
-        <v>21648.69212072948</v>
+        <v>24656.53941042209</v>
       </c>
       <c r="AA32" s="4">
         <f>IF(Y32=0,0,Z32/Y32)</f>
@@ -2823,7 +2817,7 @@
         <v>172903.801774421</v>
       </c>
       <c r="AC32" s="3">
-        <v>39.10155138786649</v>
+        <v>43.98924531132798</v>
       </c>
       <c r="AD32" s="4">
         <f>IF(AB32=0,0,AC32/AB32)</f>
@@ -2850,7 +2844,7 @@
         <v>422.0532339939541</v>
       </c>
       <c r="G33" s="3">
-        <v>58.43364202621579</v>
+        <v>65.17460356458911</v>
       </c>
       <c r="H33" s="4">
         <f>IF(F33=0,0,G33/F33)</f>
@@ -2860,7 +2854,7 @@
         <v>968.8874507802924</v>
       </c>
       <c r="J33" s="3">
-        <v>42.90436372769834</v>
+        <v>48.93446618463355</v>
       </c>
       <c r="K33" s="4">
         <f>IF(I33=0,0,J33/I33)</f>
@@ -2870,7 +2864,7 @@
         <v>15897.14811387405</v>
       </c>
       <c r="M33" s="3">
-        <v>4.837213344274089</v>
+        <v>5.71674261646904</v>
       </c>
       <c r="N33" s="4">
         <f>IF(L33=0,0,M33/L33)</f>
@@ -2880,7 +2874,7 @@
         <v>427.6878840211459</v>
       </c>
       <c r="P33" s="3">
-        <v>5.825020013755769</v>
+        <v>6.033024517372309</v>
       </c>
       <c r="Q33" s="4">
         <f>IF(O33=0,0,P33/O33)</f>
@@ -2890,7 +2884,7 @@
         <v>13022.28479122008</v>
       </c>
       <c r="T33" s="3">
-        <v>1802.94680046093</v>
+        <v>2010.936489554548</v>
       </c>
       <c r="U33" s="4">
         <f>IF(S33=0,0,T33/S33)</f>
@@ -2900,7 +2894,7 @@
         <v>24716781.60947407</v>
       </c>
       <c r="W33" s="3">
-        <v>861731.9117797464</v>
+        <v>982871.2588993013</v>
       </c>
       <c r="X33" s="4">
         <f>IF(V33=0,0,W33/V33)</f>
@@ -2910,7 +2904,7 @@
         <v>2216806.226901517</v>
       </c>
       <c r="Z33" s="3">
-        <v>30569.74919843301</v>
+        <v>34690.28850875841</v>
       </c>
       <c r="AA33" s="4">
         <f>IF(Y33=0,0,Z33/Y33)</f>
@@ -2920,7 +2914,7 @@
         <v>179047.6330362356</v>
       </c>
       <c r="AC33" s="3">
-        <v>53.76463315828005</v>
+        <v>63.54002100523212</v>
       </c>
       <c r="AD33" s="4">
         <f>IF(AB33=0,0,AC33/AB33)</f>
@@ -2947,7 +2941,7 @@
         <v>382.0743136549376</v>
       </c>
       <c r="G34" s="3">
-        <v>70.32625266599533</v>
+        <v>77.8855817338635</v>
       </c>
       <c r="H34" s="4">
         <f>IF(F34=0,0,G34/F34)</f>
@@ -2957,7 +2951,7 @@
         <v>792.6568327877751</v>
       </c>
       <c r="J34" s="3">
-        <v>47.95450258267846</v>
+        <v>54.7024904162623</v>
       </c>
       <c r="K34" s="4">
         <f>IF(I34=0,0,J34/I34)</f>
@@ -2967,7 +2961,7 @@
         <v>14099.36149543928</v>
       </c>
       <c r="M34" s="3">
-        <v>7.771691316105425</v>
+        <v>7.918256656212733</v>
       </c>
       <c r="N34" s="4">
         <f>IF(L34=0,0,M34/L34)</f>
@@ -2977,7 +2971,7 @@
         <v>410.8336896551561</v>
       </c>
       <c r="P34" s="3">
-        <v>6.801244757992798</v>
+        <v>7.485334139126877</v>
       </c>
       <c r="Q34" s="4">
         <f>IF(O34=0,0,P34/O34)</f>
@@ -2987,7 +2981,7 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T34" s="3">
-        <v>2169.888575072522</v>
+        <v>2403.128669031234</v>
       </c>
       <c r="U34" s="4">
         <f>IF(S34=0,0,T34/S34)</f>
@@ -2997,7 +2991,7 @@
         <v>22756394.15398703</v>
       </c>
       <c r="W34" s="3">
-        <v>1108078.306488663</v>
+        <v>1263898.368850708</v>
       </c>
       <c r="X34" s="4">
         <f>IF(V34=0,0,W34/V34)</f>
@@ -3007,7 +3001,7 @@
         <v>2114085.557833027</v>
       </c>
       <c r="Z34" s="3">
-        <v>36469.94504468259</v>
+        <v>41680.40197755746</v>
       </c>
       <c r="AA34" s="4">
         <f>IF(Y34=0,0,Z34/Y34)</f>
@@ -3017,7 +3011,7 @@
         <v>158763.7032537926</v>
       </c>
       <c r="AC34" s="3">
-        <v>86.34925931482576</v>
+        <v>87.97849062262685</v>
       </c>
       <c r="AD34" s="4">
         <f>IF(AB34=0,0,AC34/AB34)</f>
@@ -3044,7 +3038,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G35" s="3">
-        <v>79.01499632789736</v>
+        <v>86.85569037143482</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
@@ -3054,7 +3048,7 @@
         <v>714.5868735320346</v>
       </c>
       <c r="J35" s="3">
-        <v>51.68573642029136</v>
+        <v>58.95966902481718</v>
       </c>
       <c r="K35" s="4">
         <f>IF(I35=0,0,J35/I35)</f>
@@ -3064,7 +3058,7 @@
         <v>12459.036398116</v>
       </c>
       <c r="M35" s="3">
-        <v>5.284773733304814</v>
+        <v>6.752045505788177</v>
       </c>
       <c r="N35" s="4">
         <f>IF(L35=0,0,M35/L35)</f>
@@ -3074,7 +3068,7 @@
         <v>388.5202631627004</v>
       </c>
       <c r="P35" s="3">
-        <v>6.425640266744071</v>
+        <v>7.643253715592786</v>
       </c>
       <c r="Q35" s="4">
         <f>IF(O35=0,0,P35/O35)</f>
@@ -3084,7 +3078,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T35" s="3">
-        <v>2437.976307448053</v>
+        <v>2679.897805903459</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
@@ -3094,7 +3088,7 @@
         <v>21413420.36871202</v>
       </c>
       <c r="W35" s="3">
-        <v>1269177.296716776</v>
+        <v>1447623.317466982</v>
       </c>
       <c r="X35" s="4">
         <f>IF(V35=0,0,W35/V35)</f>
@@ -3104,7 +3098,7 @@
         <v>1925897.452986733</v>
       </c>
       <c r="Z35" s="3">
-        <v>35243.3810336343</v>
+        <v>39964.18840772193</v>
       </c>
       <c r="AA35" s="4">
         <f>IF(Y35=0,0,Z35/Y35)</f>
@@ -3114,7 +3108,7 @@
         <v>140314.2879239626</v>
       </c>
       <c r="AC35" s="3">
-        <v>58.65232708177064</v>
+        <v>74.94464016004349</v>
       </c>
       <c r="AD35" s="4">
         <f>IF(AB35=0,0,AC35/AB35)</f>
@@ -3141,7 +3135,7 @@
         <v>297.4602934996698</v>
       </c>
       <c r="G36" s="3">
-        <v>75.51235895096086</v>
+        <v>82.75070857381445</v>
       </c>
       <c r="H36" s="4">
         <f>IF(F36=0,0,G36/F36)</f>
@@ -3151,7 +3145,7 @@
         <v>607.1996095192959</v>
       </c>
       <c r="J36" s="3">
-        <v>49.91319984393473</v>
+        <v>56.92850932440988</v>
       </c>
       <c r="K36" s="4">
         <f>IF(I36=0,0,J36/I36)</f>
@@ -3161,7 +3155,7 @@
         <v>9475.405513778041</v>
       </c>
       <c r="M36" s="3">
-        <v>8.366401425374672</v>
+        <v>9.540724531468005</v>
       </c>
       <c r="N36" s="4">
         <f>IF(L36=0,0,M36/L36)</f>
@@ -3171,7 +3165,7 @@
         <v>285.742923347472</v>
       </c>
       <c r="P36" s="3">
-        <v>6.236481271973287</v>
+        <v>6.937234701249923</v>
       </c>
       <c r="Q36" s="4">
         <f>IF(O36=0,0,P36/O36)</f>
@@ -3181,7 +3175,7 @@
         <v>9178.019131321482</v>
       </c>
       <c r="T36" s="3">
-        <v>2329.903823294328</v>
+        <v>2553.240224049334</v>
       </c>
       <c r="U36" s="4">
         <f>IF(S36=0,0,T36/S36)</f>
@@ -3191,7 +3185,7 @@
         <v>19850211.7121278</v>
       </c>
       <c r="W36" s="3">
-        <v>1356137.905176748</v>
+        <v>1546922.86282469</v>
       </c>
       <c r="X36" s="4">
         <f>IF(V36=0,0,W36/V36)</f>
@@ -3201,7 +3195,7 @@
         <v>1405792.016991551</v>
       </c>
       <c r="Z36" s="3">
-        <v>30795.86643654411</v>
+        <v>35215.72640739055</v>
       </c>
       <c r="AA36" s="4">
         <f>IF(Y36=0,0,Z36/Y36)</f>
@@ -3211,7 +3205,7 @@
         <v>106730.9429757299</v>
       </c>
       <c r="AC36" s="3">
-        <v>92.86618454611744</v>
+        <v>105.9000350087299</v>
       </c>
       <c r="AD36" s="4">
         <f>IF(AB36=0,0,AC36/AB36)</f>
@@ -3358,20 +3352,20 @@
         <v>0</v>
       </c>
       <c r="F41" s="3">
-        <v>0</v>
+        <v>412.7408750394843</v>
       </c>
       <c r="G41" s="3">
-        <v>0</v>
+        <v>23.42409718172002</v>
       </c>
       <c r="H41" s="4">
         <f>IF(F41=0,0,G41/F41)</f>
         <v>0</v>
       </c>
       <c r="I41" s="3">
-        <v>1024.476057384201</v>
+        <v>1026.204299813583</v>
       </c>
       <c r="J41" s="3">
-        <v>32.68368291760166</v>
+        <v>6.332670651874505</v>
       </c>
       <c r="K41" s="4">
         <f>IF(I41=0,0,J41/I41)</f>
@@ -3381,7 +3375,7 @@
         <v>15352.83741703859</v>
       </c>
       <c r="M41" s="3">
-        <v>3.522455788802355</v>
+        <v>0.5863035025261343</v>
       </c>
       <c r="N41" s="4">
         <f>IF(L41=0,0,M41/L41)</f>
@@ -3391,27 +3385,27 @@
         <v>503.5634310516943</v>
       </c>
       <c r="P41" s="3">
-        <v>3.068380574589828</v>
+        <v>0.7976752452995279</v>
       </c>
       <c r="Q41" s="4">
         <f>IF(O41=0,0,P41/O41)</f>
         <v>0</v>
       </c>
       <c r="S41" s="3">
-        <v>0</v>
+        <v>12734.95565684622</v>
       </c>
       <c r="T41" s="3">
-        <v>0</v>
+        <v>722.7412087119392</v>
       </c>
       <c r="U41" s="4">
         <f>IF(S41=0,0,T41/S41)</f>
         <v>0</v>
       </c>
       <c r="V41" s="3">
-        <v>25177467.03377928</v>
+        <v>25286285.18025935</v>
       </c>
       <c r="W41" s="3">
-        <v>626042.9301561825</v>
+        <v>124252.6863578595</v>
       </c>
       <c r="X41" s="4">
         <f>IF(V41=0,0,W41/V41)</f>
@@ -3421,7 +3415,7 @@
         <v>2561085.175981381</v>
       </c>
       <c r="Z41" s="3">
-        <v>21648.69212072948</v>
+        <v>4301.107752270065</v>
       </c>
       <c r="AA41" s="4">
         <f>IF(Y41=0,0,Z41/Y41)</f>
@@ -3431,7 +3425,7 @@
         <v>172903.801774421</v>
       </c>
       <c r="AC41" s="3">
-        <v>39.10155138786649</v>
+        <v>6.516925231320783</v>
       </c>
       <c r="AD41" s="4">
         <f>IF(AB41=0,0,AC41/AB41)</f>
@@ -3455,20 +3449,20 @@
         <v>0</v>
       </c>
       <c r="F42" s="3">
-        <v>0</v>
+        <v>422.0532339939548</v>
       </c>
       <c r="G42" s="3">
-        <v>0</v>
+        <v>32.39383284579316</v>
       </c>
       <c r="H42" s="4">
         <f>IF(F42=0,0,G42/F42)</f>
         <v>0</v>
       </c>
       <c r="I42" s="3">
-        <v>968.8874507802924</v>
+        <v>971.1037573173985</v>
       </c>
       <c r="J42" s="3">
-        <v>42.90436372769834</v>
+        <v>8.271399086192949</v>
       </c>
       <c r="K42" s="4">
         <f>IF(I42=0,0,J42/I42)</f>
@@ -3478,7 +3472,7 @@
         <v>15897.14811387405</v>
       </c>
       <c r="M42" s="3">
-        <v>4.837213344274089</v>
+        <v>2.204028858903795</v>
       </c>
       <c r="N42" s="4">
         <f>IF(L42=0,0,M42/L42)</f>
@@ -3488,27 +3482,27 @@
         <v>427.6878840211459</v>
       </c>
       <c r="P42" s="3">
-        <v>5.825020013755769</v>
+        <v>0.7658804311889107</v>
       </c>
       <c r="Q42" s="4">
         <f>IF(O42=0,0,P42/O42)</f>
         <v>0</v>
       </c>
       <c r="S42" s="3">
-        <v>0</v>
+        <v>13022.2847912201</v>
       </c>
       <c r="T42" s="3">
-        <v>0</v>
+        <v>999.4988376351139</v>
       </c>
       <c r="U42" s="4">
         <f>IF(S42=0,0,T42/S42)</f>
         <v>0</v>
       </c>
       <c r="V42" s="3">
-        <v>24716781.60947407</v>
+        <v>24859901.01601297</v>
       </c>
       <c r="W42" s="3">
-        <v>861731.9117797464</v>
+        <v>171453.208100237</v>
       </c>
       <c r="X42" s="4">
         <f>IF(V42=0,0,W42/V42)</f>
@@ -3518,7 +3512,7 @@
         <v>2216806.226901517</v>
       </c>
       <c r="Z42" s="3">
-        <v>30569.74919843301</v>
+        <v>5397.532345701009</v>
       </c>
       <c r="AA42" s="4">
         <f>IF(Y42=0,0,Z42/Y42)</f>
@@ -3528,7 +3522,7 @@
         <v>179047.6330362356</v>
       </c>
       <c r="AC42" s="3">
-        <v>53.76463315828005</v>
+        <v>24.43846961739473</v>
       </c>
       <c r="AD42" s="4">
         <f>IF(AB42=0,0,AC42/AB42)</f>
@@ -3552,20 +3546,20 @@
         <v>0</v>
       </c>
       <c r="F43" s="3">
-        <v>0</v>
+        <v>382.0743136549376</v>
       </c>
       <c r="G43" s="3">
-        <v>0</v>
+        <v>45.49713331928587</v>
       </c>
       <c r="H43" s="4">
         <f>IF(F43=0,0,G43/F43)</f>
         <v>0</v>
       </c>
       <c r="I43" s="3">
-        <v>792.6568327877751</v>
+        <v>795.3294661601195</v>
       </c>
       <c r="J43" s="3">
-        <v>47.95450258267846</v>
+        <v>9.250731927022105</v>
       </c>
       <c r="K43" s="4">
         <f>IF(I43=0,0,J43/I43)</f>
@@ -3575,7 +3569,7 @@
         <v>14099.36149543928</v>
       </c>
       <c r="M43" s="3">
-        <v>7.771691316105425</v>
+        <v>2.494237892366946</v>
       </c>
       <c r="N43" s="4">
         <f>IF(L43=0,0,M43/L43)</f>
@@ -3585,27 +3579,27 @@
         <v>410.8336896551561</v>
       </c>
       <c r="P43" s="3">
-        <v>6.801244757992798</v>
+        <v>0.6260496127711959</v>
       </c>
       <c r="Q43" s="4">
         <f>IF(O43=0,0,P43/O43)</f>
         <v>0</v>
       </c>
       <c r="S43" s="3">
-        <v>0</v>
+        <v>11788.75109364953</v>
       </c>
       <c r="T43" s="3">
-        <v>0</v>
+        <v>1403.795965881249</v>
       </c>
       <c r="U43" s="4">
         <f>IF(S43=0,0,T43/S43)</f>
         <v>0</v>
       </c>
       <c r="V43" s="3">
-        <v>22756394.15398703</v>
+        <v>22936296.40445412</v>
       </c>
       <c r="W43" s="3">
-        <v>1108078.306488663</v>
+        <v>221609.0820698142</v>
       </c>
       <c r="X43" s="4">
         <f>IF(V43=0,0,W43/V43)</f>
@@ -3615,7 +3609,7 @@
         <v>2114085.557833027</v>
       </c>
       <c r="Z43" s="3">
-        <v>36469.94504468259</v>
+        <v>6329.655924388207</v>
       </c>
       <c r="AA43" s="4">
         <f>IF(Y43=0,0,Z43/Y43)</f>
@@ -3625,7 +3619,7 @@
         <v>158763.7032537926</v>
       </c>
       <c r="AC43" s="3">
-        <v>86.34925931482576</v>
+        <v>27.69693223305512</v>
       </c>
       <c r="AD43" s="4">
         <f>IF(AB43=0,0,AC43/AB43)</f>
@@ -3649,20 +3643,20 @@
         <v>0</v>
       </c>
       <c r="F44" s="3">
-        <v>0</v>
+        <v>338.6701578384149</v>
       </c>
       <c r="G44" s="3">
-        <v>0</v>
+        <v>48.79942009843676</v>
       </c>
       <c r="H44" s="4">
         <f>IF(F44=0,0,G44/F44)</f>
         <v>0</v>
       </c>
       <c r="I44" s="3">
-        <v>714.5868735320346</v>
+        <v>717.4492241565633</v>
       </c>
       <c r="J44" s="3">
-        <v>51.68573642029136</v>
+        <v>9.464455356970662</v>
       </c>
       <c r="K44" s="4">
         <f>IF(I44=0,0,J44/I44)</f>
@@ -3672,7 +3666,7 @@
         <v>12459.036398116</v>
       </c>
       <c r="M44" s="3">
-        <v>5.284773733304814</v>
+        <v>2.502058168889955</v>
       </c>
       <c r="N44" s="4">
         <f>IF(L44=0,0,M44/L44)</f>
@@ -3682,27 +3676,27 @@
         <v>388.5202631627004</v>
       </c>
       <c r="P44" s="3">
-        <v>6.425640266744071</v>
+        <v>1.11741603567038</v>
       </c>
       <c r="Q44" s="4">
         <f>IF(O44=0,0,P44/O44)</f>
         <v>0</v>
       </c>
       <c r="S44" s="3">
-        <v>0</v>
+        <v>10449.53311676904</v>
       </c>
       <c r="T44" s="3">
-        <v>0</v>
+        <v>1505.686711968985</v>
       </c>
       <c r="U44" s="4">
         <f>IF(S44=0,0,T44/S44)</f>
         <v>0</v>
       </c>
       <c r="V44" s="3">
-        <v>21413420.36871202</v>
+        <v>21610890.70116934</v>
       </c>
       <c r="W44" s="3">
-        <v>1269177.296716776</v>
+        <v>242173.5070957839</v>
       </c>
       <c r="X44" s="4">
         <f>IF(V44=0,0,W44/V44)</f>
@@ -3712,7 +3706,7 @@
         <v>1925897.452986733</v>
       </c>
       <c r="Z44" s="3">
-        <v>35243.3810336343</v>
+        <v>5809.098253916716</v>
       </c>
       <c r="AA44" s="4">
         <f>IF(Y44=0,0,Z44/Y44)</f>
@@ -3722,7 +3716,7 @@
         <v>140314.2879239626</v>
       </c>
       <c r="AC44" s="3">
-        <v>58.65232708177064</v>
+        <v>27.69693223305512</v>
       </c>
       <c r="AD44" s="4">
         <f>IF(AB44=0,0,AC44/AB44)</f>
@@ -3746,20 +3740,20 @@
         <v>0</v>
       </c>
       <c r="F45" s="3">
-        <v>0</v>
+        <v>297.4602934996698</v>
       </c>
       <c r="G45" s="3">
-        <v>0</v>
+        <v>50.94083911201337</v>
       </c>
       <c r="H45" s="4">
         <f>IF(F45=0,0,G45/F45)</f>
         <v>0</v>
       </c>
       <c r="I45" s="3">
-        <v>607.1996095192959</v>
+        <v>610.1638407046684</v>
       </c>
       <c r="J45" s="3">
-        <v>49.91319984393473</v>
+        <v>9.162136177603854</v>
       </c>
       <c r="K45" s="4">
         <f>IF(I45=0,0,J45/I45)</f>
@@ -3769,7 +3763,7 @@
         <v>9475.405513778041</v>
       </c>
       <c r="M45" s="3">
-        <v>8.366401425374672</v>
+        <v>2.647848884297535</v>
       </c>
       <c r="N45" s="4">
         <f>IF(L45=0,0,M45/L45)</f>
@@ -3779,27 +3773,27 @@
         <v>285.742923347472</v>
       </c>
       <c r="P45" s="3">
-        <v>6.236481271973287</v>
+        <v>0.7667368651648867</v>
       </c>
       <c r="Q45" s="4">
         <f>IF(O45=0,0,P45/O45)</f>
         <v>0</v>
       </c>
       <c r="S45" s="3">
-        <v>0</v>
+        <v>9178.019131321482</v>
       </c>
       <c r="T45" s="3">
-        <v>0</v>
+        <v>1571.759344532979</v>
       </c>
       <c r="U45" s="4">
         <f>IF(S45=0,0,T45/S45)</f>
         <v>0</v>
       </c>
       <c r="V45" s="3">
-        <v>19850211.7121278</v>
+        <v>20059051.99524085</v>
       </c>
       <c r="W45" s="3">
-        <v>1356137.905176748</v>
+        <v>259185.2599577568</v>
       </c>
       <c r="X45" s="4">
         <f>IF(V45=0,0,W45/V45)</f>
@@ -3809,7 +3803,7 @@
         <v>1405792.016991551</v>
       </c>
       <c r="Z45" s="3">
-        <v>30795.86643654411</v>
+        <v>5319.448695129715</v>
       </c>
       <c r="AA45" s="4">
         <f>IF(Y45=0,0,Z45/Y45)</f>
@@ -3819,7 +3813,7 @@
         <v>106730.9429757299</v>
       </c>
       <c r="AC45" s="3">
-        <v>92.86618454611744</v>
+        <v>29.32616354089987</v>
       </c>
       <c r="AD45" s="4">
         <f>IF(AB45=0,0,AC45/AB45)</f>
@@ -3958,28 +3952,28 @@
         <v>0</v>
       </c>
       <c r="D50" s="3">
-        <f>J50+G50</f>
+        <f>G50+J50</f>
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>P50+M50</f>
+        <f>M50+P50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G50" s="3">
-        <v>58.98240259960006</v>
+        <v>55.04951209333916</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
         <v>0</v>
       </c>
       <c r="I50" s="3">
-        <v>382.3073643284126</v>
+        <v>382.3073643284127</v>
       </c>
       <c r="J50" s="6">
-        <v>8.688572781210823</v>
+        <v>7.728037475080812</v>
       </c>
       <c r="K50" s="7">
         <f>IF(I50=0,0,J50/I50)</f>
@@ -4009,7 +4003,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T50" s="3">
-        <v>834.7483796180522</v>
+        <v>779.0881516072866</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
@@ -4019,7 +4013,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W50" s="6">
-        <v>206244.2943557147</v>
+        <v>183396.5001733974</v>
       </c>
       <c r="X50" s="7">
         <f>IF(V50=0,0,W50/V50)</f>
@@ -4055,18 +4049,18 @@
         <v>0</v>
       </c>
       <c r="D51" s="3">
-        <f>J51+G51</f>
+        <f>G51+J51</f>
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>P51+M51</f>
+        <f>M51+P51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
-        <v>147.7607036391231</v>
+        <v>147.7607036391234</v>
       </c>
       <c r="G51" s="3">
-        <v>59.41247823140037</v>
+        <v>55.83301727702623</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
@@ -4076,7 +4070,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J51" s="6">
-        <v>7.531359140255693</v>
+        <v>6.745118358334934</v>
       </c>
       <c r="K51" s="7">
         <f>IF(I51=0,0,J51/I51)</f>
@@ -4103,20 +4097,20 @@
         <v>0</v>
       </c>
       <c r="S51" s="3">
-        <v>2091.183174942718</v>
+        <v>2091.183174942721</v>
       </c>
       <c r="T51" s="3">
-        <v>840.8350244635603</v>
+        <v>790.1767077474119</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
         <v>0</v>
       </c>
       <c r="V51" s="3">
-        <v>7100767.677214348</v>
+        <v>7100767.677214347</v>
       </c>
       <c r="W51" s="6">
-        <v>238006.6357756928</v>
+        <v>213135.3226955337</v>
       </c>
       <c r="X51" s="7">
         <f>IF(V51=0,0,W51/V51)</f>
@@ -4152,18 +4146,18 @@
         <v>0</v>
       </c>
       <c r="D52" s="3">
-        <f>J52+G52</f>
+        <f>G52+J52</f>
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>P52+M52</f>
+        <f>M52+P52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G52" s="3">
-        <v>59.19812501773821</v>
+        <v>55.74658849855057</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
@@ -4173,7 +4167,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J52" s="6">
-        <v>8.333503383573669</v>
+        <v>7.433932887340605</v>
       </c>
       <c r="K52" s="7">
         <f>IF(I52=0,0,J52/I52)</f>
@@ -4203,7 +4197,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T52" s="3">
-        <v>837.8013908731305</v>
+        <v>788.9535245672573</v>
       </c>
       <c r="U52" s="4">
         <f>IF(S52=0,0,T52/S52)</f>
@@ -4213,7 +4207,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W52" s="6">
-        <v>279483.1369019002</v>
+        <v>249256.9665041761</v>
       </c>
       <c r="X52" s="7">
         <f>IF(V52=0,0,W52/V52)</f>
@@ -4249,18 +4243,18 @@
         <v>0</v>
       </c>
       <c r="D53" s="3">
-        <f>J53+G53</f>
+        <f>G53+J53</f>
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>P53+M53</f>
+        <f>M53+P53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G53" s="3">
-        <v>27.88815467106969</v>
+        <v>25.48769675026658</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
@@ -4270,7 +4264,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J53" s="6">
-        <v>3.251090114021907</v>
+        <v>2.88069493231611</v>
       </c>
       <c r="K53" s="7">
         <f>IF(I53=0,0,J53/I53)</f>
@@ -4300,7 +4294,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T53" s="3">
-        <v>394.6870743846378</v>
+        <v>360.7145966384487</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
@@ -4310,7 +4304,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W53" s="6">
-        <v>115470.6967978468</v>
+        <v>102299.5457925303</v>
       </c>
       <c r="X53" s="7">
         <f>IF(V53=0,0,W53/V53)</f>
@@ -4346,18 +4340,18 @@
         <v>0</v>
       </c>
       <c r="D54" s="3">
-        <f>J54+G54</f>
+        <f>G54+J54</f>
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>P54+M54</f>
+        <f>M54+P54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
-        <v>93.49564395607474</v>
+        <v>93.49564395607489</v>
       </c>
       <c r="G54" s="3">
-        <v>16.26254254897413</v>
+        <v>14.82314301600723</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
@@ -4367,7 +4361,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J54" s="6">
-        <v>2.460393484535132</v>
+        <v>2.194074902868248</v>
       </c>
       <c r="K54" s="7">
         <f>IF(I54=0,0,J54/I54)</f>
@@ -4394,10 +4388,10 @@
         <v>0</v>
       </c>
       <c r="S54" s="3">
-        <v>1323.19698509889</v>
+        <v>1323.196985098892</v>
       </c>
       <c r="T54" s="3">
-        <v>230.1556132492615</v>
+        <v>209.784513144647</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>
@@ -4407,7 +4401,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W54" s="6">
-        <v>96394.34072632995</v>
+        <v>85955.24938089401</v>
       </c>
       <c r="X54" s="7">
         <f>IF(V54=0,0,W54/V54)</f>
@@ -4566,28 +4560,28 @@
         <v>0</v>
       </c>
       <c r="D59" s="3">
-        <f>J59+G59</f>
+        <f>G59+J59</f>
         <v>0</v>
       </c>
       <c r="E59" s="3">
-        <f>P59+M59</f>
+        <f>M59+P59</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G59" s="3">
-        <v>105.1172530897168</v>
+        <v>101.6478618860977</v>
       </c>
       <c r="H59" s="4">
         <f>IF(F59=0,0,G59/F59)</f>
         <v>0</v>
       </c>
       <c r="I59" s="3">
-        <v>382.3073643284126</v>
+        <v>382.3073643284127</v>
       </c>
       <c r="J59" s="6">
-        <v>30.38027252396196</v>
+        <v>27.06745242213167</v>
       </c>
       <c r="K59" s="7">
         <f>IF(I59=0,0,J59/I59)</f>
@@ -4617,7 +4611,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T59" s="3">
-        <v>1487.671793945145</v>
+        <v>1438.571239240006</v>
       </c>
       <c r="U59" s="4">
         <f>IF(S59=0,0,T59/S59)</f>
@@ -4627,7 +4621,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W59" s="6">
-        <v>763318.428798628</v>
+        <v>679501.0839667805</v>
       </c>
       <c r="X59" s="7">
         <f>IF(V59=0,0,W59/V59)</f>
@@ -4663,18 +4657,18 @@
         <v>0</v>
       </c>
       <c r="D60" s="3">
-        <f>J60+G60</f>
+        <f>G60+J60</f>
         <v>0</v>
       </c>
       <c r="E60" s="3">
-        <f>P60+M60</f>
+        <f>M60+P60</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
-        <v>147.7607036391231</v>
+        <v>147.7607036391234</v>
       </c>
       <c r="G60" s="3">
-        <v>102.74200724521</v>
+        <v>99.75691769012525</v>
       </c>
       <c r="H60" s="4">
         <f>IF(F60=0,0,G60/F60)</f>
@@ -4684,7 +4678,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J60" s="6">
-        <v>25.02248949374902</v>
+        <v>22.43247551696055</v>
       </c>
       <c r="K60" s="7">
         <f>IF(I60=0,0,J60/I60)</f>
@@ -4711,20 +4705,20 @@
         <v>0</v>
       </c>
       <c r="S60" s="3">
-        <v>2091.183174942718</v>
+        <v>2091.183174942721</v>
       </c>
       <c r="T60" s="3">
-        <v>1454.056130077462</v>
+        <v>1411.809653852386</v>
       </c>
       <c r="U60" s="4">
         <f>IF(S60=0,0,T60/S60)</f>
         <v>0</v>
       </c>
       <c r="V60" s="3">
-        <v>7100767.677214348</v>
+        <v>7100767.677214347</v>
       </c>
       <c r="W60" s="6">
-        <v>836476.8330573244</v>
+        <v>749637.100508377</v>
       </c>
       <c r="X60" s="7">
         <f>IF(V60=0,0,W60/V60)</f>
@@ -4760,18 +4754,18 @@
         <v>0</v>
       </c>
       <c r="D61" s="3">
-        <f>J61+G61</f>
+        <f>G61+J61</f>
         <v>0</v>
       </c>
       <c r="E61" s="3">
-        <f>P61+M61</f>
+        <f>M61+P61</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G61" s="3">
-        <v>97.488226988148</v>
+        <v>94.84760082701457</v>
       </c>
       <c r="H61" s="4">
         <f>IF(F61=0,0,G61/F61)</f>
@@ -4781,7 +4775,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J61" s="6">
-        <v>26.68454090976095</v>
+        <v>23.85461403009552</v>
       </c>
       <c r="K61" s="7">
         <f>IF(I61=0,0,J61/I61)</f>
@@ -4811,7 +4805,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T61" s="3">
-        <v>1379.702011507161</v>
+        <v>1342.330553037646</v>
       </c>
       <c r="U61" s="4">
         <f>IF(S61=0,0,T61/S61)</f>
@@ -4821,7 +4815,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W61" s="6">
-        <v>949876.6631412003</v>
+        <v>848608.1942622317</v>
       </c>
       <c r="X61" s="7">
         <f>IF(V61=0,0,W61/V61)</f>
@@ -4857,18 +4851,18 @@
         <v>0</v>
       </c>
       <c r="D62" s="3">
-        <f>J62+G62</f>
+        <f>G62+J62</f>
         <v>0</v>
       </c>
       <c r="E62" s="3">
-        <f>P62+M62</f>
+        <f>M62+P62</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G62" s="3">
-        <v>62.28901992946252</v>
+        <v>59.08004047660047</v>
       </c>
       <c r="H62" s="4">
         <f>IF(F62=0,0,G62/F62)</f>
@@ -4878,7 +4872,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J62" s="6">
-        <v>11.86059618587699</v>
+        <v>10.52490515259787</v>
       </c>
       <c r="K62" s="7">
         <f>IF(I62=0,0,J62/I62)</f>
@@ -4908,7 +4902,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T62" s="3">
-        <v>881.545277276785</v>
+        <v>836.1301995511723</v>
       </c>
       <c r="U62" s="4">
         <f>IF(S62=0,0,T62/S62)</f>
@@ -4918,7 +4912,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W62" s="6">
-        <v>432629.1184659526</v>
+        <v>383703.346976216</v>
       </c>
       <c r="X62" s="7">
         <f>IF(V62=0,0,W62/V62)</f>
@@ -4954,18 +4948,18 @@
         <v>0</v>
       </c>
       <c r="D63" s="3">
-        <f>J63+G63</f>
+        <f>G63+J63</f>
         <v>0</v>
       </c>
       <c r="E63" s="3">
-        <f>P63+M63</f>
+        <f>M63+P63</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
-        <v>93.49564395607474</v>
+        <v>93.49564395607489</v>
       </c>
       <c r="G63" s="3">
-        <v>40.86638015373266</v>
+        <v>38.47283650311636</v>
       </c>
       <c r="H63" s="4">
         <f>IF(F63=0,0,G63/F63)</f>
@@ -4975,7 +4969,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J63" s="6">
-        <v>9.160355738468613</v>
+        <v>8.174381605417016</v>
       </c>
       <c r="K63" s="7">
         <f>IF(I63=0,0,J63/I63)</f>
@@ -5002,10 +4996,10 @@
         <v>0</v>
       </c>
       <c r="S63" s="3">
-        <v>1323.19698509889</v>
+        <v>1323.196985098892</v>
       </c>
       <c r="T63" s="3">
-        <v>578.3613944274117</v>
+        <v>544.4867708814627</v>
       </c>
       <c r="U63" s="4">
         <f>IF(S63=0,0,T63/S63)</f>
@@ -5015,7 +5009,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W63" s="6">
-        <v>365344.9764395468</v>
+        <v>325951.4286683677</v>
       </c>
       <c r="X63" s="7">
         <f>IF(V63=0,0,W63/V63)</f>
@@ -5174,28 +5168,28 @@
         <v>0</v>
       </c>
       <c r="D68" s="3">
-        <f>J68+G68</f>
+        <f>G68+J68</f>
         <v>0</v>
       </c>
       <c r="E68" s="3">
-        <f>P68+M68</f>
+        <f>M68+P68</f>
         <v>0</v>
       </c>
       <c r="F68" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G68" s="3">
-        <v>98.37588727255864</v>
+        <v>94.65713618175391</v>
       </c>
       <c r="H68" s="4">
         <f>IF(F68=0,0,G68/F68)</f>
         <v>0</v>
       </c>
       <c r="I68" s="3">
-        <v>382.3073643284126</v>
+        <v>382.3073643284127</v>
       </c>
       <c r="J68" s="6">
-        <v>25.16365196989442</v>
+        <v>22.4094333642202</v>
       </c>
       <c r="K68" s="7">
         <f>IF(I68=0,0,J68/I68)</f>
@@ -5225,7 +5219,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T68" s="3">
-        <v>1392.264622581063</v>
+        <v>1339.635002381882</v>
       </c>
       <c r="U68" s="4">
         <f>IF(S68=0,0,T68/S68)</f>
@@ -5235,7 +5229,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W68" s="6">
-        <v>623324.3944149893</v>
+        <v>554700.6611577384</v>
       </c>
       <c r="X68" s="7">
         <f>IF(V68=0,0,W68/V68)</f>
@@ -5271,18 +5265,18 @@
         <v>0</v>
       </c>
       <c r="D69" s="3">
-        <f>J69+G69</f>
+        <f>G69+J69</f>
         <v>0</v>
       </c>
       <c r="E69" s="3">
-        <f>P69+M69</f>
+        <f>M69+P69</f>
         <v>0</v>
       </c>
       <c r="F69" s="3">
-        <v>147.7607036391231</v>
+        <v>147.7607036391234</v>
       </c>
       <c r="G69" s="3">
-        <v>96.54985248064197</v>
+        <v>93.32656566805846</v>
       </c>
       <c r="H69" s="4">
         <f>IF(F69=0,0,G69/F69)</f>
@@ -5292,7 +5286,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J69" s="6">
-        <v>21.00591395392729</v>
+        <v>18.8267058367451</v>
       </c>
       <c r="K69" s="7">
         <f>IF(I69=0,0,J69/I69)</f>
@@ -5319,20 +5313,20 @@
         <v>0</v>
       </c>
       <c r="S69" s="3">
-        <v>2091.183174942718</v>
+        <v>2091.183174942721</v>
       </c>
       <c r="T69" s="3">
-        <v>1366.421667453817</v>
+        <v>1320.804104837496</v>
       </c>
       <c r="U69" s="4">
         <f>IF(S69=0,0,T69/S69)</f>
         <v>0</v>
       </c>
       <c r="V69" s="3">
-        <v>7100767.677214348</v>
+        <v>7100767.677214347</v>
       </c>
       <c r="W69" s="6">
-        <v>692794.2038804609</v>
+        <v>620735.8681268226</v>
       </c>
       <c r="X69" s="7">
         <f>IF(V69=0,0,W69/V69)</f>
@@ -5368,18 +5362,18 @@
         <v>0</v>
       </c>
       <c r="D70" s="3">
-        <f>J70+G70</f>
+        <f>G70+J70</f>
         <v>0</v>
       </c>
       <c r="E70" s="3">
-        <f>P70+M70</f>
+        <f>M70+P70</f>
         <v>0</v>
       </c>
       <c r="F70" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G70" s="3">
-        <v>92.20871899130873</v>
+        <v>89.3261468773603</v>
       </c>
       <c r="H70" s="4">
         <f>IF(F70=0,0,G70/F70)</f>
@@ -5389,7 +5383,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J70" s="6">
-        <v>22.61656617855842</v>
+        <v>20.20687125075571</v>
       </c>
       <c r="K70" s="7">
         <f>IF(I70=0,0,J70/I70)</f>
@@ -5419,7 +5413,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T70" s="3">
-        <v>1304.983781131581</v>
+        <v>1264.188182865007</v>
       </c>
       <c r="U70" s="4">
         <f>IF(S70=0,0,T70/S70)</f>
@@ -5429,7 +5423,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W70" s="6">
-        <v>794041.0575617198</v>
+        <v>709040.6150101619</v>
       </c>
       <c r="X70" s="7">
         <f>IF(V70=0,0,W70/V70)</f>
@@ -5465,18 +5459,18 @@
         <v>0</v>
       </c>
       <c r="D71" s="3">
-        <f>J71+G71</f>
+        <f>G71+J71</f>
         <v>0</v>
       </c>
       <c r="E71" s="3">
-        <f>P71+M71</f>
+        <f>M71+P71</f>
         <v>0</v>
       </c>
       <c r="F71" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G71" s="3">
-        <v>56.33344127694023</v>
+        <v>53.09835934079247</v>
       </c>
       <c r="H71" s="4">
         <f>IF(F71=0,0,G71/F71)</f>
@@ -5486,7 +5480,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J71" s="6">
-        <v>9.710502579285997</v>
+        <v>8.613532581916079</v>
       </c>
       <c r="K71" s="7">
         <f>IF(I71=0,0,J71/I71)</f>
@@ -5516,7 +5510,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T71" s="3">
-        <v>797.2589577853753</v>
+        <v>751.4744646974439</v>
       </c>
       <c r="U71" s="4">
         <f>IF(S71=0,0,T71/S71)</f>
@@ -5526,7 +5520,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W71" s="6">
-        <v>351805.066879469</v>
+        <v>311924.34926455</v>
       </c>
       <c r="X71" s="7">
         <f>IF(V71=0,0,W71/V71)</f>
@@ -5562,18 +5556,18 @@
         <v>0</v>
       </c>
       <c r="D72" s="3">
-        <f>J72+G72</f>
+        <f>G72+J72</f>
         <v>0</v>
       </c>
       <c r="E72" s="3">
-        <f>P72+M72</f>
+        <f>M72+P72</f>
         <v>0</v>
       </c>
       <c r="F72" s="3">
-        <v>93.49564395607474</v>
+        <v>93.49564395607489</v>
       </c>
       <c r="G72" s="3">
-        <v>36.20808203369902</v>
+        <v>33.88385898245032</v>
       </c>
       <c r="H72" s="4">
         <f>IF(F72=0,0,G72/F72)</f>
@@ -5583,7 +5577,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J72" s="6">
-        <v>7.45877905144963</v>
+        <v>6.654744068362823</v>
       </c>
       <c r="K72" s="7">
         <f>IF(I72=0,0,J72/I72)</f>
@@ -5610,10 +5604,10 @@
         <v>0</v>
       </c>
       <c r="S72" s="3">
-        <v>1323.19698509889</v>
+        <v>1323.196985098892</v>
       </c>
       <c r="T72" s="3">
-        <v>512.4348360626584</v>
+        <v>479.5412722132613</v>
       </c>
       <c r="U72" s="4">
         <f>IF(S72=0,0,T72/S72)</f>
@@ -5623,7 +5617,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W72" s="6">
-        <v>296120.1093025655</v>
+        <v>264152.6459177388</v>
       </c>
       <c r="X72" s="7">
         <f>IF(V72=0,0,W72/V72)</f>
@@ -5647,1222 +5641,6 @@
       </c>
       <c r="AD72" s="4">
         <f>IF(AB72=0,0,AC72/AB72)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:30">
-      <c r="A74" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="75" spans="1:30">
-      <c r="B75" t="s">
-        <v>28</v>
-      </c>
-      <c r="C75" s="3">
-        <f>C77+C78+C79+C80+C81</f>
-        <v>0</v>
-      </c>
-      <c r="D75" s="3">
-        <f>D77+D78+D79+D80+D81</f>
-        <v>0</v>
-      </c>
-      <c r="E75" s="3">
-        <f>E77+E78+E79+E80+E81</f>
-        <v>0</v>
-      </c>
-      <c r="F75" s="3">
-        <f>F77+F78+F79+F80+F81</f>
-        <v>0</v>
-      </c>
-      <c r="G75" s="3">
-        <f>G77+G78+G79+G80+G81</f>
-        <v>0</v>
-      </c>
-      <c r="H75" s="4">
-        <f>IF(F75=0,0,G75/F75)</f>
-        <v>0</v>
-      </c>
-      <c r="I75" s="3">
-        <f>I77+I78+I79+I80+I81</f>
-        <v>0</v>
-      </c>
-      <c r="J75" s="3">
-        <f>J77+J78+J79+J80+J81</f>
-        <v>0</v>
-      </c>
-      <c r="K75" s="4">
-        <f>IF(I75=0,0,J75/I75)</f>
-        <v>0</v>
-      </c>
-      <c r="L75" s="3">
-        <f>L77+L78+L79+L80+L81</f>
-        <v>0</v>
-      </c>
-      <c r="M75" s="3">
-        <f>M77+M78+M79+M80+M81</f>
-        <v>0</v>
-      </c>
-      <c r="N75" s="4">
-        <f>IF(L75=0,0,M75/L75)</f>
-        <v>0</v>
-      </c>
-      <c r="O75" s="3">
-        <f>O77+O78+O79+O80+O81</f>
-        <v>0</v>
-      </c>
-      <c r="P75" s="3">
-        <f>P77+P78+P79+P80+P81</f>
-        <v>0</v>
-      </c>
-      <c r="Q75" s="4">
-        <f>IF(O75=0,0,P75/O75)</f>
-        <v>0</v>
-      </c>
-      <c r="S75" s="3">
-        <f>S77+S78+S79+S80+S81</f>
-        <v>0</v>
-      </c>
-      <c r="T75" s="3">
-        <f>T77+T78+T79+T80+T81</f>
-        <v>0</v>
-      </c>
-      <c r="U75" s="4">
-        <f>IF(S75=0,0,T75/S75)</f>
-        <v>0</v>
-      </c>
-      <c r="V75" s="3">
-        <f>V77+V78+V79+V80+V81</f>
-        <v>0</v>
-      </c>
-      <c r="W75" s="3">
-        <f>W77+W78+W79+W80+W81</f>
-        <v>0</v>
-      </c>
-      <c r="X75" s="4">
-        <f>IF(V75=0,0,W75/V75)</f>
-        <v>0</v>
-      </c>
-      <c r="Y75" s="3">
-        <f>Y77+Y78+Y79+Y80+Y81</f>
-        <v>0</v>
-      </c>
-      <c r="Z75" s="3">
-        <f>Z77+Z78+Z79+Z80+Z81</f>
-        <v>0</v>
-      </c>
-      <c r="AA75" s="4">
-        <f>IF(Y75=0,0,Z75/Y75)</f>
-        <v>0</v>
-      </c>
-      <c r="AB75" s="3">
-        <f>AB77+AB78+AB79+AB80+AB81</f>
-        <v>0</v>
-      </c>
-      <c r="AC75" s="3">
-        <f>AC77+AC78+AC79+AC80+AC81</f>
-        <v>0</v>
-      </c>
-      <c r="AD75" s="4">
-        <f>IF(AB75=0,0,AC75/AB75)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:30">
-      <c r="A76" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="77" spans="1:30">
-      <c r="B77" t="s">
-        <v>30</v>
-      </c>
-      <c r="C77" s="3">
-        <f>J77+M77+G77+P77</f>
-        <v>0</v>
-      </c>
-      <c r="D77" s="3">
-        <f>G77</f>
-        <v>0</v>
-      </c>
-      <c r="E77" s="3">
-        <f>J77+M77+P77</f>
-        <v>0</v>
-      </c>
-      <c r="F77" s="3">
-        <v>412.7408750394843</v>
-      </c>
-      <c r="G77" s="3">
-        <v>146.8879599840255</v>
-      </c>
-      <c r="H77" s="4">
-        <f>IF(F77=0,0,G77/F77)</f>
-        <v>0</v>
-      </c>
-      <c r="I77" s="3">
-        <v>0</v>
-      </c>
-      <c r="J77" s="3">
-        <v>0</v>
-      </c>
-      <c r="K77" s="4">
-        <f>IF(I77=0,0,J77/I77)</f>
-        <v>0</v>
-      </c>
-      <c r="L77" s="3">
-        <v>0</v>
-      </c>
-      <c r="M77" s="3">
-        <v>0</v>
-      </c>
-      <c r="N77" s="4">
-        <f>IF(L77=0,0,M77/L77)</f>
-        <v>0</v>
-      </c>
-      <c r="O77" s="3">
-        <v>0</v>
-      </c>
-      <c r="P77" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q77" s="4">
-        <f>IF(O77=0,0,P77/O77)</f>
-        <v>0</v>
-      </c>
-      <c r="S77" s="3">
-        <v>12734.95565684622</v>
-      </c>
-      <c r="T77" s="3">
-        <v>4532.169625172735</v>
-      </c>
-      <c r="U77" s="4">
-        <f>IF(S77=0,0,T77/S77)</f>
-        <v>0</v>
-      </c>
-      <c r="V77" s="3">
-        <v>0</v>
-      </c>
-      <c r="W77" s="3">
-        <v>0</v>
-      </c>
-      <c r="X77" s="4">
-        <f>IF(V77=0,0,W77/V77)</f>
-        <v>0</v>
-      </c>
-      <c r="Y77" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z77" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA77" s="4">
-        <f>IF(Y77=0,0,Z77/Y77)</f>
-        <v>0</v>
-      </c>
-      <c r="AB77" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC77" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD77" s="4">
-        <f>IF(AB77=0,0,AC77/AB77)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:30">
-      <c r="B78" t="s">
-        <v>31</v>
-      </c>
-      <c r="C78" s="3">
-        <f>J78+M78+G78+P78</f>
-        <v>0</v>
-      </c>
-      <c r="D78" s="3">
-        <f>G78</f>
-        <v>0</v>
-      </c>
-      <c r="E78" s="3">
-        <f>J78+M78+P78</f>
-        <v>0</v>
-      </c>
-      <c r="F78" s="3">
-        <v>422.0532339939541</v>
-      </c>
-      <c r="G78" s="3">
-        <v>141.7344183926904</v>
-      </c>
-      <c r="H78" s="4">
-        <f>IF(F78=0,0,G78/F78)</f>
-        <v>0</v>
-      </c>
-      <c r="I78" s="3">
-        <v>0</v>
-      </c>
-      <c r="J78" s="3">
-        <v>0</v>
-      </c>
-      <c r="K78" s="4">
-        <f>IF(I78=0,0,J78/I78)</f>
-        <v>0</v>
-      </c>
-      <c r="L78" s="3">
-        <v>0</v>
-      </c>
-      <c r="M78" s="3">
-        <v>0</v>
-      </c>
-      <c r="N78" s="4">
-        <f>IF(L78=0,0,M78/L78)</f>
-        <v>0</v>
-      </c>
-      <c r="O78" s="3">
-        <v>0</v>
-      </c>
-      <c r="P78" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q78" s="4">
-        <f>IF(O78=0,0,P78/O78)</f>
-        <v>0</v>
-      </c>
-      <c r="S78" s="3">
-        <v>13022.28479122008</v>
-      </c>
-      <c r="T78" s="3">
-        <v>4373.159147630166</v>
-      </c>
-      <c r="U78" s="4">
-        <f>IF(S78=0,0,T78/S78)</f>
-        <v>0</v>
-      </c>
-      <c r="V78" s="3">
-        <v>0</v>
-      </c>
-      <c r="W78" s="3">
-        <v>0</v>
-      </c>
-      <c r="X78" s="4">
-        <f>IF(V78=0,0,W78/V78)</f>
-        <v>0</v>
-      </c>
-      <c r="Y78" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z78" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA78" s="4">
-        <f>IF(Y78=0,0,Z78/Y78)</f>
-        <v>0</v>
-      </c>
-      <c r="AB78" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC78" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD78" s="4">
-        <f>IF(AB78=0,0,AC78/AB78)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="1:30">
-      <c r="B79" t="s">
-        <v>32</v>
-      </c>
-      <c r="C79" s="3">
-        <f>J79+M79+G79+P79</f>
-        <v>0</v>
-      </c>
-      <c r="D79" s="3">
-        <f>G79</f>
-        <v>0</v>
-      </c>
-      <c r="E79" s="3">
-        <f>J79+M79+P79</f>
-        <v>0</v>
-      </c>
-      <c r="F79" s="3">
-        <v>382.0743136549376</v>
-      </c>
-      <c r="G79" s="3">
-        <v>124.6559480289836</v>
-      </c>
-      <c r="H79" s="4">
-        <f>IF(F79=0,0,G79/F79)</f>
-        <v>0</v>
-      </c>
-      <c r="I79" s="3">
-        <v>0</v>
-      </c>
-      <c r="J79" s="3">
-        <v>0</v>
-      </c>
-      <c r="K79" s="4">
-        <f>IF(I79=0,0,J79/I79)</f>
-        <v>0</v>
-      </c>
-      <c r="L79" s="3">
-        <v>0</v>
-      </c>
-      <c r="M79" s="3">
-        <v>0</v>
-      </c>
-      <c r="N79" s="4">
-        <f>IF(L79=0,0,M79/L79)</f>
-        <v>0</v>
-      </c>
-      <c r="O79" s="3">
-        <v>0</v>
-      </c>
-      <c r="P79" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q79" s="4">
-        <f>IF(O79=0,0,P79/O79)</f>
-        <v>0</v>
-      </c>
-      <c r="S79" s="3">
-        <v>11788.75109364953</v>
-      </c>
-      <c r="T79" s="3">
-        <v>3846.209732339612</v>
-      </c>
-      <c r="U79" s="4">
-        <f>IF(S79=0,0,T79/S79)</f>
-        <v>0</v>
-      </c>
-      <c r="V79" s="3">
-        <v>0</v>
-      </c>
-      <c r="W79" s="3">
-        <v>0</v>
-      </c>
-      <c r="X79" s="4">
-        <f>IF(V79=0,0,W79/V79)</f>
-        <v>0</v>
-      </c>
-      <c r="Y79" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z79" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA79" s="4">
-        <f>IF(Y79=0,0,Z79/Y79)</f>
-        <v>0</v>
-      </c>
-      <c r="AB79" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC79" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD79" s="4">
-        <f>IF(AB79=0,0,AC79/AB79)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:30">
-      <c r="B80" t="s">
-        <v>33</v>
-      </c>
-      <c r="C80" s="3">
-        <f>J80+M80+G80+P80</f>
-        <v>0</v>
-      </c>
-      <c r="D80" s="3">
-        <f>G80</f>
-        <v>0</v>
-      </c>
-      <c r="E80" s="3">
-        <f>J80+M80+P80</f>
-        <v>0</v>
-      </c>
-      <c r="F80" s="3">
-        <v>338.6701578384149</v>
-      </c>
-      <c r="G80" s="3">
-        <v>106.5823973125179</v>
-      </c>
-      <c r="H80" s="4">
-        <f>IF(F80=0,0,G80/F80)</f>
-        <v>0</v>
-      </c>
-      <c r="I80" s="3">
-        <v>0</v>
-      </c>
-      <c r="J80" s="3">
-        <v>0</v>
-      </c>
-      <c r="K80" s="4">
-        <f>IF(I80=0,0,J80/I80)</f>
-        <v>0</v>
-      </c>
-      <c r="L80" s="3">
-        <v>0</v>
-      </c>
-      <c r="M80" s="3">
-        <v>0</v>
-      </c>
-      <c r="N80" s="4">
-        <f>IF(L80=0,0,M80/L80)</f>
-        <v>0</v>
-      </c>
-      <c r="O80" s="3">
-        <v>0</v>
-      </c>
-      <c r="P80" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q80" s="4">
-        <f>IF(O80=0,0,P80/O80)</f>
-        <v>0</v>
-      </c>
-      <c r="S80" s="3">
-        <v>10449.53311676904</v>
-      </c>
-      <c r="T80" s="3">
-        <v>3288.557508256084</v>
-      </c>
-      <c r="U80" s="4">
-        <f>IF(S80=0,0,T80/S80)</f>
-        <v>0</v>
-      </c>
-      <c r="V80" s="3">
-        <v>0</v>
-      </c>
-      <c r="W80" s="3">
-        <v>0</v>
-      </c>
-      <c r="X80" s="4">
-        <f>IF(V80=0,0,W80/V80)</f>
-        <v>0</v>
-      </c>
-      <c r="Y80" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z80" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA80" s="4">
-        <f>IF(Y80=0,0,Z80/Y80)</f>
-        <v>0</v>
-      </c>
-      <c r="AB80" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC80" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD80" s="4">
-        <f>IF(AB80=0,0,AC80/AB80)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:30">
-      <c r="B81" t="s">
-        <v>34</v>
-      </c>
-      <c r="C81" s="3">
-        <f>J81+M81+G81+P81</f>
-        <v>0</v>
-      </c>
-      <c r="D81" s="3">
-        <f>G81</f>
-        <v>0</v>
-      </c>
-      <c r="E81" s="3">
-        <f>J81+M81+P81</f>
-        <v>0</v>
-      </c>
-      <c r="F81" s="3">
-        <v>297.4602934996698</v>
-      </c>
-      <c r="G81" s="3">
-        <v>93.75383596516214</v>
-      </c>
-      <c r="H81" s="4">
-        <f>IF(F81=0,0,G81/F81)</f>
-        <v>0</v>
-      </c>
-      <c r="I81" s="3">
-        <v>0</v>
-      </c>
-      <c r="J81" s="3">
-        <v>0</v>
-      </c>
-      <c r="K81" s="4">
-        <f>IF(I81=0,0,J81/I81)</f>
-        <v>0</v>
-      </c>
-      <c r="L81" s="3">
-        <v>0</v>
-      </c>
-      <c r="M81" s="3">
-        <v>0</v>
-      </c>
-      <c r="N81" s="4">
-        <f>IF(L81=0,0,M81/L81)</f>
-        <v>0</v>
-      </c>
-      <c r="O81" s="3">
-        <v>0</v>
-      </c>
-      <c r="P81" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q81" s="4">
-        <f>IF(O81=0,0,P81/O81)</f>
-        <v>0</v>
-      </c>
-      <c r="S81" s="3">
-        <v>9178.019131321482</v>
-      </c>
-      <c r="T81" s="3">
-        <v>2892.73734655274</v>
-      </c>
-      <c r="U81" s="4">
-        <f>IF(S81=0,0,T81/S81)</f>
-        <v>0</v>
-      </c>
-      <c r="V81" s="3">
-        <v>0</v>
-      </c>
-      <c r="W81" s="3">
-        <v>0</v>
-      </c>
-      <c r="X81" s="4">
-        <f>IF(V81=0,0,W81/V81)</f>
-        <v>0</v>
-      </c>
-      <c r="Y81" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z81" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA81" s="4">
-        <f>IF(Y81=0,0,Z81/Y81)</f>
-        <v>0</v>
-      </c>
-      <c r="AB81" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC81" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD81" s="4">
-        <f>IF(AB81=0,0,AC81/AB81)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:30">
-      <c r="A83" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="84" spans="1:30">
-      <c r="B84" t="s">
-        <v>28</v>
-      </c>
-      <c r="C84" s="3">
-        <f>C86+C87+C88+C89+C90</f>
-        <v>0</v>
-      </c>
-      <c r="D84" s="3">
-        <f>D86+D87+D88+D89+D90</f>
-        <v>0</v>
-      </c>
-      <c r="E84" s="3">
-        <f>E86+E87+E88+E89+E90</f>
-        <v>0</v>
-      </c>
-      <c r="F84" s="3">
-        <f>F86+F87+F88+F89+F90</f>
-        <v>0</v>
-      </c>
-      <c r="G84" s="3">
-        <f>G86+G87+G88+G89+G90</f>
-        <v>0</v>
-      </c>
-      <c r="H84" s="4">
-        <f>IF(F84=0,0,G84/F84)</f>
-        <v>0</v>
-      </c>
-      <c r="I84" s="3">
-        <f>I86+I87+I88+I89+I90</f>
-        <v>0</v>
-      </c>
-      <c r="J84" s="3">
-        <f>J86+J87+J88+J89+J90</f>
-        <v>0</v>
-      </c>
-      <c r="K84" s="4">
-        <f>IF(I84=0,0,J84/I84)</f>
-        <v>0</v>
-      </c>
-      <c r="L84" s="3">
-        <f>L86+L87+L88+L89+L90</f>
-        <v>0</v>
-      </c>
-      <c r="M84" s="3">
-        <f>M86+M87+M88+M89+M90</f>
-        <v>0</v>
-      </c>
-      <c r="N84" s="4">
-        <f>IF(L84=0,0,M84/L84)</f>
-        <v>0</v>
-      </c>
-      <c r="O84" s="3">
-        <f>O86+O87+O88+O89+O90</f>
-        <v>0</v>
-      </c>
-      <c r="P84" s="3">
-        <f>P86+P87+P88+P89+P90</f>
-        <v>0</v>
-      </c>
-      <c r="Q84" s="4">
-        <f>IF(O84=0,0,P84/O84)</f>
-        <v>0</v>
-      </c>
-      <c r="S84" s="3">
-        <f>S86+S87+S88+S89+S90</f>
-        <v>0</v>
-      </c>
-      <c r="T84" s="3">
-        <f>T86+T87+T88+T89+T90</f>
-        <v>0</v>
-      </c>
-      <c r="U84" s="4">
-        <f>IF(S84=0,0,T84/S84)</f>
-        <v>0</v>
-      </c>
-      <c r="V84" s="3">
-        <f>V86+V87+V88+V89+V90</f>
-        <v>0</v>
-      </c>
-      <c r="W84" s="3">
-        <f>W86+W87+W88+W89+W90</f>
-        <v>0</v>
-      </c>
-      <c r="X84" s="4">
-        <f>IF(V84=0,0,W84/V84)</f>
-        <v>0</v>
-      </c>
-      <c r="Y84" s="3">
-        <f>Y86+Y87+Y88+Y89+Y90</f>
-        <v>0</v>
-      </c>
-      <c r="Z84" s="3">
-        <f>Z86+Z87+Z88+Z89+Z90</f>
-        <v>0</v>
-      </c>
-      <c r="AA84" s="4">
-        <f>IF(Y84=0,0,Z84/Y84)</f>
-        <v>0</v>
-      </c>
-      <c r="AB84" s="3">
-        <f>AB86+AB87+AB88+AB89+AB90</f>
-        <v>0</v>
-      </c>
-      <c r="AC84" s="3">
-        <f>AC86+AC87+AC88+AC89+AC90</f>
-        <v>0</v>
-      </c>
-      <c r="AD84" s="4">
-        <f>IF(AB84=0,0,AC84/AB84)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:30">
-      <c r="A85" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="86" spans="1:30">
-      <c r="B86" t="s">
-        <v>30</v>
-      </c>
-      <c r="C86" s="3">
-        <f>J86+M86+G86+P86</f>
-        <v>0</v>
-      </c>
-      <c r="D86" s="3">
-        <f>G86</f>
-        <v>0</v>
-      </c>
-      <c r="E86" s="3">
-        <f>J86+M86+P86</f>
-        <v>0</v>
-      </c>
-      <c r="F86" s="3">
-        <v>412.7408750394843</v>
-      </c>
-      <c r="G86" s="3">
-        <v>270.621528830763</v>
-      </c>
-      <c r="H86" s="4">
-        <f>IF(F86=0,0,G86/F86)</f>
-        <v>0</v>
-      </c>
-      <c r="I86" s="3">
-        <v>0</v>
-      </c>
-      <c r="J86" s="3">
-        <v>0</v>
-      </c>
-      <c r="K86" s="4">
-        <f>IF(I86=0,0,J86/I86)</f>
-        <v>0</v>
-      </c>
-      <c r="L86" s="3">
-        <v>0</v>
-      </c>
-      <c r="M86" s="3">
-        <v>0</v>
-      </c>
-      <c r="N86" s="4">
-        <f>IF(L86=0,0,M86/L86)</f>
-        <v>0</v>
-      </c>
-      <c r="O86" s="3">
-        <v>0</v>
-      </c>
-      <c r="P86" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q86" s="4">
-        <f>IF(O86=0,0,P86/O86)</f>
-        <v>0</v>
-      </c>
-      <c r="S86" s="3">
-        <v>12734.95565684622</v>
-      </c>
-      <c r="T86" s="3">
-        <v>8349.919714440704</v>
-      </c>
-      <c r="U86" s="4">
-        <f>IF(S86=0,0,T86/S86)</f>
-        <v>0</v>
-      </c>
-      <c r="V86" s="3">
-        <v>0</v>
-      </c>
-      <c r="W86" s="3">
-        <v>0</v>
-      </c>
-      <c r="X86" s="4">
-        <f>IF(V86=0,0,W86/V86)</f>
-        <v>0</v>
-      </c>
-      <c r="Y86" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z86" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA86" s="4">
-        <f>IF(Y86=0,0,Z86/Y86)</f>
-        <v>0</v>
-      </c>
-      <c r="AB86" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC86" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD86" s="4">
-        <f>IF(AB86=0,0,AC86/AB86)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="1:30">
-      <c r="B87" t="s">
-        <v>31</v>
-      </c>
-      <c r="C87" s="3">
-        <f>J87+M87+G87+P87</f>
-        <v>0</v>
-      </c>
-      <c r="D87" s="3">
-        <f>G87</f>
-        <v>0</v>
-      </c>
-      <c r="E87" s="3">
-        <f>J87+M87+P87</f>
-        <v>0</v>
-      </c>
-      <c r="F87" s="3">
-        <v>422.0532339939541</v>
-      </c>
-      <c r="G87" s="3">
-        <v>268.8415075664349</v>
-      </c>
-      <c r="H87" s="4">
-        <f>IF(F87=0,0,G87/F87)</f>
-        <v>0</v>
-      </c>
-      <c r="I87" s="3">
-        <v>0</v>
-      </c>
-      <c r="J87" s="3">
-        <v>0</v>
-      </c>
-      <c r="K87" s="4">
-        <f>IF(I87=0,0,J87/I87)</f>
-        <v>0</v>
-      </c>
-      <c r="L87" s="3">
-        <v>0</v>
-      </c>
-      <c r="M87" s="3">
-        <v>0</v>
-      </c>
-      <c r="N87" s="4">
-        <f>IF(L87=0,0,M87/L87)</f>
-        <v>0</v>
-      </c>
-      <c r="O87" s="3">
-        <v>0</v>
-      </c>
-      <c r="P87" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q87" s="4">
-        <f>IF(O87=0,0,P87/O87)</f>
-        <v>0</v>
-      </c>
-      <c r="S87" s="3">
-        <v>13022.28479122008</v>
-      </c>
-      <c r="T87" s="3">
-        <v>8294.997865793428</v>
-      </c>
-      <c r="U87" s="4">
-        <f>IF(S87=0,0,T87/S87)</f>
-        <v>0</v>
-      </c>
-      <c r="V87" s="3">
-        <v>0</v>
-      </c>
-      <c r="W87" s="3">
-        <v>0</v>
-      </c>
-      <c r="X87" s="4">
-        <f>IF(V87=0,0,W87/V87)</f>
-        <v>0</v>
-      </c>
-      <c r="Y87" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z87" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA87" s="4">
-        <f>IF(Y87=0,0,Z87/Y87)</f>
-        <v>0</v>
-      </c>
-      <c r="AB87" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC87" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD87" s="4">
-        <f>IF(AB87=0,0,AC87/AB87)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="1:30">
-      <c r="B88" t="s">
-        <v>32</v>
-      </c>
-      <c r="C88" s="3">
-        <f>J88+M88+G88+P88</f>
-        <v>0</v>
-      </c>
-      <c r="D88" s="3">
-        <f>G88</f>
-        <v>0</v>
-      </c>
-      <c r="E88" s="3">
-        <f>J88+M88+P88</f>
-        <v>0</v>
-      </c>
-      <c r="F88" s="3">
-        <v>382.0743136549376</v>
-      </c>
-      <c r="G88" s="3">
-        <v>239.83782878063</v>
-      </c>
-      <c r="H88" s="4">
-        <f>IF(F88=0,0,G88/F88)</f>
-        <v>0</v>
-      </c>
-      <c r="I88" s="3">
-        <v>0</v>
-      </c>
-      <c r="J88" s="3">
-        <v>0</v>
-      </c>
-      <c r="K88" s="4">
-        <f>IF(I88=0,0,J88/I88)</f>
-        <v>0</v>
-      </c>
-      <c r="L88" s="3">
-        <v>0</v>
-      </c>
-      <c r="M88" s="3">
-        <v>0</v>
-      </c>
-      <c r="N88" s="4">
-        <f>IF(L88=0,0,M88/L88)</f>
-        <v>0</v>
-      </c>
-      <c r="O88" s="3">
-        <v>0</v>
-      </c>
-      <c r="P88" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q88" s="4">
-        <f>IF(O88=0,0,P88/O88)</f>
-        <v>0</v>
-      </c>
-      <c r="S88" s="3">
-        <v>11788.75109364953</v>
-      </c>
-      <c r="T88" s="3">
-        <v>7400.100884273723</v>
-      </c>
-      <c r="U88" s="4">
-        <f>IF(S88=0,0,T88/S88)</f>
-        <v>0</v>
-      </c>
-      <c r="V88" s="3">
-        <v>0</v>
-      </c>
-      <c r="W88" s="3">
-        <v>0</v>
-      </c>
-      <c r="X88" s="4">
-        <f>IF(V88=0,0,W88/V88)</f>
-        <v>0</v>
-      </c>
-      <c r="Y88" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z88" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA88" s="4">
-        <f>IF(Y88=0,0,Z88/Y88)</f>
-        <v>0</v>
-      </c>
-      <c r="AB88" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC88" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD88" s="4">
-        <f>IF(AB88=0,0,AC88/AB88)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="1:30">
-      <c r="B89" t="s">
-        <v>33</v>
-      </c>
-      <c r="C89" s="3">
-        <f>J89+M89+G89+P89</f>
-        <v>0</v>
-      </c>
-      <c r="D89" s="3">
-        <f>G89</f>
-        <v>0</v>
-      </c>
-      <c r="E89" s="3">
-        <f>J89+M89+P89</f>
-        <v>0</v>
-      </c>
-      <c r="F89" s="3">
-        <v>338.6701578384149</v>
-      </c>
-      <c r="G89" s="3">
-        <v>208.6917795068874</v>
-      </c>
-      <c r="H89" s="4">
-        <f>IF(F89=0,0,G89/F89)</f>
-        <v>0</v>
-      </c>
-      <c r="I89" s="3">
-        <v>0</v>
-      </c>
-      <c r="J89" s="3">
-        <v>0</v>
-      </c>
-      <c r="K89" s="4">
-        <f>IF(I89=0,0,J89/I89)</f>
-        <v>0</v>
-      </c>
-      <c r="L89" s="3">
-        <v>0</v>
-      </c>
-      <c r="M89" s="3">
-        <v>0</v>
-      </c>
-      <c r="N89" s="4">
-        <f>IF(L89=0,0,M89/L89)</f>
-        <v>0</v>
-      </c>
-      <c r="O89" s="3">
-        <v>0</v>
-      </c>
-      <c r="P89" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q89" s="4">
-        <f>IF(O89=0,0,P89/O89)</f>
-        <v>0</v>
-      </c>
-      <c r="S89" s="3">
-        <v>10449.53311676904</v>
-      </c>
-      <c r="T89" s="3">
-        <v>6439.101912826773</v>
-      </c>
-      <c r="U89" s="4">
-        <f>IF(S89=0,0,T89/S89)</f>
-        <v>0</v>
-      </c>
-      <c r="V89" s="3">
-        <v>0</v>
-      </c>
-      <c r="W89" s="3">
-        <v>0</v>
-      </c>
-      <c r="X89" s="4">
-        <f>IF(V89=0,0,W89/V89)</f>
-        <v>0</v>
-      </c>
-      <c r="Y89" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z89" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA89" s="4">
-        <f>IF(Y89=0,0,Z89/Y89)</f>
-        <v>0</v>
-      </c>
-      <c r="AB89" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC89" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD89" s="4">
-        <f>IF(AB89=0,0,AC89/AB89)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="1:30">
-      <c r="B90" t="s">
-        <v>34</v>
-      </c>
-      <c r="C90" s="3">
-        <f>J90+M90+G90+P90</f>
-        <v>0</v>
-      </c>
-      <c r="D90" s="3">
-        <f>G90</f>
-        <v>0</v>
-      </c>
-      <c r="E90" s="3">
-        <f>J90+M90+P90</f>
-        <v>0</v>
-      </c>
-      <c r="F90" s="3">
-        <v>297.4602934996698</v>
-      </c>
-      <c r="G90" s="3">
-        <v>183.4401220978906</v>
-      </c>
-      <c r="H90" s="4">
-        <f>IF(F90=0,0,G90/F90)</f>
-        <v>0</v>
-      </c>
-      <c r="I90" s="3">
-        <v>0</v>
-      </c>
-      <c r="J90" s="3">
-        <v>0</v>
-      </c>
-      <c r="K90" s="4">
-        <f>IF(I90=0,0,J90/I90)</f>
-        <v>0</v>
-      </c>
-      <c r="L90" s="3">
-        <v>0</v>
-      </c>
-      <c r="M90" s="3">
-        <v>0</v>
-      </c>
-      <c r="N90" s="4">
-        <f>IF(L90=0,0,M90/L90)</f>
-        <v>0</v>
-      </c>
-      <c r="O90" s="3">
-        <v>0</v>
-      </c>
-      <c r="P90" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q90" s="4">
-        <f>IF(O90=0,0,P90/O90)</f>
-        <v>0</v>
-      </c>
-      <c r="S90" s="3">
-        <v>9178.019131321482</v>
-      </c>
-      <c r="T90" s="3">
-        <v>5659.972059659981</v>
-      </c>
-      <c r="U90" s="4">
-        <f>IF(S90=0,0,T90/S90)</f>
-        <v>0</v>
-      </c>
-      <c r="V90" s="3">
-        <v>0</v>
-      </c>
-      <c r="W90" s="3">
-        <v>0</v>
-      </c>
-      <c r="X90" s="4">
-        <f>IF(V90=0,0,W90/V90)</f>
-        <v>0</v>
-      </c>
-      <c r="Y90" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z90" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA90" s="4">
-        <f>IF(Y90=0,0,Z90/Y90)</f>
-        <v>0</v>
-      </c>
-      <c r="AB90" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC90" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD90" s="4">
-        <f>IF(AB90=0,0,AC90/AB90)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
run with updated data
</commit_message>
<xml_diff>
--- a/5000_analyze_results/results_spreadsheet.xlsx
+++ b/5000_analyze_results/results_spreadsheet.xlsx
@@ -263,7 +263,7 @@
     <t>Annual Child Deaths Averted (%)</t>
   </si>
   <si>
-    <t>India -- Rice-- 80% PDS vs none</t>
+    <t>India -- Rice-- Current PDS fortification vs none</t>
   </si>
   <si>
     <t>National</t>
@@ -287,7 +287,7 @@
     <t>Wealthiest</t>
   </si>
   <si>
-    <t>India -- Rice-- 80% PDS with increased folate vs none</t>
+    <t>India -- Rice-- Scaled-up PDS and industry fortification with increased folate vs none</t>
   </si>
   <si>
     <t>Nigeria -- Bouillon</t>
@@ -923,37 +923,37 @@
         <v>362.8529849538489</v>
       </c>
       <c r="G5" s="3">
-        <v>15.87131876495009</v>
+        <v>12.63948471625394</v>
       </c>
       <c r="H5" s="4">
         <f>IF(F5=0,0,G5/F5)</f>
         <v>0</v>
       </c>
       <c r="I5" s="3">
-        <v>4771.261231090824</v>
+        <v>4770.95717689731</v>
       </c>
       <c r="J5" s="3">
-        <v>288.4337566118361</v>
+        <v>227.2989874536637</v>
       </c>
       <c r="K5" s="4">
         <f>IF(I5=0,0,J5/I5)</f>
         <v>0</v>
       </c>
       <c r="L5" s="3">
-        <v>17957.14040242062</v>
+        <v>17865.36054925314</v>
       </c>
       <c r="M5" s="3">
-        <v>44.43225446508453</v>
+        <v>21.65626037991047</v>
       </c>
       <c r="N5" s="4">
         <f>IF(L5=0,0,M5/L5)</f>
         <v>0</v>
       </c>
       <c r="O5" s="3">
-        <v>506.7963637284521</v>
+        <v>498.0330422263939</v>
       </c>
       <c r="P5" s="3">
-        <v>15.14918337618344</v>
+        <v>10.65439426484809</v>
       </c>
       <c r="Q5" s="4">
         <f>IF(O5=0,0,P5/O5)</f>
@@ -963,37 +963,37 @@
         <v>4684.597214204819</v>
       </c>
       <c r="T5" s="3">
-        <v>204.9059502197524</v>
+        <v>163.1815014510039</v>
       </c>
       <c r="U5" s="4">
         <f>IF(S5=0,0,T5/S5)</f>
         <v>0</v>
       </c>
       <c r="V5" s="3">
-        <v>131696392.1412486</v>
+        <v>131693773.0318688</v>
       </c>
       <c r="W5" s="3">
-        <v>6289843.2834488</v>
+        <v>4951659.460940793</v>
       </c>
       <c r="X5" s="4">
         <f>IF(V5=0,0,W5/V5)</f>
         <v>0</v>
       </c>
       <c r="Y5" s="3">
-        <v>3016543.050471412</v>
+        <v>3015958.720793084</v>
       </c>
       <c r="Z5" s="3">
-        <v>83032.52589576412</v>
+        <v>60837.61671482259</v>
       </c>
       <c r="AA5" s="4">
         <f>IF(Y5=0,0,Z5/Y5)</f>
         <v>0</v>
       </c>
       <c r="AB5" s="3">
-        <v>200318.014600175</v>
+        <v>199267.9177921558</v>
       </c>
       <c r="AC5" s="3">
-        <v>493.8569486366468</v>
+        <v>240.7198813628347</v>
       </c>
       <c r="AD5" s="4">
         <f>IF(AB5=0,0,AC5/AB5)</f>
@@ -1020,37 +1020,37 @@
         <v>320.5427437766894</v>
       </c>
       <c r="G6" s="3">
-        <v>11.4178093054627</v>
+        <v>9.074264240933234</v>
       </c>
       <c r="H6" s="4">
         <f>IF(F6=0,0,G6/F6)</f>
         <v>0</v>
       </c>
       <c r="I6" s="3">
-        <v>4315.21265961095</v>
+        <v>4315.385289601074</v>
       </c>
       <c r="J6" s="3">
-        <v>254.1003600447956</v>
+        <v>200.2233643732518</v>
       </c>
       <c r="K6" s="4">
         <f>IF(I6=0,0,J6/I6)</f>
         <v>0</v>
       </c>
       <c r="L6" s="3">
-        <v>14810.98291993852</v>
+        <v>14745.99462597537</v>
       </c>
       <c r="M6" s="3">
-        <v>28.82721546485461</v>
+        <v>25.98758979552239</v>
       </c>
       <c r="N6" s="4">
         <f>IF(L6=0,0,M6/L6)</f>
         <v>0</v>
       </c>
       <c r="O6" s="3">
-        <v>297.573370209569</v>
+        <v>290.5430769057631</v>
       </c>
       <c r="P6" s="3">
-        <v>8.009454753871308</v>
+        <v>6.01854625810642</v>
       </c>
       <c r="Q6" s="4">
         <f>IF(O6=0,0,P6/O6)</f>
@@ -1060,37 +1060,37 @@
         <v>4138.352740079671</v>
       </c>
       <c r="T6" s="3">
-        <v>147.4091157648745</v>
+        <v>117.1528821498905</v>
       </c>
       <c r="U6" s="4">
         <f>IF(S6=0,0,T6/S6)</f>
         <v>0</v>
       </c>
       <c r="V6" s="3">
-        <v>123352422.8520256</v>
+        <v>123347857.654681</v>
       </c>
       <c r="W6" s="3">
-        <v>5823141.870583907</v>
+        <v>4587770.16940327</v>
       </c>
       <c r="X6" s="4">
         <f>IF(V6=0,0,W6/V6)</f>
         <v>0</v>
       </c>
       <c r="Y6" s="3">
-        <v>1788522.531513863</v>
+        <v>1789154.954169832</v>
       </c>
       <c r="Z6" s="3">
-        <v>45063.12004884495</v>
+        <v>35204.0596326089</v>
       </c>
       <c r="AA6" s="4">
         <f>IF(Y6=0,0,Z6/Y6)</f>
         <v>0</v>
       </c>
       <c r="AB6" s="3">
-        <v>165227.6716058255</v>
+        <v>164556.1108996349</v>
       </c>
       <c r="AC6" s="3">
-        <v>320.4047520423192</v>
+        <v>288.8638576354133</v>
       </c>
       <c r="AD6" s="4">
         <f>IF(AB6=0,0,AC6/AB6)</f>
@@ -1117,37 +1117,37 @@
         <v>287.7720482472399</v>
       </c>
       <c r="G7" s="3">
-        <v>9.581140009551017</v>
+        <v>7.610121026612585</v>
       </c>
       <c r="H7" s="4">
         <f>IF(F7=0,0,G7/F7)</f>
         <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>4220.065012527612</v>
+        <v>4219.566052104662</v>
       </c>
       <c r="J7" s="3">
-        <v>227.9834892376838</v>
+        <v>179.6543713526069</v>
       </c>
       <c r="K7" s="4">
         <f>IF(I7=0,0,J7/I7)</f>
         <v>0</v>
       </c>
       <c r="L7" s="3">
-        <v>13140.17641177926</v>
+        <v>13471.87729543747</v>
       </c>
       <c r="M7" s="3">
-        <v>23.20586178746074</v>
+        <v>12.99224385871738</v>
       </c>
       <c r="N7" s="4">
         <f>IF(L7=0,0,M7/L7)</f>
         <v>0</v>
       </c>
       <c r="O7" s="3">
-        <v>350.6722046220511</v>
+        <v>365.4556715009266</v>
       </c>
       <c r="P7" s="3">
-        <v>7.443215477898834</v>
+        <v>4.144179226859298</v>
       </c>
       <c r="Q7" s="4">
         <f>IF(O7=0,0,P7/O7)</f>
@@ -1157,37 +1157,37 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T7" s="3">
-        <v>123.6968790634523</v>
+        <v>98.25012674365871</v>
       </c>
       <c r="U7" s="4">
         <f>IF(S7=0,0,T7/S7)</f>
         <v>0</v>
       </c>
       <c r="V7" s="3">
-        <v>121045766.1486471</v>
+        <v>121037522.2666742</v>
       </c>
       <c r="W7" s="3">
-        <v>5290763.08339116</v>
+        <v>4168961.673235625</v>
       </c>
       <c r="X7" s="4">
         <f>IF(V7=0,0,W7/V7)</f>
         <v>0</v>
       </c>
       <c r="Y7" s="3">
-        <v>2261372.687672075</v>
+        <v>2253925.490084493</v>
       </c>
       <c r="Z7" s="3">
-        <v>51512.38835039269</v>
+        <v>42081.355435153</v>
       </c>
       <c r="AA7" s="4">
         <f>IF(Y7=0,0,Z7/Y7)</f>
         <v>0</v>
       </c>
       <c r="AB7" s="3">
-        <v>146579.1514136479</v>
+        <v>150305.4939229549</v>
       </c>
       <c r="AC7" s="3">
-        <v>257.7692366055271</v>
+        <v>144.4319288176775</v>
       </c>
       <c r="AD7" s="4">
         <f>IF(AB7=0,0,AC7/AB7)</f>
@@ -1214,37 +1214,37 @@
         <v>271.3548595424364</v>
       </c>
       <c r="G8" s="3">
-        <v>8.370468320719199</v>
+        <v>6.644413322735986</v>
       </c>
       <c r="H8" s="4">
         <f>IF(F8=0,0,G8/F8)</f>
         <v>0</v>
       </c>
       <c r="I8" s="3">
-        <v>3866.462901477351</v>
+        <v>3865.872986383962</v>
       </c>
       <c r="J8" s="3">
-        <v>196.466800308214</v>
+        <v>154.4857842407785</v>
       </c>
       <c r="K8" s="4">
         <f>IF(I8=0,0,J8/I8)</f>
         <v>0</v>
       </c>
       <c r="L8" s="3">
-        <v>12529.63951354596</v>
+        <v>12349.08716881772</v>
       </c>
       <c r="M8" s="3">
-        <v>24.70940240938403</v>
+        <v>21.6557056759987</v>
       </c>
       <c r="N8" s="4">
         <f>IF(L8=0,0,M8/L8)</f>
         <v>0</v>
       </c>
       <c r="O8" s="3">
-        <v>341.4996444598856</v>
+        <v>301.3694049551027</v>
       </c>
       <c r="P8" s="3">
-        <v>9.412116673423151</v>
+        <v>6.676028088355379</v>
       </c>
       <c r="Q8" s="4">
         <f>IF(O8=0,0,P8/O8)</f>
@@ -1254,37 +1254,37 @@
         <v>3503.314763237015</v>
       </c>
       <c r="T8" s="3">
-        <v>108.0665564369497</v>
+        <v>85.78240067578145</v>
       </c>
       <c r="U8" s="4">
         <f>IF(S8=0,0,T8/S8)</f>
         <v>0</v>
       </c>
       <c r="V8" s="3">
-        <v>114934295.1461658</v>
+        <v>114934351.5045501</v>
       </c>
       <c r="W8" s="3">
-        <v>4795957.281183481</v>
+        <v>3775258.761166275</v>
       </c>
       <c r="X8" s="4">
         <f>IF(V8=0,0,W8/V8)</f>
         <v>0</v>
       </c>
       <c r="Y8" s="3">
-        <v>2020070.981660255</v>
+        <v>2008507.025186675</v>
       </c>
       <c r="Z8" s="3">
-        <v>43199.51716528833</v>
+        <v>31981.83013071725</v>
       </c>
       <c r="AA8" s="4">
         <f>IF(Y8=0,0,Z8/Y8)</f>
         <v>0</v>
       </c>
       <c r="AB8" s="3">
-        <v>139766.3345807479</v>
+        <v>137739.9161158149</v>
       </c>
       <c r="AC8" s="3">
-        <v>274.6326446077146</v>
+        <v>240.7198813628347</v>
       </c>
       <c r="AD8" s="4">
         <f>IF(AB8=0,0,AC8/AB8)</f>
@@ -1311,37 +1311,37 @@
         <v>231.1015430943892</v>
       </c>
       <c r="G9" s="3">
-        <v>2.991144416980329</v>
+        <v>2.363675314597349</v>
       </c>
       <c r="H9" s="4">
         <f>IF(F9=0,0,G9/F9)</f>
         <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>3364.297008165505</v>
+        <v>3364.304643388201</v>
       </c>
       <c r="J9" s="3">
-        <v>97.66824302014476</v>
+        <v>77.03199338765815</v>
       </c>
       <c r="K9" s="4">
         <f>IF(I9=0,0,J9/I9)</f>
         <v>0</v>
       </c>
       <c r="L9" s="3">
-        <v>11856.76378900309</v>
+        <v>12093.93485421385</v>
       </c>
       <c r="M9" s="3">
-        <v>9.969833238497376</v>
+        <v>0</v>
       </c>
       <c r="N9" s="4">
         <f>IF(L9=0,0,M9/L9)</f>
         <v>0</v>
       </c>
       <c r="O9" s="3">
-        <v>209.6942036708812</v>
+        <v>206.7182104708461</v>
       </c>
       <c r="P9" s="3">
-        <v>1.931132451062644</v>
+        <v>0.3066137045201031</v>
       </c>
       <c r="Q9" s="4">
         <f>IF(O9=0,0,P9/O9)</f>
@@ -1351,37 +1351,37 @@
         <v>2983.6261237209</v>
       </c>
       <c r="T9" s="3">
-        <v>38.61703605622006</v>
+        <v>30.5161243070811</v>
       </c>
       <c r="U9" s="4">
         <f>IF(S9=0,0,T9/S9)</f>
         <v>0</v>
       </c>
       <c r="V9" s="3">
-        <v>107056308.1865083</v>
+        <v>107054766.0433076</v>
       </c>
       <c r="W9" s="3">
-        <v>2591118.408128396</v>
+        <v>2041884.244128227</v>
       </c>
       <c r="X9" s="4">
         <f>IF(V9=0,0,W9/V9)</f>
         <v>0</v>
       </c>
       <c r="Y9" s="3">
-        <v>1277060.928257236</v>
+        <v>1264316.28918259</v>
       </c>
       <c r="Z9" s="3">
-        <v>14249.94927478419</v>
+        <v>11927.05845476408</v>
       </c>
       <c r="AA9" s="4">
         <f>IF(Y9=0,0,Z9/Y9)</f>
         <v>0</v>
       </c>
       <c r="AB9" s="3">
-        <v>132271.7542529008</v>
+        <v>134899.4215157334</v>
       </c>
       <c r="AC9" s="3">
-        <v>110.8166811575065</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="4">
         <f>IF(AB9=0,0,AC9/AB9)</f>
@@ -1531,37 +1531,37 @@
         <v>362.8529849538489</v>
       </c>
       <c r="G14" s="3">
-        <v>151.0014963206652</v>
+        <v>138.7727230203952</v>
       </c>
       <c r="H14" s="4">
         <f>IF(F14=0,0,G14/F14)</f>
         <v>0</v>
       </c>
       <c r="I14" s="3">
-        <v>4771.261231090824</v>
+        <v>4770.95717689731</v>
       </c>
       <c r="J14" s="3">
-        <v>472.7991412386447</v>
+        <v>410.5749562188024</v>
       </c>
       <c r="K14" s="4">
         <f>IF(I14=0,0,J14/I14)</f>
         <v>0</v>
       </c>
       <c r="L14" s="3">
-        <v>17957.14040242062</v>
+        <v>17865.36054925314</v>
       </c>
       <c r="M14" s="3">
-        <v>75.86299411857873</v>
+        <v>30.31804345500842</v>
       </c>
       <c r="N14" s="4">
         <f>IF(L14=0,0,M14/L14)</f>
         <v>0</v>
       </c>
       <c r="O14" s="3">
-        <v>506.7963637284521</v>
+        <v>498.0330422263939</v>
       </c>
       <c r="P14" s="3">
-        <v>20.73168748441845</v>
+        <v>24.10262712994427</v>
       </c>
       <c r="Q14" s="4">
         <f>IF(O14=0,0,P14/O14)</f>
@@ -1571,37 +1571,37 @@
         <v>4684.597214204819</v>
       </c>
       <c r="T14" s="3">
-        <v>1949.498056615184</v>
+        <v>1791.619026509166</v>
       </c>
       <c r="U14" s="4">
         <f>IF(S14=0,0,T14/S14)</f>
         <v>0</v>
       </c>
       <c r="V14" s="3">
-        <v>131696392.1412486</v>
+        <v>131693773.0318688</v>
       </c>
       <c r="W14" s="3">
-        <v>10296243.37165028</v>
+        <v>8933486.13431564</v>
       </c>
       <c r="X14" s="4">
         <f>IF(V14=0,0,W14/V14)</f>
         <v>0</v>
       </c>
       <c r="Y14" s="3">
-        <v>3016543.050471412</v>
+        <v>3015958.720793084</v>
       </c>
       <c r="Z14" s="3">
-        <v>109981.4259164366</v>
+        <v>93059.91173374001</v>
       </c>
       <c r="AA14" s="4">
         <f>IF(Y14=0,0,Z14/Y14)</f>
         <v>0</v>
       </c>
       <c r="AB14" s="3">
-        <v>200318.014600175</v>
+        <v>199267.9177921558</v>
       </c>
       <c r="AC14" s="3">
-        <v>843.170400111354</v>
+        <v>337.0078339079628</v>
       </c>
       <c r="AD14" s="4">
         <f>IF(AB14=0,0,AC14/AB14)</f>
@@ -1628,37 +1628,37 @@
         <v>320.5427437766894</v>
       </c>
       <c r="G15" s="3">
-        <v>121.1169850777707</v>
+        <v>110.5955742937957</v>
       </c>
       <c r="H15" s="4">
         <f>IF(F15=0,0,G15/F15)</f>
         <v>0</v>
       </c>
       <c r="I15" s="3">
-        <v>4315.21265961095</v>
+        <v>4315.385289601074</v>
       </c>
       <c r="J15" s="3">
-        <v>433.8825937981489</v>
+        <v>375.4759901001896</v>
       </c>
       <c r="K15" s="4">
         <f>IF(I15=0,0,J15/I15)</f>
         <v>0</v>
       </c>
       <c r="L15" s="3">
-        <v>14810.98291993852</v>
+        <v>14745.99462597537</v>
       </c>
       <c r="M15" s="3">
-        <v>50.71796651635692</v>
+        <v>43.31262777722441</v>
       </c>
       <c r="N15" s="4">
         <f>IF(L15=0,0,M15/L15)</f>
         <v>0</v>
       </c>
       <c r="O15" s="3">
-        <v>297.573370209569</v>
+        <v>290.5430769057631</v>
       </c>
       <c r="P15" s="3">
-        <v>8.989639123106667</v>
+        <v>6.431601228599495</v>
       </c>
       <c r="Q15" s="4">
         <f>IF(O15=0,0,P15/O15)</f>
@@ -1668,37 +1668,37 @@
         <v>4138.352740079671</v>
       </c>
       <c r="T15" s="3">
-        <v>1563.675412399809</v>
+        <v>1427.839209607146</v>
       </c>
       <c r="U15" s="4">
         <f>IF(S15=0,0,T15/S15)</f>
         <v>0</v>
       </c>
       <c r="V15" s="3">
-        <v>123352422.8520256</v>
+        <v>123347857.654681</v>
       </c>
       <c r="W15" s="3">
-        <v>9963665.358672738</v>
+        <v>8596318.405286953</v>
       </c>
       <c r="X15" s="4">
         <f>IF(V15=0,0,W15/V15)</f>
         <v>0</v>
       </c>
       <c r="Y15" s="3">
-        <v>1788522.531513863</v>
+        <v>1789154.954169832</v>
       </c>
       <c r="Z15" s="3">
-        <v>62487.2058478808</v>
+        <v>54537.43664395972</v>
       </c>
       <c r="AA15" s="4">
         <f>IF(Y15=0,0,Z15/Y15)</f>
         <v>0</v>
       </c>
       <c r="AB15" s="3">
-        <v>165227.6716058255</v>
+        <v>164556.1108996349</v>
       </c>
       <c r="AC15" s="3">
-        <v>563.7196389315941</v>
+        <v>481.4397627256694</v>
       </c>
       <c r="AD15" s="4">
         <f>IF(AB15=0,0,AC15/AB15)</f>
@@ -1725,37 +1725,37 @@
         <v>287.7720482472399</v>
       </c>
       <c r="G16" s="3">
-        <v>110.0570853730647</v>
+        <v>98.44054470138161</v>
       </c>
       <c r="H16" s="4">
         <f>IF(F16=0,0,G16/F16)</f>
         <v>0</v>
       </c>
       <c r="I16" s="3">
-        <v>4220.065012527612</v>
+        <v>4219.566052104662</v>
       </c>
       <c r="J16" s="3">
-        <v>424.9209438963709</v>
+        <v>354.4411187710422</v>
       </c>
       <c r="K16" s="4">
         <f>IF(I16=0,0,J16/I16)</f>
         <v>0</v>
       </c>
       <c r="L16" s="3">
-        <v>13140.17641177926</v>
+        <v>13471.87729543747</v>
       </c>
       <c r="M16" s="3">
-        <v>42.06335874866135</v>
+        <v>30.32200998448022</v>
       </c>
       <c r="N16" s="4">
         <f>IF(L16=0,0,M16/L16)</f>
         <v>0</v>
       </c>
       <c r="O16" s="3">
-        <v>350.6722046220511</v>
+        <v>365.4556715009266</v>
       </c>
       <c r="P16" s="3">
-        <v>11.13475204433734</v>
+        <v>7.960420500028704</v>
       </c>
       <c r="Q16" s="4">
         <f>IF(O16=0,0,P16/O16)</f>
@@ -1765,37 +1765,37 @@
         <v>3715.268142871963</v>
       </c>
       <c r="T16" s="3">
-        <v>1420.887072508819</v>
+        <v>1270.912244339263</v>
       </c>
       <c r="U16" s="4">
         <f>IF(S16=0,0,T16/S16)</f>
         <v>0</v>
       </c>
       <c r="V16" s="3">
-        <v>121045766.1486471</v>
+        <v>121037522.2666742</v>
       </c>
       <c r="W16" s="3">
-        <v>9877037.894057438</v>
+        <v>8230446.57875894</v>
       </c>
       <c r="X16" s="4">
         <f>IF(V16=0,0,W16/V16)</f>
         <v>0</v>
       </c>
       <c r="Y16" s="3">
-        <v>2261372.687672075</v>
+        <v>2253925.490084493</v>
       </c>
       <c r="Z16" s="3">
-        <v>75340.05412221793</v>
+        <v>67859.19145028805</v>
       </c>
       <c r="AA16" s="4">
         <f>IF(Y16=0,0,Z16/Y16)</f>
         <v>0</v>
       </c>
       <c r="AB16" s="3">
-        <v>146579.1514136479</v>
+        <v>150305.4939229549</v>
       </c>
       <c r="AC16" s="3">
-        <v>467.3573074903397</v>
+        <v>337.0078339079628</v>
       </c>
       <c r="AD16" s="4">
         <f>IF(AB16=0,0,AC16/AB16)</f>
@@ -1822,37 +1822,37 @@
         <v>271.3548595424364</v>
       </c>
       <c r="G17" s="3">
-        <v>102.5231161409741</v>
+        <v>89.47986825818086</v>
       </c>
       <c r="H17" s="4">
         <f>IF(F17=0,0,G17/F17)</f>
         <v>0</v>
       </c>
       <c r="I17" s="3">
-        <v>3866.462901477351</v>
+        <v>3865.872986383962</v>
       </c>
       <c r="J17" s="3">
-        <v>388.7186102795378</v>
+        <v>312.110257018093</v>
       </c>
       <c r="K17" s="4">
         <f>IF(I17=0,0,J17/I17)</f>
         <v>0</v>
       </c>
       <c r="L17" s="3">
-        <v>12529.63951354596</v>
+        <v>12349.08716881772</v>
       </c>
       <c r="M17" s="3">
-        <v>47.90031315631606</v>
+        <v>38.98261468011327</v>
       </c>
       <c r="N17" s="4">
         <f>IF(L17=0,0,M17/L17)</f>
         <v>0</v>
       </c>
       <c r="O17" s="3">
-        <v>341.4996444598856</v>
+        <v>301.3694049551027</v>
       </c>
       <c r="P17" s="3">
-        <v>12.01612042955466</v>
+        <v>7.130259819960396</v>
       </c>
       <c r="Q17" s="4">
         <f>IF(O17=0,0,P17/O17)</f>
@@ -1862,37 +1862,37 @@
         <v>3503.314763237015</v>
       </c>
       <c r="T17" s="3">
-        <v>1323.620100098366</v>
+        <v>1155.225832365698</v>
       </c>
       <c r="U17" s="4">
         <f>IF(S17=0,0,T17/S17)</f>
         <v>0</v>
       </c>
       <c r="V17" s="3">
-        <v>114934295.1461658</v>
+        <v>114934351.5045501</v>
       </c>
       <c r="W17" s="3">
-        <v>9507866.130370662</v>
+        <v>7630632.786527395</v>
       </c>
       <c r="X17" s="4">
         <f>IF(V17=0,0,W17/V17)</f>
         <v>0</v>
       </c>
       <c r="Y17" s="3">
-        <v>2020070.981660255</v>
+        <v>2008507.025186675</v>
       </c>
       <c r="Z17" s="3">
-        <v>64454.20863336418</v>
+        <v>52998.46135947411</v>
       </c>
       <c r="AA17" s="4">
         <f>IF(Y17=0,0,Z17/Y17)</f>
         <v>0</v>
       </c>
       <c r="AB17" s="3">
-        <v>139766.3345807479</v>
+        <v>137739.9161158149</v>
       </c>
       <c r="AC17" s="3">
-        <v>532.4018812131835</v>
+        <v>433.2957864531199</v>
       </c>
       <c r="AD17" s="4">
         <f>IF(AB17=0,0,AC17/AB17)</f>
@@ -1919,37 +1919,37 @@
         <v>231.1015430943892</v>
       </c>
       <c r="G18" s="3">
-        <v>67.11521448847459</v>
+        <v>52.18407847809815</v>
       </c>
       <c r="H18" s="4">
         <f>IF(F18=0,0,G18/F18)</f>
         <v>0</v>
       </c>
       <c r="I18" s="3">
-        <v>3364.297008165505</v>
+        <v>3364.304643388201</v>
       </c>
       <c r="J18" s="3">
-        <v>311.568357023593</v>
+        <v>218.1918313057371</v>
       </c>
       <c r="K18" s="4">
         <f>IF(I18=0,0,J18/I18)</f>
         <v>0</v>
       </c>
       <c r="L18" s="3">
-        <v>11856.76378900309</v>
+        <v>12093.93485421385</v>
       </c>
       <c r="M18" s="3">
-        <v>28.82798583594151</v>
+        <v>4.331137135382741</v>
       </c>
       <c r="N18" s="4">
         <f>IF(L18=0,0,M18/L18)</f>
         <v>0</v>
       </c>
       <c r="O18" s="3">
-        <v>209.6942036708812</v>
+        <v>206.7182104708461</v>
       </c>
       <c r="P18" s="3">
-        <v>4.980074249699042</v>
+        <v>3.648974865616794</v>
       </c>
       <c r="Q18" s="4">
         <f>IF(O18=0,0,P18/O18)</f>
@@ -1959,37 +1959,37 @@
         <v>2983.6261237209</v>
       </c>
       <c r="T18" s="3">
-        <v>866.487971329369</v>
+        <v>673.7202084624901</v>
       </c>
       <c r="U18" s="4">
         <f>IF(S18=0,0,T18/S18)</f>
         <v>0</v>
       </c>
       <c r="V18" s="3">
-        <v>107056308.1865083</v>
+        <v>107054766.0433076</v>
       </c>
       <c r="W18" s="3">
-        <v>8317990.791051477</v>
+        <v>5806302.713304117</v>
       </c>
       <c r="X18" s="4">
         <f>IF(V18=0,0,W18/V18)</f>
         <v>0</v>
       </c>
       <c r="Y18" s="3">
-        <v>1277060.928257236</v>
+        <v>1264316.28918259</v>
       </c>
       <c r="Z18" s="3">
-        <v>31125.77512872219</v>
+        <v>25537.37112693419</v>
       </c>
       <c r="AA18" s="4">
         <f>IF(Y18=0,0,Z18/Y18)</f>
         <v>0</v>
       </c>
       <c r="AB18" s="3">
-        <v>132271.7542529008</v>
+        <v>134899.4215157334</v>
       </c>
       <c r="AC18" s="3">
-        <v>320.4047520423192</v>
+        <v>48.14397627257858</v>
       </c>
       <c r="AD18" s="4">
         <f>IF(AB18=0,0,AC18/AB18)</f>
@@ -2146,30 +2146,30 @@
         <v>0</v>
       </c>
       <c r="I23" s="3">
-        <v>1024.476057384201</v>
+        <v>1024.354560880719</v>
       </c>
       <c r="J23" s="3">
-        <v>151.6692552821839</v>
+        <v>151.5846734435843</v>
       </c>
       <c r="K23" s="4">
         <f>IF(I23=0,0,J23/I23)</f>
         <v>0</v>
       </c>
       <c r="L23" s="3">
-        <v>15352.83741703859</v>
+        <v>14912.92546688904</v>
       </c>
       <c r="M23" s="3">
-        <v>69.56725985433347</v>
+        <v>49.77988587578945</v>
       </c>
       <c r="N23" s="4">
         <f>IF(L23=0,0,M23/L23)</f>
         <v>0</v>
       </c>
       <c r="O23" s="3">
-        <v>503.5634310516943</v>
+        <v>513.4798818030744</v>
       </c>
       <c r="P23" s="3">
-        <v>21.01036396919185</v>
+        <v>27.03285584600665</v>
       </c>
       <c r="Q23" s="4">
         <f>IF(O23=0,0,P23/O23)</f>
@@ -2186,30 +2186,30 @@
         <v>0</v>
       </c>
       <c r="V23" s="3">
-        <v>25177467.03377928</v>
+        <v>25179040.28609852</v>
       </c>
       <c r="W23" s="3">
-        <v>2945174.443318196</v>
+        <v>2944045.7732535</v>
       </c>
       <c r="X23" s="4">
         <f>IF(V23=0,0,W23/V23)</f>
         <v>0</v>
       </c>
       <c r="Y23" s="3">
-        <v>2561085.175981381</v>
+        <v>2561859.505516207</v>
       </c>
       <c r="Z23" s="3">
-        <v>116196.6057628184</v>
+        <v>117190.545564875</v>
       </c>
       <c r="AA23" s="4">
         <f>IF(Y23=0,0,Z23/Y23)</f>
         <v>0</v>
       </c>
       <c r="AB23" s="3">
-        <v>172903.801774421</v>
+        <v>167937.2280679461</v>
       </c>
       <c r="AC23" s="3">
-        <v>772.255639909883</v>
+        <v>554.786800846312</v>
       </c>
       <c r="AD23" s="4">
         <f>IF(AB23=0,0,AC23/AB23)</f>
@@ -2243,30 +2243,30 @@
         <v>0</v>
       </c>
       <c r="I24" s="3">
-        <v>968.8874507802924</v>
+        <v>969.191110200812</v>
       </c>
       <c r="J24" s="3">
-        <v>150.8926468475667</v>
+        <v>150.9258526370303</v>
       </c>
       <c r="K24" s="4">
         <f>IF(I24=0,0,J24/I24)</f>
         <v>0</v>
       </c>
       <c r="L24" s="3">
-        <v>15897.14811387405</v>
+        <v>15496.18877972349</v>
       </c>
       <c r="M24" s="3">
-        <v>66.02582374739833</v>
+        <v>49.9134009951558</v>
       </c>
       <c r="N24" s="4">
         <f>IF(L24=0,0,M24/L24)</f>
         <v>0</v>
       </c>
       <c r="O24" s="3">
-        <v>427.6878840211459</v>
+        <v>401.8379348471553</v>
       </c>
       <c r="P24" s="3">
-        <v>21.73464126741991</v>
+        <v>15.73672244196298</v>
       </c>
       <c r="Q24" s="4">
         <f>IF(O24=0,0,P24/O24)</f>
@@ -2283,30 +2283,30 @@
         <v>0</v>
       </c>
       <c r="V24" s="3">
-        <v>24716781.60947407</v>
+        <v>24722331.14126323</v>
       </c>
       <c r="W24" s="3">
-        <v>3073981.15008124</v>
+        <v>3073867.312957134</v>
       </c>
       <c r="X24" s="4">
         <f>IF(V24=0,0,W24/V24)</f>
         <v>0</v>
       </c>
       <c r="Y24" s="3">
-        <v>2216806.226901517</v>
+        <v>2224473.065341928</v>
       </c>
       <c r="Z24" s="3">
-        <v>113084.6469390318</v>
+        <v>113091.1539099128</v>
       </c>
       <c r="AA24" s="4">
         <f>IF(Y24=0,0,Z24/Y24)</f>
         <v>0</v>
       </c>
       <c r="AB24" s="3">
-        <v>179047.6330362356</v>
+        <v>174496.7661250112</v>
       </c>
       <c r="AC24" s="3">
-        <v>733.1540885220165</v>
+        <v>554.786800846312</v>
       </c>
       <c r="AD24" s="4">
         <f>IF(AB24=0,0,AC24/AB24)</f>
@@ -2340,30 +2340,30 @@
         <v>0</v>
       </c>
       <c r="I25" s="3">
-        <v>792.6568327877751</v>
+        <v>792.6603703485911</v>
       </c>
       <c r="J25" s="3">
-        <v>138.7460097809298</v>
+        <v>138.7121411177468</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
         <v>0</v>
       </c>
       <c r="L25" s="3">
-        <v>14099.36149543928</v>
+        <v>13908.71537534086</v>
       </c>
       <c r="M25" s="3">
-        <v>48.02046110171266</v>
+        <v>58.82691208174825</v>
       </c>
       <c r="N25" s="4">
         <f>IF(L25=0,0,M25/L25)</f>
         <v>0</v>
       </c>
       <c r="O25" s="3">
-        <v>410.8336896551561</v>
+        <v>403.1015048057993</v>
       </c>
       <c r="P25" s="3">
-        <v>20.00392896381795</v>
+        <v>16.62349251975317</v>
       </c>
       <c r="Q25" s="4">
         <f>IF(O25=0,0,P25/O25)</f>
@@ -2380,30 +2380,30 @@
         <v>0</v>
       </c>
       <c r="V25" s="3">
-        <v>22756394.15398703</v>
+        <v>22755823.62356573</v>
       </c>
       <c r="W25" s="3">
-        <v>3255095.686233584</v>
+        <v>3251875.766117409</v>
       </c>
       <c r="X25" s="4">
         <f>IF(V25=0,0,W25/V25)</f>
         <v>0</v>
       </c>
       <c r="Y25" s="3">
-        <v>2114085.557833027</v>
+        <v>2110145.586964646</v>
       </c>
       <c r="Z25" s="3">
-        <v>104646.7324492342</v>
+        <v>107560.2286611539</v>
       </c>
       <c r="AA25" s="4">
         <f>IF(Y25=0,0,Z25/Y25)</f>
         <v>0</v>
       </c>
       <c r="AB25" s="3">
-        <v>158763.7032537926</v>
+        <v>156580.4159094453</v>
       </c>
       <c r="AC25" s="3">
-        <v>532.758637659339</v>
+        <v>652.6903539368068</v>
       </c>
       <c r="AD25" s="4">
         <f>IF(AB25=0,0,AC25/AB25)</f>
@@ -2437,30 +2437,30 @@
         <v>0</v>
       </c>
       <c r="I26" s="3">
-        <v>714.5868735320346</v>
+        <v>714.9995999658563</v>
       </c>
       <c r="J26" s="3">
-        <v>127.9421658211542</v>
+        <v>128.1332900039845</v>
       </c>
       <c r="K26" s="4">
         <f>IF(I26=0,0,J26/I26)</f>
         <v>0</v>
       </c>
       <c r="L26" s="3">
-        <v>12459.036398116</v>
+        <v>12302.18440833913</v>
       </c>
       <c r="M26" s="3">
-        <v>33.00900104676187</v>
+        <v>14.68251907597482</v>
       </c>
       <c r="N26" s="4">
         <f>IF(L26=0,0,M26/L26)</f>
         <v>0</v>
       </c>
       <c r="O26" s="3">
-        <v>388.5202631627004</v>
+        <v>394.000120021803</v>
       </c>
       <c r="P26" s="3">
-        <v>16.30620732857898</v>
+        <v>24.40948152676935</v>
       </c>
       <c r="Q26" s="4">
         <f>IF(O26=0,0,P26/O26)</f>
@@ -2477,30 +2477,30 @@
         <v>0</v>
       </c>
       <c r="V26" s="3">
-        <v>21413420.36871202</v>
+        <v>21415342.77124955</v>
       </c>
       <c r="W26" s="3">
-        <v>3188030.275738072</v>
+        <v>3188343.04784625</v>
       </c>
       <c r="X26" s="4">
         <f>IF(V26=0,0,W26/V26)</f>
         <v>0</v>
       </c>
       <c r="Y26" s="3">
-        <v>1925897.452986733</v>
+        <v>1934522.442889356</v>
       </c>
       <c r="Z26" s="3">
-        <v>86993.32044937275</v>
+        <v>85664.27164695086</v>
       </c>
       <c r="AA26" s="4">
         <f>IF(Y26=0,0,Z26/Y26)</f>
         <v>0</v>
       </c>
       <c r="AB26" s="3">
-        <v>140314.2879239626</v>
+        <v>138598.7966584856</v>
       </c>
       <c r="AC26" s="3">
-        <v>366.5770442610374</v>
+        <v>163.1725884842162</v>
       </c>
       <c r="AD26" s="4">
         <f>IF(AB26=0,0,AC26/AB26)</f>
@@ -2534,30 +2534,30 @@
         <v>0</v>
       </c>
       <c r="I27" s="3">
-        <v>607.1996095192959</v>
+        <v>607.5227834345628</v>
       </c>
       <c r="J27" s="3">
-        <v>115.4369858740715</v>
+        <v>115.499531697674</v>
       </c>
       <c r="K27" s="4">
         <f>IF(I27=0,0,J27/I27)</f>
         <v>0</v>
       </c>
       <c r="L27" s="3">
-        <v>9475.405513778041</v>
+        <v>9346.35620700917</v>
       </c>
       <c r="M27" s="3">
-        <v>26.1176055910252</v>
+        <v>17.61839148277417</v>
       </c>
       <c r="N27" s="4">
         <f>IF(L27=0,0,M27/L27)</f>
         <v>0</v>
       </c>
       <c r="O27" s="3">
-        <v>285.742923347472</v>
+        <v>287.6026494045061</v>
       </c>
       <c r="P27" s="3">
-        <v>14.29403973296256</v>
+        <v>23.00427726469026</v>
       </c>
       <c r="Q27" s="4">
         <f>IF(O27=0,0,P27/O27)</f>
@@ -2574,30 +2574,30 @@
         <v>0</v>
       </c>
       <c r="V27" s="3">
-        <v>19850211.7121278</v>
+        <v>19855184.90001665</v>
       </c>
       <c r="W27" s="3">
-        <v>3182528.287519272</v>
+        <v>3181428.078000424</v>
       </c>
       <c r="X27" s="4">
         <f>IF(V27=0,0,W27/V27)</f>
         <v>0</v>
       </c>
       <c r="Y27" s="3">
-        <v>1405792.016991551</v>
+        <v>1414713.074069254</v>
       </c>
       <c r="Z27" s="3">
-        <v>72425.83938977448</v>
+        <v>70698.23862089752</v>
       </c>
       <c r="AA27" s="4">
         <f>IF(Y27=0,0,Z27/Y27)</f>
         <v>0</v>
       </c>
       <c r="AB27" s="3">
-        <v>106730.9429757299</v>
+        <v>105311.5886077074</v>
       </c>
       <c r="AC27" s="3">
-        <v>290.0031727931782</v>
+        <v>195.8071061810624</v>
       </c>
       <c r="AD27" s="4">
         <f>IF(AB27=0,0,AC27/AB27)</f>
@@ -2747,37 +2747,37 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G32" s="3">
-        <v>35.73618465235695</v>
+        <v>88.917209540012</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
         <v>0</v>
       </c>
       <c r="I32" s="3">
-        <v>1024.476057384201</v>
+        <v>1024.354560880719</v>
       </c>
       <c r="J32" s="3">
-        <v>37.27986362662178</v>
+        <v>37.4211717676142</v>
       </c>
       <c r="K32" s="4">
         <f>IF(I32=0,0,J32/I32)</f>
         <v>0</v>
       </c>
       <c r="L32" s="3">
-        <v>15352.83741703859</v>
+        <v>14912.92546688904</v>
       </c>
       <c r="M32" s="3">
-        <v>3.962234379850328</v>
+        <v>5.872274373358116</v>
       </c>
       <c r="N32" s="4">
         <f>IF(L32=0,0,M32/L32)</f>
         <v>0</v>
       </c>
       <c r="O32" s="3">
-        <v>503.5634310516943</v>
+        <v>513.4798818030744</v>
       </c>
       <c r="P32" s="3">
-        <v>3.925692564837344</v>
+        <v>8.763104271617543</v>
       </c>
       <c r="Q32" s="4">
         <f>IF(O32=0,0,P32/O32)</f>
@@ -2787,37 +2787,37 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T32" s="3">
-        <v>1102.625774219956</v>
+        <v>2743.505160505925</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
         <v>0</v>
       </c>
       <c r="V32" s="3">
-        <v>25177467.03377928</v>
+        <v>25179040.28609852</v>
       </c>
       <c r="W32" s="3">
-        <v>714061.0112777613</v>
+        <v>716874.4105257355</v>
       </c>
       <c r="X32" s="4">
         <f>IF(V32=0,0,W32/V32)</f>
         <v>0</v>
       </c>
       <c r="Y32" s="3">
-        <v>2561085.175981381</v>
+        <v>2561859.505516207</v>
       </c>
       <c r="Z32" s="3">
-        <v>24656.53941042209</v>
+        <v>25832.67439714307</v>
       </c>
       <c r="AA32" s="4">
         <f>IF(Y32=0,0,Z32/Y32)</f>
         <v>0</v>
       </c>
       <c r="AB32" s="3">
-        <v>172903.801774421</v>
+        <v>167937.2280679461</v>
       </c>
       <c r="AC32" s="3">
-        <v>43.98924531132798</v>
+        <v>65.26903539369232</v>
       </c>
       <c r="AD32" s="4">
         <f>IF(AB32=0,0,AC32/AB32)</f>
@@ -2844,37 +2844,37 @@
         <v>422.0532339939541</v>
       </c>
       <c r="G33" s="3">
-        <v>65.17460356458911</v>
+        <v>119.3410127560627</v>
       </c>
       <c r="H33" s="4">
         <f>IF(F33=0,0,G33/F33)</f>
         <v>0</v>
       </c>
       <c r="I33" s="3">
-        <v>968.8874507802924</v>
+        <v>969.191110200812</v>
       </c>
       <c r="J33" s="3">
-        <v>48.93446618463355</v>
+        <v>48.78491642388643</v>
       </c>
       <c r="K33" s="4">
         <f>IF(I33=0,0,J33/I33)</f>
         <v>0</v>
       </c>
       <c r="L33" s="3">
-        <v>15897.14811387405</v>
+        <v>15496.18877972349</v>
       </c>
       <c r="M33" s="3">
-        <v>5.71674261646904</v>
+        <v>2.935737240042537</v>
       </c>
       <c r="N33" s="4">
         <f>IF(L33=0,0,M33/L33)</f>
         <v>0</v>
       </c>
       <c r="O33" s="3">
-        <v>427.6878840211459</v>
+        <v>401.8379348471553</v>
       </c>
       <c r="P33" s="3">
-        <v>6.033024517372309</v>
+        <v>6.341134637456737</v>
       </c>
       <c r="Q33" s="4">
         <f>IF(O33=0,0,P33/O33)</f>
@@ -2884,37 +2884,37 @@
         <v>13022.28479122008</v>
       </c>
       <c r="T33" s="3">
-        <v>2010.936489554548</v>
+        <v>3682.219516897101</v>
       </c>
       <c r="U33" s="4">
         <f>IF(S33=0,0,T33/S33)</f>
         <v>0</v>
       </c>
       <c r="V33" s="3">
-        <v>24716781.60947407</v>
+        <v>24722331.14126323</v>
       </c>
       <c r="W33" s="3">
-        <v>982871.2588993013</v>
+        <v>982144.0085640848</v>
       </c>
       <c r="X33" s="4">
         <f>IF(V33=0,0,W33/V33)</f>
         <v>0</v>
       </c>
       <c r="Y33" s="3">
-        <v>2216806.226901517</v>
+        <v>2224473.065341928</v>
       </c>
       <c r="Z33" s="3">
-        <v>34690.28850875841</v>
+        <v>34909.89877598826</v>
       </c>
       <c r="AA33" s="4">
         <f>IF(Y33=0,0,Z33/Y33)</f>
         <v>0</v>
       </c>
       <c r="AB33" s="3">
-        <v>179047.6330362356</v>
+        <v>174496.7661250112</v>
       </c>
       <c r="AC33" s="3">
-        <v>63.54002100523212</v>
+        <v>32.63451769683161</v>
       </c>
       <c r="AD33" s="4">
         <f>IF(AB33=0,0,AC33/AB33)</f>
@@ -2941,37 +2941,37 @@
         <v>382.0743136549376</v>
       </c>
       <c r="G34" s="3">
-        <v>77.8855817338635</v>
+        <v>119.4634252945786</v>
       </c>
       <c r="H34" s="4">
         <f>IF(F34=0,0,G34/F34)</f>
         <v>0</v>
       </c>
       <c r="I34" s="3">
-        <v>792.6568327877751</v>
+        <v>792.6603703485911</v>
       </c>
       <c r="J34" s="3">
-        <v>54.7024904162623</v>
+        <v>54.52997860636842</v>
       </c>
       <c r="K34" s="4">
         <f>IF(I34=0,0,J34/I34)</f>
         <v>0</v>
       </c>
       <c r="L34" s="3">
-        <v>14099.36149543928</v>
+        <v>13908.71537534086</v>
       </c>
       <c r="M34" s="3">
-        <v>7.918256656212733</v>
+        <v>17.6161303497944</v>
       </c>
       <c r="N34" s="4">
         <f>IF(L34=0,0,M34/L34)</f>
         <v>0</v>
       </c>
       <c r="O34" s="3">
-        <v>410.8336896551561</v>
+        <v>403.1015048057993</v>
       </c>
       <c r="P34" s="3">
-        <v>7.485334139126877</v>
+        <v>9.918853932482365</v>
       </c>
       <c r="Q34" s="4">
         <f>IF(O34=0,0,P34/O34)</f>
@@ -2981,37 +2981,37 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T34" s="3">
-        <v>2403.128669031234</v>
+        <v>3685.99650712055</v>
       </c>
       <c r="U34" s="4">
         <f>IF(S34=0,0,T34/S34)</f>
         <v>0</v>
       </c>
       <c r="V34" s="3">
-        <v>22756394.15398703</v>
+        <v>22755823.62356573</v>
       </c>
       <c r="W34" s="3">
-        <v>1263898.368850708</v>
+        <v>1260214.302773219</v>
       </c>
       <c r="X34" s="4">
         <f>IF(V34=0,0,W34/V34)</f>
         <v>0</v>
       </c>
       <c r="Y34" s="3">
-        <v>2114085.557833027</v>
+        <v>2110145.586964646</v>
       </c>
       <c r="Z34" s="3">
-        <v>41680.40197755746</v>
+        <v>40082.94062629784</v>
       </c>
       <c r="AA34" s="4">
         <f>IF(Y34=0,0,Z34/Y34)</f>
         <v>0</v>
       </c>
       <c r="AB34" s="3">
-        <v>158763.7032537926</v>
+        <v>156580.4159094453</v>
       </c>
       <c r="AC34" s="3">
-        <v>87.97849062262685</v>
+        <v>195.807106181077</v>
       </c>
       <c r="AD34" s="4">
         <f>IF(AB34=0,0,AC34/AB34)</f>
@@ -3038,37 +3038,37 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G35" s="3">
-        <v>86.85569037143482</v>
+        <v>117.3536742164378</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
         <v>0</v>
       </c>
       <c r="I35" s="3">
-        <v>714.5868735320346</v>
+        <v>714.9995999658563</v>
       </c>
       <c r="J35" s="3">
-        <v>58.95966902481718</v>
+        <v>58.96629333495523</v>
       </c>
       <c r="K35" s="4">
         <f>IF(I35=0,0,J35/I35)</f>
         <v>0</v>
       </c>
       <c r="L35" s="3">
-        <v>12459.036398116</v>
+        <v>12302.18440833913</v>
       </c>
       <c r="M35" s="3">
-        <v>6.752045505788177</v>
+        <v>14.68228815255128</v>
       </c>
       <c r="N35" s="4">
         <f>IF(L35=0,0,M35/L35)</f>
         <v>0</v>
       </c>
       <c r="O35" s="3">
-        <v>388.5202631627004</v>
+        <v>394.000120021803</v>
       </c>
       <c r="P35" s="3">
-        <v>7.643253715592786</v>
+        <v>8.086287446427276</v>
       </c>
       <c r="Q35" s="4">
         <f>IF(O35=0,0,P35/O35)</f>
@@ -3078,37 +3078,37 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T35" s="3">
-        <v>2679.897805903459</v>
+        <v>3620.900976118114</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
         <v>0</v>
       </c>
       <c r="V35" s="3">
-        <v>21413420.36871202</v>
+        <v>21415342.77124955</v>
       </c>
       <c r="W35" s="3">
-        <v>1447623.317466982</v>
+        <v>1447070.019652024</v>
       </c>
       <c r="X35" s="4">
         <f>IF(V35=0,0,W35/V35)</f>
         <v>0</v>
       </c>
       <c r="Y35" s="3">
-        <v>1925897.452986733</v>
+        <v>1934522.442889356</v>
       </c>
       <c r="Z35" s="3">
-        <v>39964.18840772193</v>
+        <v>38781.5464501197</v>
       </c>
       <c r="AA35" s="4">
         <f>IF(Y35=0,0,Z35/Y35)</f>
         <v>0</v>
       </c>
       <c r="AB35" s="3">
-        <v>140314.2879239626</v>
+        <v>138598.7966584856</v>
       </c>
       <c r="AC35" s="3">
-        <v>74.94464016004349</v>
+        <v>163.1725884842162</v>
       </c>
       <c r="AD35" s="4">
         <f>IF(AB35=0,0,AC35/AB35)</f>
@@ -3135,37 +3135,37 @@
         <v>297.4602934996698</v>
       </c>
       <c r="G36" s="3">
-        <v>82.75070857381445</v>
+        <v>106.3158412713952</v>
       </c>
       <c r="H36" s="4">
         <f>IF(F36=0,0,G36/F36)</f>
         <v>0</v>
       </c>
       <c r="I36" s="3">
-        <v>607.1996095192959</v>
+        <v>607.5227834345628</v>
       </c>
       <c r="J36" s="3">
-        <v>56.92850932440988</v>
+        <v>56.9564015864773</v>
       </c>
       <c r="K36" s="4">
         <f>IF(I36=0,0,J36/I36)</f>
         <v>0</v>
       </c>
       <c r="L36" s="3">
-        <v>9475.405513778041</v>
+        <v>9346.35620700917</v>
       </c>
       <c r="M36" s="3">
-        <v>9.540724531468005</v>
+        <v>8.808966507997363</v>
       </c>
       <c r="N36" s="4">
         <f>IF(L36=0,0,M36/L36)</f>
         <v>0</v>
       </c>
       <c r="O36" s="3">
-        <v>285.742923347472</v>
+        <v>287.6026494045061</v>
       </c>
       <c r="P36" s="3">
-        <v>6.937234701249923</v>
+        <v>12.65641432294366</v>
       </c>
       <c r="Q36" s="4">
         <f>IF(O36=0,0,P36/O36)</f>
@@ -3175,37 +3175,37 @@
         <v>9178.019131321482</v>
       </c>
       <c r="T36" s="3">
-        <v>2553.240224049334</v>
+        <v>3280.333027549058</v>
       </c>
       <c r="U36" s="4">
         <f>IF(S36=0,0,T36/S36)</f>
         <v>0</v>
       </c>
       <c r="V36" s="3">
-        <v>19850211.7121278</v>
+        <v>19855184.90001665</v>
       </c>
       <c r="W36" s="3">
-        <v>1546922.86282469</v>
+        <v>1544839.312856581</v>
       </c>
       <c r="X36" s="4">
         <f>IF(V36=0,0,W36/V36)</f>
         <v>0</v>
       </c>
       <c r="Y36" s="3">
-        <v>1405792.016991551</v>
+        <v>1414713.074069254</v>
       </c>
       <c r="Z36" s="3">
-        <v>35215.72640739055</v>
+        <v>34259.20168789942</v>
       </c>
       <c r="AA36" s="4">
         <f>IF(Y36=0,0,Z36/Y36)</f>
         <v>0</v>
       </c>
       <c r="AB36" s="3">
-        <v>106730.9429757299</v>
+        <v>105311.5886077074</v>
       </c>
       <c r="AC36" s="3">
-        <v>105.9000350087299</v>
+        <v>97.90355309052393</v>
       </c>
       <c r="AD36" s="4">
         <f>IF(AB36=0,0,AC36/AB36)</f>
@@ -3362,30 +3362,30 @@
         <v>0</v>
       </c>
       <c r="I41" s="3">
-        <v>1026.204299813583</v>
+        <v>1026.0828033101</v>
       </c>
       <c r="J41" s="3">
-        <v>6.332670651874505</v>
+        <v>6.296699012307799</v>
       </c>
       <c r="K41" s="4">
         <f>IF(I41=0,0,J41/I41)</f>
         <v>0</v>
       </c>
       <c r="L41" s="3">
-        <v>15352.83741703859</v>
+        <v>14912.92546688904</v>
       </c>
       <c r="M41" s="3">
-        <v>0.5863035025261343</v>
+        <v>0</v>
       </c>
       <c r="N41" s="4">
         <f>IF(L41=0,0,M41/L41)</f>
         <v>0</v>
       </c>
       <c r="O41" s="3">
-        <v>503.5634310516943</v>
+        <v>513.4798818030744</v>
       </c>
       <c r="P41" s="3">
-        <v>0.7976752452995279</v>
+        <v>4.496294947286602</v>
       </c>
       <c r="Q41" s="4">
         <f>IF(O41=0,0,P41/O41)</f>
@@ -3402,30 +3402,30 @@
         <v>0</v>
       </c>
       <c r="V41" s="3">
-        <v>25286285.18025935</v>
+        <v>25287858.4325786</v>
       </c>
       <c r="W41" s="3">
-        <v>124252.6863578595</v>
+        <v>124543.3070078939</v>
       </c>
       <c r="X41" s="4">
         <f>IF(V41=0,0,W41/V41)</f>
         <v>0</v>
       </c>
       <c r="Y41" s="3">
-        <v>2561085.175981381</v>
+        <v>2561859.505516207</v>
       </c>
       <c r="Z41" s="3">
-        <v>4301.107752270065</v>
+        <v>4619.949325433467</v>
       </c>
       <c r="AA41" s="4">
         <f>IF(Y41=0,0,Z41/Y41)</f>
         <v>0</v>
       </c>
       <c r="AB41" s="3">
-        <v>172903.801774421</v>
+        <v>167937.2280679461</v>
       </c>
       <c r="AC41" s="3">
-        <v>6.516925231320783</v>
+        <v>0</v>
       </c>
       <c r="AD41" s="4">
         <f>IF(AB41=0,0,AC41/AB41)</f>
@@ -3459,30 +3459,30 @@
         <v>0</v>
       </c>
       <c r="I42" s="3">
-        <v>971.1037573173985</v>
+        <v>971.4074167379182</v>
       </c>
       <c r="J42" s="3">
-        <v>8.271399086192949</v>
+        <v>8.202031324924203</v>
       </c>
       <c r="K42" s="4">
         <f>IF(I42=0,0,J42/I42)</f>
         <v>0</v>
       </c>
       <c r="L42" s="3">
-        <v>15897.14811387405</v>
+        <v>15496.18877972349</v>
       </c>
       <c r="M42" s="3">
-        <v>2.204028858903795</v>
+        <v>2.936306209888309</v>
       </c>
       <c r="N42" s="4">
         <f>IF(L42=0,0,M42/L42)</f>
         <v>0</v>
       </c>
       <c r="O42" s="3">
-        <v>427.6878840211459</v>
+        <v>401.8379348471553</v>
       </c>
       <c r="P42" s="3">
-        <v>0.7658804311889107</v>
+        <v>2.065827537484292</v>
       </c>
       <c r="Q42" s="4">
         <f>IF(O42=0,0,P42/O42)</f>
@@ -3499,30 +3499,30 @@
         <v>0</v>
       </c>
       <c r="V42" s="3">
-        <v>24859901.01601297</v>
+        <v>24865450.54780213</v>
       </c>
       <c r="W42" s="3">
-        <v>171453.208100237</v>
+        <v>171780.3006582037</v>
       </c>
       <c r="X42" s="4">
         <f>IF(V42=0,0,W42/V42)</f>
         <v>0</v>
       </c>
       <c r="Y42" s="3">
-        <v>2216806.226901517</v>
+        <v>2224473.065341928</v>
       </c>
       <c r="Z42" s="3">
-        <v>5397.532345701009</v>
+        <v>5823.738938398659</v>
       </c>
       <c r="AA42" s="4">
         <f>IF(Y42=0,0,Z42/Y42)</f>
         <v>0</v>
       </c>
       <c r="AB42" s="3">
-        <v>179047.6330362356</v>
+        <v>174496.7661250112</v>
       </c>
       <c r="AC42" s="3">
-        <v>24.43846961739473</v>
+        <v>32.63451769683161</v>
       </c>
       <c r="AD42" s="4">
         <f>IF(AB42=0,0,AC42/AB42)</f>
@@ -3556,30 +3556,30 @@
         <v>0</v>
       </c>
       <c r="I43" s="3">
-        <v>795.3294661601195</v>
+        <v>795.3330037209355</v>
       </c>
       <c r="J43" s="3">
-        <v>9.250731927022105</v>
+        <v>9.273915266624302</v>
       </c>
       <c r="K43" s="4">
         <f>IF(I43=0,0,J43/I43)</f>
         <v>0</v>
       </c>
       <c r="L43" s="3">
-        <v>14099.36149543928</v>
+        <v>13908.71537534086</v>
       </c>
       <c r="M43" s="3">
-        <v>2.494237892366946</v>
+        <v>5.872356832668185</v>
       </c>
       <c r="N43" s="4">
         <f>IF(L43=0,0,M43/L43)</f>
         <v>0</v>
       </c>
       <c r="O43" s="3">
-        <v>410.8336896551561</v>
+        <v>403.1015048057993</v>
       </c>
       <c r="P43" s="3">
-        <v>0.6260496127711959</v>
+        <v>0.05710813306475757</v>
       </c>
       <c r="Q43" s="4">
         <f>IF(O43=0,0,P43/O43)</f>
@@ -3596,30 +3596,30 @@
         <v>0</v>
       </c>
       <c r="V43" s="3">
-        <v>22936296.40445412</v>
+        <v>22935725.87403282</v>
       </c>
       <c r="W43" s="3">
-        <v>221609.0820698142</v>
+        <v>221433.0388277955</v>
       </c>
       <c r="X43" s="4">
         <f>IF(V43=0,0,W43/V43)</f>
         <v>0</v>
       </c>
       <c r="Y43" s="3">
-        <v>2114085.557833027</v>
+        <v>2110145.586964646</v>
       </c>
       <c r="Z43" s="3">
-        <v>6329.655924388207</v>
+        <v>6734.714861723594</v>
       </c>
       <c r="AA43" s="4">
         <f>IF(Y43=0,0,Z43/Y43)</f>
         <v>0</v>
       </c>
       <c r="AB43" s="3">
-        <v>158763.7032537926</v>
+        <v>156580.4159094453</v>
       </c>
       <c r="AC43" s="3">
-        <v>27.69693223305512</v>
+        <v>65.26903539366322</v>
       </c>
       <c r="AD43" s="4">
         <f>IF(AB43=0,0,AC43/AB43)</f>
@@ -3653,30 +3653,30 @@
         <v>0</v>
       </c>
       <c r="I44" s="3">
-        <v>717.4492241565633</v>
+        <v>717.861950590385</v>
       </c>
       <c r="J44" s="3">
-        <v>9.464455356970662</v>
+        <v>9.510016093718004</v>
       </c>
       <c r="K44" s="4">
         <f>IF(I44=0,0,J44/I44)</f>
         <v>0</v>
       </c>
       <c r="L44" s="3">
-        <v>12459.036398116</v>
+        <v>12302.18440833913</v>
       </c>
       <c r="M44" s="3">
-        <v>2.502058168889955</v>
+        <v>0</v>
       </c>
       <c r="N44" s="4">
         <f>IF(L44=0,0,M44/L44)</f>
         <v>0</v>
       </c>
       <c r="O44" s="3">
-        <v>388.5202631627004</v>
+        <v>394.000120021803</v>
       </c>
       <c r="P44" s="3">
-        <v>1.11741603567038</v>
+        <v>0.05215326621627901</v>
       </c>
       <c r="Q44" s="4">
         <f>IF(O44=0,0,P44/O44)</f>
@@ -3693,30 +3693,30 @@
         <v>0</v>
       </c>
       <c r="V44" s="3">
-        <v>21610890.70116934</v>
+        <v>21612813.10370687</v>
       </c>
       <c r="W44" s="3">
-        <v>242173.5070957839</v>
+        <v>242971.4505351149</v>
       </c>
       <c r="X44" s="4">
         <f>IF(V44=0,0,W44/V44)</f>
         <v>0</v>
       </c>
       <c r="Y44" s="3">
-        <v>1925897.452986733</v>
+        <v>1934522.442889356</v>
       </c>
       <c r="Z44" s="3">
-        <v>5809.098253916716</v>
+        <v>5530.925248759333</v>
       </c>
       <c r="AA44" s="4">
         <f>IF(Y44=0,0,Z44/Y44)</f>
         <v>0</v>
       </c>
       <c r="AB44" s="3">
-        <v>140314.2879239626</v>
+        <v>138598.7966584856</v>
       </c>
       <c r="AC44" s="3">
-        <v>27.69693223305512</v>
+        <v>0</v>
       </c>
       <c r="AD44" s="4">
         <f>IF(AB44=0,0,AC44/AB44)</f>
@@ -3750,30 +3750,30 @@
         <v>0</v>
       </c>
       <c r="I45" s="3">
-        <v>610.1638407046684</v>
+        <v>610.4870146199353</v>
       </c>
       <c r="J45" s="3">
-        <v>9.162136177603854</v>
+        <v>9.196495682844892</v>
       </c>
       <c r="K45" s="4">
         <f>IF(I45=0,0,J45/I45)</f>
         <v>0</v>
       </c>
       <c r="L45" s="3">
-        <v>9475.405513778041</v>
+        <v>9346.35620700917</v>
       </c>
       <c r="M45" s="3">
-        <v>2.647848884297535</v>
+        <v>0</v>
       </c>
       <c r="N45" s="4">
         <f>IF(L45=0,0,M45/L45)</f>
         <v>0</v>
       </c>
       <c r="O45" s="3">
-        <v>285.742923347472</v>
+        <v>287.6026494045061</v>
       </c>
       <c r="P45" s="3">
-        <v>0.7667368651648867</v>
+        <v>4.031415386218636</v>
       </c>
       <c r="Q45" s="4">
         <f>IF(O45=0,0,P45/O45)</f>
@@ -3790,30 +3790,30 @@
         <v>0</v>
       </c>
       <c r="V45" s="3">
-        <v>20059051.99524085</v>
+        <v>20064025.1831297</v>
       </c>
       <c r="W45" s="3">
-        <v>259185.2599577568</v>
+        <v>259400.8911685646</v>
       </c>
       <c r="X45" s="4">
         <f>IF(V45=0,0,W45/V45)</f>
         <v>0</v>
       </c>
       <c r="Y45" s="3">
-        <v>1405792.016991551</v>
+        <v>1414713.074069254</v>
       </c>
       <c r="Z45" s="3">
-        <v>5319.448695129715</v>
+        <v>5465.855539949844</v>
       </c>
       <c r="AA45" s="4">
         <f>IF(Y45=0,0,Z45/Y45)</f>
         <v>0</v>
       </c>
       <c r="AB45" s="3">
-        <v>106730.9429757299</v>
+        <v>105311.5886077074</v>
       </c>
       <c r="AC45" s="3">
-        <v>29.32616354089987</v>
+        <v>0</v>
       </c>
       <c r="AD45" s="4">
         <f>IF(AB45=0,0,AC45/AB45)</f>
@@ -3956,14 +3956,14 @@
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>M50+P50</f>
+        <f>P50+M50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G50" s="3">
-        <v>55.04951209333916</v>
+        <v>51.92733117123122</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
@@ -3973,7 +3973,7 @@
         <v>382.3073643284127</v>
       </c>
       <c r="J50" s="6">
-        <v>7.728037475080812</v>
+        <v>7.051351267046877</v>
       </c>
       <c r="K50" s="7">
         <f>IF(I50=0,0,J50/I50)</f>
@@ -4003,7 +4003,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T50" s="3">
-        <v>779.0881516072866</v>
+        <v>734.9014899804904</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
@@ -4013,7 +4013,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W50" s="6">
-        <v>183396.5001733974</v>
+        <v>167025.0117590204</v>
       </c>
       <c r="X50" s="7">
         <f>IF(V50=0,0,W50/V50)</f>
@@ -4053,14 +4053,14 @@
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>M51+P51</f>
+        <f>P51+M51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
         <v>147.7607036391234</v>
       </c>
       <c r="G51" s="3">
-        <v>55.83301727702623</v>
+        <v>52.79180338461813</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
@@ -4070,7 +4070,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J51" s="6">
-        <v>6.745118358334934</v>
+        <v>6.16437173703697</v>
       </c>
       <c r="K51" s="7">
         <f>IF(I51=0,0,J51/I51)</f>
@@ -4100,7 +4100,7 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T51" s="3">
-        <v>790.1767077474119</v>
+        <v>747.1359319079959</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
@@ -4110,7 +4110,7 @@
         <v>7100767.677214347</v>
       </c>
       <c r="W51" s="6">
-        <v>213135.3226955337</v>
+        <v>194405.0614645267</v>
       </c>
       <c r="X51" s="7">
         <f>IF(V51=0,0,W51/V51)</f>
@@ -4150,14 +4150,14 @@
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>M52+P52</f>
+        <f>P52+M52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G52" s="3">
-        <v>55.74658849855057</v>
+        <v>52.90475626033849</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
@@ -4167,7 +4167,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J52" s="6">
-        <v>7.433932887340605</v>
+        <v>6.801510224238125</v>
       </c>
       <c r="K52" s="7">
         <f>IF(I52=0,0,J52/I52)</f>
@@ -4197,7 +4197,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T52" s="3">
-        <v>788.9535245672573</v>
+        <v>748.7344973415004</v>
       </c>
       <c r="U52" s="4">
         <f>IF(S52=0,0,T52/S52)</f>
@@ -4207,7 +4207,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W52" s="6">
-        <v>249256.9665041761</v>
+        <v>227563.8985600341</v>
       </c>
       <c r="X52" s="7">
         <f>IF(V52=0,0,W52/V52)</f>
@@ -4247,14 +4247,14 @@
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>M53+P53</f>
+        <f>P53+M53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G53" s="3">
-        <v>25.48769675026658</v>
+        <v>23.699202858531</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
@@ -4264,7 +4264,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J53" s="6">
-        <v>2.88069493231611</v>
+        <v>2.625191036125732</v>
       </c>
       <c r="K53" s="7">
         <f>IF(I53=0,0,J53/I53)</f>
@@ -4294,7 +4294,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T53" s="3">
-        <v>360.7145966384487</v>
+        <v>335.4029390544426</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
@@ -4304,7 +4304,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W53" s="6">
-        <v>102299.5457925303</v>
+        <v>93146.59233288839</v>
       </c>
       <c r="X53" s="7">
         <f>IF(V53=0,0,W53/V53)</f>
@@ -4344,14 +4344,14 @@
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>M54+P54</f>
+        <f>P54+M54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
         <v>93.49564395607489</v>
       </c>
       <c r="G54" s="3">
-        <v>14.82314301600723</v>
+        <v>13.70139980823128</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
@@ -4361,7 +4361,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J54" s="6">
-        <v>2.194074902868248</v>
+        <v>1.998294804040721</v>
       </c>
       <c r="K54" s="7">
         <f>IF(I54=0,0,J54/I54)</f>
@@ -4391,7 +4391,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T54" s="3">
-        <v>209.784513144647</v>
+        <v>193.909043788218</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>
@@ -4401,7 +4401,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W54" s="6">
-        <v>85955.24938089401</v>
+        <v>78240.83772586659</v>
       </c>
       <c r="X54" s="7">
         <f>IF(V54=0,0,W54/V54)</f>
@@ -4564,14 +4564,14 @@
         <v>0</v>
       </c>
       <c r="E59" s="3">
-        <f>M59+P59</f>
+        <f>P59+M59</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
         <v>155.3366697637048</v>
       </c>
       <c r="G59" s="3">
-        <v>101.6478618860977</v>
+        <v>98.78915154595843</v>
       </c>
       <c r="H59" s="4">
         <f>IF(F59=0,0,G59/F59)</f>
@@ -4581,7 +4581,7 @@
         <v>382.3073643284127</v>
       </c>
       <c r="J59" s="6">
-        <v>27.06745242213167</v>
+        <v>25.04314403465664</v>
       </c>
       <c r="K59" s="7">
         <f>IF(I59=0,0,J59/I59)</f>
@@ -4611,7 +4611,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T59" s="3">
-        <v>1438.571239240006</v>
+        <v>1398.113344697664</v>
       </c>
       <c r="U59" s="4">
         <f>IF(S59=0,0,T59/S59)</f>
@@ -4621,7 +4621,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W59" s="6">
-        <v>679501.0839667805</v>
+        <v>624818.6004041024</v>
       </c>
       <c r="X59" s="7">
         <f>IF(V59=0,0,W59/V59)</f>
@@ -4661,14 +4661,14 @@
         <v>0</v>
       </c>
       <c r="E60" s="3">
-        <f>M60+P60</f>
+        <f>P60+M60</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
         <v>147.7607036391234</v>
       </c>
       <c r="G60" s="3">
-        <v>99.75691769012525</v>
+        <v>97.13343978236543</v>
       </c>
       <c r="H60" s="4">
         <f>IF(F60=0,0,G60/F60)</f>
@@ -4678,7 +4678,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J60" s="6">
-        <v>22.43247551696055</v>
+        <v>20.88002309512856</v>
       </c>
       <c r="K60" s="7">
         <f>IF(I60=0,0,J60/I60)</f>
@@ -4708,7 +4708,7 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T60" s="3">
-        <v>1411.809653852386</v>
+        <v>1374.680886017467</v>
       </c>
       <c r="U60" s="4">
         <f>IF(S60=0,0,T60/S60)</f>
@@ -4718,7 +4718,7 @@
         <v>7100767.677214347</v>
       </c>
       <c r="W60" s="6">
-        <v>749637.100508377</v>
+        <v>693698.8487645769</v>
       </c>
       <c r="X60" s="7">
         <f>IF(V60=0,0,W60/V60)</f>
@@ -4758,14 +4758,14 @@
         <v>0</v>
       </c>
       <c r="E61" s="3">
-        <f>M61+P61</f>
+        <f>P61+M61</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
         <v>134.4880808162132</v>
       </c>
       <c r="G61" s="3">
-        <v>94.84760082701457</v>
+        <v>92.60233179008993</v>
       </c>
       <c r="H61" s="4">
         <f>IF(F61=0,0,G61/F61)</f>
@@ -4775,7 +4775,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J61" s="6">
-        <v>23.85461403009552</v>
+        <v>22.29461296479261</v>
       </c>
       <c r="K61" s="7">
         <f>IF(I61=0,0,J61/I61)</f>
@@ -4805,7 +4805,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T61" s="3">
-        <v>1342.330553037646</v>
+        <v>1310.554385778021</v>
       </c>
       <c r="U61" s="4">
         <f>IF(S61=0,0,T61/S61)</f>
@@ -4815,7 +4815,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W61" s="6">
-        <v>848608.1942622317</v>
+        <v>788440.6003954103</v>
       </c>
       <c r="X61" s="7">
         <f>IF(V61=0,0,W61/V61)</f>
@@ -4855,14 +4855,14 @@
         <v>0</v>
       </c>
       <c r="E62" s="3">
-        <f>M62+P62</f>
+        <f>P62+M62</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
         <v>118.5139506930648</v>
       </c>
       <c r="G62" s="3">
-        <v>59.08004047660047</v>
+        <v>56.58851159007293</v>
       </c>
       <c r="H62" s="4">
         <f>IF(F62=0,0,G62/F62)</f>
@@ -4872,7 +4872,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J62" s="6">
-        <v>10.52490515259787</v>
+        <v>9.68772199998633</v>
       </c>
       <c r="K62" s="7">
         <f>IF(I62=0,0,J62/I62)</f>
@@ -4902,7 +4902,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T62" s="3">
-        <v>836.1301995511723</v>
+        <v>800.868840075549</v>
       </c>
       <c r="U62" s="4">
         <f>IF(S62=0,0,T62/S62)</f>
@@ -4912,7 +4912,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W62" s="6">
-        <v>383703.346976216</v>
+        <v>352143.6781484308</v>
       </c>
       <c r="X62" s="7">
         <f>IF(V62=0,0,W62/V62)</f>
@@ -4952,14 +4952,14 @@
         <v>0</v>
       </c>
       <c r="E63" s="3">
-        <f>M63+P63</f>
+        <f>P63+M63</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
         <v>93.49564395607489</v>
       </c>
       <c r="G63" s="3">
-        <v>38.47283650311636</v>
+        <v>36.54054007239058</v>
       </c>
       <c r="H63" s="4">
         <f>IF(F63=0,0,G63/F63)</f>
@@ -4969,7 +4969,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J63" s="6">
-        <v>8.174381605417016</v>
+        <v>7.506574384869266</v>
       </c>
       <c r="K63" s="7">
         <f>IF(I63=0,0,J63/I63)</f>
@@ -4999,7 +4999,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T63" s="3">
-        <v>544.4867708814627</v>
+        <v>517.1399480427974</v>
       </c>
       <c r="U63" s="4">
         <f>IF(S63=0,0,T63/S63)</f>
@@ -5009,7 +5009,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W63" s="6">
-        <v>325951.4286683677</v>
+        <v>298724.0740778223</v>
       </c>
       <c r="X63" s="7">
         <f>IF(V63=0,0,W63/V63)</f>
@@ -5172,7 +5172,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="3">
-        <f>M68+P68</f>
+        <f>P68+M68</f>
         <v>0</v>
       </c>
       <c r="F68" s="3">
@@ -5269,7 +5269,7 @@
         <v>0</v>
       </c>
       <c r="E69" s="3">
-        <f>M69+P69</f>
+        <f>P69+M69</f>
         <v>0</v>
       </c>
       <c r="F69" s="3">
@@ -5366,7 +5366,7 @@
         <v>0</v>
       </c>
       <c r="E70" s="3">
-        <f>M70+P70</f>
+        <f>P70+M70</f>
         <v>0</v>
       </c>
       <c r="F70" s="3">
@@ -5463,7 +5463,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="3">
-        <f>M71+P71</f>
+        <f>P71+M71</f>
         <v>0</v>
       </c>
       <c r="F71" s="3">
@@ -5560,7 +5560,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="3">
-        <f>M72+P72</f>
+        <f>P72+M72</f>
         <v>0</v>
       </c>
       <c r="F72" s="3">

</xml_diff>

<commit_message>
add scale-up vs. current for India/rice
</commit_message>
<xml_diff>
--- a/5000_analyze_results/results_spreadsheet.xlsx
+++ b/5000_analyze_results/results_spreadsheet.xlsx
@@ -19,58 +19,6 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="J48" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Based on correlation between serum folate and hemoglobin</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K48" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Based on correlation between serum folate and hemoglobin</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W48" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Based on correlation between serum folate and hemoglobin</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X48" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Based on correlation between serum folate and hemoglobin</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="J57" authorId="0">
       <text>
         <r>
@@ -175,12 +123,64 @@
         </r>
       </text>
     </comment>
+    <comment ref="J75" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Based on correlation between serum folate and hemoglobin</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K75" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Based on correlation between serum folate and hemoglobin</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W75" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Based on correlation between serum folate and hemoglobin</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X75" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Based on correlation between serum folate and hemoglobin</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="43">
   <si>
     <t>DALYs Averted by Fortification (1000s)</t>
   </si>
@@ -288,6 +288,9 @@
   </si>
   <si>
     <t>India -- Rice-- Scaled-up PDS and industry fortification with increased folate vs none</t>
+  </si>
+  <si>
+    <t>India -- Rice-- Scale-up beyond current PDS fortification</t>
   </si>
   <si>
     <t>Nigeria -- Bouillon</t>
@@ -686,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD72"/>
+  <dimension ref="A1:AD81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -2136,80 +2139,80 @@
         <v>0</v>
       </c>
       <c r="F23" s="3">
-        <v>412.7408750394843</v>
+        <v>350.2135002375949</v>
       </c>
       <c r="G23" s="3">
-        <v>203.0197823281202</v>
+        <v>126.1332383041412</v>
       </c>
       <c r="H23" s="4">
         <f>IF(F23=0,0,G23/F23)</f>
         <v>0</v>
       </c>
       <c r="I23" s="3">
-        <v>1024.476057384201</v>
+        <v>4544.075240942104</v>
       </c>
       <c r="J23" s="3">
-        <v>151.6692552821839</v>
+        <v>183.377095729081</v>
       </c>
       <c r="K23" s="4">
         <f>IF(I23=0,0,J23/I23)</f>
         <v>0</v>
       </c>
       <c r="L23" s="3">
-        <v>15352.83741703859</v>
+        <v>17921.59458137977</v>
       </c>
       <c r="M23" s="3">
-        <v>69.56725985433347</v>
+        <v>27.52917778772116</v>
       </c>
       <c r="N23" s="4">
         <f>IF(L23=0,0,M23/L23)</f>
         <v>0</v>
       </c>
       <c r="O23" s="3">
-        <v>503.5634310516943</v>
+        <v>495.9444735664641</v>
       </c>
       <c r="P23" s="3">
-        <v>21.01036396919185</v>
+        <v>7.481059255957137</v>
       </c>
       <c r="Q23" s="4">
         <f>IF(O23=0,0,P23/O23)</f>
         <v>0</v>
       </c>
       <c r="S23" s="3">
-        <v>12734.95565684622</v>
+        <v>4521.415712753815</v>
       </c>
       <c r="T23" s="3">
-        <v>6264.094694192449</v>
+        <v>1628.437525058162</v>
       </c>
       <c r="U23" s="4">
         <f>IF(S23=0,0,T23/S23)</f>
         <v>0</v>
       </c>
       <c r="V23" s="3">
-        <v>25177467.03377928</v>
+        <v>126742195.0259868</v>
       </c>
       <c r="W23" s="3">
-        <v>2945174.443318196</v>
+        <v>3982425.375684574</v>
       </c>
       <c r="X23" s="4">
         <f>IF(V23=0,0,W23/V23)</f>
         <v>0</v>
       </c>
       <c r="Y23" s="3">
-        <v>2561085.175981381</v>
+        <v>2951242.405431581</v>
       </c>
       <c r="Z23" s="3">
-        <v>116196.6057628184</v>
+        <v>32833.07583494857</v>
       </c>
       <c r="AA23" s="4">
         <f>IF(Y23=0,0,Z23/Y23)</f>
         <v>0</v>
       </c>
       <c r="AB23" s="3">
-        <v>172903.801774421</v>
+        <v>199922.9290412657</v>
       </c>
       <c r="AC23" s="3">
-        <v>772.255639909883</v>
+        <v>305.9504023261252</v>
       </c>
       <c r="AD23" s="4">
         <f>IF(AB23=0,0,AC23/AB23)</f>
@@ -2233,80 +2236,80 @@
         <v>0</v>
       </c>
       <c r="F24" s="3">
-        <v>422.0532339939541</v>
+        <v>311.4684795357562</v>
       </c>
       <c r="G24" s="3">
-        <v>198.5663656707619</v>
+        <v>101.5213100528625</v>
       </c>
       <c r="H24" s="4">
         <f>IF(F24=0,0,G24/F24)</f>
         <v>0</v>
       </c>
       <c r="I24" s="3">
-        <v>968.8874507802924</v>
+        <v>4115.061938775183</v>
       </c>
       <c r="J24" s="3">
-        <v>150.8926468475667</v>
+        <v>175.1483470106083</v>
       </c>
       <c r="K24" s="4">
         <f>IF(I24=0,0,J24/I24)</f>
         <v>0</v>
       </c>
       <c r="L24" s="3">
-        <v>15897.14811387405</v>
+        <v>14788.44110493821</v>
       </c>
       <c r="M24" s="3">
-        <v>66.02582374739833</v>
+        <v>19.50661562452465</v>
       </c>
       <c r="N24" s="4">
         <f>IF(L24=0,0,M24/L24)</f>
         <v>0</v>
       </c>
       <c r="O24" s="3">
-        <v>427.6878840211459</v>
+        <v>292.0445785383909</v>
       </c>
       <c r="P24" s="3">
-        <v>21.73464126741991</v>
+        <v>2.180210262297885</v>
       </c>
       <c r="Q24" s="4">
         <f>IF(O24=0,0,P24/O24)</f>
         <v>0</v>
       </c>
       <c r="S24" s="3">
-        <v>13022.28479122008</v>
+        <v>4021.199857929781</v>
       </c>
       <c r="T24" s="3">
-        <v>6126.686293225393</v>
+        <v>1310.686327457256</v>
       </c>
       <c r="U24" s="4">
         <f>IF(S24=0,0,T24/S24)</f>
         <v>0</v>
       </c>
       <c r="V24" s="3">
-        <v>24716781.60947407</v>
+        <v>118766080.2208486</v>
       </c>
       <c r="W24" s="3">
-        <v>3073981.15008124</v>
+        <v>4011188.986341327</v>
       </c>
       <c r="X24" s="4">
         <f>IF(V24=0,0,W24/V24)</f>
         <v>0</v>
       </c>
       <c r="Y24" s="3">
-        <v>2216806.226901517</v>
+        <v>1753068.388397526</v>
       </c>
       <c r="Z24" s="3">
-        <v>113084.6469390318</v>
+        <v>19783.04635228659</v>
       </c>
       <c r="AA24" s="4">
         <f>IF(Y24=0,0,Z24/Y24)</f>
         <v>0</v>
       </c>
       <c r="AB24" s="3">
-        <v>179047.6330362356</v>
+        <v>164977.1295440781</v>
       </c>
       <c r="AC24" s="3">
-        <v>733.1540885220165</v>
+        <v>216.8152457429387</v>
       </c>
       <c r="AD24" s="4">
         <f>IF(AB24=0,0,AC24/AB24)</f>
@@ -2330,80 +2333,80 @@
         <v>0</v>
       </c>
       <c r="F25" s="3">
-        <v>382.0743136549376</v>
+        <v>280.1619272206273</v>
       </c>
       <c r="G25" s="3">
-        <v>154.1818427005811</v>
+        <v>90.83042367476904</v>
       </c>
       <c r="H25" s="4">
         <f>IF(F25=0,0,G25/F25)</f>
         <v>0</v>
       </c>
       <c r="I25" s="3">
-        <v>792.6568327877751</v>
+        <v>4040.491935003149</v>
       </c>
       <c r="J25" s="3">
-        <v>138.7460097809298</v>
+        <v>174.9214101983323</v>
       </c>
       <c r="K25" s="4">
         <f>IF(I25=0,0,J25/I25)</f>
         <v>0</v>
       </c>
       <c r="L25" s="3">
-        <v>14099.36149543928</v>
+        <v>13121.09243386837</v>
       </c>
       <c r="M25" s="3">
-        <v>48.02046110171266</v>
+        <v>16.47687015608139</v>
       </c>
       <c r="N25" s="4">
         <f>IF(L25=0,0,M25/L25)</f>
         <v>0</v>
       </c>
       <c r="O25" s="3">
-        <v>410.8336896551561</v>
+        <v>344.935183132892</v>
       </c>
       <c r="P25" s="3">
-        <v>20.00392896381795</v>
+        <v>3.880373961144243</v>
       </c>
       <c r="Q25" s="4">
         <f>IF(O25=0,0,P25/O25)</f>
         <v>0</v>
       </c>
       <c r="S25" s="3">
-        <v>11788.75109364953</v>
+        <v>3617.018016128304</v>
       </c>
       <c r="T25" s="3">
-        <v>4757.219477462471</v>
+        <v>1172.662117595605</v>
       </c>
       <c r="U25" s="4">
         <f>IF(S25=0,0,T25/S25)</f>
         <v>0</v>
       </c>
       <c r="V25" s="3">
-        <v>22756394.15398703</v>
+        <v>116878553.0684172</v>
       </c>
       <c r="W25" s="3">
-        <v>3255095.686233584</v>
+        <v>4060793.245081708</v>
       </c>
       <c r="X25" s="4">
         <f>IF(V25=0,0,W25/V25)</f>
         <v>0</v>
       </c>
       <c r="Y25" s="3">
-        <v>2114085.557833027</v>
+        <v>2220801.451734822</v>
       </c>
       <c r="Z25" s="3">
-        <v>104646.7324492342</v>
+        <v>24803.95321792085</v>
       </c>
       <c r="AA25" s="4">
         <f>IF(Y25=0,0,Z25/Y25)</f>
         <v>0</v>
       </c>
       <c r="AB25" s="3">
-        <v>158763.7032537926</v>
+        <v>146367.154284477</v>
       </c>
       <c r="AC25" s="3">
-        <v>532.758637659339</v>
+        <v>183.0884297384764</v>
       </c>
       <c r="AD25" s="4">
         <f>IF(AB25=0,0,AC25/AB25)</f>
@@ -2427,80 +2430,80 @@
         <v>0</v>
       </c>
       <c r="F26" s="3">
-        <v>338.6701578384149</v>
+        <v>264.7104462197004</v>
       </c>
       <c r="G26" s="3">
-        <v>120.7918882652273</v>
+        <v>82.83545493544487</v>
       </c>
       <c r="H26" s="4">
         <f>IF(F26=0,0,G26/F26)</f>
         <v>0</v>
       </c>
       <c r="I26" s="3">
-        <v>714.5868735320346</v>
+        <v>3711.723400478158</v>
       </c>
       <c r="J26" s="3">
-        <v>127.9421658211542</v>
+        <v>157.5814734089011</v>
       </c>
       <c r="K26" s="4">
         <f>IF(I26=0,0,J26/I26)</f>
         <v>0</v>
       </c>
       <c r="L26" s="3">
-        <v>12459.036398116</v>
+        <v>12509.4824404558</v>
       </c>
       <c r="M26" s="3">
-        <v>33.00900104676187</v>
+        <v>19.07299118544161</v>
       </c>
       <c r="N26" s="4">
         <f>IF(L26=0,0,M26/L26)</f>
         <v>0</v>
       </c>
       <c r="O26" s="3">
-        <v>388.5202631627004</v>
+        <v>334.1065712533387</v>
       </c>
       <c r="P26" s="3">
-        <v>16.30620732857898</v>
+        <v>3.852939512438141</v>
       </c>
       <c r="Q26" s="4">
         <f>IF(O26=0,0,P26/O26)</f>
         <v>0</v>
       </c>
       <c r="S26" s="3">
-        <v>10449.53311676904</v>
+        <v>3417.532362561234</v>
       </c>
       <c r="T26" s="3">
-        <v>3726.985704086702</v>
+        <v>1069.443431689916</v>
       </c>
       <c r="U26" s="4">
         <f>IF(S26=0,0,T26/S26)</f>
         <v>0</v>
       </c>
       <c r="V26" s="3">
-        <v>21413420.36871202</v>
+        <v>111157067.1148831</v>
       </c>
       <c r="W26" s="3">
-        <v>3188030.275738072</v>
+        <v>3853045.254141852</v>
       </c>
       <c r="X26" s="4">
         <f>IF(V26=0,0,W26/V26)</f>
         <v>0</v>
       </c>
       <c r="Y26" s="3">
-        <v>1925897.452986733</v>
+        <v>1986227.953294863</v>
       </c>
       <c r="Z26" s="3">
-        <v>86993.32044937275</v>
+        <v>21040.67771757673</v>
       </c>
       <c r="AA26" s="4">
         <f>IF(Y26=0,0,Z26/Y26)</f>
         <v>0</v>
       </c>
       <c r="AB26" s="3">
-        <v>140314.2879239626</v>
+        <v>139542.2921601469</v>
       </c>
       <c r="AC26" s="3">
-        <v>366.5770442610374</v>
+        <v>211.9971291708644</v>
       </c>
       <c r="AD26" s="4">
         <f>IF(AB26=0,0,AC26/AB26)</f>
@@ -2524,80 +2527,80 @@
         <v>0</v>
       </c>
       <c r="F27" s="3">
-        <v>297.4602934996698</v>
+        <v>228.7378677797919</v>
       </c>
       <c r="G27" s="3">
-        <v>100.604253937639</v>
+        <v>49.8204031635008</v>
       </c>
       <c r="H27" s="4">
         <f>IF(F27=0,0,G27/F27)</f>
         <v>0</v>
       </c>
       <c r="I27" s="3">
-        <v>607.1996095192959</v>
+        <v>3287.366635081595</v>
       </c>
       <c r="J27" s="3">
-        <v>115.4369858740715</v>
+        <v>141.1674286687611</v>
       </c>
       <c r="K27" s="4">
         <f>IF(I27=0,0,J27/I27)</f>
         <v>0</v>
       </c>
       <c r="L27" s="3">
-        <v>9475.405513778041</v>
+        <v>11848.74438110083</v>
       </c>
       <c r="M27" s="3">
-        <v>26.1176055910252</v>
+        <v>11.70584179613739</v>
       </c>
       <c r="N27" s="4">
         <f>IF(L27=0,0,M27/L27)</f>
         <v>0</v>
       </c>
       <c r="O27" s="3">
-        <v>285.742923347472</v>
+        <v>207.9711932231975</v>
       </c>
       <c r="P27" s="3">
-        <v>14.29403973296256</v>
+        <v>2.10708170880744</v>
       </c>
       <c r="Q27" s="4">
         <f>IF(O27=0,0,P27/O27)</f>
         <v>0</v>
       </c>
       <c r="S27" s="3">
-        <v>9178.019131321482</v>
+        <v>2953.109999413819</v>
       </c>
       <c r="T27" s="3">
-        <v>3104.104270417525</v>
+        <v>643.204084155409</v>
       </c>
       <c r="U27" s="4">
         <f>IF(S27=0,0,T27/S27)</f>
         <v>0</v>
       </c>
       <c r="V27" s="3">
-        <v>19850211.7121278</v>
+        <v>105015702.2458295</v>
       </c>
       <c r="W27" s="3">
-        <v>3182528.287519272</v>
+        <v>3765958.107265323</v>
       </c>
       <c r="X27" s="4">
         <f>IF(V27=0,0,W27/V27)</f>
         <v>0</v>
       </c>
       <c r="Y27" s="3">
-        <v>1405792.016991551</v>
+        <v>1265807.171489435</v>
       </c>
       <c r="Z27" s="3">
-        <v>72425.83938977448</v>
+        <v>12359.89525352535</v>
       </c>
       <c r="AA27" s="4">
         <f>IF(Y27=0,0,Z27/Y27)</f>
         <v>0</v>
       </c>
       <c r="AB27" s="3">
-        <v>106730.9429757299</v>
+        <v>132182.6190963176</v>
       </c>
       <c r="AC27" s="3">
-        <v>290.0031727931782</v>
+        <v>130.0891474457458</v>
       </c>
       <c r="AD27" s="4">
         <f>IF(AB27=0,0,AC27/AB27)</f>
@@ -2747,7 +2750,7 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G32" s="3">
-        <v>88.917209540012</v>
+        <v>203.0197823281202</v>
       </c>
       <c r="H32" s="4">
         <f>IF(F32=0,0,G32/F32)</f>
@@ -2757,7 +2760,7 @@
         <v>1024.476057384201</v>
       </c>
       <c r="J32" s="3">
-        <v>37.42618266519206</v>
+        <v>151.6692552821839</v>
       </c>
       <c r="K32" s="4">
         <f>IF(I32=0,0,J32/I32)</f>
@@ -2767,7 +2770,7 @@
         <v>15352.83741703859</v>
       </c>
       <c r="M32" s="3">
-        <v>8.513003026653081</v>
+        <v>69.56725985433347</v>
       </c>
       <c r="N32" s="4">
         <f>IF(L32=0,0,M32/L32)</f>
@@ -2777,7 +2780,7 @@
         <v>503.5634310516943</v>
       </c>
       <c r="P32" s="3">
-        <v>4.035215178299462</v>
+        <v>21.01036396919185</v>
       </c>
       <c r="Q32" s="4">
         <f>IF(O32=0,0,P32/O32)</f>
@@ -2787,7 +2790,7 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T32" s="3">
-        <v>2743.505160505925</v>
+        <v>6264.094694192449</v>
       </c>
       <c r="U32" s="4">
         <f>IF(S32=0,0,T32/S32)</f>
@@ -2797,7 +2800,7 @@
         <v>25177467.03377928</v>
       </c>
       <c r="W32" s="3">
-        <v>716915.3751159273</v>
+        <v>2945174.443318196</v>
       </c>
       <c r="X32" s="4">
         <f>IF(V32=0,0,W32/V32)</f>
@@ -2807,7 +2810,7 @@
         <v>2561085.175981381</v>
       </c>
       <c r="Z32" s="3">
-        <v>26434.5692036259</v>
+        <v>116196.6057628184</v>
       </c>
       <c r="AA32" s="4">
         <f>IF(Y32=0,0,Z32/Y32)</f>
@@ -2817,7 +2820,7 @@
         <v>172903.801774421</v>
       </c>
       <c r="AC32" s="3">
-        <v>94.49541585397674</v>
+        <v>772.255639909883</v>
       </c>
       <c r="AD32" s="4">
         <f>IF(AB32=0,0,AC32/AB32)</f>
@@ -2844,7 +2847,7 @@
         <v>422.0532339939541</v>
       </c>
       <c r="G33" s="3">
-        <v>119.3410127560627</v>
+        <v>198.5663656707619</v>
       </c>
       <c r="H33" s="4">
         <f>IF(F33=0,0,G33/F33)</f>
@@ -2854,7 +2857,7 @@
         <v>968.8874507802924</v>
       </c>
       <c r="J33" s="3">
-        <v>48.89668702791759</v>
+        <v>150.8926468475667</v>
       </c>
       <c r="K33" s="4">
         <f>IF(I33=0,0,J33/I33)</f>
@@ -2864,7 +2867,7 @@
         <v>15897.14811387405</v>
       </c>
       <c r="M33" s="3">
-        <v>12.76530790260248</v>
+        <v>66.02582374739833</v>
       </c>
       <c r="N33" s="4">
         <f>IF(L33=0,0,M33/L33)</f>
@@ -2874,7 +2877,7 @@
         <v>427.6878840211459</v>
       </c>
       <c r="P33" s="3">
-        <v>6.028749298481445</v>
+        <v>21.73464126741991</v>
       </c>
       <c r="Q33" s="4">
         <f>IF(O33=0,0,P33/O33)</f>
@@ -2884,7 +2887,7 @@
         <v>13022.28479122008</v>
       </c>
       <c r="T33" s="3">
-        <v>3682.219516897101</v>
+        <v>6126.686293225393</v>
       </c>
       <c r="U33" s="4">
         <f>IF(S33=0,0,T33/S33)</f>
@@ -2894,7 +2897,7 @@
         <v>24716781.60947407</v>
       </c>
       <c r="W33" s="3">
-        <v>982157.0316114575</v>
+        <v>3073981.15008124</v>
       </c>
       <c r="X33" s="4">
         <f>IF(V33=0,0,W33/V33)</f>
@@ -2904,7 +2907,7 @@
         <v>2216806.226901517</v>
       </c>
       <c r="Z33" s="3">
-        <v>34210.39940629248</v>
+        <v>113084.6469390318</v>
       </c>
       <c r="AA33" s="4">
         <f>IF(Y33=0,0,Z33/Y33)</f>
@@ -2914,7 +2917,7 @@
         <v>179047.6330362356</v>
       </c>
       <c r="AC33" s="3">
-        <v>141.743123780936</v>
+        <v>733.1540885220165</v>
       </c>
       <c r="AD33" s="4">
         <f>IF(AB33=0,0,AC33/AB33)</f>
@@ -2941,7 +2944,7 @@
         <v>382.0743136549376</v>
       </c>
       <c r="G34" s="3">
-        <v>119.4634252945786</v>
+        <v>154.1818427005811</v>
       </c>
       <c r="H34" s="4">
         <f>IF(F34=0,0,G34/F34)</f>
@@ -2951,7 +2954,7 @@
         <v>792.6568327877751</v>
       </c>
       <c r="J34" s="3">
-        <v>54.5890911232098</v>
+        <v>138.7460097809298</v>
       </c>
       <c r="K34" s="4">
         <f>IF(I34=0,0,J34/I34)</f>
@@ -2961,7 +2964,7 @@
         <v>14099.36149543928</v>
       </c>
       <c r="M34" s="3">
-        <v>13.51587385891005</v>
+        <v>48.02046110171266</v>
       </c>
       <c r="N34" s="4">
         <f>IF(L34=0,0,M34/L34)</f>
@@ -2971,7 +2974,7 @@
         <v>410.8336896551561</v>
       </c>
       <c r="P34" s="3">
-        <v>7.356626560289995</v>
+        <v>20.00392896381795</v>
       </c>
       <c r="Q34" s="4">
         <f>IF(O34=0,0,P34/O34)</f>
@@ -2981,7 +2984,7 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T34" s="3">
-        <v>3685.99650712055</v>
+        <v>4757.219477462471</v>
       </c>
       <c r="U34" s="4">
         <f>IF(S34=0,0,T34/S34)</f>
@@ -2991,7 +2994,7 @@
         <v>22756394.15398703</v>
       </c>
       <c r="W34" s="3">
-        <v>1261498.724129144</v>
+        <v>3255095.686233584</v>
       </c>
       <c r="X34" s="4">
         <f>IF(V34=0,0,W34/V34)</f>
@@ -3001,7 +3004,7 @@
         <v>2114085.557833027</v>
       </c>
       <c r="Z34" s="3">
-        <v>40224.46724295756</v>
+        <v>104646.7324492342</v>
       </c>
       <c r="AA34" s="4">
         <f>IF(Y34=0,0,Z34/Y34)</f>
@@ -3011,7 +3014,7 @@
         <v>158763.7032537926</v>
       </c>
       <c r="AC34" s="3">
-        <v>149.8892803200579</v>
+        <v>532.758637659339</v>
       </c>
       <c r="AD34" s="4">
         <f>IF(AB34=0,0,AC34/AB34)</f>
@@ -3038,7 +3041,7 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G35" s="3">
-        <v>117.3536742164378</v>
+        <v>120.7918882652273</v>
       </c>
       <c r="H35" s="4">
         <f>IF(F35=0,0,G35/F35)</f>
@@ -3048,7 +3051,7 @@
         <v>714.5868735320346</v>
       </c>
       <c r="J35" s="3">
-        <v>58.87230459435971</v>
+        <v>127.9421658211542</v>
       </c>
       <c r="K35" s="4">
         <f>IF(I35=0,0,J35/I35)</f>
@@ -3058,7 +3061,7 @@
         <v>12459.036398116</v>
       </c>
       <c r="M35" s="3">
-        <v>13.5043200882338</v>
+        <v>33.00900104676187</v>
       </c>
       <c r="N35" s="4">
         <f>IF(L35=0,0,M35/L35)</f>
@@ -3068,7 +3071,7 @@
         <v>388.5202631627004</v>
       </c>
       <c r="P35" s="3">
-        <v>7.537730635970249</v>
+        <v>16.30620732857898</v>
       </c>
       <c r="Q35" s="4">
         <f>IF(O35=0,0,P35/O35)</f>
@@ -3078,7 +3081,7 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T35" s="3">
-        <v>3620.900976118114</v>
+        <v>3726.985704086702</v>
       </c>
       <c r="U35" s="4">
         <f>IF(S35=0,0,T35/S35)</f>
@@ -3088,7 +3091,7 @@
         <v>21413420.36871202</v>
       </c>
       <c r="W35" s="3">
-        <v>1446105.459525652</v>
+        <v>3188030.275738072</v>
       </c>
       <c r="X35" s="4">
         <f>IF(V35=0,0,W35/V35)</f>
@@ -3098,7 +3101,7 @@
         <v>1925897.452986733</v>
       </c>
       <c r="Z35" s="3">
-        <v>38916.56609589816</v>
+        <v>86993.32044937275</v>
       </c>
       <c r="AA35" s="4">
         <f>IF(Y35=0,0,Z35/Y35)</f>
@@ -3108,7 +3111,7 @@
         <v>140314.2879239626</v>
       </c>
       <c r="AC35" s="3">
-        <v>149.8892803200579</v>
+        <v>366.5770442610374</v>
       </c>
       <c r="AD35" s="4">
         <f>IF(AB35=0,0,AC35/AB35)</f>
@@ -3135,7 +3138,7 @@
         <v>297.4602934996698</v>
       </c>
       <c r="G36" s="3">
-        <v>106.3158412713952</v>
+        <v>100.604253937639</v>
       </c>
       <c r="H36" s="4">
         <f>IF(F36=0,0,G36/F36)</f>
@@ -3145,7 +3148,7 @@
         <v>607.1996095192959</v>
       </c>
       <c r="J36" s="3">
-        <v>56.87764650202414</v>
+        <v>115.4369858740715</v>
       </c>
       <c r="K36" s="4">
         <f>IF(I36=0,0,J36/I36)</f>
@@ -3155,7 +3158,7 @@
         <v>9475.405513778041</v>
       </c>
       <c r="M36" s="3">
-        <v>12.91396182483621</v>
+        <v>26.1176055910252</v>
       </c>
       <c r="N36" s="4">
         <f>IF(L36=0,0,M36/L36)</f>
@@ -3165,7 +3168,7 @@
         <v>285.742923347472</v>
       </c>
       <c r="P36" s="3">
-        <v>6.662558508813381</v>
+        <v>14.29403973296256</v>
       </c>
       <c r="Q36" s="4">
         <f>IF(O36=0,0,P36/O36)</f>
@@ -3175,7 +3178,7 @@
         <v>9178.019131321482</v>
       </c>
       <c r="T36" s="3">
-        <v>3280.333027549058</v>
+        <v>3104.104270417525</v>
       </c>
       <c r="U36" s="4">
         <f>IF(S36=0,0,T36/S36)</f>
@@ -3185,7 +3188,7 @@
         <v>19850211.7121278</v>
       </c>
       <c r="W36" s="3">
-        <v>1545620.805538651</v>
+        <v>3182528.287519272</v>
       </c>
       <c r="X36" s="4">
         <f>IF(V36=0,0,W36/V36)</f>
@@ -3195,7 +3198,7 @@
         <v>1405792.016991551</v>
       </c>
       <c r="Z36" s="3">
-        <v>34472.30498424848</v>
+        <v>72425.83938977448</v>
       </c>
       <c r="AA36" s="4">
         <f>IF(Y36=0,0,Z36/Y36)</f>
@@ -3205,7 +3208,7 @@
         <v>106730.9429757299</v>
       </c>
       <c r="AC36" s="3">
-        <v>143.3723550887371</v>
+        <v>290.0031727931782</v>
       </c>
       <c r="AD36" s="4">
         <f>IF(AB36=0,0,AC36/AB36)</f>
@@ -3355,17 +3358,17 @@
         <v>412.7408750394843</v>
       </c>
       <c r="G41" s="3">
-        <v>23.42409718172002</v>
+        <v>88.917209540012</v>
       </c>
       <c r="H41" s="4">
         <f>IF(F41=0,0,G41/F41)</f>
         <v>0</v>
       </c>
       <c r="I41" s="3">
-        <v>1026.204299813583</v>
+        <v>1024.476057384201</v>
       </c>
       <c r="J41" s="3">
-        <v>6.332670651874505</v>
+        <v>37.42618266519206</v>
       </c>
       <c r="K41" s="4">
         <f>IF(I41=0,0,J41/I41)</f>
@@ -3375,7 +3378,7 @@
         <v>15352.83741703859</v>
       </c>
       <c r="M41" s="3">
-        <v>0.5863035025261343</v>
+        <v>8.513003026653081</v>
       </c>
       <c r="N41" s="4">
         <f>IF(L41=0,0,M41/L41)</f>
@@ -3385,7 +3388,7 @@
         <v>503.5634310516943</v>
       </c>
       <c r="P41" s="3">
-        <v>0.7976752452995279</v>
+        <v>4.035215178299462</v>
       </c>
       <c r="Q41" s="4">
         <f>IF(O41=0,0,P41/O41)</f>
@@ -3395,17 +3398,17 @@
         <v>12734.95565684622</v>
       </c>
       <c r="T41" s="3">
-        <v>722.7412087119392</v>
+        <v>2743.505160505925</v>
       </c>
       <c r="U41" s="4">
         <f>IF(S41=0,0,T41/S41)</f>
         <v>0</v>
       </c>
       <c r="V41" s="3">
-        <v>25286285.18025935</v>
+        <v>25177467.03377928</v>
       </c>
       <c r="W41" s="3">
-        <v>124252.6863578595</v>
+        <v>716915.3751159273</v>
       </c>
       <c r="X41" s="4">
         <f>IF(V41=0,0,W41/V41)</f>
@@ -3415,7 +3418,7 @@
         <v>2561085.175981381</v>
       </c>
       <c r="Z41" s="3">
-        <v>4301.107752270065</v>
+        <v>26434.5692036259</v>
       </c>
       <c r="AA41" s="4">
         <f>IF(Y41=0,0,Z41/Y41)</f>
@@ -3425,7 +3428,7 @@
         <v>172903.801774421</v>
       </c>
       <c r="AC41" s="3">
-        <v>6.516925231320783</v>
+        <v>94.49541585397674</v>
       </c>
       <c r="AD41" s="4">
         <f>IF(AB41=0,0,AC41/AB41)</f>
@@ -3449,20 +3452,20 @@
         <v>0</v>
       </c>
       <c r="F42" s="3">
-        <v>422.0532339939548</v>
+        <v>422.0532339939541</v>
       </c>
       <c r="G42" s="3">
-        <v>32.39383284579316</v>
+        <v>119.3410127560627</v>
       </c>
       <c r="H42" s="4">
         <f>IF(F42=0,0,G42/F42)</f>
         <v>0</v>
       </c>
       <c r="I42" s="3">
-        <v>971.1037573173985</v>
+        <v>968.8874507802924</v>
       </c>
       <c r="J42" s="3">
-        <v>8.271399086192949</v>
+        <v>48.89668702791759</v>
       </c>
       <c r="K42" s="4">
         <f>IF(I42=0,0,J42/I42)</f>
@@ -3472,7 +3475,7 @@
         <v>15897.14811387405</v>
       </c>
       <c r="M42" s="3">
-        <v>2.204028858903795</v>
+        <v>12.76530790260248</v>
       </c>
       <c r="N42" s="4">
         <f>IF(L42=0,0,M42/L42)</f>
@@ -3482,27 +3485,27 @@
         <v>427.6878840211459</v>
       </c>
       <c r="P42" s="3">
-        <v>0.7658804311889107</v>
+        <v>6.028749298481445</v>
       </c>
       <c r="Q42" s="4">
         <f>IF(O42=0,0,P42/O42)</f>
         <v>0</v>
       </c>
       <c r="S42" s="3">
-        <v>13022.2847912201</v>
+        <v>13022.28479122008</v>
       </c>
       <c r="T42" s="3">
-        <v>999.4988376351139</v>
+        <v>3682.219516897101</v>
       </c>
       <c r="U42" s="4">
         <f>IF(S42=0,0,T42/S42)</f>
         <v>0</v>
       </c>
       <c r="V42" s="3">
-        <v>24859901.01601297</v>
+        <v>24716781.60947407</v>
       </c>
       <c r="W42" s="3">
-        <v>171453.208100237</v>
+        <v>982157.0316114575</v>
       </c>
       <c r="X42" s="4">
         <f>IF(V42=0,0,W42/V42)</f>
@@ -3512,7 +3515,7 @@
         <v>2216806.226901517</v>
       </c>
       <c r="Z42" s="3">
-        <v>5397.532345701009</v>
+        <v>34210.39940629248</v>
       </c>
       <c r="AA42" s="4">
         <f>IF(Y42=0,0,Z42/Y42)</f>
@@ -3522,7 +3525,7 @@
         <v>179047.6330362356</v>
       </c>
       <c r="AC42" s="3">
-        <v>24.43846961739473</v>
+        <v>141.743123780936</v>
       </c>
       <c r="AD42" s="4">
         <f>IF(AB42=0,0,AC42/AB42)</f>
@@ -3549,17 +3552,17 @@
         <v>382.0743136549376</v>
       </c>
       <c r="G43" s="3">
-        <v>45.49713331928587</v>
+        <v>119.4634252945786</v>
       </c>
       <c r="H43" s="4">
         <f>IF(F43=0,0,G43/F43)</f>
         <v>0</v>
       </c>
       <c r="I43" s="3">
-        <v>795.3294661601195</v>
+        <v>792.6568327877751</v>
       </c>
       <c r="J43" s="3">
-        <v>9.250773828173406</v>
+        <v>54.5890911232098</v>
       </c>
       <c r="K43" s="4">
         <f>IF(I43=0,0,J43/I43)</f>
@@ -3569,7 +3572,7 @@
         <v>14099.36149543928</v>
       </c>
       <c r="M43" s="3">
-        <v>2.494237892366946</v>
+        <v>13.51587385891005</v>
       </c>
       <c r="N43" s="4">
         <f>IF(L43=0,0,M43/L43)</f>
@@ -3579,7 +3582,7 @@
         <v>410.8336896551561</v>
       </c>
       <c r="P43" s="3">
-        <v>0.6260496127711959</v>
+        <v>7.356626560289995</v>
       </c>
       <c r="Q43" s="4">
         <f>IF(O43=0,0,P43/O43)</f>
@@ -3589,17 +3592,17 @@
         <v>11788.75109364953</v>
       </c>
       <c r="T43" s="3">
-        <v>1403.795965881249</v>
+        <v>3685.99650712055</v>
       </c>
       <c r="U43" s="4">
         <f>IF(S43=0,0,T43/S43)</f>
         <v>0</v>
       </c>
       <c r="V43" s="3">
-        <v>22936296.40445412</v>
+        <v>22756394.15398703</v>
       </c>
       <c r="W43" s="3">
-        <v>221609.0820698142</v>
+        <v>1261498.724129144</v>
       </c>
       <c r="X43" s="4">
         <f>IF(V43=0,0,W43/V43)</f>
@@ -3609,7 +3612,7 @@
         <v>2114085.557833027</v>
       </c>
       <c r="Z43" s="3">
-        <v>6329.655924388207</v>
+        <v>40224.46724295756</v>
       </c>
       <c r="AA43" s="4">
         <f>IF(Y43=0,0,Z43/Y43)</f>
@@ -3619,7 +3622,7 @@
         <v>158763.7032537926</v>
       </c>
       <c r="AC43" s="3">
-        <v>27.69693223305512</v>
+        <v>149.8892803200579</v>
       </c>
       <c r="AD43" s="4">
         <f>IF(AB43=0,0,AC43/AB43)</f>
@@ -3646,17 +3649,17 @@
         <v>338.6701578384149</v>
       </c>
       <c r="G44" s="3">
-        <v>48.79942009843676</v>
+        <v>117.3536742164378</v>
       </c>
       <c r="H44" s="4">
         <f>IF(F44=0,0,G44/F44)</f>
         <v>0</v>
       </c>
       <c r="I44" s="3">
-        <v>717.4492241565633</v>
+        <v>714.5868735320346</v>
       </c>
       <c r="J44" s="3">
-        <v>9.464455356970662</v>
+        <v>58.87230459435971</v>
       </c>
       <c r="K44" s="4">
         <f>IF(I44=0,0,J44/I44)</f>
@@ -3666,7 +3669,7 @@
         <v>12459.036398116</v>
       </c>
       <c r="M44" s="3">
-        <v>2.502058168889955</v>
+        <v>13.5043200882338</v>
       </c>
       <c r="N44" s="4">
         <f>IF(L44=0,0,M44/L44)</f>
@@ -3676,7 +3679,7 @@
         <v>388.5202631627004</v>
       </c>
       <c r="P44" s="3">
-        <v>1.11741603567038</v>
+        <v>7.537730635970249</v>
       </c>
       <c r="Q44" s="4">
         <f>IF(O44=0,0,P44/O44)</f>
@@ -3686,17 +3689,17 @@
         <v>10449.53311676904</v>
       </c>
       <c r="T44" s="3">
-        <v>1505.686711968985</v>
+        <v>3620.900976118114</v>
       </c>
       <c r="U44" s="4">
         <f>IF(S44=0,0,T44/S44)</f>
         <v>0</v>
       </c>
       <c r="V44" s="3">
-        <v>21610890.70116934</v>
+        <v>21413420.36871202</v>
       </c>
       <c r="W44" s="3">
-        <v>242173.5070957839</v>
+        <v>1446105.459525652</v>
       </c>
       <c r="X44" s="4">
         <f>IF(V44=0,0,W44/V44)</f>
@@ -3706,7 +3709,7 @@
         <v>1925897.452986733</v>
       </c>
       <c r="Z44" s="3">
-        <v>5809.098253916716</v>
+        <v>38916.56609589816</v>
       </c>
       <c r="AA44" s="4">
         <f>IF(Y44=0,0,Z44/Y44)</f>
@@ -3716,7 +3719,7 @@
         <v>140314.2879239626</v>
       </c>
       <c r="AC44" s="3">
-        <v>27.69693223305512</v>
+        <v>149.8892803200579</v>
       </c>
       <c r="AD44" s="4">
         <f>IF(AB44=0,0,AC44/AB44)</f>
@@ -3743,17 +3746,17 @@
         <v>297.4602934996698</v>
       </c>
       <c r="G45" s="3">
-        <v>50.94083911201337</v>
+        <v>106.3158412713952</v>
       </c>
       <c r="H45" s="4">
         <f>IF(F45=0,0,G45/F45)</f>
         <v>0</v>
       </c>
       <c r="I45" s="3">
-        <v>610.1638407046684</v>
+        <v>607.1996095192959</v>
       </c>
       <c r="J45" s="3">
-        <v>9.162136177603854</v>
+        <v>56.87764650202414</v>
       </c>
       <c r="K45" s="4">
         <f>IF(I45=0,0,J45/I45)</f>
@@ -3763,7 +3766,7 @@
         <v>9475.405513778041</v>
       </c>
       <c r="M45" s="3">
-        <v>2.647848884297535</v>
+        <v>12.91396182483621</v>
       </c>
       <c r="N45" s="4">
         <f>IF(L45=0,0,M45/L45)</f>
@@ -3773,7 +3776,7 @@
         <v>285.742923347472</v>
       </c>
       <c r="P45" s="3">
-        <v>0.7667368651648867</v>
+        <v>6.662558508813381</v>
       </c>
       <c r="Q45" s="4">
         <f>IF(O45=0,0,P45/O45)</f>
@@ -3783,17 +3786,17 @@
         <v>9178.019131321482</v>
       </c>
       <c r="T45" s="3">
-        <v>1571.759344532979</v>
+        <v>3280.333027549058</v>
       </c>
       <c r="U45" s="4">
         <f>IF(S45=0,0,T45/S45)</f>
         <v>0</v>
       </c>
       <c r="V45" s="3">
-        <v>20059051.99524085</v>
+        <v>19850211.7121278</v>
       </c>
       <c r="W45" s="3">
-        <v>259185.2599577568</v>
+        <v>1545620.805538651</v>
       </c>
       <c r="X45" s="4">
         <f>IF(V45=0,0,W45/V45)</f>
@@ -3803,7 +3806,7 @@
         <v>1405792.016991551</v>
       </c>
       <c r="Z45" s="3">
-        <v>5319.448695129715</v>
+        <v>34472.30498424848</v>
       </c>
       <c r="AA45" s="4">
         <f>IF(Y45=0,0,Z45/Y45)</f>
@@ -3813,7 +3816,7 @@
         <v>106730.9429757299</v>
       </c>
       <c r="AC45" s="3">
-        <v>29.32616354089987</v>
+        <v>143.3723550887371</v>
       </c>
       <c r="AD45" s="4">
         <f>IF(AB45=0,0,AC45/AB45)</f>
@@ -3857,11 +3860,11 @@
         <f>I50+I51+I52+I53+I54</f>
         <v>0</v>
       </c>
-      <c r="J48" s="6">
+      <c r="J48" s="3">
         <f>J50+J51+J52+J53+J54</f>
         <v>0</v>
       </c>
-      <c r="K48" s="7">
+      <c r="K48" s="4">
         <f>IF(I48=0,0,J48/I48)</f>
         <v>0</v>
       </c>
@@ -3905,11 +3908,11 @@
         <f>V50+V51+V52+V53+V54</f>
         <v>0</v>
       </c>
-      <c r="W48" s="6">
+      <c r="W48" s="3">
         <f>W50+W51+W52+W53+W54</f>
         <v>0</v>
       </c>
-      <c r="X48" s="7">
+      <c r="X48" s="4">
         <f>IF(V48=0,0,W48/V48)</f>
         <v>0</v>
       </c>
@@ -3952,88 +3955,88 @@
         <v>0</v>
       </c>
       <c r="D50" s="3">
-        <f>J50+G50</f>
+        <f>G50</f>
         <v>0</v>
       </c>
       <c r="E50" s="3">
-        <f>M50+P50</f>
+        <f>J50+M50+P50</f>
         <v>0</v>
       </c>
       <c r="F50" s="3">
-        <v>155.3366697637048</v>
+        <v>412.7408750394843</v>
       </c>
       <c r="G50" s="3">
-        <v>51.92733117123122</v>
+        <v>23.42409718172002</v>
       </c>
       <c r="H50" s="4">
         <f>IF(F50=0,0,G50/F50)</f>
         <v>0</v>
       </c>
       <c r="I50" s="3">
-        <v>382.3073643284127</v>
-      </c>
-      <c r="J50" s="6">
-        <v>7.051351267046877</v>
-      </c>
-      <c r="K50" s="7">
+        <v>1026.204299813583</v>
+      </c>
+      <c r="J50" s="3">
+        <v>6.332670651874505</v>
+      </c>
+      <c r="K50" s="4">
         <f>IF(I50=0,0,J50/I50)</f>
         <v>0</v>
       </c>
       <c r="L50" s="3">
-        <v>0</v>
+        <v>15352.83741703859</v>
       </c>
       <c r="M50" s="3">
-        <v>0</v>
+        <v>0.5863035025261343</v>
       </c>
       <c r="N50" s="4">
         <f>IF(L50=0,0,M50/L50)</f>
         <v>0</v>
       </c>
       <c r="O50" s="3">
-        <v>0</v>
+        <v>503.5634310516943</v>
       </c>
       <c r="P50" s="3">
-        <v>0</v>
+        <v>0.7976752452995279</v>
       </c>
       <c r="Q50" s="4">
         <f>IF(O50=0,0,P50/O50)</f>
         <v>0</v>
       </c>
       <c r="S50" s="3">
-        <v>2198.402026122217</v>
+        <v>12734.95565684622</v>
       </c>
       <c r="T50" s="3">
-        <v>734.9014899804904</v>
+        <v>722.7412087119392</v>
       </c>
       <c r="U50" s="4">
         <f>IF(S50=0,0,T50/S50)</f>
         <v>0</v>
       </c>
       <c r="V50" s="3">
-        <v>9070418.669545408</v>
-      </c>
-      <c r="W50" s="6">
-        <v>167025.0117590204</v>
-      </c>
-      <c r="X50" s="7">
+        <v>25286285.18025935</v>
+      </c>
+      <c r="W50" s="3">
+        <v>124252.6863578595</v>
+      </c>
+      <c r="X50" s="4">
         <f>IF(V50=0,0,W50/V50)</f>
         <v>0</v>
       </c>
       <c r="Y50" s="3">
-        <v>0</v>
+        <v>2561085.175981381</v>
       </c>
       <c r="Z50" s="3">
-        <v>0</v>
+        <v>4301.107752270065</v>
       </c>
       <c r="AA50" s="4">
         <f>IF(Y50=0,0,Z50/Y50)</f>
         <v>0</v>
       </c>
       <c r="AB50" s="3">
-        <v>0</v>
+        <v>172903.801774421</v>
       </c>
       <c r="AC50" s="3">
-        <v>0</v>
+        <v>6.516925231320783</v>
       </c>
       <c r="AD50" s="4">
         <f>IF(AB50=0,0,AC50/AB50)</f>
@@ -4049,88 +4052,88 @@
         <v>0</v>
       </c>
       <c r="D51" s="3">
-        <f>J51+G51</f>
+        <f>G51</f>
         <v>0</v>
       </c>
       <c r="E51" s="3">
-        <f>M51+P51</f>
+        <f>J51+M51+P51</f>
         <v>0</v>
       </c>
       <c r="F51" s="3">
-        <v>147.7607036391234</v>
+        <v>422.0532339939548</v>
       </c>
       <c r="G51" s="3">
-        <v>52.79180338461813</v>
+        <v>32.39383284579316</v>
       </c>
       <c r="H51" s="4">
         <f>IF(F51=0,0,G51/F51)</f>
         <v>0</v>
       </c>
       <c r="I51" s="3">
-        <v>245.090682899663</v>
-      </c>
-      <c r="J51" s="6">
-        <v>6.16437173703697</v>
-      </c>
-      <c r="K51" s="7">
+        <v>971.1037573173985</v>
+      </c>
+      <c r="J51" s="3">
+        <v>8.271399086192949</v>
+      </c>
+      <c r="K51" s="4">
         <f>IF(I51=0,0,J51/I51)</f>
         <v>0</v>
       </c>
       <c r="L51" s="3">
-        <v>0</v>
+        <v>15897.14811387405</v>
       </c>
       <c r="M51" s="3">
-        <v>0</v>
+        <v>2.204028858903795</v>
       </c>
       <c r="N51" s="4">
         <f>IF(L51=0,0,M51/L51)</f>
         <v>0</v>
       </c>
       <c r="O51" s="3">
-        <v>0</v>
+        <v>427.6878840211459</v>
       </c>
       <c r="P51" s="3">
-        <v>0</v>
+        <v>0.7658804311889107</v>
       </c>
       <c r="Q51" s="4">
         <f>IF(O51=0,0,P51/O51)</f>
         <v>0</v>
       </c>
       <c r="S51" s="3">
-        <v>2091.183174942721</v>
+        <v>13022.2847912201</v>
       </c>
       <c r="T51" s="3">
-        <v>747.1359319079959</v>
+        <v>999.4988376351139</v>
       </c>
       <c r="U51" s="4">
         <f>IF(S51=0,0,T51/S51)</f>
         <v>0</v>
       </c>
       <c r="V51" s="3">
-        <v>7100767.677214347</v>
-      </c>
-      <c r="W51" s="6">
-        <v>194405.0614645267</v>
-      </c>
-      <c r="X51" s="7">
+        <v>24859901.01601297</v>
+      </c>
+      <c r="W51" s="3">
+        <v>171453.208100237</v>
+      </c>
+      <c r="X51" s="4">
         <f>IF(V51=0,0,W51/V51)</f>
         <v>0</v>
       </c>
       <c r="Y51" s="3">
-        <v>0</v>
+        <v>2216806.226901517</v>
       </c>
       <c r="Z51" s="3">
-        <v>0</v>
+        <v>5397.532345701009</v>
       </c>
       <c r="AA51" s="4">
         <f>IF(Y51=0,0,Z51/Y51)</f>
         <v>0</v>
       </c>
       <c r="AB51" s="3">
-        <v>0</v>
+        <v>179047.6330362356</v>
       </c>
       <c r="AC51" s="3">
-        <v>0</v>
+        <v>24.43846961739473</v>
       </c>
       <c r="AD51" s="4">
         <f>IF(AB51=0,0,AC51/AB51)</f>
@@ -4146,88 +4149,88 @@
         <v>0</v>
       </c>
       <c r="D52" s="3">
-        <f>J52+G52</f>
+        <f>G52</f>
         <v>0</v>
       </c>
       <c r="E52" s="3">
-        <f>M52+P52</f>
+        <f>J52+M52+P52</f>
         <v>0</v>
       </c>
       <c r="F52" s="3">
-        <v>134.4880808162132</v>
+        <v>382.0743136549376</v>
       </c>
       <c r="G52" s="3">
-        <v>52.90475626033849</v>
+        <v>45.49713331928587</v>
       </c>
       <c r="H52" s="4">
         <f>IF(F52=0,0,G52/F52)</f>
         <v>0</v>
       </c>
       <c r="I52" s="3">
-        <v>200.4130880433794</v>
-      </c>
-      <c r="J52" s="6">
-        <v>6.801510224238125</v>
-      </c>
-      <c r="K52" s="7">
+        <v>795.3294661601195</v>
+      </c>
+      <c r="J52" s="3">
+        <v>9.250773828173406</v>
+      </c>
+      <c r="K52" s="4">
         <f>IF(I52=0,0,J52/I52)</f>
         <v>0</v>
       </c>
       <c r="L52" s="3">
-        <v>0</v>
+        <v>14099.36149543928</v>
       </c>
       <c r="M52" s="3">
-        <v>0</v>
+        <v>2.494237892366946</v>
       </c>
       <c r="N52" s="4">
         <f>IF(L52=0,0,M52/L52)</f>
         <v>0</v>
       </c>
       <c r="O52" s="3">
-        <v>0</v>
+        <v>410.8336896551561</v>
       </c>
       <c r="P52" s="3">
-        <v>0</v>
+        <v>0.6260496127711959</v>
       </c>
       <c r="Q52" s="4">
         <f>IF(O52=0,0,P52/O52)</f>
         <v>0</v>
       </c>
       <c r="S52" s="3">
-        <v>1903.342396907326</v>
+        <v>11788.75109364953</v>
       </c>
       <c r="T52" s="3">
-        <v>748.7344973415004</v>
+        <v>1403.795965881249</v>
       </c>
       <c r="U52" s="4">
         <f>IF(S52=0,0,T52/S52)</f>
         <v>0</v>
       </c>
       <c r="V52" s="3">
-        <v>6292834.208210533</v>
-      </c>
-      <c r="W52" s="6">
-        <v>227563.8985600341</v>
-      </c>
-      <c r="X52" s="7">
+        <v>22936296.40445412</v>
+      </c>
+      <c r="W52" s="3">
+        <v>221609.0820698142</v>
+      </c>
+      <c r="X52" s="4">
         <f>IF(V52=0,0,W52/V52)</f>
         <v>0</v>
       </c>
       <c r="Y52" s="3">
-        <v>0</v>
+        <v>2114085.557833027</v>
       </c>
       <c r="Z52" s="3">
-        <v>0</v>
+        <v>6329.655924388207</v>
       </c>
       <c r="AA52" s="4">
         <f>IF(Y52=0,0,Z52/Y52)</f>
         <v>0</v>
       </c>
       <c r="AB52" s="3">
-        <v>0</v>
+        <v>158763.7032537926</v>
       </c>
       <c r="AC52" s="3">
-        <v>0</v>
+        <v>27.69693223305512</v>
       </c>
       <c r="AD52" s="4">
         <f>IF(AB52=0,0,AC52/AB52)</f>
@@ -4243,88 +4246,88 @@
         <v>0</v>
       </c>
       <c r="D53" s="3">
-        <f>J53+G53</f>
+        <f>G53</f>
         <v>0</v>
       </c>
       <c r="E53" s="3">
-        <f>M53+P53</f>
+        <f>J53+M53+P53</f>
         <v>0</v>
       </c>
       <c r="F53" s="3">
-        <v>118.5139506930648</v>
+        <v>338.6701578384149</v>
       </c>
       <c r="G53" s="3">
-        <v>23.699202858531</v>
+        <v>48.79942009843676</v>
       </c>
       <c r="H53" s="4">
         <f>IF(F53=0,0,G53/F53)</f>
         <v>0</v>
       </c>
       <c r="I53" s="3">
-        <v>193.9015574705648</v>
-      </c>
-      <c r="J53" s="6">
-        <v>2.625191036125732</v>
-      </c>
-      <c r="K53" s="7">
+        <v>717.4492241565633</v>
+      </c>
+      <c r="J53" s="3">
+        <v>9.464455356970662</v>
+      </c>
+      <c r="K53" s="4">
         <f>IF(I53=0,0,J53/I53)</f>
         <v>0</v>
       </c>
       <c r="L53" s="3">
-        <v>0</v>
+        <v>12459.036398116</v>
       </c>
       <c r="M53" s="3">
-        <v>0</v>
+        <v>2.502058168889955</v>
       </c>
       <c r="N53" s="4">
         <f>IF(L53=0,0,M53/L53)</f>
         <v>0</v>
       </c>
       <c r="O53" s="3">
-        <v>0</v>
+        <v>388.5202631627004</v>
       </c>
       <c r="P53" s="3">
-        <v>0</v>
+        <v>1.11741603567038</v>
       </c>
       <c r="Q53" s="4">
         <f>IF(O53=0,0,P53/O53)</f>
         <v>0</v>
       </c>
       <c r="S53" s="3">
-        <v>1677.268540156761</v>
+        <v>10449.53311676904</v>
       </c>
       <c r="T53" s="3">
-        <v>335.4029390544426</v>
+        <v>1505.686711968985</v>
       </c>
       <c r="U53" s="4">
         <f>IF(S53=0,0,T53/S53)</f>
         <v>0</v>
       </c>
       <c r="V53" s="3">
-        <v>6053045.584847068</v>
-      </c>
-      <c r="W53" s="6">
-        <v>93146.59233288839</v>
-      </c>
-      <c r="X53" s="7">
+        <v>21610890.70116934</v>
+      </c>
+      <c r="W53" s="3">
+        <v>242173.5070957839</v>
+      </c>
+      <c r="X53" s="4">
         <f>IF(V53=0,0,W53/V53)</f>
         <v>0</v>
       </c>
       <c r="Y53" s="3">
-        <v>0</v>
+        <v>1925897.452986733</v>
       </c>
       <c r="Z53" s="3">
-        <v>0</v>
+        <v>5809.098253916716</v>
       </c>
       <c r="AA53" s="4">
         <f>IF(Y53=0,0,Z53/Y53)</f>
         <v>0</v>
       </c>
       <c r="AB53" s="3">
-        <v>0</v>
+        <v>140314.2879239626</v>
       </c>
       <c r="AC53" s="3">
-        <v>0</v>
+        <v>27.69693223305512</v>
       </c>
       <c r="AD53" s="4">
         <f>IF(AB53=0,0,AC53/AB53)</f>
@@ -4340,88 +4343,88 @@
         <v>0</v>
       </c>
       <c r="D54" s="3">
-        <f>J54+G54</f>
+        <f>G54</f>
         <v>0</v>
       </c>
       <c r="E54" s="3">
-        <f>M54+P54</f>
+        <f>J54+M54+P54</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
-        <v>93.49564395607489</v>
+        <v>297.4602934996698</v>
       </c>
       <c r="G54" s="3">
-        <v>13.70139980823128</v>
+        <v>50.94083911201337</v>
       </c>
       <c r="H54" s="4">
         <f>IF(F54=0,0,G54/F54)</f>
         <v>0</v>
       </c>
       <c r="I54" s="3">
-        <v>136.6145524202559</v>
-      </c>
-      <c r="J54" s="6">
-        <v>1.998294804040721</v>
-      </c>
-      <c r="K54" s="7">
+        <v>610.1638407046684</v>
+      </c>
+      <c r="J54" s="3">
+        <v>9.162136177603854</v>
+      </c>
+      <c r="K54" s="4">
         <f>IF(I54=0,0,J54/I54)</f>
         <v>0</v>
       </c>
       <c r="L54" s="3">
-        <v>0</v>
+        <v>9475.405513778041</v>
       </c>
       <c r="M54" s="3">
-        <v>0</v>
+        <v>2.647848884297535</v>
       </c>
       <c r="N54" s="4">
         <f>IF(L54=0,0,M54/L54)</f>
         <v>0</v>
       </c>
       <c r="O54" s="3">
-        <v>0</v>
+        <v>285.742923347472</v>
       </c>
       <c r="P54" s="3">
-        <v>0</v>
+        <v>0.7667368651648867</v>
       </c>
       <c r="Q54" s="4">
         <f>IF(O54=0,0,P54/O54)</f>
         <v>0</v>
       </c>
       <c r="S54" s="3">
-        <v>1323.196985098892</v>
+        <v>9178.019131321482</v>
       </c>
       <c r="T54" s="3">
-        <v>193.909043788218</v>
+        <v>1571.759344532979</v>
       </c>
       <c r="U54" s="4">
         <f>IF(S54=0,0,T54/S54)</f>
         <v>0</v>
       </c>
       <c r="V54" s="3">
-        <v>4890905.466101354</v>
-      </c>
-      <c r="W54" s="6">
-        <v>78240.83772586659</v>
-      </c>
-      <c r="X54" s="7">
+        <v>20059051.99524085</v>
+      </c>
+      <c r="W54" s="3">
+        <v>259185.2599577568</v>
+      </c>
+      <c r="X54" s="4">
         <f>IF(V54=0,0,W54/V54)</f>
         <v>0</v>
       </c>
       <c r="Y54" s="3">
-        <v>0</v>
+        <v>1405792.016991551</v>
       </c>
       <c r="Z54" s="3">
-        <v>0</v>
+        <v>5319.448695129715</v>
       </c>
       <c r="AA54" s="4">
         <f>IF(Y54=0,0,Z54/Y54)</f>
         <v>0</v>
       </c>
       <c r="AB54" s="3">
-        <v>0</v>
+        <v>106730.9429757299</v>
       </c>
       <c r="AC54" s="3">
-        <v>0</v>
+        <v>29.32616354089987</v>
       </c>
       <c r="AD54" s="4">
         <f>IF(AB54=0,0,AC54/AB54)</f>
@@ -4560,7 +4563,7 @@
         <v>0</v>
       </c>
       <c r="D59" s="3">
-        <f>J59+G59</f>
+        <f>G59+J59</f>
         <v>0</v>
       </c>
       <c r="E59" s="3">
@@ -4571,7 +4574,7 @@
         <v>155.3366697637048</v>
       </c>
       <c r="G59" s="3">
-        <v>98.78915154595843</v>
+        <v>51.92733117123122</v>
       </c>
       <c r="H59" s="4">
         <f>IF(F59=0,0,G59/F59)</f>
@@ -4581,7 +4584,7 @@
         <v>382.3073643284127</v>
       </c>
       <c r="J59" s="6">
-        <v>25.04314403465664</v>
+        <v>7.051351267046877</v>
       </c>
       <c r="K59" s="7">
         <f>IF(I59=0,0,J59/I59)</f>
@@ -4611,7 +4614,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T59" s="3">
-        <v>1398.113344697664</v>
+        <v>734.9014899804904</v>
       </c>
       <c r="U59" s="4">
         <f>IF(S59=0,0,T59/S59)</f>
@@ -4621,7 +4624,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W59" s="6">
-        <v>624818.6004041024</v>
+        <v>167025.0117590204</v>
       </c>
       <c r="X59" s="7">
         <f>IF(V59=0,0,W59/V59)</f>
@@ -4657,7 +4660,7 @@
         <v>0</v>
       </c>
       <c r="D60" s="3">
-        <f>J60+G60</f>
+        <f>G60+J60</f>
         <v>0</v>
       </c>
       <c r="E60" s="3">
@@ -4668,7 +4671,7 @@
         <v>147.7607036391234</v>
       </c>
       <c r="G60" s="3">
-        <v>97.13343978236543</v>
+        <v>52.79180338461813</v>
       </c>
       <c r="H60" s="4">
         <f>IF(F60=0,0,G60/F60)</f>
@@ -4678,7 +4681,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J60" s="6">
-        <v>20.88002309512856</v>
+        <v>6.16437173703697</v>
       </c>
       <c r="K60" s="7">
         <f>IF(I60=0,0,J60/I60)</f>
@@ -4708,7 +4711,7 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T60" s="3">
-        <v>1374.680886017467</v>
+        <v>747.1359319079959</v>
       </c>
       <c r="U60" s="4">
         <f>IF(S60=0,0,T60/S60)</f>
@@ -4718,7 +4721,7 @@
         <v>7100767.677214347</v>
       </c>
       <c r="W60" s="6">
-        <v>693698.8487645769</v>
+        <v>194405.0614645267</v>
       </c>
       <c r="X60" s="7">
         <f>IF(V60=0,0,W60/V60)</f>
@@ -4754,7 +4757,7 @@
         <v>0</v>
       </c>
       <c r="D61" s="3">
-        <f>J61+G61</f>
+        <f>G61+J61</f>
         <v>0</v>
       </c>
       <c r="E61" s="3">
@@ -4765,7 +4768,7 @@
         <v>134.4880808162132</v>
       </c>
       <c r="G61" s="3">
-        <v>92.60233179008993</v>
+        <v>52.90475626033849</v>
       </c>
       <c r="H61" s="4">
         <f>IF(F61=0,0,G61/F61)</f>
@@ -4775,7 +4778,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J61" s="6">
-        <v>22.29461296479261</v>
+        <v>6.801510224238125</v>
       </c>
       <c r="K61" s="7">
         <f>IF(I61=0,0,J61/I61)</f>
@@ -4805,7 +4808,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T61" s="3">
-        <v>1310.554385778021</v>
+        <v>748.7344973415004</v>
       </c>
       <c r="U61" s="4">
         <f>IF(S61=0,0,T61/S61)</f>
@@ -4815,7 +4818,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W61" s="6">
-        <v>788440.6003954103</v>
+        <v>227563.8985600341</v>
       </c>
       <c r="X61" s="7">
         <f>IF(V61=0,0,W61/V61)</f>
@@ -4851,7 +4854,7 @@
         <v>0</v>
       </c>
       <c r="D62" s="3">
-        <f>J62+G62</f>
+        <f>G62+J62</f>
         <v>0</v>
       </c>
       <c r="E62" s="3">
@@ -4862,7 +4865,7 @@
         <v>118.5139506930648</v>
       </c>
       <c r="G62" s="3">
-        <v>56.58851159007293</v>
+        <v>23.699202858531</v>
       </c>
       <c r="H62" s="4">
         <f>IF(F62=0,0,G62/F62)</f>
@@ -4872,7 +4875,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J62" s="6">
-        <v>9.68772199998633</v>
+        <v>2.625191036125732</v>
       </c>
       <c r="K62" s="7">
         <f>IF(I62=0,0,J62/I62)</f>
@@ -4902,7 +4905,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T62" s="3">
-        <v>800.868840075549</v>
+        <v>335.4029390544426</v>
       </c>
       <c r="U62" s="4">
         <f>IF(S62=0,0,T62/S62)</f>
@@ -4912,7 +4915,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W62" s="6">
-        <v>352143.6781484308</v>
+        <v>93146.59233288839</v>
       </c>
       <c r="X62" s="7">
         <f>IF(V62=0,0,W62/V62)</f>
@@ -4948,7 +4951,7 @@
         <v>0</v>
       </c>
       <c r="D63" s="3">
-        <f>J63+G63</f>
+        <f>G63+J63</f>
         <v>0</v>
       </c>
       <c r="E63" s="3">
@@ -4959,7 +4962,7 @@
         <v>93.49564395607489</v>
       </c>
       <c r="G63" s="3">
-        <v>36.54054007239058</v>
+        <v>13.70139980823128</v>
       </c>
       <c r="H63" s="4">
         <f>IF(F63=0,0,G63/F63)</f>
@@ -4969,7 +4972,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J63" s="6">
-        <v>7.506574384869266</v>
+        <v>1.998294804040721</v>
       </c>
       <c r="K63" s="7">
         <f>IF(I63=0,0,J63/I63)</f>
@@ -4999,7 +5002,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T63" s="3">
-        <v>517.1399480427974</v>
+        <v>193.909043788218</v>
       </c>
       <c r="U63" s="4">
         <f>IF(S63=0,0,T63/S63)</f>
@@ -5009,7 +5012,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W63" s="6">
-        <v>298724.0740778223</v>
+        <v>78240.83772586659</v>
       </c>
       <c r="X63" s="7">
         <f>IF(V63=0,0,W63/V63)</f>
@@ -5168,7 +5171,7 @@
         <v>0</v>
       </c>
       <c r="D68" s="3">
-        <f>J68+G68</f>
+        <f>G68+J68</f>
         <v>0</v>
       </c>
       <c r="E68" s="3">
@@ -5179,7 +5182,7 @@
         <v>155.3366697637048</v>
       </c>
       <c r="G68" s="3">
-        <v>94.65713618175391</v>
+        <v>98.78915154595843</v>
       </c>
       <c r="H68" s="4">
         <f>IF(F68=0,0,G68/F68)</f>
@@ -5189,7 +5192,7 @@
         <v>382.3073643284127</v>
       </c>
       <c r="J68" s="6">
-        <v>22.4094333642202</v>
+        <v>25.04314403465664</v>
       </c>
       <c r="K68" s="7">
         <f>IF(I68=0,0,J68/I68)</f>
@@ -5219,7 +5222,7 @@
         <v>2198.402026122217</v>
       </c>
       <c r="T68" s="3">
-        <v>1339.635002381882</v>
+        <v>1398.113344697664</v>
       </c>
       <c r="U68" s="4">
         <f>IF(S68=0,0,T68/S68)</f>
@@ -5229,7 +5232,7 @@
         <v>9070418.669545408</v>
       </c>
       <c r="W68" s="6">
-        <v>554700.6611577384</v>
+        <v>624818.6004041024</v>
       </c>
       <c r="X68" s="7">
         <f>IF(V68=0,0,W68/V68)</f>
@@ -5265,7 +5268,7 @@
         <v>0</v>
       </c>
       <c r="D69" s="3">
-        <f>J69+G69</f>
+        <f>G69+J69</f>
         <v>0</v>
       </c>
       <c r="E69" s="3">
@@ -5276,7 +5279,7 @@
         <v>147.7607036391234</v>
       </c>
       <c r="G69" s="3">
-        <v>93.32656566805846</v>
+        <v>97.13343978236543</v>
       </c>
       <c r="H69" s="4">
         <f>IF(F69=0,0,G69/F69)</f>
@@ -5286,7 +5289,7 @@
         <v>245.090682899663</v>
       </c>
       <c r="J69" s="6">
-        <v>18.8267058367451</v>
+        <v>20.88002309512856</v>
       </c>
       <c r="K69" s="7">
         <f>IF(I69=0,0,J69/I69)</f>
@@ -5316,7 +5319,7 @@
         <v>2091.183174942721</v>
       </c>
       <c r="T69" s="3">
-        <v>1320.804104837496</v>
+        <v>1374.680886017467</v>
       </c>
       <c r="U69" s="4">
         <f>IF(S69=0,0,T69/S69)</f>
@@ -5326,7 +5329,7 @@
         <v>7100767.677214347</v>
       </c>
       <c r="W69" s="6">
-        <v>620735.8681268226</v>
+        <v>693698.8487645769</v>
       </c>
       <c r="X69" s="7">
         <f>IF(V69=0,0,W69/V69)</f>
@@ -5362,7 +5365,7 @@
         <v>0</v>
       </c>
       <c r="D70" s="3">
-        <f>J70+G70</f>
+        <f>G70+J70</f>
         <v>0</v>
       </c>
       <c r="E70" s="3">
@@ -5373,7 +5376,7 @@
         <v>134.4880808162132</v>
       </c>
       <c r="G70" s="3">
-        <v>89.3261468773603</v>
+        <v>92.60233179008993</v>
       </c>
       <c r="H70" s="4">
         <f>IF(F70=0,0,G70/F70)</f>
@@ -5383,7 +5386,7 @@
         <v>200.4130880433794</v>
       </c>
       <c r="J70" s="6">
-        <v>20.20687125075571</v>
+        <v>22.29461296479261</v>
       </c>
       <c r="K70" s="7">
         <f>IF(I70=0,0,J70/I70)</f>
@@ -5413,7 +5416,7 @@
         <v>1903.342396907326</v>
       </c>
       <c r="T70" s="3">
-        <v>1264.188182865007</v>
+        <v>1310.554385778021</v>
       </c>
       <c r="U70" s="4">
         <f>IF(S70=0,0,T70/S70)</f>
@@ -5423,7 +5426,7 @@
         <v>6292834.208210533</v>
       </c>
       <c r="W70" s="6">
-        <v>709040.6150101619</v>
+        <v>788440.6003954103</v>
       </c>
       <c r="X70" s="7">
         <f>IF(V70=0,0,W70/V70)</f>
@@ -5459,7 +5462,7 @@
         <v>0</v>
       </c>
       <c r="D71" s="3">
-        <f>J71+G71</f>
+        <f>G71+J71</f>
         <v>0</v>
       </c>
       <c r="E71" s="3">
@@ -5470,7 +5473,7 @@
         <v>118.5139506930648</v>
       </c>
       <c r="G71" s="3">
-        <v>53.09835934079247</v>
+        <v>56.58851159007293</v>
       </c>
       <c r="H71" s="4">
         <f>IF(F71=0,0,G71/F71)</f>
@@ -5480,7 +5483,7 @@
         <v>193.9015574705648</v>
       </c>
       <c r="J71" s="6">
-        <v>8.613532581916079</v>
+        <v>9.68772199998633</v>
       </c>
       <c r="K71" s="7">
         <f>IF(I71=0,0,J71/I71)</f>
@@ -5510,7 +5513,7 @@
         <v>1677.268540156761</v>
       </c>
       <c r="T71" s="3">
-        <v>751.4744646974439</v>
+        <v>800.868840075549</v>
       </c>
       <c r="U71" s="4">
         <f>IF(S71=0,0,T71/S71)</f>
@@ -5520,7 +5523,7 @@
         <v>6053045.584847068</v>
       </c>
       <c r="W71" s="6">
-        <v>311924.34926455</v>
+        <v>352143.6781484308</v>
       </c>
       <c r="X71" s="7">
         <f>IF(V71=0,0,W71/V71)</f>
@@ -5556,7 +5559,7 @@
         <v>0</v>
       </c>
       <c r="D72" s="3">
-        <f>J72+G72</f>
+        <f>G72+J72</f>
         <v>0</v>
       </c>
       <c r="E72" s="3">
@@ -5567,7 +5570,7 @@
         <v>93.49564395607489</v>
       </c>
       <c r="G72" s="3">
-        <v>33.88385898245032</v>
+        <v>36.54054007239058</v>
       </c>
       <c r="H72" s="4">
         <f>IF(F72=0,0,G72/F72)</f>
@@ -5577,7 +5580,7 @@
         <v>136.6145524202559</v>
       </c>
       <c r="J72" s="6">
-        <v>6.654744068362823</v>
+        <v>7.506574384869266</v>
       </c>
       <c r="K72" s="7">
         <f>IF(I72=0,0,J72/I72)</f>
@@ -5607,7 +5610,7 @@
         <v>1323.196985098892</v>
       </c>
       <c r="T72" s="3">
-        <v>479.5412722132613</v>
+        <v>517.1399480427974</v>
       </c>
       <c r="U72" s="4">
         <f>IF(S72=0,0,T72/S72)</f>
@@ -5617,7 +5620,7 @@
         <v>4890905.466101354</v>
       </c>
       <c r="W72" s="6">
-        <v>264152.6459177388</v>
+        <v>298724.0740778223</v>
       </c>
       <c r="X72" s="7">
         <f>IF(V72=0,0,W72/V72)</f>
@@ -5641,6 +5644,614 @@
       </c>
       <c r="AD72" s="4">
         <f>IF(AB72=0,0,AC72/AB72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:30">
+      <c r="A74" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="75" spans="1:30">
+      <c r="B75" t="s">
+        <v>28</v>
+      </c>
+      <c r="C75" s="3">
+        <f>C77+C78+C79+C80+C81</f>
+        <v>0</v>
+      </c>
+      <c r="D75" s="3">
+        <f>D77+D78+D79+D80+D81</f>
+        <v>0</v>
+      </c>
+      <c r="E75" s="3">
+        <f>E77+E78+E79+E80+E81</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="3">
+        <f>F77+F78+F79+F80+F81</f>
+        <v>0</v>
+      </c>
+      <c r="G75" s="3">
+        <f>G77+G78+G79+G80+G81</f>
+        <v>0</v>
+      </c>
+      <c r="H75" s="4">
+        <f>IF(F75=0,0,G75/F75)</f>
+        <v>0</v>
+      </c>
+      <c r="I75" s="3">
+        <f>I77+I78+I79+I80+I81</f>
+        <v>0</v>
+      </c>
+      <c r="J75" s="6">
+        <f>J77+J78+J79+J80+J81</f>
+        <v>0</v>
+      </c>
+      <c r="K75" s="7">
+        <f>IF(I75=0,0,J75/I75)</f>
+        <v>0</v>
+      </c>
+      <c r="L75" s="3">
+        <f>L77+L78+L79+L80+L81</f>
+        <v>0</v>
+      </c>
+      <c r="M75" s="3">
+        <f>M77+M78+M79+M80+M81</f>
+        <v>0</v>
+      </c>
+      <c r="N75" s="4">
+        <f>IF(L75=0,0,M75/L75)</f>
+        <v>0</v>
+      </c>
+      <c r="O75" s="3">
+        <f>O77+O78+O79+O80+O81</f>
+        <v>0</v>
+      </c>
+      <c r="P75" s="3">
+        <f>P77+P78+P79+P80+P81</f>
+        <v>0</v>
+      </c>
+      <c r="Q75" s="4">
+        <f>IF(O75=0,0,P75/O75)</f>
+        <v>0</v>
+      </c>
+      <c r="S75" s="3">
+        <f>S77+S78+S79+S80+S81</f>
+        <v>0</v>
+      </c>
+      <c r="T75" s="3">
+        <f>T77+T78+T79+T80+T81</f>
+        <v>0</v>
+      </c>
+      <c r="U75" s="4">
+        <f>IF(S75=0,0,T75/S75)</f>
+        <v>0</v>
+      </c>
+      <c r="V75" s="3">
+        <f>V77+V78+V79+V80+V81</f>
+        <v>0</v>
+      </c>
+      <c r="W75" s="6">
+        <f>W77+W78+W79+W80+W81</f>
+        <v>0</v>
+      </c>
+      <c r="X75" s="7">
+        <f>IF(V75=0,0,W75/V75)</f>
+        <v>0</v>
+      </c>
+      <c r="Y75" s="3">
+        <f>Y77+Y78+Y79+Y80+Y81</f>
+        <v>0</v>
+      </c>
+      <c r="Z75" s="3">
+        <f>Z77+Z78+Z79+Z80+Z81</f>
+        <v>0</v>
+      </c>
+      <c r="AA75" s="4">
+        <f>IF(Y75=0,0,Z75/Y75)</f>
+        <v>0</v>
+      </c>
+      <c r="AB75" s="3">
+        <f>AB77+AB78+AB79+AB80+AB81</f>
+        <v>0</v>
+      </c>
+      <c r="AC75" s="3">
+        <f>AC77+AC78+AC79+AC80+AC81</f>
+        <v>0</v>
+      </c>
+      <c r="AD75" s="4">
+        <f>IF(AB75=0,0,AC75/AB75)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:30">
+      <c r="A76" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="77" spans="1:30">
+      <c r="B77" t="s">
+        <v>30</v>
+      </c>
+      <c r="C77" s="3">
+        <f>J77+M77+G77+P77</f>
+        <v>0</v>
+      </c>
+      <c r="D77" s="3">
+        <f>G77+J77</f>
+        <v>0</v>
+      </c>
+      <c r="E77" s="3">
+        <f>M77+P77</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="3">
+        <v>155.3366697637048</v>
+      </c>
+      <c r="G77" s="3">
+        <v>94.65713618175391</v>
+      </c>
+      <c r="H77" s="4">
+        <f>IF(F77=0,0,G77/F77)</f>
+        <v>0</v>
+      </c>
+      <c r="I77" s="3">
+        <v>382.3073643284127</v>
+      </c>
+      <c r="J77" s="6">
+        <v>22.4094333642202</v>
+      </c>
+      <c r="K77" s="7">
+        <f>IF(I77=0,0,J77/I77)</f>
+        <v>0</v>
+      </c>
+      <c r="L77" s="3">
+        <v>0</v>
+      </c>
+      <c r="M77" s="3">
+        <v>0</v>
+      </c>
+      <c r="N77" s="4">
+        <f>IF(L77=0,0,M77/L77)</f>
+        <v>0</v>
+      </c>
+      <c r="O77" s="3">
+        <v>0</v>
+      </c>
+      <c r="P77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="4">
+        <f>IF(O77=0,0,P77/O77)</f>
+        <v>0</v>
+      </c>
+      <c r="S77" s="3">
+        <v>2198.402026122217</v>
+      </c>
+      <c r="T77" s="3">
+        <v>1339.635002381882</v>
+      </c>
+      <c r="U77" s="4">
+        <f>IF(S77=0,0,T77/S77)</f>
+        <v>0</v>
+      </c>
+      <c r="V77" s="3">
+        <v>9070418.669545408</v>
+      </c>
+      <c r="W77" s="6">
+        <v>554700.6611577384</v>
+      </c>
+      <c r="X77" s="7">
+        <f>IF(V77=0,0,W77/V77)</f>
+        <v>0</v>
+      </c>
+      <c r="Y77" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="4">
+        <f>IF(Y77=0,0,Z77/Y77)</f>
+        <v>0</v>
+      </c>
+      <c r="AB77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD77" s="4">
+        <f>IF(AB77=0,0,AC77/AB77)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:30">
+      <c r="B78" t="s">
+        <v>31</v>
+      </c>
+      <c r="C78" s="3">
+        <f>J78+M78+G78+P78</f>
+        <v>0</v>
+      </c>
+      <c r="D78" s="3">
+        <f>G78+J78</f>
+        <v>0</v>
+      </c>
+      <c r="E78" s="3">
+        <f>M78+P78</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="3">
+        <v>147.7607036391234</v>
+      </c>
+      <c r="G78" s="3">
+        <v>93.32656566805846</v>
+      </c>
+      <c r="H78" s="4">
+        <f>IF(F78=0,0,G78/F78)</f>
+        <v>0</v>
+      </c>
+      <c r="I78" s="3">
+        <v>245.090682899663</v>
+      </c>
+      <c r="J78" s="6">
+        <v>18.8267058367451</v>
+      </c>
+      <c r="K78" s="7">
+        <f>IF(I78=0,0,J78/I78)</f>
+        <v>0</v>
+      </c>
+      <c r="L78" s="3">
+        <v>0</v>
+      </c>
+      <c r="M78" s="3">
+        <v>0</v>
+      </c>
+      <c r="N78" s="4">
+        <f>IF(L78=0,0,M78/L78)</f>
+        <v>0</v>
+      </c>
+      <c r="O78" s="3">
+        <v>0</v>
+      </c>
+      <c r="P78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="4">
+        <f>IF(O78=0,0,P78/O78)</f>
+        <v>0</v>
+      </c>
+      <c r="S78" s="3">
+        <v>2091.183174942721</v>
+      </c>
+      <c r="T78" s="3">
+        <v>1320.804104837496</v>
+      </c>
+      <c r="U78" s="4">
+        <f>IF(S78=0,0,T78/S78)</f>
+        <v>0</v>
+      </c>
+      <c r="V78" s="3">
+        <v>7100767.677214347</v>
+      </c>
+      <c r="W78" s="6">
+        <v>620735.8681268226</v>
+      </c>
+      <c r="X78" s="7">
+        <f>IF(V78=0,0,W78/V78)</f>
+        <v>0</v>
+      </c>
+      <c r="Y78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="4">
+        <f>IF(Y78=0,0,Z78/Y78)</f>
+        <v>0</v>
+      </c>
+      <c r="AB78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD78" s="4">
+        <f>IF(AB78=0,0,AC78/AB78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:30">
+      <c r="B79" t="s">
+        <v>32</v>
+      </c>
+      <c r="C79" s="3">
+        <f>J79+M79+G79+P79</f>
+        <v>0</v>
+      </c>
+      <c r="D79" s="3">
+        <f>G79+J79</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="3">
+        <f>M79+P79</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="3">
+        <v>134.4880808162132</v>
+      </c>
+      <c r="G79" s="3">
+        <v>89.3261468773603</v>
+      </c>
+      <c r="H79" s="4">
+        <f>IF(F79=0,0,G79/F79)</f>
+        <v>0</v>
+      </c>
+      <c r="I79" s="3">
+        <v>200.4130880433794</v>
+      </c>
+      <c r="J79" s="6">
+        <v>20.20687125075571</v>
+      </c>
+      <c r="K79" s="7">
+        <f>IF(I79=0,0,J79/I79)</f>
+        <v>0</v>
+      </c>
+      <c r="L79" s="3">
+        <v>0</v>
+      </c>
+      <c r="M79" s="3">
+        <v>0</v>
+      </c>
+      <c r="N79" s="4">
+        <f>IF(L79=0,0,M79/L79)</f>
+        <v>0</v>
+      </c>
+      <c r="O79" s="3">
+        <v>0</v>
+      </c>
+      <c r="P79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="4">
+        <f>IF(O79=0,0,P79/O79)</f>
+        <v>0</v>
+      </c>
+      <c r="S79" s="3">
+        <v>1903.342396907326</v>
+      </c>
+      <c r="T79" s="3">
+        <v>1264.188182865007</v>
+      </c>
+      <c r="U79" s="4">
+        <f>IF(S79=0,0,T79/S79)</f>
+        <v>0</v>
+      </c>
+      <c r="V79" s="3">
+        <v>6292834.208210533</v>
+      </c>
+      <c r="W79" s="6">
+        <v>709040.6150101619</v>
+      </c>
+      <c r="X79" s="7">
+        <f>IF(V79=0,0,W79/V79)</f>
+        <v>0</v>
+      </c>
+      <c r="Y79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="4">
+        <f>IF(Y79=0,0,Z79/Y79)</f>
+        <v>0</v>
+      </c>
+      <c r="AB79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD79" s="4">
+        <f>IF(AB79=0,0,AC79/AB79)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:30">
+      <c r="B80" t="s">
+        <v>33</v>
+      </c>
+      <c r="C80" s="3">
+        <f>J80+M80+G80+P80</f>
+        <v>0</v>
+      </c>
+      <c r="D80" s="3">
+        <f>G80+J80</f>
+        <v>0</v>
+      </c>
+      <c r="E80" s="3">
+        <f>M80+P80</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="3">
+        <v>118.5139506930648</v>
+      </c>
+      <c r="G80" s="3">
+        <v>53.09835934079247</v>
+      </c>
+      <c r="H80" s="4">
+        <f>IF(F80=0,0,G80/F80)</f>
+        <v>0</v>
+      </c>
+      <c r="I80" s="3">
+        <v>193.9015574705648</v>
+      </c>
+      <c r="J80" s="6">
+        <v>8.613532581916079</v>
+      </c>
+      <c r="K80" s="7">
+        <f>IF(I80=0,0,J80/I80)</f>
+        <v>0</v>
+      </c>
+      <c r="L80" s="3">
+        <v>0</v>
+      </c>
+      <c r="M80" s="3">
+        <v>0</v>
+      </c>
+      <c r="N80" s="4">
+        <f>IF(L80=0,0,M80/L80)</f>
+        <v>0</v>
+      </c>
+      <c r="O80" s="3">
+        <v>0</v>
+      </c>
+      <c r="P80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="4">
+        <f>IF(O80=0,0,P80/O80)</f>
+        <v>0</v>
+      </c>
+      <c r="S80" s="3">
+        <v>1677.268540156761</v>
+      </c>
+      <c r="T80" s="3">
+        <v>751.4744646974439</v>
+      </c>
+      <c r="U80" s="4">
+        <f>IF(S80=0,0,T80/S80)</f>
+        <v>0</v>
+      </c>
+      <c r="V80" s="3">
+        <v>6053045.584847068</v>
+      </c>
+      <c r="W80" s="6">
+        <v>311924.34926455</v>
+      </c>
+      <c r="X80" s="7">
+        <f>IF(V80=0,0,W80/V80)</f>
+        <v>0</v>
+      </c>
+      <c r="Y80" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="4">
+        <f>IF(Y80=0,0,Z80/Y80)</f>
+        <v>0</v>
+      </c>
+      <c r="AB80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD80" s="4">
+        <f>IF(AB80=0,0,AC80/AB80)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="2:30">
+      <c r="B81" t="s">
+        <v>34</v>
+      </c>
+      <c r="C81" s="3">
+        <f>J81+M81+G81+P81</f>
+        <v>0</v>
+      </c>
+      <c r="D81" s="3">
+        <f>G81+J81</f>
+        <v>0</v>
+      </c>
+      <c r="E81" s="3">
+        <f>M81+P81</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="3">
+        <v>93.49564395607489</v>
+      </c>
+      <c r="G81" s="3">
+        <v>33.88385898245032</v>
+      </c>
+      <c r="H81" s="4">
+        <f>IF(F81=0,0,G81/F81)</f>
+        <v>0</v>
+      </c>
+      <c r="I81" s="3">
+        <v>136.6145524202559</v>
+      </c>
+      <c r="J81" s="6">
+        <v>6.654744068362823</v>
+      </c>
+      <c r="K81" s="7">
+        <f>IF(I81=0,0,J81/I81)</f>
+        <v>0</v>
+      </c>
+      <c r="L81" s="3">
+        <v>0</v>
+      </c>
+      <c r="M81" s="3">
+        <v>0</v>
+      </c>
+      <c r="N81" s="4">
+        <f>IF(L81=0,0,M81/L81)</f>
+        <v>0</v>
+      </c>
+      <c r="O81" s="3">
+        <v>0</v>
+      </c>
+      <c r="P81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q81" s="4">
+        <f>IF(O81=0,0,P81/O81)</f>
+        <v>0</v>
+      </c>
+      <c r="S81" s="3">
+        <v>1323.196985098892</v>
+      </c>
+      <c r="T81" s="3">
+        <v>479.5412722132613</v>
+      </c>
+      <c r="U81" s="4">
+        <f>IF(S81=0,0,T81/S81)</f>
+        <v>0</v>
+      </c>
+      <c r="V81" s="3">
+        <v>4890905.466101354</v>
+      </c>
+      <c r="W81" s="6">
+        <v>264152.6459177388</v>
+      </c>
+      <c r="X81" s="7">
+        <f>IF(V81=0,0,W81/V81)</f>
+        <v>0</v>
+      </c>
+      <c r="Y81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="4">
+        <f>IF(Y81=0,0,Z81/Y81)</f>
+        <v>0</v>
+      </c>
+      <c r="AB81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD81" s="4">
+        <f>IF(AB81=0,0,AC81/AB81)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>